<commit_message>
v2.22: cierre de caja con Id único (alta o actualización).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E246"/>
+  <dimension ref="A1:E248"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4593,9 +4593,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="247">
+      <c r="A247" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="B247" t="str">
+        <v>14:45</v>
+      </c>
+      <c r="C247" t="str">
+        <v>Cierre de caja: borrar legacy y upsert por Id</v>
+      </c>
+      <c r="D247" t="str">
+        <v>Se eliminaron 329 tesorerías cargadas con el Excel de cajas cerradas (sin Id) y 169 parejas de conciliación asociadas. El cierre nuevo (docs/Caja/cierre_CIERRE-…, columna Id) hace alta/actualización por origen_id cierre|{Id}; la columna Caja elige Galicia o Mercado Pago. Si ya había tesorería tesoreria_*.xlsx del mismo movimiento, se retira para no duplicar. sql/supabase_cb_borrar_tesoreria_cierre_legacy.sql y sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql.</v>
+      </c>
+      <c r="E247" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="B248" t="str">
+        <v>14:56</v>
+      </c>
+      <c r="C248" t="str">
+        <v>Despliegue v2.22 producción</v>
+      </c>
+      <c r="D248" t="str">
+        <v>Push a main y Vercel --prod: cierre de caja con Id único (alta o actualización); se eliminó la tesorería legacy de CIERRE sin Id. APP_VERSION 2.22.</v>
+      </c>
+      <c r="E248" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E246"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E248"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5085,7 +5119,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto; Ingreso→crédito y Egreso→débito; historial de caja ya cerrada. El archivo debe llamarse MP_… en la solapa Mercado Pago y Galicia_… en Banco Galicia (primera palabra antes del _). Filas Pendiente y totales del pie no se cargan. Tesorería no duplica si ya existe misma fecha, monto, descripción, categoría y cliente (aunque el Excel sea de otro formato). La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql y sql/supabase_conciliacion_bancaria_manual_grupo.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id cierre|{Id}) sin duplicar ni dejar datos viejos. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx no duplica si ya existe misma fecha, monto, descripción, categoría y cliente. Al subir un cierre con Id, se retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql y sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5232,7 +5266,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5954,9 +5988,20 @@
         <v>Despliegue v2.21: Conciliación Bancaria — extracto Galicia ya no incluye el saldo en el ID; un reexport del banco con saldo corrido no duplica movimientos (dedupe por fecha, importe y descripción). Se eliminaron 17 copias del último upload. Producción Vercel.</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>2.22</v>
+      </c>
+      <c r="B66" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Despliegue v2.22: Conciliación Bancaria — cierre de caja con Id único (cierre_CIERRE-…): alta o actualización por el mismo Id; la columna Caja elige Mercado Pago o Galicia. Se eliminó la tesorería legacy de cajas cerradas sin Id. sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C66"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.23: tesorería con Id actualiza categoría y cuenta.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E248"/>
+  <dimension ref="A1:E251"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4627,9 +4627,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="249">
+      <c r="A249" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="B249" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C249" t="str">
+        <v>Borrar tesorería anterior a septiembre 2026</v>
+      </c>
+      <c r="D249" t="str">
+        <v>Se eliminaron 361 movimientos de tesorería (Galicia 320, Mercado Pago 41) con fecha &lt; 01/09/2026, de ambas interfaces, y 240 parejas (confirmadas incluidas). El extracto banco no se tocó. Queda tesorería desde el 01/09/2026. sql/supabase_cb_borrar_tesoreria_antes_20260901.sql.</v>
+      </c>
+      <c r="E249" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="B250" t="str">
+        <v>17:25</v>
+      </c>
+      <c r="C250" t="str">
+        <v>Cierre MP: actualizar cuenta por Id</v>
+      </c>
+      <c r="D250" t="str">
+        <v>El 2.402,91 (PROYECTO ELECTRICO 10000053) no tomaba Imp. deb. y cred. bancario: el upload no usaba el Id y saltaba la fila como duplicado. Se actualizaron 25 filas de MP_CIERRE-310520260010_3.xlsx (Id + categoría/cuenta). El parser ahora usa Id en tesorería y cierre (origen_id id|{Id}), adopta la fila vieja y actualiza sin exigir misma cuenta. sql/supabase_cb_adoptar_id_tesoreria.sql.</v>
+      </c>
+      <c r="E250" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="B251" t="str">
+        <v>17:27</v>
+      </c>
+      <c r="C251" t="str">
+        <v>Despliegue v2.23 producción</v>
+      </c>
+      <c r="D251" t="str">
+        <v>Push a main y Vercel --prod: tesorería/cierre con Id actualiza categoría y cuenta sobre el mismo movimiento; cache-bust del JS. APP_VERSION 2.23.</v>
+      </c>
+      <c r="E251" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E248"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E251"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5119,7 +5170,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id cierre|{Id}) sin duplicar ni dejar datos viejos. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx no duplica si ya existe misma fecha, monto, descripción, categoría y cliente. Al subir un cierre con Id, se retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql y sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx no duplica si ya existe misma fecha, monto, descripción, categoría y cliente. Al subir un cierre con Id, se retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql y sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5266,7 +5317,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -5999,9 +6050,20 @@
         <v>Despliegue v2.22: Conciliación Bancaria — cierre de caja con Id único (cierre_CIERRE-…): alta o actualización por el mismo Id; la columna Caja elige Mercado Pago o Galicia. Se eliminó la tesorería legacy de cajas cerradas sin Id. sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2.23</v>
+      </c>
+      <c r="B67" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Despliegue v2.23: Conciliación Bancaria — el Id de tesorería/cierre actualiza categoría y cuenta en el mismo movimiento (no lo salta como duplicado). Cache-bust del JS de conciliación. sql/supabase_cb_adoptar_id_tesoreria.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C67"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.24: categoría y cuenta contable en tesorería (todas las tablas).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E251"/>
+  <dimension ref="A1:E253"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4678,9 +4678,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="B252" t="str">
+        <v>21:05</v>
+      </c>
+      <c r="C252" t="str">
+        <v>Categoría y cuenta en tesorería (todas las tablas)</v>
+      </c>
+      <c r="D252" t="str">
+        <v>Conciliación Bancaria: columnas Categoría y Cuenta contable también en Solo sistema y en Conciliación manual (lista de tesorería). Sugeridos/Confirmados ya las tenían. El Excel de Solo sistema las exporta. Encabezados ordenables y sticky.</v>
+      </c>
+      <c r="E252" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="B253" t="str">
+        <v>21:07</v>
+      </c>
+      <c r="C253" t="str">
+        <v>Despliegue v2.24 producción</v>
+      </c>
+      <c r="D253" t="str">
+        <v>Push a main y Vercel --prod: Categoría y Cuenta contable en Solo sistema y Conciliación manual. APP_VERSION 2.24.</v>
+      </c>
+      <c r="E253" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E251"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E253"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5170,7 +5204,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx no duplica si ya existe misma fecha, monto, descripción, categoría y cliente. Al subir un cierre con Id, se retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos y Confirmados, entre Sistema e Importe aparecen Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql y sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx no duplica si ya existe misma fecha, monto, descripción, categoría y cliente. Al subir un cierre con Id, se retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql y sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5317,7 +5351,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6061,9 +6095,20 @@
         <v>Despliegue v2.23: Conciliación Bancaria — el Id de tesorería/cierre actualiza categoría y cuenta en el mismo movimiento (no lo salta como duplicado). Cache-bust del JS de conciliación. sql/supabase_cb_adoptar_id_tesoreria.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>2.24</v>
+      </c>
+      <c r="B68" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Despliegue v2.24: Conciliación Bancaria — columnas Categoría y Cuenta contable en Solo sistema y en Conciliación manual (tesorería), además de Sugeridos/Confirmados. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C68"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.25: tesorería abierta MP y Galicia con Id (alta o actualización).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E253"/>
+  <dimension ref="A1:E256"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4712,9 +4712,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B254" t="str">
+        <v>10:28</v>
+      </c>
+      <c r="C254" t="str">
+        <v>Tesorería abierta: Id único y borrar sin Id</v>
+      </c>
+      <c r="D254" t="str">
+        <v>La tesorería tesoreria_*.xlsx ahora trae columna Id (p. ej. tesoreria_mercadopago_2026-09-15). El upload usa origen_id id|{Id}: alta o actualización si cambió un dato; filas sin Id se omiten. Se eliminaron 318 tesorerías de esta interfaz cargadas sin Id (Galicia 151, Mercado Pago 167) y 303 parejas de conciliación. No se tocó extracto ni cierre de caja. sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql.</v>
+      </c>
+      <c r="E254" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B255" t="str">
+        <v>11:28</v>
+      </c>
+      <c r="C255" t="str">
+        <v>Tesorería Galicia con Id (misma interfaz)</v>
+      </c>
+      <c r="D255" t="str">
+        <v>tesoreria_transferencia_galicia_2026-09-15 trae las mismas columnas que MP (Tipo, Id, Fecha, Crédito, Débito). Mismo proceso: origen_id id|{Id}, alta o actualización, omitir filas sin Id. Las 151 tesorerías Galicia sin Id ya estaban borradas. La detección prioriza tesorería frente al extracto CC para no cargar el Excel de sistema como banco.</v>
+      </c>
+      <c r="E255" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B256" t="str">
+        <v>11:32</v>
+      </c>
+      <c r="C256" t="str">
+        <v>Despliegue v2.25 producción</v>
+      </c>
+      <c r="D256" t="str">
+        <v>Push a main y Vercel --prod: tesorería abierta (MP y Galicia) con Id único, alta o actualización; se eliminó la tesorería de esa interfaz cargada sin Id. APP_VERSION 2.25.</v>
+      </c>
+      <c r="E256" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E253"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E256"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5204,7 +5255,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx no duplica si ya existe misma fecha, monto, descripción, categoría y cliente. Al subir un cierre con Id, se retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (mismas columnas Tipo/Fecha/Crédito/Débito). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql y sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql y sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5351,7 +5402,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6106,9 +6157,20 @@
         <v>Despliegue v2.24: Conciliación Bancaria — columnas Categoría y Cuenta contable en Solo sistema y en Conciliación manual (tesorería), además de Sugeridos/Confirmados. Producción Vercel.</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>2.25</v>
+      </c>
+      <c r="B69" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Despliegue v2.25: Conciliación Bancaria — tesorería abierta tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id: alta o actualización por origen_id id|{Id}; filas sin Id no se cargan. Se eliminaron 318 tesorerías de esa interfaz sin Id y 303 parejas. Detección prioriza tesorería vs extracto Galicia. sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C69"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.26: sugerencias con tolerancia por monto y fecha cercana primero.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E256"/>
+  <dimension ref="A1:E258"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4763,9 +4763,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="257">
+      <c r="A257" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B257" t="str">
+        <v>14:20</v>
+      </c>
+      <c r="C257" t="str">
+        <v>Sugerencias: tolerancia por monto y fecha cercana primero</v>
+      </c>
+      <c r="D257" t="str">
+        <v>El match automático ya no usa ±$1 fijo: montos &lt; $100 toleran 1 centavo; luego $1 / $10 / $100 según el tamaño. Primero empareja fecha cercana (±14 días), después lo que resta con fecha lejana. Coincidencia exacta de monto y fecha: badge verde. Evita que un Imp. Ley 25413 de $4,80 se pare con uno de $5,08 de otro mes.</v>
+      </c>
+      <c r="E257" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B258" t="str">
+        <v>14:25</v>
+      </c>
+      <c r="C258" t="str">
+        <v>Despliegue v2.26 producción</v>
+      </c>
+      <c r="D258" t="str">
+        <v>Push a main y Vercel --prod: sugerencias con tolerancia según tamaño del importe, fecha cercana primero y badge verde si coinciden monto y fecha exactos. APP_VERSION 2.26.</v>
+      </c>
+      <c r="E258" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E256"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E258"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5255,7 +5289,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe (misma fecha, fecha cercana ±14 días o fecha lejana, tolerancia ±$1) y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql y sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql y sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5402,7 +5436,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6168,9 +6202,20 @@
         <v>Despliegue v2.25: Conciliación Bancaria — tesorería abierta tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id: alta o actualización por origen_id id|{Id}; filas sin Id no se cargan. Se eliminaron 318 tesorerías de esa interfaz sin Id y 303 parejas. Detección prioriza tesorería vs extracto Galicia. sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>2.26</v>
+      </c>
+      <c r="B70" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Despliegue v2.26: Conciliación Bancaria — tolerancia de match según tamaño del importe (centavos / $1 / $10 / $100); primero fecha cercana y después lejana; badge verde si coinciden monto y fecha exactos. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C70"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.27: tesorería abierta ausente a solapa A eliminar.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E258"/>
+  <dimension ref="A1:E260"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4797,9 +4797,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="259">
+      <c r="A259" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B259" t="str">
+        <v>17:10</v>
+      </c>
+      <c r="C259" t="str">
+        <v>Tesorería abierta ausente: solapa A eliminar</v>
+      </c>
+      <c r="D259" t="str">
+        <v>Al cargar tesoreria_*.xlsx con Id, los movimientos de tesorería abierta que ya estaban en base y no vienen en el archivo no se borran solos: pasan a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada). El cierre de caja no entra en esta lógica. sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql.</v>
+      </c>
+      <c r="E259" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B260" t="str">
+        <v>17:22</v>
+      </c>
+      <c r="C260" t="str">
+        <v>Despliegue v2.27 producción</v>
+      </c>
+      <c r="D260" t="str">
+        <v>Push a main y Vercel --prod: solapa A eliminar para tesorería abierta cuyo Id no vino en el último tesoreria_*.xlsx; baja confirmada (y pareja asociada). APP_VERSION 2.27.</v>
+      </c>
+      <c r="E260" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E258"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E260"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5289,7 +5323,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql y sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql y sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5436,7 +5470,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6213,9 +6247,20 @@
         <v>Despliegue v2.26: Conciliación Bancaria — tolerancia de match según tamaño del importe (centavos / $1 / $10 / $100); primero fecha cercana y después lejana; badge verde si coinciden monto y fecha exactos. Producción Vercel.</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>2.27</v>
+      </c>
+      <c r="B71" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Despliegue v2.27: Conciliación Bancaria — al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen van a la solapa A eliminar para confirmar la baja definitiva (Id, fecha, importe, categoría, cuenta, descripción). sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C71"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6417,7 +6462,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
Conciliación: filtros amplios en modal (extracto/sistema/categoría/cuenta).
El buscar sigue en la toolbar; conciliación manual replica el mismo esquema.
Bitácora actualizada y fallback local del helper de fechas LyP.

Co-authored-by: Lucas M Bustos <lucas.bustos.martin@gmail.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E260"/>
+  <dimension ref="A1:E261"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4831,9 +4831,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="261">
+      <c r="A261" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B261" t="str">
+        <v>17:49</v>
+      </c>
+      <c r="C261" t="str">
+        <v>Filtros amplios en modal (conciliación)</v>
+      </c>
+      <c r="D261" t="str">
+        <v>Conciliación Bancaria: los filtros pasan a un modal (mes extracto, mes sistema, categoría, cuenta contable) con opciones dinámicas y badge de cantidad activa. El buscar sigue amplio en la toolbar. Conciliación manual replica el mismo esquema (hereda filtros de la vista). Cache-bust JS/CSS ?v=2.28.</v>
+      </c>
+      <c r="E261" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E260"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E261"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5323,7 +5340,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros de mes y de concepto del extracto (además de buscar); el control se marca en naranja cuando hay filtro activo. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismos filtros Mes / Concepto del extracto / Buscar que la vista; si ya estaban activos, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql y sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql y sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql.</v>
       </c>
     </row>
     <row r="61">

</xml_diff>

<commit_message>
Conciliación manual: modal casi fullscreen para no aplastar la derecha.
Ancho/alto ~viewport, grilla 1fr/1.2fr con minmax(0) y pick tables más altas.

Co-authored-by: Lucas M Bustos <lucas.bustos.martin@gmail.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E261"/>
+  <dimension ref="A1:E262"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4848,9 +4848,26 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="262">
+      <c r="A262" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B262" t="str">
+        <v>18:11</v>
+      </c>
+      <c r="C262" t="str">
+        <v>Modal conciliación manual a casi fullscreen</v>
+      </c>
+      <c r="D262" t="str">
+        <v>El modal de Conciliación manual pasa a casi todo el viewport (márgenes mínimos) para que la columna derecha (tesorería) no quede aplastada. Grilla 1fr / 1.2fr con minmax(0), tablas pick más altas y sticky thead intacto. Cache-bust ?v=2.29.</v>
+      </c>
+      <c r="E262" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E261"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E262"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.28: filtros modal conciliación y modal manual fullscreen
Co-authored-by: Lucas M Bustos <lucas.bustos.martin@gmail.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E262"/>
+  <dimension ref="A1:E263"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4865,9 +4865,26 @@
         <v>Ajuste</v>
       </c>
     </row>
+    <row r="263">
+      <c r="A263" t="str">
+        <v>__HOY__</v>
+      </c>
+      <c r="B263" t="str">
+        <v>__AHORA__</v>
+      </c>
+      <c r="C263" t="str">
+        <v>Despliegue v2.28 producción</v>
+      </c>
+      <c r="D263" t="str">
+        <v>Push a main y Vercel --prod: filtros amplios en modal (mes extracto, mes sistema, categoría, cuenta contable) en Conciliación Bancaria y manual; modal manual casi fullscreen. APP_VERSION 2.28.</v>
+      </c>
+      <c r="E263" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E262"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E263"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5504,7 +5521,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6292,9 +6309,20 @@
         <v>Despliegue v2.27: Conciliación Bancaria — al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen van a la solapa A eliminar para confirmar la baja definitiva (Id, fecha, importe, categoría, cuenta, descripción). sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>2.28</v>
+      </c>
+      <c r="B72" t="str">
+        <v>__HOY__</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Despliegue v2.28: Conciliación Bancaria — filtros en modal (mes extracto, mes sistema, categoría, cuenta contable) con badge; buscar amplio en toolbar; mismo esquema en Conciliación manual. Modal manual casi fullscreen para columna tesorería. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C72"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix timeout al subir cierre de caja Galicia en conciliación
Fragmenta adopción/retiro/upsert en lotes de 100, optimiza RPCs SQL
(set-based + índice) y muestra mensaje claro en español ante statement timeout.

Co-authored-by: Lucas M Bustos <lucas.bustos.martin@gmail.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E263"/>
+  <dimension ref="A1:E264"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4882,9 +4882,26 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="B264" t="str">
+        <v>15:12</v>
+      </c>
+      <c r="C264" t="str">
+        <v>Fix timeout upload cierre Galicia</v>
+      </c>
+      <c r="D264" t="str">
+        <v>Al subir cierre de caja Galicia (~2.500 filas) fallaba con “canceling statement due to statement timeout”: cb_adoptar_id_tesoreria y cb_retirar_tesoreria_duplicada_por_cierre iban en un solo RPC fila a fila. Ahora el cliente fragmenta en lotes de 100, adopción set-based + índice hash fecha/monto, statement_timeout local 90s en guardar/adoptar/retirar/sugerencias, y mensaje de error en español (sin el string crudo de Postgres). SQL a correr en Supabase: sql/supabase_cb_upload_tesoreria_lotes.sql. Cache-bust JS ?v=2.30.</v>
+      </c>
+      <c r="E264" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E263"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E264"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5374,7 +5391,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql y sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento en lotes (evita timeout de Postgres en archivos grandes); si el servidor corta por tiempo, la UI muestra un mensaje claro en español. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql y sql/supabase_cb_upload_tesoreria_lotes.sql.</v>
       </c>
     </row>
     <row r="61">

</xml_diff>

<commit_message>
v2.29: conciliación sin timeout al recálcular sugerencias; regla de alinear main con lo publicado.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E263"/>
+  <dimension ref="A1:E266"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4882,9 +4882,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="B264" t="str">
+        <v>15:45</v>
+      </c>
+      <c r="C264" t="str">
+        <v>Upload conciliación: timeout al recálcular sugerencias</v>
+      </c>
+      <c r="D264" t="str">
+        <v>Sobre v2.28: el cierre de caja Galicia cortaba con “canceling statement due to statement timeout” en cb_reemplazar_sugerencias (trigger de solapamiento por fila, 8s). El chequeo quedó en un solo scan por statement (misma regla: un movimiento no puede estar en dos conciliaciones activas). RPC de carga con timeout 60s; adoptar/retirar en lotes de 250. sql/supabase_cb_upload_sin_timeout.sql.</v>
+      </c>
+      <c r="E264" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="B265" t="str">
+        <v>15:50</v>
+      </c>
+      <c r="C265" t="str">
+        <v>Regla: main local vs último publicado</v>
+      </c>
+      <c r="D265" t="str">
+        <v>Regla alwaysApply sync-main-publicado: antes de editar o desplegar, git fetch y alinear main local con origin/main / Vercel. Evita implementar sobre una versión vieja. Referenciada en bitacora-tareas y reglas-fornitalia.</v>
+      </c>
+      <c r="E265" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="B266" t="str">
+        <v>15:50</v>
+      </c>
+      <c r="C266" t="str">
+        <v>Despliegue v2.29 producción</v>
+      </c>
+      <c r="D266" t="str">
+        <v>Push a main y Vercel --prod: Conciliación Bancaria sin timeout al recálcular sugerencias (trigger statement-level; RPC 60s; lotes 250). Regla de alinear main local con lo publicado. APP_VERSION 2.29.</v>
+      </c>
+      <c r="E266" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E263"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E266"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5374,7 +5425,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql y sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql y sql/supabase_cb_upload_sin_timeout.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5521,7 +5572,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6320,9 +6371,20 @@
         <v>Despliegue v2.28: Conciliación Bancaria — filtros en modal (mes extracto, mes sistema, categoría, cuenta contable) con badge; buscar amplio en toolbar; mismo esquema en Conciliación manual. Modal manual casi fullscreen para columna tesorería. Producción Vercel.</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>2.29</v>
+      </c>
+      <c r="B73" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Despliegue v2.29: Conciliación Bancaria — upload de cierre/tesorería sin timeout al recálcular sugerencias (chequeo de solapamiento por statement; RPC 60s; lotes de 250). Regla sync-main-publicado. sql/supabase_cb_upload_sin_timeout.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C73"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.30: eliminar movimiento del extracto Galicia desde Solo banco.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E266"/>
+  <dimension ref="A1:E268"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4933,9 +4933,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="267">
+      <c r="A267" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="B267" t="str">
+        <v>16:58</v>
+      </c>
+      <c r="C267" t="str">
+        <v>Eliminar extracto Galicia en Solo banco</v>
+      </c>
+      <c r="D267" t="str">
+        <v>En Conciliación Bancaria, solapa Solo banco de Galicia: papelera junto al ojito para borrar un movimiento del extracto que no esté en sugerido/confirmado (permiso cargar). Confirmación previa. RPC cb_borrar_movimiento_banco_galicia. sql/supabase_cb_borrar_movimiento_banco_galicia.sql.</v>
+      </c>
+      <c r="E267" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="B268" t="str">
+        <v>17:35</v>
+      </c>
+      <c r="C268" t="str">
+        <v>Despliegue v2.30 producción</v>
+      </c>
+      <c r="D268" t="str">
+        <v>Push a main y Vercel --prod: Solo banco Galicia con papelera para eliminar un movimiento del extracto no conciliado. sql/supabase_cb_borrar_movimiento_banco_galicia.sql. APP_VERSION 2.30.</v>
+      </c>
+      <c r="E268" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E266"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E268"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5425,7 +5459,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql y sql/supabase_cb_upload_sin_timeout.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql y sql/supabase_cb_borrar_movimiento_banco_galicia.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5572,7 +5606,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6382,9 +6416,20 @@
         <v>Despliegue v2.29: Conciliación Bancaria — upload de cierre/tesorería sin timeout al recálcular sugerencias (chequeo de solapamiento por statement; RPC 60s; lotes de 250). Regla sync-main-publicado. sql/supabase_cb_upload_sin_timeout.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>2.30</v>
+      </c>
+      <c r="B74" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Despliegue v2.30: Conciliación Bancaria — Solo banco Galicia: papelera para eliminar un movimiento del extracto no conciliado. sql/supabase_cb_borrar_movimiento_banco_galicia.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C74"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6586,7 +6631,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.31: adjuntos en Gestión de Proyectos (proyecto, entregable y tarea).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E268"/>
+  <dimension ref="A1:E274"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -4967,9 +4967,111 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="269">
+      <c r="A269" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B269" t="str">
+        <v>09:29</v>
+      </c>
+      <c r="C269" t="str">
+        <v>Informe Word costeo importación agosto 2026</v>
+      </c>
+      <c r="D269" t="str">
+        <v>Análisis del Excel Fornitalia_costo_Agosto_importacion_2026.xlsx (landed cost por ítem vs NIC 2). Word en docs/ANALISIS_COSTEO_IMPORTACION_AGOSTO_2026.docx con veredicto, KPIs, fórmula, pileta B34 y costos unitarios. Regenerar: python3 scripts/generar-informe-costeo-importacion-agosto-2026.py.</v>
+      </c>
+      <c r="E269" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B270" t="str">
+        <v>09:49</v>
+      </c>
+      <c r="C270" t="str">
+        <v>Word costeo: tablas fuera de página</v>
+      </c>
+      <c r="D270" t="str">
+        <v>El .docx se veía en 2 páginas: anchos de tabla en EMU interpretados como twips. Se regeneró docs/ANALISIS_COSTEO_IMPORTACION_AGOSTO_2026.docx con anchos en dxa (~17 cm).</v>
+      </c>
+      <c r="E270" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B271" t="str">
+        <v>10:02</v>
+      </c>
+      <c r="C271" t="str">
+        <v>Word costeo: notas al pie FOB SIM landed</v>
+      </c>
+      <c r="D271" t="str">
+        <v>En docs/ANALISIS_COSTEO_IMPORTACION_AGOSTO_2026.docx, llamada a nota al pie en la primera aparición de SIM, FOB y landed, con definición en español al pie de página.</v>
+      </c>
+      <c r="E271" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B272" t="str">
+        <v>10:15</v>
+      </c>
+      <c r="C272" t="str">
+        <v>Word costeo: español AR y notas cortas</v>
+      </c>
+      <c r="D272" t="str">
+        <v>Se reemplazó pileta por gastos a prorratear; landed por costo de internación; stand/kit/invoice al español argentino. Notas al pie breves para SIM, TC, BNA, FOB, NCM, NIC 2, IIBB, ND, TRP, Ley 25.413 y cuenta y orden.</v>
+      </c>
+      <c r="E272" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B273" t="str">
+        <v>10:40</v>
+      </c>
+      <c r="C273" t="str">
+        <v>GP: archivos adjuntos en proyecto, entregable y tarea</v>
+      </c>
+      <c r="D273" t="str">
+        <v>Gestión de Proyectos: adjuntos por fecha + descripción + archivo (mismo esquema que horas) en proyecto, entregable y tarea. Bucket privado gp-archivos en Storage, URL firmada para ver. Solapa Archivos y hoja Excel. sql/supabase_gp_archivos.sql.</v>
+      </c>
+      <c r="E273" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B274" t="str">
+        <v>11:00</v>
+      </c>
+      <c r="C274" t="str">
+        <v>Despliegue v2.31 producción</v>
+      </c>
+      <c r="D274" t="str">
+        <v>Push a main y Vercel --prod: Gestión de Proyectos con archivos adjuntos (fecha, descripción, archivo) en proyecto, entregable y tarea. Bucket privado gp-archivos, URL firmada, solapa Archivos y hoja Excel. sql/supabase_gp_archivos.sql. APP_VERSION 2.31.</v>
+      </c>
+      <c r="E274" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E268"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E274"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5451,7 +5553,7 @@
         <v>Gestión de Proyectos</v>
       </c>
       <c r="B59" t="str">
-        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Solapa Horas cons.: conciliación diaria. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
+        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Archivos adjuntos por fecha (descripción + archivo en Storage gp-archivos) en proyecto, entregable y tarea; solapa Archivos y hoja Excel. Solapa Horas cons.: conciliación diaria. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
       </c>
     </row>
     <row r="60">
@@ -5606,7 +5708,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6427,9 +6529,20 @@
         <v>Despliegue v2.30: Conciliación Bancaria — Solo banco Galicia: papelera para eliminar un movimiento del extracto no conciliado. sql/supabase_cb_borrar_movimiento_banco_galicia.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>2.31</v>
+      </c>
+      <c r="B75" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Despliegue v2.31: Gestión de Proyectos — archivos adjuntos por fecha (descripción + archivo) en proyecto, entregable y tarea; Storage privado gp-archivos y URL firmada; solapa Archivos y hoja Excel. sql/supabase_gp_archivos.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C75"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6617,7 +6730,7 @@
         <v>Gestión de Proyectos</v>
       </c>
       <c r="B13" t="str">
-        <v>ABM de planes de trabajo (proyecto, entregables, tareas y dependencias), To-Do jerárquico, Gantt one-page con avance y SPI, horas consumidas por fecha con observaciones (proyecto, entregable y tarea), export Excel/PDF, permisos por perfil.</v>
+        <v>ABM de planes de trabajo (proyecto, entregables, tareas y dependencias), To-Do jerárquico, Gantt one-page con avance y SPI, horas consumidas y archivos adjuntos por fecha (proyecto, entregable y tarea; Storage gp-archivos), export Excel/PDF, permisos por perfil.</v>
       </c>
       <c r="C13">
         <v>40</v>

</xml_diff>

<commit_message>
v2.32: menú Cajas (físicas) Galicia-f y Morba-s/f (ARS).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E274"/>
+  <dimension ref="A1:E279"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5069,16 +5069,101 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="275">
+      <c r="A275" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B275" t="str">
+        <v>11:40</v>
+      </c>
+      <c r="C275" t="str">
+        <v>Menú Cajas (físicas): Galicia-f (ARS)</v>
+      </c>
+      <c r="D275" t="str">
+        <v>Nuevo menú para cajas no conciliables. Arranca Galicia-f (ARS) con tesoreria_efectivo_pesos_… y cierre_PES-… (misma lógica de Id que conciliación, sin extracto ni match). El saldo de cierre alimenta una línea más en Saldos extractos. sql/supabase_cajas_fisicas.sql.</v>
+      </c>
+      <c r="E275" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B276" t="str">
+        <v>11:45</v>
+      </c>
+      <c r="C276" t="str">
+        <v>Nombre de caja Galicia-f (ARS)</v>
+      </c>
+      <c r="D276" t="str">
+        <v>La caja física de efectivo pesos se muestra como Galicia-f (ARS) en Cajas (físicas) y en Saldos extractos (solapa, consolidado, gráfico y Excel).</v>
+      </c>
+      <c r="E276" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B277" t="str">
+        <v>11:50</v>
+      </c>
+      <c r="C277" t="str">
+        <v>Cajas físicas: sin Apertura de Caja</v>
+      </c>
+      <c r="D277" t="str">
+        <v>Cajas (físicas) ya no carga Apertura de Caja (igual que conciliación). Se borraron las aperturas ya subidas. El monto de apertura, si viene en el Excel, solo se usa para el corte de Saldos extractos. sql/supabase_cf_borrar_apertura_caja.sql.</v>
+      </c>
+      <c r="E277" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B278" t="str">
+        <v>11:55</v>
+      </c>
+      <c r="C278" t="str">
+        <v>Cajas físicas: orden y filtros</v>
+      </c>
+      <c r="D278" t="str">
+        <v>Cajas (físicas): encabezados ordenables (asc/desc) y filtros en modal como Conciliación Bancaria (mes, tipo, categoría, cuenta contable) con badge; el buscar sigue en la toolbar. El Excel respeta el listado filtrado.</v>
+      </c>
+      <c r="E278" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B279" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="C279" t="str">
+        <v>Caja física Morba-s/f (ARS)</v>
+      </c>
+      <c r="D279" t="str">
+        <v>Nueva solapa Morba-s/f (ARS) en Cajas (físicas) para tesoreria_transferencia_morba_… y cierre_MOR-… (canal morba_sf, no conciliable). El saldo alimenta Saldos extractos (solapa, consolidado, gráfico y Excel). Si el archivo se sube en Conciliación Bancaria, se rechaza y se indica Cajas (físicas). sql/supabase_cajas_fisicas_morba.sql.</v>
+      </c>
+      <c r="E279" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E274"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E279"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B67"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -5566,55 +5651,63 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Saldos extractos</v>
+        <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago, Banco Galicia y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia: PDF de resumen de cuenta (saldo inicial/cierre del período). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia + MP (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql y sql/supabase_saldos_extractos_mercadopago.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Galicia-f (ARS) (efectivo pesos: tesoreria_efectivo_pesos_… / cierre_PES-…) y Morba-s/f (ARS) (Transferencia Morba: tesoreria_transferencia_morba_… / cierre_MOR-…). Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. Apertura de Caja y filas Pendiente no se cargan (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Tesorería abierta: los Ids que ya no vienen van a A eliminar. Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql y sql/supabase_cf_borrar_apertura_caja.sql.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago, Banco Galicia, Galicia-f (ARS), Morba-s/f (ARS) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia: PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia-f (ARS) y Morba-s/f (ARS): saldos de cajas físicas que se actualizan desde el menú Cajas (físicas). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia + MP + Galicia-f (ARS) + Morba-s/f (ARS) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql y sql/supabase_cajas_fisicas_morba.sql.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B63" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B64" t="str">
-        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B65" t="str">
-        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
+        <v>Log de excluidos en upload</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
         <v>Análisis financiero extracto (PDF)</v>
       </c>
-      <c r="B66" t="str">
+      <c r="B67" t="str">
         <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B67"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5708,7 +5801,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6540,16 +6633,27 @@
         <v>Despliegue v2.31: Gestión de Proyectos — archivos adjuntos por fecha (descripción + archivo) en proyecto, entregable y tarea; Storage privado gp-archivos y URL firmada; solapa Archivos y hoja Excel. sql/supabase_gp_archivos.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>2.32</v>
+      </c>
+      <c r="B76" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Despliegue v2.32: menú Cajas (físicas) no conciliables — Galicia-f (ARS) (tesoreria_efectivo_pesos / cierre_PES) y Morba-s/f (ARS) (tesoreria_transferencia_morba / cierre_MOR); sin Apertura de Caja; orden y filtros; saldos en Saldos extractos (solapas y consolidado). sql/supabase_cajas_fisicas.sql y sql/supabase_cajas_fisicas_morba.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C76"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -6758,7 +6862,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (resumen PDF) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (resumen PDF), Galicia-f (ARS) y Morba-s/f (ARS) (cajas físicas desde Cajas) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>
@@ -6767,9 +6871,23 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Cajas (físicas)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Menú de cajas no conciliables. Galicia-f (ARS) (efectivo pesos) y Morba-s/f (ARS) (Transferencia Morba) con tesorería abierta y cierre de caja por Id, sin extracto ni match. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
+      </c>
+      <c r="C16">
+        <v>8</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6795,7 +6913,7 @@
         <v>Frontend</v>
       </c>
       <c r="B2" t="str">
-        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria y Saldos extractos en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.* y fornitalia-saldos-extractos.*). Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia con pdf.js en el navegador.</v>
+        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas) y Saldos extractos en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.* y fornitalia-saldos-extractos.*). Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia con pdf.js en el navegador.</v>
       </c>
     </row>
     <row r="3">
@@ -6803,7 +6921,7 @@
         <v>Datos</v>
       </c>
       <c r="B3" t="str">
-        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia, cb_movimiento, cb_match, eb_saldo_extracto. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
+        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia, cb_movimiento, cb_match, cf_movimiento, eb_saldo_extracto. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
v2.33: conciliación manual de dos movimientos del mismo extracto.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E281"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5154,9 +5154,43 @@
         <v>Implementacion</v>
       </c>
     </row>
+    <row r="280">
+      <c r="A280" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B280" t="str">
+        <v>16:45</v>
+      </c>
+      <c r="C280" t="str">
+        <v>Conciliación manual solo extracto</v>
+      </c>
+      <c r="D280" t="str">
+        <v>Conciliación manual admite dos o más movimientos del mismo extracto sin tesorería (crédito por transferencia errónea y débito de la devolución). Justificación obligatoria; van a Confirmados con badge solo extracto. sql/supabase_cb_confirmar_manual_solo_extracto.sql.</v>
+      </c>
+      <c r="E280" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B281" t="str">
+        <v>17:40</v>
+      </c>
+      <c r="C281" t="str">
+        <v>Despliegue v2.33 producción</v>
+      </c>
+      <c r="D281" t="str">
+        <v>Push a main y Vercel --prod: conciliación manual de dos o más movimientos del mismo extracto sin tesorería (transferencia por error y devolución). APP_VERSION 2.33.</v>
+      </c>
+      <c r="E281" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E279"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E281"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5646,7 +5680,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql y sql/supabase_cb_borrar_movimiento_banco_galicia.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql y sql/supabase_cb_confirmar_manual_solo_extracto.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5801,7 +5835,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6644,9 +6678,20 @@
         <v>Despliegue v2.32: menú Cajas (físicas) no conciliables — Galicia-f (ARS) (tesoreria_efectivo_pesos / cierre_PES) y Morba-s/f (ARS) (tesoreria_transferencia_morba / cierre_MOR); sin Apertura de Caja; orden y filtros; saldos en Saldos extractos (solapas y consolidado). sql/supabase_cajas_fisicas.sql y sql/supabase_cajas_fisicas_morba.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>2.33</v>
+      </c>
+      <c r="B77" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Despliegue v2.33: Conciliación Bancaria — conciliación manual de dos o más movimientos del mismo extracto sin tesorería (crédito por transferencia errónea y débito de la devolución; badge solo extracto). sql/supabase_cb_confirmar_manual_solo_extracto.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C76"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C77"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6848,7 +6893,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.34: Confirmados solo extracto muestra crédito y débito.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E281"/>
+  <dimension ref="A1:E283"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5188,9 +5188,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="282">
+      <c r="A282" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B282" t="str">
+        <v>17:55</v>
+      </c>
+      <c r="C282" t="str">
+        <v>Confirmados solo extracto: crédito y débito</v>
+      </c>
+      <c r="D282" t="str">
+        <v>En Confirmados, la conciliación solo extracto muestra el crédito y el débito (no la suma neta en 0,00). El Excel exporta ambos importes como número.</v>
+      </c>
+      <c r="E282" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B283" t="str">
+        <v>18:05</v>
+      </c>
+      <c r="C283" t="str">
+        <v>Despliegue v2.34 producción</v>
+      </c>
+      <c r="D283" t="str">
+        <v>Push a main y Vercel --prod: Confirmados solo extracto muestra crédito y débito (no la suma neta en 0,00). APP_VERSION 2.34.</v>
+      </c>
+      <c r="E283" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E281"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E283"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5680,7 +5714,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql y sql/supabase_cb_confirmar_manual_solo_extracto.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql y sql/supabase_cb_confirmar_manual_solo_extracto.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5835,7 +5869,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6689,9 +6723,20 @@
         <v>Despliegue v2.33: Conciliación Bancaria — conciliación manual de dos o más movimientos del mismo extracto sin tesorería (crédito por transferencia errónea y débito de la devolución; badge solo extracto). sql/supabase_cb_confirmar_manual_solo_extracto.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>2.34</v>
+      </c>
+      <c r="B78" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Despliegue v2.34: Conciliación Bancaria — Confirmados solo extracto muestra crédito y débito (no la suma neta en 0,00); Excel con ambos importes numéricos. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C77"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C78"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6893,7 +6938,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.35: MP Solo banco No requiere conciliación.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E283"/>
+  <dimension ref="A1:E285"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5222,9 +5222,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="284">
+      <c r="A284" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B284" t="str">
+        <v>18:55</v>
+      </c>
+      <c r="C284" t="str">
+        <v>MP Solo banco: No requiere conciliación</v>
+      </c>
+      <c r="D284" t="str">
+        <v>En Mercado Pago, Solo banco permite marcar un movimiento como No requiere conciliación con justificación. No se borra del extracto; va a la solapa No requiere y se puede deshacer. sql/supabase_cb_mp_no_requiere_conciliacion.sql.</v>
+      </c>
+      <c r="E284" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B285" t="str">
+        <v>19:05</v>
+      </c>
+      <c r="C285" t="str">
+        <v>Despliegue v2.35 producción</v>
+      </c>
+      <c r="D285" t="str">
+        <v>Push a main y Vercel --prod: Mercado Pago Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere). APP_VERSION 2.35.</v>
+      </c>
+      <c r="E285" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E283"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E285"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5714,7 +5748,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql y sql/supabase_cb_confirmar_manual_solo_extracto.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6938,7 +6972,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.36: Impuestos MP, extracto Galicia PDF y confirmar todos en Sugeridos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E285"/>
+  <dimension ref="A1:E296"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5256,16 +5256,203 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="286">
+      <c r="A286" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B286" t="str">
+        <v>11:50</v>
+      </c>
+      <c r="C286" t="str">
+        <v>Menú Impuestos: Mercado Pago CIBBPP</v>
+      </c>
+      <c r="D286" t="str">
+        <v>Nuevo menú Impuestos, primera solapa Mercado Pago. Upload de Reporte-Percepción-CIBBPP (IIBB Reg. General Buenos Aires, icono de ayuda). Cruce por Número de movimiento contra el extracto MP: columnas En extracto y Conciliado. sql/supabase_impuestos.sql.</v>
+      </c>
+      <c r="E286" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B287" t="str">
+        <v>11:55</v>
+      </c>
+      <c r="C287" t="str">
+        <v>Impuestos CIBBPP: percibido no conciliado</v>
+      </c>
+      <c r="D287" t="str">
+        <v>En la card Percibido de CIBBPP se muestra debajo el monto percibido que todavía no está conciliado (incluye sin extracto y en extracto sin confirmar).</v>
+      </c>
+      <c r="E287" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B288" t="str">
+        <v>12:05</v>
+      </c>
+      <c r="C288" t="str">
+        <v>Impuestos MP: combo CIBBPP y CIBCPP</v>
+      </c>
+      <c r="D288" t="str">
+        <v>El régimen de percepción es un combo: CIBBPP (IIBB Reg. General Buenos Aires) y CIBCPP (IIBB Rég. General CABA). Cada uno tiene su listado, cruce y upload; el tercero se suma después.</v>
+      </c>
+      <c r="E288" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B289" t="str">
+        <v>12:10</v>
+      </c>
+      <c r="C289" t="str">
+        <v>Impuestos MP: combo CIVAPP</v>
+      </c>
+      <c r="D289" t="str">
+        <v>Tercer régimen en el combo de Mercado Pago: CIVAPP — Percepción IVA. Mismo upload y cruce por Número de movimiento contra el extracto.</v>
+      </c>
+      <c r="E289" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B290" t="str">
+        <v>12:15</v>
+      </c>
+      <c r="C290" t="str">
+        <v>Impuestos MP: filtros Mes, extracto y conciliado</v>
+      </c>
+      <c r="D290" t="str">
+        <v>Impuestos Mercado Pago: botón Filtros (modal como Cajas) con Mes, En extracto MP y Conciliado (Sí / No / No requiere). El buscar queda en la toolbar. Tabla, KPIs y Excel respetan los filtros; al cambiar de régimen se limpian.</v>
+      </c>
+      <c r="E290" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B291" t="str">
+        <v>12:45</v>
+      </c>
+      <c r="C291" t="str">
+        <v>Impuestos: conciliación manual con tesorería MP</v>
+      </c>
+      <c r="D291" t="str">
+        <v>Botón Conciliación manual en Impuestos: las percepciones no conciliadas se filtran por tipo de archivo, se pueden seleccionar todas y se concilian con un único movimiento de tesorería Mercado Pago (justificación y diferencia). No crea match en Conciliación Bancaria. sql/supabase_impuestos_conciliacion_manual.sql.</v>
+      </c>
+      <c r="E291" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B292" t="str">
+        <v>13:05</v>
+      </c>
+      <c r="C292" t="str">
+        <v>Confirmados: conciliación manual de impuestos</v>
+      </c>
+      <c r="D292" t="str">
+        <v>El tesorería de la conciliación manual de Impuestos aparece en Confirmados de Conciliación Bancaria (Mercado Pago) con criterio Conciliación manual de impuestos, sin usar el cargo del extracto. Las tres ya hechas se backfillearon. Deshacer limpia las percepciones. sql/supabase_cb_match_impuestos.sql.</v>
+      </c>
+      <c r="E292" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B293" t="str">
+        <v>14:10</v>
+      </c>
+      <c r="C293" t="str">
+        <v>Sugeridos: máximo 4 días de diferencia</v>
+      </c>
+      <c r="D293" t="str">
+        <v>Las sugerencias de Conciliación Bancaria ya no emparejan extracto y tesorería si las fechas difieren en más de 4 días. Lo más lejano queda en Solo banco / Solo sistema (se puede conciliar a mano). Al abrir el módulo se recálculan las sugerencias viejas fuera de esa ventana.</v>
+      </c>
+      <c r="E293" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B294" t="str">
+        <v>14:35</v>
+      </c>
+      <c r="C294" t="str">
+        <v>Galicia: extracto PDF sin duplicar vs Excel</v>
+      </c>
+      <c r="D294" t="str">
+        <v>Conciliación Bancaria admite el PDF Extracto_Cuentas_Galicia_… (resumen de cuenta corriente) como extracto Galicia. No duplica movimientos ya cargados por Excel: misma fecha, importe y concepto (el saldo del banco puede cambiar). El Excel Extracto_CC… sigue valiendo.</v>
+      </c>
+      <c r="E294" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B295" t="str">
+        <v>14:55</v>
+      </c>
+      <c r="C295" t="str">
+        <v>Sugeridos: check confirmar todos los listados</v>
+      </c>
+      <c r="D295" t="str">
+        <v>En Conciliación Bancaria → Sugeridos hay un check Confirmar todos los listados: confirma las sugerencias visibles (respeta filtros) y las pasa a Confirmados. sql/supabase_cb_confirmar_sugeridos.sql.</v>
+      </c>
+      <c r="E295" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B296" t="str">
+        <v>15:10</v>
+      </c>
+      <c r="C296" t="str">
+        <v>Despliegue v2.36 producción</v>
+      </c>
+      <c r="D296" t="str">
+        <v>Push a main y Vercel --prod: Impuestos MP (CIBBPP/CIBCPP/CIVAPP y conciliación manual en Confirmados); extracto Galicia PDF; Sugeridos máximo 4 días y check confirmar todos. APP_VERSION 2.36.</v>
+      </c>
+      <c r="E296" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E285"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E296"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B67"/>
+  <dimension ref="A1:B68"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -5748,7 +5935,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto CC (fecha+débito/crédito+descripción; no duplica si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), primero fecha cercana (±14 días) y después fecha lejana. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5769,47 +5956,55 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Impuestos</v>
       </c>
       <c r="B63" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql y sql/supabase_cb_match_impuestos.sql.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B64" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B65" t="str">
-        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B66" t="str">
-        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
+        <v>Log de excluidos en upload</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
         <v>Análisis financiero extracto (PDF)</v>
       </c>
-      <c r="B67" t="str">
+      <c r="B68" t="str">
         <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B68"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5903,7 +6098,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C80"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6768,16 +6963,38 @@
         <v>Despliegue v2.34: Conciliación Bancaria — Confirmados solo extracto muestra crédito y débito (no la suma neta en 0,00); Excel con ambos importes numéricos. Producción Vercel.</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>2.35</v>
+      </c>
+      <c r="B79" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Despliegue v2.35: Conciliación Bancaria — Mercado Pago Solo banco: marcar No requiere conciliación con justificación (no se borra del extracto; solapa No requiere; se puede deshacer). sql/supabase_cb_mp_no_requiere_conciliacion.sql. Producción Vercel.</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>2.36</v>
+      </c>
+      <c r="B80" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Despliegue v2.36: Impuestos Mercado Pago (combo CIBBPP/CIBCPP/CIVAPP, conciliación manual de percepciones con tesorería en Confirmados); extracto Galicia PDF Extracto_Cuentas_Galicia_… sin duplicar vs Excel; Sugeridos solo ±4 días y check Confirmar todos los listados. sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql, sql/supabase_cb_match_impuestos.sql, sql/supabase_cb_confirmar_sugeridos.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C78"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C80"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -6972,7 +7189,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar, sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar (Galicia: Excel CC o PDF Extracto_Cuentas_Galicia_…, sin repetir lo ya cargado), sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>
@@ -7009,9 +7226,23 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Impuestos</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Menú Impuestos (Mercado Pago): combo de percepción CIBBPP (IIBB Reg. General Buenos Aires), CIBCPP (IIBB Rég. General CABA) y CIVAPP (Percepción IVA), cruce por Número de movimiento con el extracto MP (en extracto / conciliado) y conciliación manual de no conciliadas con un movimiento de tesorería MP (queda en Confirmados). Excel y permisos en Seguridad.</v>
+      </c>
+      <c r="C17">
+        <v>8</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D17"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7037,7 +7268,7 @@
         <v>Frontend</v>
       </c>
       <c r="B2" t="str">
-        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas) y Saldos extractos en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.* y fornitalia-saldos-extractos.*). Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia con pdf.js en el navegador.</v>
+        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas), Saldos extractos e Impuestos en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.*, fornitalia-saldos-extractos.* y fornitalia-impuestos.*). Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia con pdf.js en el navegador.</v>
       </c>
     </row>
     <row r="3">
@@ -7045,7 +7276,7 @@
         <v>Datos</v>
       </c>
       <c r="B3" t="str">
-        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia, cb_movimiento, cb_match, cf_movimiento, eb_saldo_extracto. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
+        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia, cb_movimiento, cb_match, cf_movimiento, eb_saldo_extracto, imp_percepcion_mp. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
v2.37: recálculo de Sugeridos no pisa Confirmados ni fechas lejanas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E296"/>
+  <dimension ref="A1:E298"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5443,9 +5443,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="297">
+      <c r="A297" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B297" t="str">
+        <v>16:25</v>
+      </c>
+      <c r="C297" t="str">
+        <v>Sugerencias: no pisar confirmados ni fechas lejanas</v>
+      </c>
+      <c r="D297" t="str">
+        <v>El recálculo de Conciliación Bancaria fallaba con “ya está en otra conciliación activa” (Galicia: 371 filas con el mismo created_at; la paginación podía omitir un confirmado y volver a sugerirlo). El RPC ahora omite pares ya confirmados, duplicados y con más de 4 días. El error, si aparece, nombra el movimiento. La carga del módulo ya no se corta si falla el recálculo. sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql.</v>
+      </c>
+      <c r="E297" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B298" t="str">
+        <v>16:45</v>
+      </c>
+      <c r="C298" t="str">
+        <v>Despliegue v2.37 producción</v>
+      </c>
+      <c r="D298" t="str">
+        <v>Push a main y Vercel --prod: recálculo de Sugeridos no pisa Confirmados ni arma pares con más de 4 días; paginación estable; el error nombra el movimiento. sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql. APP_VERSION 2.37.</v>
+      </c>
+      <c r="E298" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E296"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E298"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5935,7 +5969,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6098,7 +6132,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -6985,9 +7019,20 @@
         <v>Despliegue v2.36: Impuestos Mercado Pago (combo CIBBPP/CIBCPP/CIVAPP, conciliación manual de percepciones con tesorería en Confirmados); extracto Galicia PDF Extracto_Cuentas_Galicia_… sin duplicar vs Excel; Sugeridos solo ±4 días y check Confirmar todos los listados. sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql, sql/supabase_cb_match_impuestos.sql, sql/supabase_cb_confirmar_sugeridos.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>2.37</v>
+      </c>
+      <c r="B81" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Despliegue v2.37: Conciliación Bancaria — recálculo de Sugeridos no pisa movimientos ya confirmados ni propone pares con más de 4 días; paginación estable de matches; si hay solape el error nombra el movimiento. sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C80"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C81"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.38: Galicia USD (PDF/CCE/cierre_DOL), Efectivo-f USD y ayuda unificada.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E298"/>
+  <dimension ref="A1:E305"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5477,9 +5477,128 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="299">
+      <c r="A299" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B299" t="str">
+        <v>16:55</v>
+      </c>
+      <c r="C299" t="str">
+        <v>Caja física Efectivo-f (USD) pesificada al MEP</v>
+      </c>
+      <c r="D299" t="str">
+        <v>Nueva solapa en Cajas (físicas) para tesoreria_efectivo_dolar_… y cierre_DOL-…. Los USD se convierten a ARS con usd_mep de tipo_de_cambio (fecha del movimiento o última cotización anterior). Se guardan ARS, USD original y TC. El saldo entra a Saldos extractos y al consolidado. sql/supabase_cajas_fisicas_dolar.sql.</v>
+      </c>
+      <c r="E299" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B300" t="str">
+        <v>17:05</v>
+      </c>
+      <c r="C300" t="str">
+        <v>Nombres Efectivo-f (ARS) y Efectivo-f (USD)</v>
+      </c>
+      <c r="D300" t="str">
+        <v>Las cajas físicas de efectivo pesos y efectivo dólar pasan a llamarse Efectivo-f (ARS) y Efectivo-f (USD) (antes Galicia-f). Solapas, Saldos extractos, consolidado y mensajes de Conciliación Bancaria.</v>
+      </c>
+      <c r="E300" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B301" t="str">
+        <v>17:26</v>
+      </c>
+      <c r="C301" t="str">
+        <v>Galicia (USD): extracto CCE y tesorería dólar</v>
+      </c>
+      <c r="D301" t="str">
+        <v>Nueva solapa Galicia (USD) en Conciliación Bancaria (canal galicia_usd, distinto de Efectivo-f USD). Extracto_CCE… y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… con Caja = Transferencia Galicia Dolar y Moneda USD: se concilia en dólares. Apertura de Caja y Pendiente no se cargan. El saldo de corte se pesifica al MEP en Saldos extractos. Banco Galicia pasa a Galicia (ARS). sql/supabase_cb_galicia_usd.sql.</v>
+      </c>
+      <c r="E301" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B302" t="str">
+        <v>17:50</v>
+      </c>
+      <c r="C302" t="str">
+        <v>Ayuda unificada con icono (como Flujo de caja)</v>
+      </c>
+      <c r="D302" t="str">
+        <v>Los textos largos de menús (Conciliación, Saldos, Cajas, Impuestos, Gestión de Proyectos, Reportes, Novedades, Seguridad) pasan al popover de ayuda al clic, el mismo método que Flujo de caja (icono + template). scripts/lib/fornitalia-help.js.</v>
+      </c>
+      <c r="E302" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B303" t="str">
+        <v>18:10</v>
+      </c>
+      <c r="C303" t="str">
+        <v>Galicia (USD): PDF Extracto_Cuentas_Galicia igual que en pesos</v>
+      </c>
+      <c r="D303" t="str">
+        <v>Conciliación Bancaria acepta el PDF de Cuenta Corriente Especial en dólares (mismo nombre Extracto_Cuentas_Galicia_… que el de pesos). Detecta el título, carga movimientos en USD en la solapa Galicia (USD) y no los mezcla con ARS. En Saldos extractos el mismo PDF arma el corte y pesifica inicial/cierre al MEP. El Excel Extracto_CCE… sigue valiendo.</v>
+      </c>
+      <c r="E303" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B304" t="str">
+        <v>18:25</v>
+      </c>
+      <c r="C304" t="str">
+        <v>Galicia (USD): cierre_DOL con Transferencia Galicia Dolar</v>
+      </c>
+      <c r="D304" t="str">
+        <v>El Excel de caja cerrada cierre_DOL-… con Caja = Transferencia Galicia Dolar se rechazaba como Efectivo-f (USD). Ahora la columna Caja manda: entra a Conciliación Galicia (USD) en dólares; si Caja es Efectivo Dolar, sigue yendo a Cajas (físicas).</v>
+      </c>
+      <c r="E304" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B305" t="str">
+        <v>18:32</v>
+      </c>
+      <c r="C305" t="str">
+        <v>Despliegue v2.38 producción</v>
+      </c>
+      <c r="D305" t="str">
+        <v>Push a main y Vercel --prod: Galicia (USD) en Conciliación (Excel CCE, PDF Extracto_Cuentas_Galicia_…, tesorería y cierre_CIERRE/cierre_DOL con Caja Transferencia Galicia Dolar); Saldos Galicia USD pesificado al MEP; caja física Efectivo-f (USD); ayuda unificada con icono. sql/supabase_cb_galicia_usd.sql y sql/supabase_cajas_fisicas_dolar.sql. APP_VERSION 2.38.</v>
+      </c>
+      <c r="E305" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E298"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E305"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5969,7 +6088,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago y Banco Galicia. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago y Galicia) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia: extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago, Galicia (ARS) y Galicia (USD). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -5977,7 +6096,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Galicia-f (ARS) (efectivo pesos: tesoreria_efectivo_pesos_… / cierre_PES-…) y Morba-s/f (ARS) (Transferencia Morba: tesoreria_transferencia_morba_… / cierre_MOR-…). Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. Apertura de Caja y filas Pendiente no se cargan (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Tesorería abierta: los Ids que ya no vienen van a A eliminar. Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql y sql/supabase_cf_borrar_apertura_caja.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS) (efectivo pesos: tesoreria_efectivo_pesos_… / cierre_PES-…), Morba-s/f (ARS) (Transferencia Morba: tesoreria_transferencia_morba_… / cierre_MOR-…) y Efectivo-f (USD) (efectivo dólar: tesoreria_efectivo_dolar_… / cierre_DOL-…). En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. Apertura de Caja y filas Pendiente no se cargan (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Tesorería abierta: los Ids que ya no vienen van a A eliminar. Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cf_borrar_apertura_caja.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -5985,7 +6104,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago, Banco Galicia, Galicia-f (ARS), Morba-s/f (ARS) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia: PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia-f (ARS) y Morba-s/f (ARS): saldos de cajas físicas que se actualizan desde el menú Cajas (físicas). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia + MP + Galicia-f (ARS) + Morba-s/f (ARS) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql y sql/supabase_cajas_fisicas_morba.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago, Galicia (ARS), Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas); Efectivo-f (USD) entra en ARS (MEP). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cb_galicia_usd.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -6132,7 +6251,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7030,9 +7149,20 @@
         <v>Despliegue v2.37: Conciliación Bancaria — recálculo de Sugeridos no pisa movimientos ya confirmados ni propone pares con más de 4 días; paginación estable de matches; si hay solape el error nombra el movimiento. sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>2.38</v>
+      </c>
+      <c r="B82" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Despliegue v2.38: Galicia (USD) en Conciliación Bancaria (Excel CCE, PDF Extracto_Cuentas_Galicia_… de cuenta en dólares, tesorería y cierre_CIERRE/cierre_DOL con Caja Transferencia Galicia Dolar; importes en USD); Saldos Galicia USD pesificado al MEP; caja física Efectivo-f (USD); ayuda de menús con el mismo icono que Flujo de caja. sql/supabase_cb_galicia_usd.sql y sql/supabase_cajas_fisicas_dolar.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C82"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7234,7 +7364,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago y Galicia). Uploads por ID sin duplicar (Galicia: Excel CC o PDF Extracto_Cuentas_Galicia_…, sin repetir lo ya cargado), sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago, Galicia ARS y Galicia USD). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>
@@ -7248,7 +7378,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (resumen PDF), Galicia-f (ARS) y Morba-s/f (ARS) (cajas físicas desde Cajas) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Efectivo-f (ARS), Morba-s/f (ARS) y Efectivo-f (USD, saldo en ARS al MEP) (cajas físicas desde Cajas) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>
@@ -7262,7 +7392,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B16" t="str">
-        <v>Menú de cajas no conciliables. Galicia-f (ARS) (efectivo pesos) y Morba-s/f (ARS) (Transferencia Morba) con tesorería abierta y cierre de caja por Id, sin extracto ni match. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
+        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba) y Efectivo-f (USD) (efectivo dólar pesificado al MEP de tipo_de_cambio) con tesorería abierta y cierre de caja por Id, sin extracto ni match. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
       </c>
       <c r="C16">
         <v>8</v>
@@ -7313,7 +7443,7 @@
         <v>Frontend</v>
       </c>
       <c r="B2" t="str">
-        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas), Saldos extractos e Impuestos en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.*, fornitalia-saldos-extractos.* y fornitalia-impuestos.*). Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia con pdf.js en el navegador.</v>
+        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas), Saldos extractos e Impuestos en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.*, fornitalia-saldos-extractos.* y fornitalia-impuestos.*). Ayuda de menús en scripts/lib/fornitalia-help.js. Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia ARS/USD con pdf.js en el navegador.</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
v2.39: suma algebraica en cards de Conciliación Bancaria.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E305"/>
+  <dimension ref="A1:E307"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5596,9 +5596,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="306">
+      <c r="A306" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B306" t="str">
+        <v>18:42</v>
+      </c>
+      <c r="C306" t="str">
+        <v>Conciliación: suma algebraica en las cards</v>
+      </c>
+      <c r="D306" t="str">
+        <v>Cada card de Conciliación Bancaria muestra, debajo de la cantidad, la suma algebraica de los importes del listado filtrado (más chica que el conteo; verde/rojo). Extracto, tesorería, sugeridos/confirmados (importe banco), solo banco/sistema, anulados, no requiere y A eliminar. Respeta buscar y filtros de mes/categoría/cuenta.</v>
+      </c>
+      <c r="E306" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B307" t="str">
+        <v>18:58</v>
+      </c>
+      <c r="C307" t="str">
+        <v>Despliegue v2.39 producción</v>
+      </c>
+      <c r="D307" t="str">
+        <v>Push a main y Vercel --prod: Conciliación Bancaria cards con suma algebraica de importes del listado filtrado (debajo de la cantidad). APP_VERSION 2.39.</v>
+      </c>
+      <c r="E307" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E305"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E307"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6088,7 +6122,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago, Galicia (ARS) y Galicia (USD). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago, Galicia (ARS) y Galicia (USD). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6251,7 +6285,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7160,9 +7194,20 @@
         <v>Despliegue v2.38: Galicia (USD) en Conciliación Bancaria (Excel CCE, PDF Extracto_Cuentas_Galicia_… de cuenta en dólares, tesorería y cierre_CIERRE/cierre_DOL con Caja Transferencia Galicia Dolar; importes en USD); Saldos Galicia USD pesificado al MEP; caja física Efectivo-f (USD); ayuda de menús con el mismo icono que Flujo de caja. sql/supabase_cb_galicia_usd.sql y sql/supabase_cajas_fisicas_dolar.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>2.39</v>
+      </c>
+      <c r="B83" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Despliegue v2.39: Conciliación Bancaria — cada card muestra, debajo de la cantidad, la suma algebraica de los importes del listado filtrado. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C83"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7364,7 +7409,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago, Galicia ARS y Galicia USD). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago, Galicia ARS y Galicia USD). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Cards con cantidad y suma algebraica del listado filtrado. Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.40: botones Mercado Pago en azul y Galicia en naranja.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E307"/>
+  <dimension ref="A1:E309"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5630,9 +5630,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="308">
+      <c r="A308" t="str">
+        <v>21/09/2026</v>
+      </c>
+      <c r="B308" t="str">
+        <v>15:15</v>
+      </c>
+      <c r="C308" t="str">
+        <v>Botones MP azul y Galicia naranja</v>
+      </c>
+      <c r="D308" t="str">
+        <v>Solapas y botones de carga de Mercado Pago pasan al azul de marca (#009EE3); Galicia (ARS/USD) al naranja. En Conciliación Bancaria, Saldos extractos e Impuestos, para distinguir el canal de un vistazo. Excel sigue verde.</v>
+      </c>
+      <c r="E308" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>21/09/2026</v>
+      </c>
+      <c r="B309" t="str">
+        <v>15:20</v>
+      </c>
+      <c r="C309" t="str">
+        <v>Despliegue v2.40 producción</v>
+      </c>
+      <c r="D309" t="str">
+        <v>Push a main y Vercel --prod: solapas y botones de carga Mercado Pago en azul de marca y Galicia (ARS/USD) en naranja (Conciliación Bancaria, Saldos extractos e Impuestos). APP_VERSION 2.40.</v>
+      </c>
+      <c r="E309" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E307"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E309"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6122,7 +6156,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago, Galicia (ARS) y Galicia (USD). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS) y Galicia (USD) (naranja). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6138,7 +6172,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago, Galicia (ARS), Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas); Efectivo-f (USD) entra en ARS (MEP). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cb_galicia_usd.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas); Efectivo-f (USD) entra en ARS (MEP). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cb_galicia_usd.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -6146,7 +6180,7 @@
         <v>Impuestos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql y sql/supabase_cb_match_impuestos.sql.</v>
+        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca): combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql y sql/supabase_cb_match_impuestos.sql.</v>
       </c>
     </row>
     <row r="64">
@@ -6285,7 +6319,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7205,9 +7239,20 @@
         <v>Despliegue v2.39: Conciliación Bancaria — cada card muestra, debajo de la cantidad, la suma algebraica de los importes del listado filtrado. Producción Vercel.</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>2.40</v>
+      </c>
+      <c r="B84" t="str">
+        <v>21/09/2026</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Despliegue v2.40: solapas y botones de carga Mercado Pago en azul de marca (#009EE3) y Galicia ARS/USD en naranja (Conciliación Bancaria, Saldos extractos e Impuestos). Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C83"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C84"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7409,7 +7454,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago, Galicia ARS y Galicia USD). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Cards con cantidad y suma algebraica del listado filtrado. Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Cards con cantidad y suma algebraica del listado filtrado. Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.41: duplicados de tesorería con descarte, conciliación manual más clara y solapa de eliminados.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E309"/>
+  <dimension ref="A1:E315"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5664,9 +5664,111 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B310" t="str">
+        <v>09:52</v>
+      </c>
+      <c r="C310" t="str">
+        <v>Potenciales duplicados en tesorería</v>
+      </c>
+      <c r="D310" t="str">
+        <v>Nueva solapa Potenciales duplicados en Conciliación Bancaria: grupos de tesorería con el mismo importe y hasta 40 días entre fechas (duplicado, triplicado o más). Card con cantidad de grupos y suma algebraica. Ojito con tabla y todos los campos de cada registro. Excel del listado filtrado. Respeta buscar y filtros de mes/categoría/cuenta.</v>
+      </c>
+      <c r="E310" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B311" t="str">
+        <v>10:18</v>
+      </c>
+      <c r="C311" t="str">
+        <v>Descartar duplicados de tesorería</v>
+      </c>
+      <c r="D311" t="str">
+        <v>En Potenciales duplicados se puede descartar un grupo (permiso confirmar). Queda persistido por el conjunto de IDs y no vuelve a listarse. Si entra un movimiento nuevo al grupo, sí se muestra. Solapa Duplicados descartados para deshacer. sql/supabase_cb_dup_tesoreria_descartar.sql.</v>
+      </c>
+      <c r="E311" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B312" t="str">
+        <v>10:20</v>
+      </c>
+      <c r="C312" t="str">
+        <v>Fix descarte de duplicados (ORDER BY DISTINCT)</v>
+      </c>
+      <c r="D312" t="str">
+        <v>La RPC cb_descartar_dup_tesoreria fallaba al confirmar: PostgreSQL exige que el ORDER BY de un SELECT DISTINCT esté en la lista. Se ordena por el UUID (x) en lugar de x::text.</v>
+      </c>
+      <c r="E312" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B313" t="str">
+        <v>11:08</v>
+      </c>
+      <c r="C313" t="str">
+        <v>Conciliación manual: contraparte y descripción</v>
+      </c>
+      <c r="D313" t="str">
+        <v>En el modal de Conciliación manual, el extracto muestra Contraparte y tesorería muestra Descripción, además de concepto, categoría y cuenta.</v>
+      </c>
+      <c r="E313" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B314" t="str">
+        <v>11:20</v>
+      </c>
+      <c r="C314" t="str">
+        <v>Solapa Tesorería eliminada</v>
+      </c>
+      <c r="D314" t="str">
+        <v>Nueva solapa en Conciliación Bancaria con tesorería borrada: papelera de Solo sistema, baja confirmada en A eliminar o reemplazo al cargar cierre/Id. Se archiva en cb_movimiento_eliminado (las bajas anteriores a esta solapa no aparecen). Ojito, card, Excel. sql/supabase_cb_tesoreria_eliminada.sql.</v>
+      </c>
+      <c r="E314" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B315" t="str">
+        <v>11:23</v>
+      </c>
+      <c r="C315" t="str">
+        <v>Despliegue v2.41 producción</v>
+      </c>
+      <c r="D315" t="str">
+        <v>Push a main y Vercel --prod: Potenciales duplicados (descartar persistente), Conciliación manual con contraparte y descripción, Tesorería eliminada. sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql. APP_VERSION 2.41.</v>
+      </c>
+      <c r="E315" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E309"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E315"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6156,7 +6258,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS) y Galicia (USD) (naranja). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS) y Galicia (USD) (naranja). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6319,7 +6421,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7250,9 +7352,20 @@
         <v>Despliegue v2.40: solapas y botones de carga Mercado Pago en azul de marca (#009EE3) y Galicia ARS/USD en naranja (Conciliación Bancaria, Saldos extractos e Impuestos). Producción Vercel.</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>2.41</v>
+      </c>
+      <c r="B85" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Despliegue v2.41: Conciliación Bancaria — Potenciales duplicados de tesorería (mismo importe, ≤40 días; descartar para que no vuelvan a entrar, con deshacer); Conciliación manual con Contraparte en extracto y Descripción en tesorería; solapa Tesorería eliminada (archivo de bajas). sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C85"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7454,7 +7567,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Cards con cantidad y suma algebraica del listado filtrado. Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos; quedan en Tesorería eliminada). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.42: tesorería histórica, popup de carga y update por Id aunque esté Pendiente.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E315"/>
+  <dimension ref="A1:E318"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5766,9 +5766,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="316">
+      <c r="A316" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B316" t="str">
+        <v>18:10</v>
+      </c>
+      <c r="C316" t="str">
+        <v>Tesorería histórica y popup de carga</v>
+      </c>
+      <c r="D316" t="str">
+        <v>Conciliación Bancaria reconoce movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto): Caja reparte MP/Galicia ARS/USD; mismo Id hace alta o actualización sin duplicar. Efectivo y Morba se omiten (van a Cajas físicas). Tras cualquier carga (extracto o tesorería) se abre un popup con nuevos, actualizados, sin cambios, sugerencias y omitidos.</v>
+      </c>
+      <c r="E316" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B317" t="str">
+        <v>18:45</v>
+      </c>
+      <c r="C317" t="str">
+        <v>Update por Id aunque esté Pendiente</v>
+      </c>
+      <c r="D317" t="str">
+        <v>El histórico omitía Status Pendiente y no actualizaba categoría/cuenta de Ids ya cargados (65 casos: p. ej. percepciones y costo MP). Ahora si el Id existe se actualiza donde esté; Pendiente nuevo no se da de alta. Se corrigieron esos 65 en tesorería.</v>
+      </c>
+      <c r="E317" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B318" t="str">
+        <v>18:55</v>
+      </c>
+      <c r="C318" t="str">
+        <v>Despliegue v2.42 producción</v>
+      </c>
+      <c r="D318" t="str">
+        <v>Push a main y Vercel --prod: tesorería histórica movimientos-historico_… (Caja reparte canales; popup de carga); update de categoría/cuenta por Id aunque el Excel traiga Pendiente. APP_VERSION 2.42.</v>
+      </c>
+      <c r="E318" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E315"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E318"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6258,7 +6309,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS) y Galicia (USD) (naranja). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja no entra en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS) y Galicia (USD) (naranja). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS y Galicia USD; Efectivo y Morba no se cargan acá (van a Cajas físicas). Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6266,7 +6317,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS) (efectivo pesos: tesoreria_efectivo_pesos_… / cierre_PES-…), Morba-s/f (ARS) (Transferencia Morba: tesoreria_transferencia_morba_… / cierre_MOR-…) y Efectivo-f (USD) (efectivo dólar: tesoreria_efectivo_dolar_… / cierre_DOL-…). En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. Apertura de Caja y filas Pendiente no se cargan (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Tesorería abierta: los Ids que ya no vienen van a A eliminar. Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cf_borrar_apertura_caja.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS) (efectivo pesos: tesoreria_efectivo_pesos_… / cierre_PES-…), Morba-s/f (ARS) (Transferencia Morba: tesoreria_transferencia_morba_… / cierre_MOR-…) y Efectivo-f (USD) (efectivo dólar: tesoreria_efectivo_dolar_… / cierre_DOL-…). En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cf_borrar_apertura_caja.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -6421,7 +6472,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7363,9 +7414,20 @@
         <v>Despliegue v2.41: Conciliación Bancaria — Potenciales duplicados de tesorería (mismo importe, ≤40 días; descartar para que no vuelvan a entrar, con deshacer); Conciliación manual con Contraparte en extracto y Descripción en tesorería; solapa Tesorería eliminada (archivo de bajas). sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>2.42</v>
+      </c>
+      <c r="B86" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Despliegue v2.42: tesorería histórica movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) reparte MP/Galicia ARS/USD y cajas físicas; popup de resumen de carga (nuevos, actualizados, sin cambios, sugerencias, omitidos); si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C86"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7567,7 +7629,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) como tesorería histórica. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos; quedan en Tesorería eliminada). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos; quedan en Tesorería eliminada). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>
@@ -7595,7 +7657,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B16" t="str">
-        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba) y Efectivo-f (USD) (efectivo dólar pesificado al MEP de tipo_de_cambio) con tesorería abierta y cierre de caja por Id, sin extracto ni match. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
+        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba) y Efectivo-f (USD) (efectivo dólar pesificado al MEP de tipo_de_cambio) con tesorería abierta, cierre de caja e histórico movimientos-historico_… por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
       </c>
       <c r="C16">
         <v>8</v>

</xml_diff>

<commit_message>
v2.43: Flujo desde tesorería, Matriz EF con estructura, Credicoop/s-f y sin caución.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E318"/>
+  <dimension ref="A1:E326"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5817,16 +5817,152 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B319" t="str">
+        <v>19:20</v>
+      </c>
+      <c r="C319" t="str">
+        <v>Flujo desde tesorería, Credicoop, s/f y sin caución</v>
+      </c>
+      <c r="D319" t="str">
+        <v>El Flujo de caja deja de leer la tabla transacciones y se arma con tesorería de Conciliación + Cajas físicas, unida a matriz_cat_cuenta_ef (Pendiente adentro). Credicoop es caja banco (botón negro). Efectivo-s/f ARS y USD en Cajas físicas. ABM Matriz EF. Se retira la columna Caución, el % G/P, el modal de marcha y el §8 del informe PDF. Se eliminan serie_cauciones.json, convertir-serie-cauciones.js y los helpers muertos del generador. sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql.</v>
+      </c>
+      <c r="E319" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B320" t="str">
+        <v>19:42</v>
+      </c>
+      <c r="C320" t="str">
+        <v>Fix SUPABASE_PAGE_SIZE al abrir Flujo</v>
+      </c>
+      <c r="D320" t="str">
+        <v>Al pasar el Flujo a tesorería se usaba SUPABASE_PAGE_SIZE en la paginación y había quedado sin definir. Se restaura const SUPABASE_PAGE_SIZE = 1000 junto al timeout de carga.</v>
+      </c>
+      <c r="E320" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B321" t="str">
+        <v>19:44</v>
+      </c>
+      <c r="C321" t="str">
+        <v>Fix getTasaAnterior al armar Flujo</v>
+      </c>
+      <c r="D321" t="str">
+        <v>Al sacar caución se borró getTasaAnterior, que no es de caución: es el fallback de cotización (MEP/CCL/Oficial) cuando el día no tiene tasa. Se restaura; montoConvertido y exports lo siguen usando.</v>
+      </c>
+      <c r="E321" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B322" t="str">
+        <v>19:55</v>
+      </c>
+      <c r="C322" t="str">
+        <v>G/P operativo: egresos de tesorería en absoluto</v>
+      </c>
+      <c r="D322" t="str">
+        <v>Tesorería guarda egreso/débito con monto negativo. El Flujo restaba ese negativo y el G/P quedaba ingresos+|egresos|. Se toma el valor absoluto al mapear (como en transacciones) y al guardar se vuelve a firmar.</v>
+      </c>
+      <c r="E322" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B323" t="str">
+        <v>20:40</v>
+      </c>
+      <c r="C323" t="str">
+        <v>EF: mismo par Ingreso/Egreso y USD al MEP</v>
+      </c>
+      <c r="D323" t="str">
+        <v>Ids 10002462 (egreso USD 15.756) y 10002864 (ingreso USD 30.000) en Efectivo Dólar, categoría Pago de Cuotas de Créditos / Intereses Bancarios. La matriz del otro tipo cubre la misma línea 6.2. El EF convierte USD a pesos con MEP de la fecha. El Flujo neto D suma 6.2/6.3 con signo (no |egreso|), para que cobro y pago se neteen.</v>
+      </c>
+      <c r="E323" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B324" t="str">
+        <v>20:56</v>
+      </c>
+      <c r="C324" t="str">
+        <v>Ordenar columnas Matriz EF</v>
+      </c>
+      <c r="D324" t="str">
+        <v>Encabezados de la grilla Matriz EF (Relaciones y Sin relación) ordenan al clic, ascendente/descendente, con indicador. El Excel exporta el orden visible.</v>
+      </c>
+      <c r="E324" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B325" t="str">
+        <v>21:15</v>
+      </c>
+      <c r="C325" t="str">
+        <v>ABM estructura EF en Matriz EF</v>
+      </c>
+      <c r="D325" t="str">
+        <v>Misma solapa Matriz EF, pestaña Estructura EF: alta/edición/baja de renglones de ef_estructura. No se pueden borrar secciones 1–6, totales A–D ni 6.1–6.3 (fórmulas), ni subítems con relaciones en la matriz o que alimentan ratios del Flujo. Renombrar sección/subítem actualiza hijas y matriz. sql/supabase_ef_estructura_abm.sql.</v>
+      </c>
+      <c r="E325" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B326" t="str">
+        <v>21:25</v>
+      </c>
+      <c r="C326" t="str">
+        <v>Despliegue v2.43 producción</v>
+      </c>
+      <c r="D326" t="str">
+        <v>Push a main y Vercel --prod: Flujo desde tesorería (Pendiente adentro); Credicoop caja banco; Efectivo-s/f ARS/USD; Matriz EF (relaciones, ordenar columnas y ABM de estructura); EF Ingreso/Egreso en la misma línea y USD×MEP; se retira caución. APP_VERSION 2.43.</v>
+      </c>
+      <c r="E326" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E318"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E326"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B68"/>
+  <dimension ref="A1:B69"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -5845,7 +5981,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa: columnas Ingresos, Egresos y G/P operativo (sin anulados ni apertura/cierre de caja; traspasos no incluidos en el import). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO; columna Caución (solo origen ARS). Proyección de ratios y caución en ARS. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda con criterios de la tabla. Exportar Flujo a Excel (mismo método que Evolución/EF: xlsx-js-style, importes numéricos, % como fracción).</v>
+        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -5981,7 +6117,7 @@
         <v>Inclusión por mes (Configuración)</v>
       </c>
       <c r="B19" t="str">
-        <v>Interruptores por cada mes con movimientos: incluir o excluir del flujo por mes, tarjetas de resumen, Evolución, Caución y agregados que usan excluirFilaFlujoOperativo. Persistencia localStorage y columna meses_excluidos en config_dashboard. Sin afectar duplicados ni export de base histórica.</v>
+        <v>Interruptores por cada mes con movimientos: incluir o excluir del flujo por mes, tarjetas de resumen, Evolución y agregados que usan excluirFilaFlujoOperativo. Persistencia localStorage y columna meses_excluidos en config_dashboard. Sin afectar duplicados ni export de base histórica.</v>
       </c>
     </row>
     <row r="20">
@@ -5997,7 +6133,7 @@
         <v>Exclusiones (flujo operativo)</v>
       </c>
       <c r="B21" t="str">
-        <v>No se incluyen en G/P operativo, Evolución ni Caución: anulados; apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito si aparecieran en datos; meses desmarcados en Configuración → Inclusión por mes (meses_excluidos en Supabase/localStorage). Base histórica y Todas las transacciones siguen completas.</v>
+        <v>No se incluyen en G/P operativo ni Evolución: apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito; meses desmarcados en Configuración → Inclusión por mes (meses_excluidos en Supabase/localStorage). Status Pendiente sí entra al Flujo. Base histórica y Todas las transacciones siguen completas.</v>
       </c>
     </row>
     <row r="22">
@@ -6005,7 +6141,7 @@
         <v>Datos</v>
       </c>
       <c r="B22" t="str">
-        <v>Transacciones y tipo de cambio desde Supabase (carga paginada de a 1000 filas por request para no truncar resultados). Cotización faltante: se usa la fecha anterior disponible.</v>
+        <v>Tesorería (Conciliación Bancaria + Cajas físicas) y tipo de cambio desde Supabase (carga paginada). La relación categoría/cuenta/tipo → EF vive en matriz_cat_cuenta_ef. Cotización faltante: se usa la fecha anterior disponible.</v>
       </c>
     </row>
     <row r="23">
@@ -6157,7 +6293,7 @@
         <v>Estado Financiero (tabla dinámica)</v>
       </c>
       <c r="B41" t="str">
-        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (hoja EF_Estructura del extracto). Columna Ítem con viñeta en detalle; períodos en columnas horizontales; subtotales y fórmulas con % del Flujo Operativo Generado. Clic en importe: modal con todas las transacciones (ef_subitem) que componen el valor del período o total. Gráficos línea (fila) y barras (columna). Exportar EF a Excel. Conciliación §7 oculta en vista y export.</v>
+        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). En ARS, USD × MEP de la fecha. Clic en importe: detalle con Ids. Gráficos y export Excel. Conciliación §7 oculta.</v>
       </c>
     </row>
     <row r="42">
@@ -6197,7 +6333,7 @@
         <v>Int. por caución</v>
       </c>
       <c r="B46" t="str">
-        <v>Columna en flujo por mes: interés mensual por colocar el sobrante de caja a la tasa diaria de la serie de cauciones. Carga Serie_Cauciones.xlsx al refrescar (o serie_cauciones.json si no hay Excel). Cálculo: base = G/P acumulado a la fecha + interés acumulado; Int T = base × tasa. Clic en el valor abre modal con marcha (G/P acum, Int T-1, Base, Tasa, Int T).</v>
+        <v>Retirado de la app: la columna Caución, el % G/P, el modal de marcha y la carga de Serie_Cauciones ya no están en el Flujo. La fila comercial se conserva por el trabajo histórico.</v>
       </c>
     </row>
     <row r="47">
@@ -6229,7 +6365,7 @@
         <v>Int. por caución proyectado</v>
       </c>
       <c r="B50" t="str">
-        <v>Punto de partida = G/P Total real + interés acumulado; tasa = promedio último mes real; días naturales; Int T-1 día 1 = (Int T-1 + Int T) último día del mes anterior. G/P acum en marcha = al inicio de cada día (real y proyectado). Ventana rodante: ingresos/egresos distintos por mes.</v>
+        <v>Retirado de la app junto con la columna Caución del Flujo.</v>
       </c>
     </row>
     <row r="51">
@@ -6237,7 +6373,7 @@
         <v>Disclaimer proyección</v>
       </c>
       <c r="B51" t="str">
-        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses, ventana rodante, y cálculo de Int. por caución proyectado.</v>
+        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses y ventana rodante.</v>
       </c>
     </row>
     <row r="52">
@@ -6253,7 +6389,7 @@
         <v>Configuración % G/P en caución</v>
       </c>
       <c r="B53" t="str">
-        <v>Combo "% G/P acum. en caución" en Configuración con escala de 5 en 5 (100, 95, 90… hasta 0). Por defecto 100 %; menor % = más liquidez (menos interés por caución).</v>
+        <v>Retirado de Configuración: el combo % G/P acum. en caución ya no se muestra. La columna pct_caucion en config_dashboard queda sin uso.</v>
       </c>
     </row>
     <row r="54">
@@ -6261,7 +6397,7 @@
         <v>Etiqueta Caución (x% cash)</v>
       </c>
       <c r="B54" t="str">
-        <v>Columna en flujo por mes: cabecera "Caución (x% cash)" donde x es el valor del parámetro % G/P; sin icono % a la izquierda. Modales de marcha y disclaimer usan "Caución".</v>
+        <v>Retirado: la columna Caución ya no forma parte del Flujo por mes.</v>
       </c>
     </row>
     <row r="55">
@@ -6277,7 +6413,7 @@
         <v>Config por usuario en Supabase</v>
       </c>
       <c r="B56" t="str">
-        <v>Tabla config_dashboard (user_id, proyección, caución, alertas y meses_excluidos JSON). Con Auth anónimo se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql; meses excluidos: supabase_config_dashboard_meses_excluidos.sql.</v>
+        <v>Tabla config_dashboard (user_id, proyección, alertas y meses_excluidos JSON). Se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql; meses excluidos: supabase_config_dashboard_meses_excluidos.sql.</v>
       </c>
     </row>
     <row r="57">
@@ -6309,7 +6445,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS) y Galicia (USD) (naranja). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS y Galicia USD; Efectivo y Morba no se cargan acá (van a Cajas físicas). Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Filas Pendiente y totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo (con o sin factura) y Morba no se cargan acá (van a Cajas físicas). Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6317,7 +6453,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS) (efectivo pesos: tesoreria_efectivo_pesos_… / cierre_PES-…), Morba-s/f (ARS) (Transferencia Morba: tesoreria_transferencia_morba_… / cierre_MOR-…) y Efectivo-f (USD) (efectivo dólar: tesoreria_efectivo_dolar_… / cierre_DOL-…). En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cf_borrar_apertura_caja.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD). En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cf_borrar_apertura_caja.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -6325,7 +6461,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas); Efectivo-f (USD) entra en ARS (MEP). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cb_galicia_usd.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas); Efectivo-f (USD) entra en ARS (MEP). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cb_galicia_usd.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -6370,15 +6506,23 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
+        <v>Matriz EF</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). Validaciones: no borrar 1–6, A–D, 6.1–6.3 ni subítems con relaciones/ratios; códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql y sql/supabase_ef_estructura_abm.sql.</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
         <v>Análisis financiero extracto (PDF)</v>
       </c>
-      <c r="B68" t="str">
+      <c r="B69" t="str">
         <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B69"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6472,7 +6616,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7425,16 +7569,27 @@
         <v>Despliegue v2.42: tesorería histórica movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) reparte MP/Galicia ARS/USD y cajas físicas; popup de resumen de carga (nuevos, actualizados, sin cambios, sugerencias, omitidos); si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Producción Vercel.</v>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>2.43</v>
+      </c>
+      <c r="B87" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Despliegue v2.43: Flujo de caja desde tesorería (cb/cf + matriz; Pendiente adentro); Credicoop caja banco; Efectivo-s/f ARS/USD; menú Matriz EF (relaciones, ordenar, ABM de ef_estructura); Estado Financiero con Ingreso/Egreso en la misma línea y USD×MEP; se retira Caución del Flujo. sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql y sql/supabase_ef_estructura_abm.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C86"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C87"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -7517,7 +7672,7 @@
         <v>Interés por caución</v>
       </c>
       <c r="B6" t="str">
-        <v>Columna Int. por caución en flujo por mes: cálculo de interés mensual por reinversión del sobrante a un día con tasa de serie de cauciones. Carga de Excel al refrescar, modal de marcha de cálculo (G/P acum, Base, Tasa, Int T). Incluye soporte para múltiples formatos de fecha y columna tasa_diaria.</v>
+        <v>Trabajo histórico ya entregado: columna Caución, serie de tasas y modal de marcha. Retirado de la app; las horas se conservan.</v>
       </c>
       <c r="C6">
         <v>5</v>
@@ -7531,7 +7686,7 @@
         <v>Proyección de flujo (próximos 3 meses)</v>
       </c>
       <c r="B7" t="str">
-        <v>Proyección de ingresos, egresos, G/P y ratios para los próximos 3 meses con configuración (mediana/promedio, meses de historia 3/6/12/24), ventana rodante; Int. por caución proyectado en cadena desde último real (G/P+interés); disclaimer de metodología bajo la proyección.</v>
+        <v>Proyección de ingresos, egresos, G/P y ratios para los próximos 3 meses con configuración (mediana/promedio, meses de historia 3/6/12/24), ventana rodante; disclaimer de metodología bajo la proyección.</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -7629,7 +7784,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos; quedan en Tesorería eliminada). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos; quedan en Tesorería eliminada). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>
@@ -7643,7 +7798,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Efectivo-f (ARS), Morba-s/f (ARS) y Efectivo-f (USD, saldo en ARS al MEP) (cajas físicas desde Cajas) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>
@@ -7657,7 +7812,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B16" t="str">
-        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba) y Efectivo-f (USD) (efectivo dólar pesificado al MEP de tipo_de_cambio) con tesorería abierta, cierre de caja e histórico movimientos-historico_… por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
+        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (histórico Caja Efectivo … sin factura; USD si la moneda es USD) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
       </c>
       <c r="C16">
         <v>8</v>
@@ -7680,9 +7835,23 @@
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Matriz EF y Flujo desde tesorería</v>
+      </c>
+      <c r="B18" t="str">
+        <v>El Flujo de caja pasa a alimentarse con tesorería (conciliación + cajas físicas) y la matriz categoría/cuenta/tipo → Estado Financiero (tabla base + ABM de relaciones y de la estructura de ítems/subítems). Incluye Status Pendiente. Se retira la columna Caución del Flujo.</v>
+      </c>
+      <c r="C18">
+        <v>24</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7708,7 +7877,7 @@
         <v>Frontend</v>
       </c>
       <c r="B2" t="str">
-        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas), Saldos extractos e Impuestos en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.*, fornitalia-saldos-extractos.* y fornitalia-impuestos.*). Ayuda de menús en scripts/lib/fornitalia-help.js. Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia ARS/USD con pdf.js en el navegador.</v>
+        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas), Saldos extractos, Impuestos y Matriz EF en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.*, fornitalia-saldos-extractos.*, fornitalia-impuestos.* y fornitalia-matriz-ef.*). Ayuda de menús en scripts/lib/fornitalia-help.js. Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia ARS/USD con pdf.js en el navegador.</v>
       </c>
     </row>
     <row r="3">
@@ -7716,7 +7885,7 @@
         <v>Datos</v>
       </c>
       <c r="B3" t="str">
-        <v>Supabase (PostgreSQL). Tablas: transacciones, tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia, cb_movimiento, cb_match, cf_movimiento, eb_saldo_extracto, imp_percepcion_mp. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
+        <v>Supabase (PostgreSQL). Tablas: transacciones (respaldo), tipo_de_cambio, config_dashboard, gp_proyecto, gp_entregable, gp_entregable_hora, gp_tarea, gp_tarea_hora, gp_proyecto_hora, gp_dependencia, cb_movimiento, cb_match, cf_movimiento, eb_saldo_extracto, imp_percepcion_mp, matriz_cat_cuenta_ef. Scripts SQL en carpeta sql/ se ejecutan en Supabase SQL Editor.</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
v2.44: retiro upload y Errores del Flujo; Matriz EF vuelve a la pantalla.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E326"/>
+  <dimension ref="A1:E330"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5953,9 +5953,77 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B327" t="str">
+        <v>21:55</v>
+      </c>
+      <c r="C327" t="str">
+        <v>Retiro upload de extracto normalizado del Flujo</v>
+      </c>
+      <c r="D327" t="str">
+        <v>Se elimina por completo de la app el botón Actualizar base desde normalizado, el modal que reemplazaba la tabla transacciones y la solapa Excluidos upload (permisos carga_normalizada y ver_solapa_excluidos_upload fuera de Seguridad). El Flujo sigue alimentado por tesorería. La escritura de ef_estructura queda solo con editar_matriz_ef.</v>
+      </c>
+      <c r="E327" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B328" t="str">
+        <v>22:10</v>
+      </c>
+      <c r="C328" t="str">
+        <v>Retiro solapa Errores del Flujo</v>
+      </c>
+      <c r="D328" t="str">
+        <v>Se elimina por completo la solapa Errores del Flujo de caja: botón, tabla, filtros, export Excel, modal de clasificación, modal de potencial duplicado y el permiso ver_solapa_errores en el menú de Seguridad. El modal mensual queda solo con Por categoría / Por cuenta. La edición de registros sigue en Todas las transacciones. Los duplicados de tesorería siguen en Conciliación Bancaria.</v>
+      </c>
+      <c r="E328" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B329" t="str">
+        <v>22:22</v>
+      </c>
+      <c r="C329" t="str">
+        <v>Fix layout Matriz EF fuera de pantalla</v>
+      </c>
+      <c r="D329" t="str">
+        <v>Al retirar Excluidos upload quedó un &lt;/div&gt; de más: el footer y las vistas (Matriz EF, Conciliación, etc.) salían de #main-content y se veían abajo del Flujo. Se restaura el cierre correcto de view-dashboard.</v>
+      </c>
+      <c r="E329" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B330" t="str">
+        <v>22:26</v>
+      </c>
+      <c r="C330" t="str">
+        <v>Despliegue v2.44 producción</v>
+      </c>
+      <c r="D330" t="str">
+        <v>Push a main y Vercel --prod: se retiran del Flujo el upload de extracto normalizado y la solapa Errores; se corrige el layout de Matriz EF (cierre HTML). APP_VERSION 2.44.</v>
+      </c>
+      <c r="E330" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E326"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E330"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5981,7 +6049,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -5997,7 +6065,7 @@
         <v>Moneda</v>
       </c>
       <c r="B4" t="str">
-        <v>Selector ARS / USD. Maestro caja→moneda (medio de pago) alineado a scripts/lib/fornitalia-moneda-por-medio.js en import normalizado y en esTransaccionUSD. En ARS: USD con monto × tipo_cambio o cotización de tabla; movimientos en ARS usan monto (no monto_cambio si viene desalineado del extracto).</v>
+        <v>Selector ARS / USD. Maestro caja→moneda (medio de pago) alineado a scripts/lib/fornitalia-moneda-por-medio.js en esTransaccionUSD. En ARS: USD con monto × tipo_cambio o cotización de tabla; movimientos en ARS usan monto (no monto_cambio si viene desalineado del extracto).</v>
       </c>
     </row>
     <row r="5">
@@ -6013,7 +6081,7 @@
         <v>Comisiones/Ventas %</v>
       </c>
       <c r="B6" t="str">
-        <v>Columna: egresos con ef_subitem «Comisiones por Ventas» ÷ ingresos con ef_subitem «Cobranzas por Ventas (Efectivo neto ingresado)» del mes (subítems canónicos EF; alias cortos se normalizan al import). Sin ef_subitem la fila no entra al ratio. Ayuda al clic en icono de columna e informe PDF (template-flujo-informe-pdf).</v>
+        <v>Columna: egresos con ef_subitem «Comisiones por Ventas» ÷ ingresos con ef_subitem «Cobranzas por Ventas (Efectivo neto ingresado)» del mes (subítems canónicos EF; alias cortos se normalizan). Sin ef_subitem la fila no entra al ratio. Ayuda al clic en icono de columna e informe PDF (template-flujo-informe-pdf).</v>
       </c>
     </row>
     <row r="7">
@@ -6053,7 +6121,7 @@
         <v>Por categoría (matriz)</v>
       </c>
       <c r="B11" t="str">
-        <v>Solapa del modal: detalle agrupado por nueva_categoria con fallback a extracto/validación (categoriaDistribucionFlujo); bloques Ingresos / Costo directo / indirecto / Otros costos; Ver para listado de transacciones.</v>
+        <v>Solapa del modal: detalle agrupado por nueva_categoria con fallback a extracto (categoriaDistribucionFlujo); bloques Ingresos / Costo directo / indirecto / Otros costos; Ver para listado de transacciones.</v>
       </c>
     </row>
     <row r="12">
@@ -6117,7 +6185,7 @@
         <v>Inclusión por mes (Configuración)</v>
       </c>
       <c r="B19" t="str">
-        <v>Interruptores por cada mes con movimientos: incluir o excluir del flujo por mes, tarjetas de resumen, Evolución y agregados que usan excluirFilaFlujoOperativo. Persistencia localStorage y columna meses_excluidos en config_dashboard. Sin afectar duplicados ni export de base histórica.</v>
+        <v>Interruptores por cada mes con movimientos: incluir o excluir del flujo por mes, tarjetas de resumen, Evolución y agregados que usan excluirFilaFlujoOperativo. Persistencia localStorage y columna meses_excluidos en config_dashboard. Sin afectar export de base histórica.</v>
       </c>
     </row>
     <row r="20">
@@ -6165,7 +6233,7 @@
         <v>Seguridad y roles</v>
       </c>
       <c r="B25" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos granulares desde Supabase: ver_solapa_* (cada solapa del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, carga_normalizada, editar_registros, assign_roles. Visor por defecto: Flujo por mes + exportar/reportes; un admin puede activar solapas y menús sueltos en Seguridad. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos granulares desde Supabase: ver_solapa_* (cada solapa del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo por mes + exportar/reportes; un admin puede activar solapas y menús sueltos en Seguridad. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
       </c>
     </row>
     <row r="26">
@@ -6197,7 +6265,7 @@
         <v>Exportar a Excel</v>
       </c>
       <c r="B29" t="str">
-        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle. Export Errores: incluye categoria_matriz y cuenta_matriz (misma lógica que el dashboard); monto como número.</v>
+        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle.</v>
       </c>
     </row>
     <row r="30">
@@ -6229,7 +6297,7 @@
         <v>Edición desde modal Errores</v>
       </c>
       <c r="B33" t="str">
-        <v>En el detalle de errores, icono de edición por registro. Abre modal para corregir: Categoría y Cuenta contable solo desde valores existentes en BD; Descripción libre. UPDATE en transacciones solo si hubo cambios respecto a la fila; si no, aviso (antes el modal cerraba sin guardar). Tras UPDATE se verifica que haya filas actualizadas; nota contextual para inconsistencia categoría/cuenta/descripción. editado y editado_detalle al guardar con cambios.</v>
+        <v>Retirado: la solapa Errores y su modal de detalle ya no están en el Flujo. La edición de registros sigue en Todas las transacciones.</v>
       </c>
     </row>
     <row r="34">
@@ -6245,7 +6313,7 @@
         <v>Tipo de error en Errores</v>
       </c>
       <c r="B35" t="str">
-        <v>Tabla de errores muestra columna Tipo de error: Inconsistencia entre Categoria, Cuenta Contable y Descripcion; o Potencial registro duplicado. Excepciones explícitas cat/cuenta (Impuestos/IIBB, Logistica/Fletes, Alquileres varias cuentas, Activos/Hornos, Mantenimiento/Ferreteria, Sueldos/Comisiones Ventas y variantes, Marketing/Creación contenido, Honorarios/Honorarios Contables) no marcan inconsistencia. Export a Excel incluye tipo_error.</v>
+        <v>Retirado: la clasificación de inconsistencia y el tipo de error ya no se calculan ni se listan en el Flujo.</v>
       </c>
     </row>
     <row r="36">
@@ -6253,7 +6321,7 @@
         <v>Detección de potencial duplicado</v>
       </c>
       <c r="B36" t="str">
-        <v>Registros con misma fecha, monto, tipo_movimiento y descripción similar se marcan como potencial duplicado. Icono Ver abre modal con comparación Este registro / Posible duplicado; acciones: Excluir de cálculos (anular) o Eliminar registro.</v>
+        <v>Retirado del Flujo: el modal de comparación Este registro / Posible duplicado ya no existe. Los duplicados de tesorería se gestionan en Conciliación Bancaria → Potenciales duplicados.</v>
       </c>
     </row>
     <row r="37">
@@ -6261,7 +6329,7 @@
         <v>Filtro por tipo de error</v>
       </c>
       <c r="B37" t="str">
-        <v>En la solapa Errores, selector para filtrar por tipo: Todos, Inconsistencia (categoría/cuenta/descripción), Potencial registro duplicado. La exportación a Excel exporta solo los registros visibles según el filtro.</v>
+        <v>Retirado: el selector Tipo de error de la solapa Errores ya no está en la app.</v>
       </c>
     </row>
     <row r="38">
@@ -6269,7 +6337,7 @@
         <v>Duplicados: condición cliente</v>
       </c>
       <c r="B38" t="str">
-        <v>Dos registros son potencial duplicado solo si coinciden en fecha, monto, tipo_movimiento, descripción similar y además cliente es igual; si cliente es distinto no se marcan como duplicado. Modal de comparación muestra id_origen y Cliente.</v>
+        <v>Retirado: esa regla de duplicados del Flujo ya no se aplica. Conciliación Bancaria usa su propio criterio (mismo importe, hasta 40 días).</v>
       </c>
     </row>
     <row r="39">
@@ -6285,7 +6353,7 @@
         <v>Evolución (tabla dinámica)</v>
       </c>
       <c r="B40" t="str">
-        <v>Solapa Evolución: Agrupar por = Nueva categoría (matriz) o Nueva cuenta contable (matriz) —prioriza nueva_categoria / nueva_cuenta_contable en BD y si faltan usa extracto con validación—; Período = Diario o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
+        <v>Solapa Evolución: Agrupar por = Nueva categoría (matriz) o Nueva cuenta contable (matriz) —prioriza nueva_categoria / nueva_cuenta_contable en BD y si faltan usa extracto—; Período = Diario o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
       </c>
     </row>
     <row r="41">
@@ -6493,7 +6561,7 @@
         <v>Upload de extracto normalizado</v>
       </c>
       <c r="B66" t="str">
-        <v>Botón en la app para reemplazar transacciones desde la hoja Normalizado (p. ej. Base_Fornitalia_To_App): incluye nueva_categoria, nueva_cuenta_contable, costo_directo/indirecto y columnas EF_Item / EF_SubItem → ef_item / ef_subitem en Supabase. Validación previa, carga en lotes y log de excluidos.</v>
+        <v>Retirado: el Flujo ya no reemplaza la tabla transacciones desde un Excel Normalizado. El botón, el modal y el permiso carga_normalizada salieron de la app. Queda el script npm run normalizar-extracto para generar el archivo.</v>
       </c>
     </row>
     <row r="67">
@@ -6501,7 +6569,7 @@
         <v>Log de excluidos en upload</v>
       </c>
       <c r="B67" t="str">
-        <v>Nueva solapa Excluidos upload con registros no insertados por error o por regla de negocio (Apertura/Cierre de Caja), persistidos en Supabase para auditoría.</v>
+        <v>Retirado: la solapa Excluidos upload y su permiso ya no están en el dashboard. La tabla de auditoría en Supabase se conserva.</v>
       </c>
     </row>
     <row r="68">
@@ -6616,7 +6684,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7580,9 +7648,20 @@
         <v>Despliegue v2.43: Flujo de caja desde tesorería (cb/cf + matriz; Pendiente adentro); Credicoop caja banco; Efectivo-s/f ARS/USD; menú Matriz EF (relaciones, ordenar, ABM de ef_estructura); Estado Financiero con Ingreso/Egreso en la misma línea y USD×MEP; se retira Caución del Flujo. sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql y sql/supabase_ef_estructura_abm.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>2.44</v>
+      </c>
+      <c r="B88" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Despliegue v2.44: se retiran del Flujo el upload de extracto normalizado (botón, modal, solapa Excluidos) y la solapa Errores (clasificación y duplicados del Flujo); se corrige el layout de Matriz EF que quedaba fuera de pantalla. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C88"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7616,7 +7695,7 @@
         <v>Normalización de datos</v>
       </c>
       <c r="B2" t="str">
-        <v>Relevamiento, limpieza y normalización de datos históricos de caja (campos de moneda, categorías, cuentas contables, flags de edición). Incluye lógica de excepciones, detección de inconsistencias y carga controlada desde extracto normalizado.</v>
+        <v>Relevamiento, limpieza y normalización de datos históricos de caja (campos de moneda, categorías, cuentas contables, flags de edición). Incluye lógica de excepciones y detección de inconsistencias. La carga desde extracto normalizado en la app quedó retirada (el Flujo se alimenta de tesorería).</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -7644,7 +7723,7 @@
         <v>Detección de duplicados y gestión de errores</v>
       </c>
       <c r="B4" t="str">
-        <v>Detección de potencial duplicado (fecha, monto, tipo, cliente, descripción similar), tipo de error (inconsistencia / duplicado), filtro por tipo, modal de comparación con id_origen y Cliente, acciones anular o eliminar registro.</v>
+        <v>Trabajo histórico ya entregado: solapa Errores, inconsistencia categoría/cuenta/descripción y potencial duplicado en el Flujo. Retirado de la app; las horas se conservan. Los duplicados de tesorería viven en Conciliación Bancaria.</v>
       </c>
       <c r="C4">
         <v>2</v>

</xml_diff>

<commit_message>
v2.45: tesorería omite Anulado y Cajas muestra el resultado de la carga.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E330"/>
+  <dimension ref="A1:E333"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6021,9 +6021,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B331" t="str">
+        <v>22:42</v>
+      </c>
+      <c r="C331" t="str">
+        <v>Cajas físicas: popup resultado de carga</v>
+      </c>
+      <c r="D331" t="str">
+        <v>Tras cargar tesorería o cierre en Cajas (físicas) se abre el mismo cartel que en Conciliación Bancaria: reconocidas, nuevas, actualizadas, sin cambios, a eliminar y omitidas (Apertura, Pendiente, otras cajas, sin Id, Id duplicado).</v>
+      </c>
+      <c r="E331" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B332" t="str">
+        <v>22:55</v>
+      </c>
+      <c r="C332" t="str">
+        <v>Omitir Status Anulado en tesorería</v>
+      </c>
+      <c r="D332" t="str">
+        <v>Se eliminaron 20 movimientos Anulado ya cargados (17 conciliación: Galicia 15 + MP 2, incl. Id 2102; 3 cajas) y 6 parejas confirmadas de Galicia que los usaban. El upload de Conciliación y Cajas ya no da de alta Anulado; si el Id existía se borra. sql/supabase_tesoreria_omitir_anulado.sql.</v>
+      </c>
+      <c r="E332" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B333" t="str">
+        <v>22:58</v>
+      </c>
+      <c r="C333" t="str">
+        <v>Despliegue v2.45 producción</v>
+      </c>
+      <c r="D333" t="str">
+        <v>Push a main y Vercel --prod: Status Anulado no entra a tesorería (se borraron 20 ya cargados); popup de resultado de carga en Cajas físicas. sql/supabase_tesoreria_omitir_anulado.sql. APP_VERSION 2.45.</v>
+      </c>
+      <c r="E333" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E330"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E333"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6513,7 +6564,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo (con o sin factura) y Morba no se cargan acá (van a Cajas físicas). Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo (con o sin factura) y Morba no se cargan acá (van a Cajas físicas). Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6521,7 +6572,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD). En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cf_borrar_apertura_caja.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD). En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -6684,7 +6735,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7659,9 +7710,20 @@
         <v>Despliegue v2.44: se retiran del Flujo el upload de extracto normalizado (botón, modal, solapa Excluidos) y la solapa Errores (clasificación y duplicados del Flujo); se corrige el layout de Matriz EF que quedaba fuera de pantalla. Producción Vercel.</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>2.45</v>
+      </c>
+      <c r="B89" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Despliegue v2.45: tesorería no carga Status Anulado (se eliminaron 20 ya cargados, incl. Id 2102; si el Id existía se borra); popup de resultado de carga en Cajas físicas. sql/supabase_tesoreria_omitir_anulado.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C88"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C89"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7891,7 +7953,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B16" t="str">
-        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (histórico Caja Efectivo … sin factura; USD si la moneda es USD) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
+        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (histórico Caja Efectivo … sin factura; USD si la moneda es USD) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Tras cada carga se abre el popup de resultado (nuevos, actualizados, sin cambios, omitidos). El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
       </c>
       <c r="C16">
         <v>8</v>

</xml_diff>

<commit_message>
v2.46: Efectivo-s/f desde tesorería y corte de saldos sin Apertura.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E333"/>
+  <dimension ref="A1:E337"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6072,9 +6072,77 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B334" t="str">
+        <v>23:40</v>
+      </c>
+      <c r="C334" t="str">
+        <v>Efectivo-s/f desde cualquier tesorería</v>
+      </c>
+      <c r="D334" t="str">
+        <v>Caja = Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) entran a Efectivo-s/f ARS/USD aunque vengan en histórico, cierre u otro Excel de tesorería (Conciliación o Cajas). El saldo de corte alimenta Saldos extractos. Antes se omitían y esas solapas quedaban vacías.</v>
+      </c>
+      <c r="E334" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>22/09/2026</v>
+      </c>
+      <c r="B335" t="str">
+        <v>23:50</v>
+      </c>
+      <c r="C335" t="str">
+        <v>Efectivo-s/f: alta de Pendiente nuevo</v>
+      </c>
+      <c r="D335" t="str">
+        <v>Los 4 de Caja Efectivo … (sin factura) quedaban en omitidos Pendiente (nuevos) porque el Id no existía. En Efectivo-s/f el Status Pendiente sí se da de alta; en tesorería banco se mantiene la regla anterior.</v>
+      </c>
+      <c r="E335" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B336" t="str">
+        <v>00:12</v>
+      </c>
+      <c r="C336" t="str">
+        <v>Saldos extractos: Apertura no entra al corte</v>
+      </c>
+      <c r="D336" t="str">
+        <v>Apertura de Caja no se suma ni alimenta Saldos extractos. El histórico no pisa el corte de tesorería/cierre (había inflado sep-2026: Efectivo-f 198 M, Morba 238 M, Efectivo-f USD 283 M). Se borran esos 3 cortes; queda tesorería/cierre. sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+      </c>
+      <c r="E336" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B337" t="str">
+        <v>00:20</v>
+      </c>
+      <c r="C337" t="str">
+        <v>Despliegue v2.46 producción</v>
+      </c>
+      <c r="D337" t="str">
+        <v>Push a main y Vercel --prod: Efectivo-s/f desde cualquier tesorería (Pendiente nuevo sí entra); Apertura no alimenta Saldos extractos; el histórico no pisa tesorería/cierre. sql/supabase_eb_borrar_saldos_historico_apertura.sql. APP_VERSION 2.46.</v>
+      </c>
+      <c r="E337" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E333"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E337"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6564,7 +6632,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo (con o sin factura) y Morba no se cargan acá (van a Cajas físicas). Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6572,7 +6640,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD). En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga (el saldo de apertura, si viene, solo alimenta el corte de Saldos extractos). Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -6580,7 +6648,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas); Efectivo-f (USD) entra en ARS (MEP). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cb_galicia_usd.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cb_galicia_usd.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -6735,7 +6803,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7721,9 +7789,20 @@
         <v>Despliegue v2.45: tesorería no carga Status Anulado (se eliminaron 20 ya cargados, incl. Id 2102; si el Id existía se borra); popup de resultado de carga en Cajas físicas. sql/supabase_tesoreria_omitir_anulado.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>2.46</v>
+      </c>
+      <c r="B90" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Despliegue v2.46: Efectivo-s/f ARS/USD desde cualquier tesorería (Pendiente nuevo sí se da de alta); Apertura de Caja no entra al corte de Saldos extractos; el histórico no pisa tesorería/cierre (se borraron los 3 cortes inflados de sep-2026). sql/supabase_eb_borrar_saldos_historico_apertura.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C89"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C90"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7953,7 +8032,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B16" t="str">
-        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (histórico Caja Efectivo … sin factura; USD si la moneda es USD) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Tras cada carga se abre el popup de resultado (nuevos, actualizados, sin cambios, omitidos). El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
+        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura), en cualquier tesorería, cierre o histórico) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Tras cada carga se abre el popup de resultado (nuevos, actualizados, sin cambios, omitidos). Apertura de Caja no entra al corte. El histórico no pisa el saldo de tesorería o cierre. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
       </c>
       <c r="C16">
         <v>8</v>

</xml_diff>

<commit_message>
v2.47: Credicoop en Saldos extractos desde tesorería.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E337"/>
+  <dimension ref="A1:E339"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6140,9 +6140,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="338">
+      <c r="A338" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B338" t="str">
+        <v>00:40</v>
+      </c>
+      <c r="C338" t="str">
+        <v>Saldos extractos: Credicoop</v>
+      </c>
+      <c r="D338" t="str">
+        <v>Solapa Credicoop y columna en el consolidado. Sin extractos históricos: el corte se arma con tesorería (Conciliación, sin Apertura). Se siembran 3 cortes desde los 4 movimientos ya cargados (saldo 500.000 al 25/08/2026). sql/supabase_eb_saldo_credicoop.sql.</v>
+      </c>
+      <c r="E338" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B339" t="str">
+        <v>00:50</v>
+      </c>
+      <c r="C339" t="str">
+        <v>Despliegue v2.47 producción</v>
+      </c>
+      <c r="D339" t="str">
+        <v>Push a main y Vercel --prod: Credicoop en Saldos extractos (solapa, consolidado, gráfico y Excel); corte desde tesorería sin extractos históricos ni Apertura. sql/supabase_eb_saldo_credicoop.sql. APP_VERSION 2.47.</v>
+      </c>
+      <c r="E339" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E337"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E339"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6648,7 +6682,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql y sql/supabase_cb_galicia_usd.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql y sql/supabase_eb_saldo_credicoop.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -6803,7 +6837,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7800,9 +7834,20 @@
         <v>Despliegue v2.46: Efectivo-s/f ARS/USD desde cualquier tesorería (Pendiente nuevo sí se da de alta); Apertura de Caja no entra al corte de Saldos extractos; el histórico no pisa tesorería/cierre (se borraron los 3 cortes inflados de sep-2026). sql/supabase_eb_borrar_saldos_historico_apertura.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>2.47</v>
+      </c>
+      <c r="B91" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Despliegue v2.47: Credicoop en Saldos extractos (solapa, consolidado, gráfico y Excel). Sin extractos históricos: el corte se arma con tesorería de Conciliación (sin Apertura); se siembran 3 cortes (saldo 500.000 al 25/08/2026). sql/supabase_eb_saldo_credicoop.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C90"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C91"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8018,7 +8063,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>

</xml_diff>

<commit_message>
v2.48: columna Usuario en tablas y aviso de nueva versión al entrar.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E339"/>
+  <dimension ref="A1:E342"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6174,16 +6174,67 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="340">
+      <c r="A340" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B340" t="str">
+        <v>12:15</v>
+      </c>
+      <c r="C340" t="str">
+        <v>Columna Usuario en tablas operativas</v>
+      </c>
+      <c r="D340" t="str">
+        <v>Se muestra quién cargó o confirmó: nombre para mostrar (LB) y al pasar el mouse el email. Persistencia created_by / updated_by / confirmado_by / descartado_by / eliminado_by / no_requiere_by. Histórico nulo atribuido a lucas.bustos.martin@gmail.com. RPC get_usuarios_mostrar. sql/supabase_usuarios_mostrar.sql.</v>
+      </c>
+      <c r="E340" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B341" t="str">
+        <v>12:25</v>
+      </c>
+      <c r="C341" t="str">
+        <v>Modal Nueva versión en cada despliegue</v>
+      </c>
+      <c r="D341" t="str">
+        <v>Como en Pandi: al iniciar sesión, si hay novedades de la versión que el usuario aún no confirmó, se muestra el modal «Nueva versión» (logo, badge y lista). El agente redacta 2–4 frases visibles en scripts/lib/fornitalia-release-blurb.js; crear-bitacora-excel.js genera fornitalia-release.json. localStorage por usuario. Sin RPC de ack.</v>
+      </c>
+      <c r="E341" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B342" t="str">
+        <v>12:35</v>
+      </c>
+      <c r="C342" t="str">
+        <v>Despliegue v2.48 producción</v>
+      </c>
+      <c r="D342" t="str">
+        <v>Push a main y Vercel --prod: columna Usuario en tablas (nombre; tooltip email) y modal «Nueva versión» al iniciar sesión. sql/supabase_usuarios_mostrar.sql. APP_VERSION 2.48.</v>
+      </c>
+      <c r="E342" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E339"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E342"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B69"/>
+  <dimension ref="A1:B71"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -6370,7 +6421,7 @@
         <v>Tablas y scroll</v>
       </c>
       <c r="B23" t="str">
-        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal.</v>
+        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal. Columna Usuario (nombre para mostrar; tooltip con email) en Conciliación, Cajas, Saldos por canal, Impuestos, Matriz EF y Todas las transacciones.</v>
       </c>
     </row>
     <row r="24">
@@ -6426,7 +6477,7 @@
         <v>Flujo de despliegue</v>
       </c>
       <c r="B30" t="str">
-        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación.</v>
+        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación. En cada despliegue el agente redacta el modal «Nueva versión» (scripts/lib/fornitalia-release-blurb.js → fornitalia-release.json).</v>
       </c>
     </row>
     <row r="31">
@@ -6741,9 +6792,25 @@
         <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Usuario en tablas</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Quién cargó, confirmó, descartó o eliminó: se ve el nombre para mostrar (ej. LB) y al pasar el mouse el email. Lo histórico de tesorería, saldos, impuestos y matriz queda a nombre de LB (lucas.bustos.martin@gmail.com). El consolidado de Saldos extractos no tiene actor por fila. rpc get_usuarios_mostrar. sql/supabase_usuarios_mostrar.sql.</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Novedades al iniciar sesión</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Tras cada despliegue, al entrar a la app se muestra el modal «Nueva versión» con 2–4 frases de lo que se nota al recargar (logo, badge de versión, lista). Una vez Entendido, no vuelve a aparecer hasta la siguiente versión. El texto lo actualiza el agente en scripts/lib/fornitalia-release-blurb.js; fornitalia-release.json se sirve por red.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B71"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6837,7 +6904,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7845,16 +7912,27 @@
         <v>Despliegue v2.47: Credicoop en Saldos extractos (solapa, consolidado, gráfico y Excel). Sin extractos históricos: el corte se arma con tesorería de Conciliación (sin Apertura); se siembran 3 cortes (saldo 500.000 al 25/08/2026). sql/supabase_eb_saldo_credicoop.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>2.48</v>
+      </c>
+      <c r="B92" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Despliegue v2.48: columna Usuario en tablas operativas (nombre para mostrar; al pasar el mouse, el email) y modal «Nueva versión» al iniciar sesión con las novedades de cada despliegue. sql/supabase_usuarios_mostrar.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C91"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C92"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -8114,9 +8192,23 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Aviso de nueva versión</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Modal «Nueva versión» al iniciar sesión después de cada despliegue, con las novedades visibles de esa versión (mismo criterio que Pandi).</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8142,7 +8234,7 @@
         <v>Frontend</v>
       </c>
       <c r="B2" t="str">
-        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas), Saldos extractos, Impuestos y Matriz EF en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.*, fornitalia-saldos-extractos.*, fornitalia-impuestos.* y fornitalia-matriz-ef.*). Ayuda de menús en scripts/lib/fornitalia-help.js. Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia ARS/USD con pdf.js en el navegador.</v>
+        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas), Saldos extractos, Impuestos y Matriz EF en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.*, fornitalia-saldos-extractos.*, fornitalia-impuestos.* y fornitalia-matriz-ef.*). Ayuda de menús en scripts/lib/fornitalia-help.js. Novedades de cada versión: scripts/lib/fornitalia-release-blurb.js → fornitalia-release.json. Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia ARS/USD con pdf.js en el navegador.</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
v2.49: carga del histórico de tesorería desde Flujo de caja para todas las cajas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E342"/>
+  <dimension ref="A1:E344"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6225,9 +6225,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B343" t="str">
+        <v>18:20</v>
+      </c>
+      <c r="C343" t="str">
+        <v>Histórico de todas las cajas desde Flujo</v>
+      </c>
+      <c r="D343" t="str">
+        <v>En Flujo de caja, botón Cargar tesorería histórica: el Excel movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) se reparte de una vez a Conciliación (MP, Galicia ARS/USD, Credicoop) y a Cajas físicas (Efectivo-f, Morba, s/f). Popup de resultado conjunto. Ya no hace falta cargarlo solapa por solapa.</v>
+      </c>
+      <c r="E343" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B344" t="str">
+        <v>18:36</v>
+      </c>
+      <c r="C344" t="str">
+        <v>Despliegue v2.49 producción</v>
+      </c>
+      <c r="D344" t="str">
+        <v>Push a main y Vercel --prod: carga del histórico de tesorería desde Flujo de caja para todas las cajas juntas. APP_VERSION 2.49.</v>
+      </c>
+      <c r="E344" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E342"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E344"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6253,7 +6287,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -6717,7 +6751,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6725,7 +6759,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -6904,7 +6938,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7923,9 +7957,20 @@
         <v>Despliegue v2.48: columna Usuario en tablas operativas (nombre para mostrar; al pasar el mouse, el email) y modal «Nueva versión» al iniciar sesión con las novedades de cada despliegue. sql/supabase_usuarios_mostrar.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>2.49</v>
+      </c>
+      <c r="B93" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Despliegue v2.49: en Flujo de caja, Cargar tesorería histórica reparte el Excel movimientos-historico_… a todas las cajas (Conciliación y Cajas físicas) en una sola carga, con popup de resultado. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C93"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.50: orden en Flujo, búsqueda por descripción y mes en curso en Saldos extractos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E344"/>
+  <dimension ref="A1:E349"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6259,9 +6259,94 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B345" t="str">
+        <v>09:52</v>
+      </c>
+      <c r="C345" t="str">
+        <v>Orden y búsqueda en tablas del Flujo</v>
+      </c>
+      <c r="D345" t="str">
+        <v>En Flujo por mes y Todas las transacciones se puede ordenar por cualquier columna (clic en el encabezado). El buscador de Todas las transacciones busca por id operación y también por descripción.</v>
+      </c>
+      <c r="E345" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B346" t="str">
+        <v>10:40</v>
+      </c>
+      <c r="C346" t="str">
+        <v>Saldos extractos: mes en curso en bancos</v>
+      </c>
+      <c r="D346" t="str">
+        <v>En Mercado Pago, Galicia ARS/USD, Credicoop y Consolidado se agrega una fila Mes en curso (celeste): último corte más los movimientos del mes, totalizado hasta hoy. No es día a día. sql/supabase_eb_saldo_mes_en_curso.sql.</v>
+      </c>
+      <c r="E346" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B347" t="str">
+        <v>11:15</v>
+      </c>
+      <c r="C347" t="str">
+        <v>Mes en curso Galicia: saldo corrido del extracto</v>
+      </c>
+      <c r="D347" t="str">
+        <v>El mes en curso de Galicia tomaba el último saldo por UUID y mostraba 62.230.449,63 (línea intermedia del 23/09, archivo (8)). Ahora usa el saldo corrido de la última fila del extracto (fecha + fila Excel): 164.444.617,56. No se excluye ningún movimiento; hay re-subidas incrementales del mismo Excel.</v>
+      </c>
+      <c r="E347" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B348" t="str">
+        <v>11:20</v>
+      </c>
+      <c r="C348" t="str">
+        <v>Mes en curso: suma créditos menos débitos</v>
+      </c>
+      <c r="D348" t="str">
+        <v>El mes en curso de bancos (Galicia ARS/USD, MP, Credicoop) se calcula como último corte más la suma algebraica crédito − débito de los movimientos del mes. No usa el saldo corrido del extracto; puede diferir si hay cheques o re-subidas duplicadas.</v>
+      </c>
+      <c r="E348" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B349" t="str">
+        <v>11:26</v>
+      </c>
+      <c r="C349" t="str">
+        <v>Despliegue v2.50 producción</v>
+      </c>
+      <c r="D349" t="str">
+        <v>Push a main y Vercel --prod: orden por columna en Flujo por mes y Todas las transacciones; buscador también por descripción; Saldos extractos con fila Mes en curso (corte + crédito − débito). sql/supabase_eb_saldo_mes_en_curso.sql. APP_VERSION 2.50.</v>
+      </c>
+      <c r="E349" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E344"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E349"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6287,7 +6372,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Icono de ayuda. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -6455,7 +6540,7 @@
         <v>Tablas y scroll</v>
       </c>
       <c r="B23" t="str">
-        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal. Columna Usuario (nombre para mostrar; tooltip con email) en Conciliación, Cajas, Saldos por canal, Impuestos, Matriz EF y Todas las transacciones.</v>
+        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal. Flujo por mes y Todas las transacciones: clic en el encabezado ordena la columna. Columna Usuario (nombre para mostrar; tooltip con email) en Conciliación, Cajas, Saldos por canal, Impuestos, Matriz EF y Todas las transacciones.</v>
       </c>
     </row>
     <row r="24">
@@ -6647,7 +6732,7 @@
         <v>Todas las transacciones</v>
       </c>
       <c r="B47" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) e id operación (texto). Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) y buscador por id operación o descripción (texto). Clic en un encabezado ordena asc/desc. Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa.</v>
       </c>
     </row>
     <row r="48">
@@ -6767,7 +6852,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql y sql/supabase_eb_saldo_credicoop.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En bancos (MP, Galicia ARS/USD, Credicoop) y en Consolidado, una fila Mes en curso (celeste) totaliza hasta hoy: último corte más la suma algebraica crédito − débito de los movimientos banco del mes (puede diferir del saldo corrido del extracto si hay cheques o re-subidas). Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -6938,7 +7023,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -7968,9 +8053,20 @@
         <v>Despliegue v2.49: en Flujo de caja, Cargar tesorería histórica reparte el Excel movimientos-historico_… a todas las cajas (Conciliación y Cajas físicas) en una sola carga, con popup de resultado. Producción Vercel.</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>2.50</v>
+      </c>
+      <c r="B94" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Despliegue v2.50: orden por columna en Flujo por mes y Todas las transacciones; el buscador de Todas también busca en descripción; Saldos extractos con fila Mes en curso (celeste) = último corte + créditos − débitos. sql/supabase_eb_saldo_mes_en_curso.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C93"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C94"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8088,7 +8184,7 @@
         <v>Listado y edición completa de transacciones</v>
       </c>
       <c r="B8" t="str">
-        <v>Solapa Todas las transacciones con listado completo, filtros por mes y categoría, y modal de edición con todos los campos y combos para valores normalizados (categoría, cuenta contable, tipo movimiento, status, medio pago, moneda, origen archivo).</v>
+        <v>Solapa Todas las transacciones con listado completo, filtros por mes y categoría, buscador por id operación o descripción, orden por columna, y modal de edición con todos los campos y combos para valores normalizados (categoría, cuenta contable, tipo movimiento, status, medio pago, moneda, origen archivo).</v>
       </c>
       <c r="C8">
         <v>2</v>
@@ -8186,7 +8282,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual, con promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En bancos, fila Mes en curso (celeste) = último corte + créditos − débitos hasta hoy. Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>

</xml_diff>

<commit_message>
v2.51: US$ en Saldos extractos, solapa Activo y reporte PDF.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E349"/>
+  <dimension ref="A1:E352"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6344,9 +6344,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B350" t="str">
+        <v>11:45</v>
+      </c>
+      <c r="C350" t="str">
+        <v>Saldos extractos: USD chiquito en cajas dólar</v>
+      </c>
+      <c r="D350" t="str">
+        <v>En Galicia (USD), Efectivo-f (USD), Efectivo-s/f (USD) y el consolidado, debajo del saldo en pesos se muestra el monto en dólares en letra chica (US$).</v>
+      </c>
+      <c r="E350" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B351" t="str">
+        <v>11:55</v>
+      </c>
+      <c r="C351" t="str">
+        <v>Saldos extractos: PDF gráfico y solapa activa</v>
+      </c>
+      <c r="D351" t="str">
+        <v>Botón PDF arma un reporte de la vista activa (cards, gráfico y tabla) e indica qué solapa está activa. La solapa seleccionada se marca con etiqueta Activo y un contorno más visible.</v>
+      </c>
+      <c r="E351" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B352" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C352" t="str">
+        <v>Despliegue v2.51 producción</v>
+      </c>
+      <c r="D352" t="str">
+        <v>Push a main y Vercel --prod: en Saldos extractos, US$ chiquito en cajas dólar; solapa Activo más visible; reporte PDF de cards, gráfico y tabla. APP_VERSION 2.51.</v>
+      </c>
+      <c r="E352" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E349"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E352"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6852,7 +6903,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En bancos (MP, Galicia ARS/USD, Credicoop) y en Consolidado, una fila Mes en curso (celeste) totaliza hasta hoy: último corte más la suma algebraica crédito − débito de los movimientos banco del mes (puede diferir del saldo corrido del extracto si hay cheques o re-subidas). Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En bancos (MP, Galicia ARS/USD, Credicoop) y en Consolidado, una fila Mes en curso (celeste) totaliza hasta hoy: último corte más la suma algebraica crédito − débito de los movimientos banco del mes (puede diferir del saldo corrido del extracto si hay cheques o re-subidas). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -7023,7 +7074,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8064,9 +8115,20 @@
         <v>Despliegue v2.50: orden por columna en Flujo por mes y Todas las transacciones; el buscador de Todas también busca en descripción; Saldos extractos con fila Mes en curso (celeste) = último corte + créditos − débitos. sql/supabase_eb_saldo_mes_en_curso.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>2.51</v>
+      </c>
+      <c r="B95" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Despliegue v2.51: Saldos extractos — US$ debajo del peso en cajas dólar; solapa Activo más visible; reporte PDF de la vista (cards, gráfico y tabla). Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C95"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8282,7 +8344,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En bancos, fila Mes en curso (celeste) = último corte + créditos − débitos hasta hoy. Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En bancos, fila Mes en curso (celeste) = último corte + créditos − débitos hasta hoy. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>

</xml_diff>

<commit_message>
v2.52: help en Saldos, solapa Activo en todas las pantallas y Home recarga el Flujo.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E352"/>
+  <dimension ref="A1:E356"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6395,9 +6395,77 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B353" t="str">
+        <v>13:10</v>
+      </c>
+      <c r="C353" t="str">
+        <v>Saldos extractos: período y help en cards</v>
+      </c>
+      <c r="D353" t="str">
+        <v>En Variación del período, debajo del importe se ve el filtro Desde / Hasta (o Todos los cortes). Las cinco cards tienen icono de ayuda (mismo método que el resto de la app) con texto breve: qué se ve y qué no es.</v>
+      </c>
+      <c r="E353" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B354" t="str">
+        <v>13:45</v>
+      </c>
+      <c r="C354" t="str">
+        <v>Solapa activa en todas las pantallas</v>
+      </c>
+      <c r="D354" t="str">
+        <v>El botón de solapa en uso se marca igual que en Saldos extractos: etiqueta Activo y contorno más visible. Aplica a Flujo (Flujo por mes, Todas, Evolución, Estado Financiero y el modal categoría/cuenta), Conciliación, Cajas físicas, Impuestos, Matriz EF y Gestión de Proyectos.</v>
+      </c>
+      <c r="E354" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B355" t="str">
+        <v>13:55</v>
+      </c>
+      <c r="C355" t="str">
+        <v>Home recarga el Flujo de caja</v>
+      </c>
+      <c r="D355" t="str">
+        <v>Al volver a Home (Flujo de caja) se recargan tesorería, cajas, tipos de cambio y la config; se recalcula la tabla. Antes solo se mostraba lo que quedó en memoria.</v>
+      </c>
+      <c r="E355" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B356" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="C356" t="str">
+        <v>Despliegue v2.52 producción</v>
+      </c>
+      <c r="D356" t="str">
+        <v>Push a main y Vercel --prod: help y período en cards de Saldos extractos; solapa Activo en todas las pantallas; Home recarga el Flujo de caja. APP_VERSION 2.52.</v>
+      </c>
+      <c r="E356" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E352"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E356"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6423,7 +6491,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. La solapa activa (Flujo por mes, Todas las transacciones, Evolución, Estado Financiero) se marca con etiqueta Activo y un contorno más visible. Al volver a Home se recargan tesorería, cajas y tipos de cambio (no queda el dato viejo en memoria). Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -6599,7 +6667,7 @@
         <v>Menú lateral</v>
       </c>
       <c r="B24" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage. Home es el Flujo de caja: cada vez que se vuelve ahí se recargan tesorería, cajas y tipos de cambio.</v>
       </c>
     </row>
     <row r="25">
@@ -6879,7 +6947,7 @@
         <v>Gestión de Proyectos</v>
       </c>
       <c r="B59" t="str">
-        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Archivos adjuntos por fecha (descripción + archivo en Storage gp-archivos) en proyecto, entregable y tarea; solapa Archivos y hoja Excel. Solapa Horas cons.: conciliación diaria. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
+        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Archivos adjuntos por fecha (descripción + archivo en Storage gp-archivos) en proyecto, entregable y tarea; solapa Archivos y hoja Excel. Solapa Horas cons.: conciliación diaria. La solapa activa (To-Do, Gantt, Horas, Archivos) se marca con etiqueta Activo y un contorno más visible. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
       </c>
     </row>
     <row r="60">
@@ -6887,7 +6955,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -6895,7 +6963,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -6903,7 +6971,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En bancos (MP, Galicia ARS/USD, Credicoop) y en Consolidado, una fila Mes en curso (celeste) totaliza hasta hoy: último corte más la suma algebraica crédito − débito de los movimientos banco del mes (puede diferir del saldo corrido del extracto si hay cheques o re-subidas). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período, promedio de saldo (cuánto queda en las cuentas) y promedio de variación. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En bancos (MP, Galicia ARS/USD, Credicoop) y en Consolidado, una fila Mes en curso (celeste) totaliza hasta hoy: último corte más la suma algebraica crédito − débito de los movimientos banco del mes (puede diferir del saldo corrido del extracto si hay cheques o re-subidas). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -6911,7 +6979,7 @@
         <v>Impuestos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca): combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql y sql/supabase_cb_match_impuestos.sql.</v>
+        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca), marcada Activo como el resto de pantallas: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql y sql/supabase_cb_match_impuestos.sql.</v>
       </c>
     </row>
     <row r="64">
@@ -6951,7 +7019,7 @@
         <v>Matriz EF</v>
       </c>
       <c r="B68" t="str">
-        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). Validaciones: no borrar 1–6, A–D, 6.1–6.3 ni subítems con relaciones/ratios; códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql y sql/supabase_ef_estructura_abm.sql.</v>
+        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6, A–D, 6.1–6.3 ni subítems con relaciones/ratios; códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql y sql/supabase_ef_estructura_abm.sql.</v>
       </c>
     </row>
     <row r="69">
@@ -7074,7 +7142,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8126,9 +8194,20 @@
         <v>Despliegue v2.51: Saldos extractos — US$ debajo del peso en cajas dólar; solapa Activo más visible; reporte PDF de la vista (cards, gráfico y tabla). Producción Vercel.</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>2.52</v>
+      </c>
+      <c r="B96" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Despliegue v2.52: Saldos extractos — help en las cards y período filtrado bajo Variación; solapa Activo en Flujo, Conciliación, Cajas, Impuestos, Matriz EF y Gestión de Proyectos; Home recarga tesorería y recalcula el Flujo. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C96"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.53: el histórico recálcula sugeridos en cada caja de Conciliación.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E356"/>
+  <dimension ref="A1:E358"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6463,9 +6463,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B357" t="str">
+        <v>17:20</v>
+      </c>
+      <c r="C357" t="str">
+        <v>Histórico: sugeridos como en cada caja</v>
+      </c>
+      <c r="D357" t="str">
+        <v>Al cargar tesorería histórica desde Flujo (o el mismo Excel en Conciliación), se recálculan los sugeridos de cada canal (MP, Galicia ARS/USD, Credicoop) con la misma lógica que al cargar tesorería solapa por solapa. Si un canal falla, el resto sigue.</v>
+      </c>
+      <c r="E357" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B358" t="str">
+        <v>19:55</v>
+      </c>
+      <c r="C358" t="str">
+        <v>Despliegue v2.53 producción</v>
+      </c>
+      <c r="D358" t="str">
+        <v>Push a main y Vercel --prod: el histórico de tesorería recálcula sugeridos en cada caja de Conciliación (igual que cargar solapa por solapa). APP_VERSION 2.53.</v>
+      </c>
+      <c r="E358" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E356"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E358"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6491,7 +6525,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. La solapa activa (Flujo por mes, Todas las transacciones, Evolución, Estado Financiero) se marca con etiqueta Activo y un contorno más visible. Al volver a Home se recargan tesorería, cajas y tipos de cambio (no queda el dato viejo en memoria). Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja y recálcula los sugeridos de Conciliación en cada canal, igual que si se cargara tesorería solapa por solapa. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. La solapa activa (Flujo por mes, Todas las transacciones, Evolución, Estado Financiero) se marca con etiqueta Activo y un contorno más visible. Al volver a Home se recargan tesorería, cajas y tipos de cambio (no queda el dato viejo en memoria). Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -6955,7 +6989,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas). En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -7142,7 +7176,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C96"/>
+  <dimension ref="A1:C97"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8205,9 +8239,20 @@
         <v>Despliegue v2.52: Saldos extractos — help en las cards y período filtrado bajo Variación; solapa Activo en Flujo, Conciliación, Cajas, Impuestos, Matriz EF y Gestión de Proyectos; Home recarga tesorería y recalcula el Flujo. Producción Vercel.</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>2.53</v>
+      </c>
+      <c r="B97" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Despliegue v2.53: tesorería histórica desde Flujo recálcula sugeridos de Conciliación en cada canal (MP, Galicia ARS/USD, Credicoop), igual que cargar caja por caja. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C96"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C97"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.54: comparar tesorería saldos con el mes en curso en Saldos extractos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E358"/>
+  <dimension ref="A1:E360"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6497,9 +6497,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>25/09/2026</v>
+      </c>
+      <c r="B359" t="str">
+        <v>15:30</v>
+      </c>
+      <c r="C359" t="str">
+        <v>Saldos extractos: comparar tesorería saldos</v>
+      </c>
+      <c r="D359" t="str">
+        <v>Botón Tesorería saldos en Saldos extractos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso. Coincide = tilde verde; si no, cruz roja con el monto de la diferencia (en cajas dólar se compara US$).</v>
+      </c>
+      <c r="E359" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>25/09/2026</v>
+      </c>
+      <c r="B360" t="str">
+        <v>20:18</v>
+      </c>
+      <c r="C360" t="str">
+        <v>Despliegue v2.54 producción</v>
+      </c>
+      <c r="D360" t="str">
+        <v>Push a main y Vercel --prod: en Saldos extractos, botón Tesorería saldos compara el Excel tesoreria_saldos con el mes en curso (tilde verde o cruz roja + diferencia). APP_VERSION 2.54.</v>
+      </c>
+      <c r="E360" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E358"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E360"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7005,7 +7039,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En bancos (MP, Galicia ARS/USD, Credicoop) y en Consolidado, una fila Mes en curso (celeste) totaliza hasta hoy: último corte más la suma algebraica crédito − débito de los movimientos banco del mes (puede diferir del saldo corrido del extracto si hay cheques o re-subidas). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En bancos (MP, Galicia ARS/USD, Credicoop) y en Consolidado, una fila Mes en curso (celeste) totaliza hasta hoy: último corte más la suma algebraica crédito − débito de los movimientos banco del mes (puede diferir del saldo corrido del extracto si hay cheques o re-subidas). Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -7176,7 +7210,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C98"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8250,9 +8284,20 @@
         <v>Despliegue v2.53: tesorería histórica desde Flujo recálcula sugeridos de Conciliación en cada canal (MP, Galicia ARS/USD, Credicoop), igual que cargar caja por caja. Producción Vercel.</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>2.54</v>
+      </c>
+      <c r="B98" t="str">
+        <v>25/09/2026</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Despliegue v2.54: Saldos extractos — botón Tesorería saldos sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara cada caja con el mes en curso (tilde verde o cruz roja + diferencia; en dólar se compara US$). Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C97"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C98"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.55: columna Observaciones en todos los listados de movimientos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E360"/>
+  <dimension ref="A1:E362"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6531,9 +6531,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B361" t="str">
+        <v>07:46</v>
+      </c>
+      <c r="C361" t="str">
+        <v>Columna Observaciones en todos los movimientos</v>
+      </c>
+      <c r="D361" t="str">
+        <v>Observaciones como columna extra (después de Descripción) en Todas las transacciones, detalle de mes, Evolución, Estado Financiero, Conciliación Bancaria, Cajas físicas, Excel y el picker de tesorería de Impuestos. El campo ya estaba guardado: en transacciones como columna; en tesorería/cajas dentro de raw.observaciones (incluido el histórico). Editar desde el Flujo actualiza raw.observaciones. sql/supabase_imp_tesoreria_observaciones.sql.</v>
+      </c>
+      <c r="E361" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B362" t="str">
+        <v>10:43</v>
+      </c>
+      <c r="C362" t="str">
+        <v>Despliegue v2.55 producción</v>
+      </c>
+      <c r="D362" t="str">
+        <v>Push a main y Vercel --prod: columna Observaciones en todos los listados de movimientos (Flujo, Conciliación, Cajas, Excel e Impuestos). APP_VERSION 2.55.</v>
+      </c>
+      <c r="E362" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E360"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E362"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6671,7 +6705,7 @@
         <v>Detalle transacciones (tabla)</v>
       </c>
       <c r="B16" t="str">
-        <v>En el modal mensual, al expandir una categoría/cuenta se muestra una tabla con títulos y filas de transacciones (Fecha, Tipo, Medio, Moneda, Monto, moneda vista, TC, Cliente, Descripción, Origen). Icono ojo por fila (operadores) abre el modal de edición con el detalle completo del registro. Scroll vertical con encabezados fijos en el detalle expandido.</v>
+        <v>En el modal mensual, al expandir una categoría/cuenta se muestra una tabla con títulos y filas de transacciones (Fecha, Tipo, Medio, Moneda, Monto, moneda vista, TC, Cliente, Descripción, Observaciones, Origen). Icono ojo por fila (operadores) abre el modal de edición con el detalle completo del registro. Scroll vertical con encabezados fijos en el detalle expandido.</v>
       </c>
     </row>
     <row r="17">
@@ -6775,7 +6809,7 @@
         <v>Exportar a Excel</v>
       </c>
       <c r="B29" t="str">
-        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle.</v>
+        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, observaciones, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle.</v>
       </c>
     </row>
     <row r="30">
@@ -6871,7 +6905,7 @@
         <v>Estado Financiero (tabla dinámica)</v>
       </c>
       <c r="B41" t="str">
-        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). En ARS, USD × MEP de la fecha. Clic en importe: detalle con Ids. Gráficos y export Excel. Conciliación §7 oculta.</v>
+        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Gráficos y export Excel. Conciliación §7 oculta.</v>
       </c>
     </row>
     <row r="42">
@@ -6887,7 +6921,7 @@
         <v>Evolución: detalle al clic y exportar</v>
       </c>
       <c r="B43" t="str">
-        <v>Clic en un valor abre modal con detalle: Fecha, Categoría (matriz), Cuenta (matriz), Descripción, Monto. Exportar Evolución a Excel: primera columna con el mismo criterio de agrupación.</v>
+        <v>Clic en un valor abre modal con detalle: Fecha, Categoría (matriz), Cuenta (matriz), Descripción, Observaciones, Monto. Exportar Evolución a Excel: primera columna con el mismo criterio de agrupación.</v>
       </c>
     </row>
     <row r="44">
@@ -6919,7 +6953,7 @@
         <v>Todas las transacciones</v>
       </c>
       <c r="B47" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas. Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) y buscador por id operación o descripción (texto). Clic en un encabezado ordena asc/desc. Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas (incluida Observaciones, después de Descripción). Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) y buscador por id operación, descripción u observaciones. Clic en un encabezado ordena asc/desc. Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa.</v>
       </c>
     </row>
     <row r="48">
@@ -6927,7 +6961,7 @@
         <v>Edición completa de registros</v>
       </c>
       <c r="B48" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), ef_item y ef_subitem (estado de flujo), origen archivo, descripción, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), ef_item y ef_subitem (estado de flujo), origen archivo, descripción, observaciones, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). En tesorería (cb/cf) observaciones se guarda en raw.observaciones. editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
       </c>
     </row>
     <row r="49">
@@ -7023,7 +7057,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -7031,7 +7065,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -7047,7 +7081,7 @@
         <v>Impuestos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca), marcada Activo como el resto de pantallas: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql y sql/supabase_cb_match_impuestos.sql.</v>
+        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca), marcada Activo como el resto de pantallas: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (listado con Observaciones; justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql, sql/supabase_cb_match_impuestos.sql y sql/supabase_imp_tesoreria_observaciones.sql.</v>
       </c>
     </row>
     <row r="64">
@@ -7210,7 +7244,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C98"/>
+  <dimension ref="A1:C99"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8295,9 +8329,20 @@
         <v>Despliegue v2.54: Saldos extractos — botón Tesorería saldos sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara cada caja con el mes en curso (tilde verde o cruz roja + diferencia; en dólar se compara US$). Producción Vercel.</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>2.55</v>
+      </c>
+      <c r="B99" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Despliegue v2.55: columna Observaciones en Todas las transacciones, detalle de mes, Evolución, Estado Financiero, Conciliación Bancaria, Cajas físicas, Excel y tesorería de Impuestos; edición desde el Flujo. sql/supabase_imp_tesoreria_observaciones.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C99"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.56: AJUSTE DE SALDOS (CAJA) entra en el Flujo de caja neto del período.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E362"/>
+  <dimension ref="A1:E364"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6565,9 +6565,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B363" t="str">
+        <v>12:14</v>
+      </c>
+      <c r="C363" t="str">
+        <v>AJUSTE DE SALDOS (CAJA) en el Flujo neto D</v>
+      </c>
+      <c r="D363" t="str">
+        <v>El ítem AJUSTE DE SALDOS (CAJA) y su subítem pasan a figurar debajo de FLUJO OPERATIVO GENERADO. No entran en A–C; sí suman o restan en (=) FLUJO DE CAJA NETO DEL PERÍODO (Ingreso +, Egreso −). La fórmula D está fija en la app; se actualizó en estructura. sql/supabase_ef_ajuste_saldos_caja.sql.</v>
+      </c>
+      <c r="E363" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B364" t="str">
+        <v>12:16</v>
+      </c>
+      <c r="C364" t="str">
+        <v>Despliegue v2.56 producción</v>
+      </c>
+      <c r="D364" t="str">
+        <v>Push a main y Vercel --prod: AJUSTE DE SALDOS (CAJA) debajo de FLUJO OPERATIVO GENERADO y en el Flujo de caja neto del período (D). APP_VERSION 2.56.</v>
+      </c>
+      <c r="E364" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E362"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E364"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6905,7 +6939,7 @@
         <v>Estado Financiero (tabla dinámica)</v>
       </c>
       <c r="B41" t="str">
-        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Gráficos y export Excel. Conciliación §7 oculta.</v>
+        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). AJUSTE DE SALDOS (CAJA) va debajo de FLUJO OPERATIVO GENERADO y entra en (=) FLUJO DE CAJA NETO DEL PERÍODO (D), no en A–C. En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Gráficos y export Excel. Conciliación §7 oculta.</v>
       </c>
     </row>
     <row r="42">
@@ -7121,7 +7155,7 @@
         <v>Matriz EF</v>
       </c>
       <c r="B68" t="str">
-        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6, A–D, 6.1–6.3 ni subítems con relaciones/ratios; códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql y sql/supabase_ef_estructura_abm.sql.</v>
+        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6 ni 1.2 (ajuste de saldos), A–D, 6.1–6.3 ni subítems con relaciones/ratios; códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql, sql/supabase_ef_estructura_abm.sql y sql/supabase_ef_ajuste_saldos_caja.sql.</v>
       </c>
     </row>
     <row r="69">
@@ -7244,7 +7278,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C100"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8340,9 +8374,20 @@
         <v>Despliegue v2.55: columna Observaciones en Todas las transacciones, detalle de mes, Evolución, Estado Financiero, Conciliación Bancaria, Cajas físicas, Excel y tesorería de Impuestos; edición desde el Flujo. sql/supabase_imp_tesoreria_observaciones.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>2.56</v>
+      </c>
+      <c r="B100" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Despliegue v2.56: AJUSTE DE SALDOS (CAJA) debajo de FLUJO OPERATIVO GENERADO; suma o resta en (=) FLUJO DE CAJA NETO DEL PERÍODO (no en A–C). sql/supabase_ef_ajuste_saldos_caja.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C99"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C100"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.57: Galicia del consolidado muestra el saldo real del extracto.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E364"/>
+  <dimension ref="A1:E366"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6599,9 +6599,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B365" t="str">
+        <v>12:40</v>
+      </c>
+      <c r="C365" t="str">
+        <v>Galicia mes en curso: saldo real del banco</v>
+      </c>
+      <c r="D365" t="str">
+        <v>En Saldos extractos / Consolidado, el mes en curso de Galicia (ARS y USD) deja de sumar todos los movimientos banco (se inflaba por re-subidas y cheques en proceso). Toma el saldo corrido de la última fila del extracto (hoy 174.998.384,31) y solo suma lo posterior a esa fecha. Tesorería y conciliación no se tocan.</v>
+      </c>
+      <c r="E365" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B366" t="str">
+        <v>16:00</v>
+      </c>
+      <c r="C366" t="str">
+        <v>Despliegue v2.57 producción</v>
+      </c>
+      <c r="D366" t="str">
+        <v>Push a main y Vercel --prod: Galicia mes en curso en Saldos extractos y Consolidado usa el saldo corrido del extracto (saldo real del banco). Tesorería no se toca. APP_VERSION 2.57.</v>
+      </c>
+      <c r="E366" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E364"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E366"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7107,7 +7141,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En bancos (MP, Galicia ARS/USD, Credicoop) y en Consolidado, una fila Mes en curso (celeste) totaliza hasta hoy: último corte más la suma algebraica crédito − débito de los movimientos banco del mes (puede diferir del saldo corrido del extracto si hay cheques o re-subidas). Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP y Credicoop, mes en curso = último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -7278,7 +7312,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C100"/>
+  <dimension ref="A1:C101"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8385,9 +8419,20 @@
         <v>Despliegue v2.56: AJUSTE DE SALDOS (CAJA) debajo de FLUJO OPERATIVO GENERADO; suma o resta en (=) FLUJO DE CAJA NETO DEL PERÍODO (no en A–C). sql/supabase_ef_ajuste_saldos_caja.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>2.57</v>
+      </c>
+      <c r="B101" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Despliegue v2.57: Saldos extractos / Consolidado — Galicia (ARS y USD) mes en curso usa el saldo corrido de la última fila del extracto (saldo real del banco), no la suma de movimientos. Tesorería y conciliación no se tocan. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C100"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C101"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8603,7 +8648,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En bancos, fila Mes en curso (celeste) = último corte + créditos − débitos hasta hoy. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En Galicia, mes en curso = saldo corrido del extracto (saldo real del banco). En MP y Credicoop, último corte + créditos − débitos. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>

</xml_diff>

<commit_message>
v2.58: el saldo de período lo arman los movimientos del Excel; el PDF solo verifica.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E366"/>
+  <dimension ref="A1:E370"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6633,9 +6633,77 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B367" t="str">
+        <v>16:15</v>
+      </c>
+      <c r="C367" t="str">
+        <v>Galicia: borrar extracto temporal que ya no está</v>
+      </c>
+      <c r="D367" t="str">
+        <v>Se eliminaron 29 movimientos banco que no están en el Extracto_CC actual: 2 cheques en proceso (23/09), 2 IIBB Capital Federal (1/09) y 25 filas del PDF de agosto. Tesorería no se tocó. El próximo Excel CC/CCE retira solo lo que ese archivo ya no trae. sql/supabase_cb_retirar_extracto_banco_ausente.sql.</v>
+      </c>
+      <c r="E367" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B368" t="str">
+        <v>16:35</v>
+      </c>
+      <c r="C368" t="str">
+        <v>Cortes nuevos: banco manda, extracto verifica</v>
+      </c>
+      <c r="D368" t="str">
+        <v>De ahora en más (no se tocan extractos ya cargados): el banco (Galicia/MP) es la fuente de verdad; tesorería es la administración de la app. Un corte nuevo Galicia = saldo del PDF + movimientos banco del período que el extracto no trajo (corte del banco), para conciliar el mes vencido movimiento a movimiento. El upload muestra extracto vs saldo banco en la app; las diferencias vs tesorería siguen en Sugeridos / Solo banco / Solo sistema. sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+      </c>
+      <c r="E368" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B369" t="str">
+        <v>16:50</v>
+      </c>
+      <c r="C369" t="str">
+        <v>Saldo de período: Excel manda, PDF solo verifica</v>
+      </c>
+      <c r="D369" t="str">
+        <v>Después del último corte, el saldo se calcula con los movimientos cargados por el Excel del extracto (CC/CCE/MP). El PDF resumen del banco no da de alta movimientos: solo muestra cuáles del período no están en su saldo. Corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se tocan.</v>
+      </c>
+      <c r="E369" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B370" t="str">
+        <v>16:55</v>
+      </c>
+      <c r="C370" t="str">
+        <v>Despliegue v2.58 producción</v>
+      </c>
+      <c r="D370" t="str">
+        <v>Push a main y Vercel --prod: saldo de período Galicia = último corte + movimientos del Excel; el PDF solo verifica y no carga movimientos; el Excel CC/CCE retira temporales que ya no trae. Extractos ya cargados no se tocan. APP_VERSION 2.58.</v>
+      </c>
+      <c r="E370" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E366"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E370"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7125,7 +7193,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental: nunca borra movimientos ya cargados; si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), si un movimiento banco temporal ya no viene en el archivo (cheque en proceso, PDF viejo) se retira; tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -7141,7 +7209,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): PDF de resumen de cuenta (saldo inicial/cierre del período). Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP y Credicoop, mes en curso = último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql y sql/supabase_eb_saldo_mes_en_curso.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP y Credicoop, mes en curso = último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -7312,7 +7380,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:C102"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8430,9 +8498,20 @@
         <v>Despliegue v2.57: Saldos extractos / Consolidado — Galicia (ARS y USD) mes en curso usa el saldo corrido de la última fila del extracto (saldo real del banco), no la suma de movimientos. Tesorería y conciliación no se tocan. Producción Vercel.</v>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>2.58</v>
+      </c>
+      <c r="B102" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Despliegue v2.58: después del último corte, el saldo de período Galicia se arma con los movimientos del Excel (CC/CCE); el PDF del banco solo verifica y no da de alta movimientos; el Excel retira del extracto lo que ya no trae. Extractos ya cargados no se recalculan. sql/supabase_eb_guardar_saldos_regla_movimientos.sql y sql/supabase_cb_retirar_extracto_banco_ausente.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C102"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.59: tesorería histórica da de alta Pendiente; el cartel muestra Sugeridos aunque sea 0.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E370"/>
+  <dimension ref="A1:E373"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -5794,7 +5794,7 @@
         <v>Update por Id aunque esté Pendiente</v>
       </c>
       <c r="D317" t="str">
-        <v>El histórico omitía Status Pendiente y no actualizaba categoría/cuenta de Ids ya cargados (65 casos: p. ej. percepciones y costo MP). Ahora si el Id existe se actualiza donde esté; Pendiente nuevo no se da de alta. Se corrigieron esos 65 en tesorería.</v>
+        <v>El histórico omitía Status Pendiente y no actualizaba categoría/cuenta de Ids ya cargados (65 casos: p. ej. percepciones y costo MP). Ahora si el Id existe se actualiza donde esté; Status Pendiente sí se da de alta. Se corrigieron esos 65 en tesorería.</v>
       </c>
       <c r="E317" t="str">
         <v>Ajuste</v>
@@ -6701,9 +6701,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B371" t="str">
+        <v>07:40</v>
+      </c>
+      <c r="C371" t="str">
+        <v>Cartel de carga: Sugeridos siempre, por caja</v>
+      </c>
+      <c r="D371" t="str">
+        <v>Al cargar tesorería histórica (Flujo o Conciliación), el resultado muestra Sugeridos de Mercado Pago, Galicia, Galicia USD y Credicoop aunque sea 0, para que se vea que el recálculo corrió. También lista los Ids nuevos. Antes, si no había parejas, la línea no aparecía.</v>
+      </c>
+      <c r="E371" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B372" t="str">
+        <v>07:50</v>
+      </c>
+      <c r="C372" t="str">
+        <v>Histórico: Pendiente sí se da de alta</v>
+      </c>
+      <c r="D372" t="str">
+        <v>El upload de tesorería (histórico, tesorería abierta y cierre) da de alta Status Pendiente. Lo único que no entra es Anulado (si el Id ya existía, se elimina). Así entran p. ej. 10003427 y 10003428 (ajustes de caja MP y Galicia del 27/09).</v>
+      </c>
+      <c r="E372" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B373" t="str">
+        <v>07:55</v>
+      </c>
+      <c r="C373" t="str">
+        <v>Despliegue v2.59 producción</v>
+      </c>
+      <c r="D373" t="str">
+        <v>Push a main y Vercel --prod: tesorería histórica da de alta Pendiente (Anulado no); el cartel muestra Sugeridos por caja aunque sea 0 y lista Ids nuevos. APP_VERSION 2.59.</v>
+      </c>
+      <c r="E373" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E370"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E373"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6729,7 +6780,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja y recálcula los sugeridos de Conciliación en cada canal, igual que si se cargara tesorería solapa por solapa. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. La solapa activa (Flujo por mes, Todas las transacciones, Evolución, Estado Financiero) se marca con etiqueta Activo y un contorno más visible. Al volver a Home se recargan tesorería, cajas y tipos de cambio (no queda el dato viejo en memoria). Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja y recálcula los sugeridos de Conciliación en cada canal; el cartel muestra Sugeridos por caja aunque sea 0, y los Ids nuevos. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. La solapa activa (Flujo por mes, Todas las transacciones, Evolución, Estado Financiero) se marca con etiqueta Activo y un contorno más visible. Al volver a Home se recargan tesorería, cajas y tipos de cambio (no queda el dato viejo en memoria). Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -7193,7 +7244,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), si un movimiento banco temporal ya no viene en el archivo (cheque en proceso, PDF viejo) se retira; tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos, cuántos cambiaron, cuántos ya estaban, cuántas sugerencias se reconocieron y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), si un movimiento banco temporal ya no viene en el archivo (cheque en proceso, PDF viejo) se retira; tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -7201,7 +7252,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Pendiente nuevo no se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -7380,7 +7431,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8330,7 +8381,7 @@
         <v>22/09/2026</v>
       </c>
       <c r="C86" t="str">
-        <v>Despliegue v2.42: tesorería histórica movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) reparte MP/Galicia ARS/USD y cajas físicas; popup de resumen de carga (nuevos, actualizados, sin cambios, sugerencias, omitidos); si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Status Pendiente (Pendiente nuevo no se da de alta). Producción Vercel.</v>
+        <v>Despliegue v2.42: tesorería histórica movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) reparte MP/Galicia ARS/USD y cajas físicas; popup de resumen de carga (nuevos, actualizados, sin cambios, sugerencias, omitidos); si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Producción Vercel.</v>
       </c>
     </row>
     <row r="87">
@@ -8509,9 +8560,20 @@
         <v>Despliegue v2.58: después del último corte, el saldo de período Galicia se arma con los movimientos del Excel (CC/CCE); el PDF del banco solo verifica y no da de alta movimientos; el Excel retira del extracto lo que ya no trae. Extractos ya cargados no se recalculan. sql/supabase_eb_guardar_saldos_regla_movimientos.sql y sql/supabase_cb_retirar_extracto_banco_ausente.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>2.59</v>
+      </c>
+      <c r="B103" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Despliegue v2.59: tesorería histórica da de alta Status Pendiente (Anulado no entra); el cartel de carga muestra Sugeridos por caja aunque sea 0 y lista los Ids nuevos. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C102"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C103"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.60: No requiere y duplicados se marcan o descartan en lote.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E373"/>
+  <dimension ref="A1:E378"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6752,9 +6752,94 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B374" t="str">
+        <v>08:20</v>
+      </c>
+      <c r="C374" t="str">
+        <v>Solo banco: No requiere en lote (MP y Galicia)</v>
+      </c>
+      <c r="D374" t="str">
+        <v>En Solo banco de Mercado Pago, Galicia ARS y Galicia USD se pueden seleccionar varios movimientos o todos los listados y marcarlos No requiere conciliación con una sola justificación. No se borran; van a la solapa No requiere. rpc cb_marcar_no_requiere_conciliacion_lote y ampliación a Galicia.</v>
+      </c>
+      <c r="E374" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B375" t="str">
+        <v>08:25</v>
+      </c>
+      <c r="C375" t="str">
+        <v>No requiere en lote: sin timeout</v>
+      </c>
+      <c r="D375" t="str">
+        <v>Marcar muchos Solo banco (p. ej. 460) ya no corta por timeout: una sola actualización por bloque de 80 y el botón muestra el avance. sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql.</v>
+      </c>
+      <c r="E375" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B376" t="str">
+        <v>08:40</v>
+      </c>
+      <c r="C376" t="str">
+        <v>Solo sistema: No requiere en lote</v>
+      </c>
+      <c r="D376" t="str">
+        <v>En Solo sistema (Mercado Pago, Galicia ARS y Galicia USD) se pueden seleccionar varios o todos los listados y marcarlos No requiere conciliación con una justificación. No se borran; van a la solapa No requiere (columna Origen: Extracto o Tesorería). sql/supabase_cb_no_requiere_conciliacion_sistema.sql.</v>
+      </c>
+      <c r="E376" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B377" t="str">
+        <v>08:50</v>
+      </c>
+      <c r="C377" t="str">
+        <v>Potenciales duplicados: descartar en lote</v>
+      </c>
+      <c r="D377" t="str">
+        <v>En Potenciales duplicados se pueden seleccionar varios grupos o todos los listados y descartarlos de una vez (confirmación única). Van a Duplicados descartados y se puede deshacer. sql/supabase_cb_dup_tesoreria_descartar_lote.sql.</v>
+      </c>
+      <c r="E377" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B378" t="str">
+        <v>08:55</v>
+      </c>
+      <c r="C378" t="str">
+        <v>Despliegue v2.60 producción</v>
+      </c>
+      <c r="D378" t="str">
+        <v>Push a main y Vercel --prod: Solo banco y Solo sistema (MP y Galicia) con selección múltiple para No requiere conciliación; Potenciales duplicados se descartan en lote. APP_VERSION 2.60.</v>
+      </c>
+      <c r="E378" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E373"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E378"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7244,7 +7329,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), si un movimiento banco temporal ya no viene en el archivo (cheque en proceso, PDF viejo) se retira; tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago Solo banco se puede marcar No requiere conciliación (justificación; no se borra; solapa No requiere; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), si un movimiento banco temporal ya no viene en el archivo (cheque en proceso, PDF viejo) se retira; tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -7431,7 +7516,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8571,9 +8656,20 @@
         <v>Despliegue v2.59: tesorería histórica da de alta Status Pendiente (Anulado no entra); el cartel de carga muestra Sugeridos por caja aunque sea 0 y lista los Ids nuevos. Producción Vercel.</v>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>2.60</v>
+      </c>
+      <c r="B104" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Despliegue v2.60: Conciliación — Solo banco y Solo sistema (Mercado Pago y Galicia) permiten marcar No requiere de a varios o todos; Potenciales duplicados se descartan en lote. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C103"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C104"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8775,7 +8871,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos; quedan en Tesorería eliminada). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos; quedan en Tesorería eliminada). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.61: A eliminar solo Pendiente; ratios del Flujo sobre Ingresos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E378"/>
+  <dimension ref="A1:E383"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6837,9 +6837,94 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B379" t="str">
+        <v>09:10</v>
+      </c>
+      <c r="C379" t="str">
+        <v>A eliminar: Pendiente del histórico</v>
+      </c>
+      <c r="D379" t="str">
+        <v>Al cargar tesoreria_*.xlsx, un Id Pendiente que había entrado por el histórico y ya no viene (p. ej. 10003427 en Mercado Pago) pasa a A eliminar. El histórico confirmado no se marca. sql/supabase_cb_tesoreria_abierta_pendiente_historico.sql.</v>
+      </c>
+      <c r="E379" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B380" t="str">
+        <v>09:20</v>
+      </c>
+      <c r="C380" t="str">
+        <v>A eliminar: solo Status Pendiente</v>
+      </c>
+      <c r="D380" t="str">
+        <v>La baja solo aplica a registros Pendiente (caja abierta), entre por tesorería o por el histórico: se pueden anular en el sistema y desaparecer. Confirmado nunca va a A eliminar. El cierre no entra. sql/supabase_cb_tesoreria_abierta_pendiente_historico.sql.</v>
+      </c>
+      <c r="E380" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B381" t="str">
+        <v>09:25</v>
+      </c>
+      <c r="C381" t="str">
+        <v>Flujo: Egresos / Ingresos simple</v>
+      </c>
+      <c r="D381" t="str">
+        <v>La última columna del Flujo por mes pasa a Egresos ÷ Ingresos (mismas columnas de la tabla). Ya no usa el Flujo Operativo Generado ni resta comisiones. Total, proyección y Excel alineados.</v>
+      </c>
+      <c r="E381" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B382" t="str">
+        <v>09:30</v>
+      </c>
+      <c r="C382" t="str">
+        <v>Flujo: ratios sobre Ingresos</v>
+      </c>
+      <c r="D382" t="str">
+        <v>Costo dir./Ingresos, Costo ind./Ingresos y Costo total/Ingreso total usan siempre Ingresos como denominador. Numeradores: §2, §3 y Egresos (costo total). Ya no se divide por el Flujo Operativo Generado.</v>
+      </c>
+      <c r="E382" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B383" t="str">
+        <v>09:35</v>
+      </c>
+      <c r="C383" t="str">
+        <v>Despliegue v2.61 producción</v>
+      </c>
+      <c r="D383" t="str">
+        <v>Push a main y Vercel --prod: A eliminar solo Pendiente (tesorería o histórico); Confirmado no se elimina. Flujo: Costo dir., Costo ind. y Costo total sobre Ingresos. APP_VERSION 2.61.</v>
+      </c>
+      <c r="E383" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E378"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E383"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6865,7 +6950,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja y recálcula los sugeridos de Conciliación en cada canal; el cartel muestra Sugeridos por caja aunque sea 0, y los Ids nuevos. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./ind. ÷ FLUJO OPERATIVO GENERADO (§2/§3); Costo total/Ingreso total = total egresos operativos ÷ FLUJO OPERATIVO GENERADO. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. La solapa activa (Flujo por mes, Todas las transacciones, Evolución, Estado Financiero) se marca con etiqueta Activo y un contorno más visible. Al volver a Home se recargan tesorería, cajas y tipos de cambio (no queda el dato viejo en memoria). Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja y recálcula los sugeridos de Conciliación en cada canal; el cartel muestra Sugeridos por caja aunque sea 0, y los Ids nuevos. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. La solapa activa (Flujo por mes, Todas las transacciones, Evolución, Estado Financiero) se marca con etiqueta Activo y un contorno más visible. Al volver a Home se recargan tesorería, cajas y tipos de cambio (no queda el dato viejo en memoria). Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -6905,7 +6990,7 @@
         <v>Egresos / Ingresos</v>
       </c>
       <c r="B7" t="str">
-        <v>Columna Egresos (icono ayuda) / Ingresos: porcentaje (egresos sin comisiones) sobre ingresos. Ayuda al clic: "Egresos - Comisiones por Venta / Ingresos".</v>
+        <v>Ratios del Flujo por mes con denominador siempre = columna Ingresos: Costo dir. / Ingresos (§2), Costo ind. / Ingresos (§3) y Costo total / Ingreso total (Egresos ÷ Ingresos). Total, proyección y Excel con la misma fórmula.</v>
       </c>
     </row>
     <row r="8">
@@ -7329,7 +7414,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), si un movimiento banco temporal ya no viene en el archivo (cheque en proceso, PDF viejo) se retira; tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada; el cierre de caja y el histórico no entran en esa lógica. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), si un movimiento banco temporal ya no viene en el archivo (cheque en proceso, PDF viejo) se retira; tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -7337,7 +7422,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Tesorería abierta: los Ids que ya no vienen van a A eliminar. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Solo Status Pendiente (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -7516,7 +7601,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C105"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8667,9 +8752,20 @@
         <v>Despliegue v2.60: Conciliación — Solo banco y Solo sistema (Mercado Pago y Galicia) permiten marcar No requiere de a varios o todos; Potenciales duplicados se descartan en lote. Producción Vercel.</v>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>2.61</v>
+      </c>
+      <c r="B105" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Despliegue v2.61: A eliminar solo Status Pendiente (caja abierta, tesorería o histórico); Confirmado nunca. Flujo de caja: Costo dir./Ingresos, Costo ind./Ingresos y Costo total/Ingreso total con denominador Ingresos. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C104"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C105"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8871,7 +8967,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería abierta (tesoreria_*.xlsx con Id), los Ids que ya no vienen en el archivo van a la solapa A eliminar para confirmar la baja definitiva (no se borran solos; quedan en Tesorería eliminada). En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.62: Flujo tipo Dashboard, gráfico G/P y PDF de una página.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E383"/>
+  <dimension ref="A1:E389"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -6922,9 +6922,111 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B384" t="str">
+        <v>12:15</v>
+      </c>
+      <c r="C384" t="str">
+        <v>Flujo: vista Dashboard (Everfit)</v>
+      </c>
+      <c r="D384" t="str">
+        <v>Flujo de caja replica la vista Dashboard de Everfit: filtro Período (último año / año / todo), gráfico G/P Mensual (barras + tendencia) y tabla con meses en columnas, filas Ingresos/Egresos/G/P y Ratios del Negocio (Comisiones/Ventas, Costo dir., Costo ind., Costo total). PDF con chips de filtros activos remarcados. scripts/lib/fornitalia-flujo-dashboard-ux.js.</v>
+      </c>
+      <c r="E384" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B385" t="str">
+        <v>12:20</v>
+      </c>
+      <c r="C385" t="str">
+        <v>Flujo: Total de ratios sin proyección</v>
+      </c>
+      <c r="D385" t="str">
+        <v>En Ratios del Negocio la columna Total suma solo meses reales. Las columnas Proy. se ven, pero no entran al porcentaje total.</v>
+      </c>
+      <c r="E385" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B386" t="str">
+        <v>12:30</v>
+      </c>
+      <c r="C386" t="str">
+        <v>PDF Flujo en una sola página</v>
+      </c>
+      <c r="D386" t="str">
+        <v>El PDF de Flujo entra en una hoja A4 apaisada: se achica el gráfico G/P si ocupa de más y se escala el reporte para que cabecera, filtros, tarjetas, gráfico y tabla queden juntos.</v>
+      </c>
+      <c r="E386" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B387" t="str">
+        <v>12:35</v>
+      </c>
+      <c r="C387" t="str">
+        <v>PDF Flujo: gráfico y columnas</v>
+      </c>
+      <c r="D387" t="str">
+        <v>El gráfico G/P del PDF vuelve a un tamaño usable (no miniatura). La tabla ajusta columnas al contenido y queda centrada, homogénea, debajo del gráfico en la misma hoja.</v>
+      </c>
+      <c r="E387" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B388" t="str">
+        <v>12:44</v>
+      </c>
+      <c r="C388" t="str">
+        <v>PDF Flujo: gráfico a todo el ancho</v>
+      </c>
+      <c r="D388" t="str">
+        <v>El gráfico G/P del PDF se estira de margen a margen (sangría chica a cada lado) y gana altura con el espacio libre de la hoja, sin salir de una página.</v>
+      </c>
+      <c r="E388" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B389" t="str">
+        <v>13:05</v>
+      </c>
+      <c r="C389" t="str">
+        <v>Despliegue v2.62 producción</v>
+      </c>
+      <c r="D389" t="str">
+        <v>Push a main y Vercel --prod: Flujo tipo Dashboard (período, gráfico G/P, tabla con meses en columnas, PDF una página). APP_VERSION 2.62.</v>
+      </c>
+      <c r="E389" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E383"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E389"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6950,7 +7052,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Tabla de caja operativa alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF (categoría + cuenta + tipo → ítem/subítem). Incluye Status Pendiente. No hay carga de extracto normalizado ni solapa Errores en esta vista. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas (Conciliación + Cajas físicas) según la columna Caja y recálcula los sugeridos de Conciliación en cada canal; el cartel muestra Sugeridos por caja aunque sea 0, y los Ids nuevos. Columnas Ingresos, Egresos y G/P operativo (sin apertura/cierre ni traspasos). Comisiones/Ventas % por subítems EF; Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. Proyección de ratios. Meses excluidos por Configuración → Inclusión por mes no aparecen en filas ni totales. Clic en un encabezado ordena asc/desc (Mes-Año, importes y ratios). Icono de ayuda. La solapa activa (Flujo por mes, Todas las transacciones, Evolución, Estado Financiero) se marca con etiqueta Activo y un contorno más visible. Al volver a Home se recargan tesorería, cajas y tipos de cambio (no queda el dato viejo en memoria). Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total de ratios no incluye proyectados. Proyección como columnas extra si el período incluye el mes en curso. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico a tamaño usable y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -6958,7 +7060,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Tres tarjetas: Ingresos totales, Egresos totales y G/P operativo (misma base operativa que la tabla Flujo por mes), en ARS o USD según selector.</v>
+        <v>Tres tarjetas: Ingresos totales, Egresos totales y G/P operativo (misma base operativa que la tabla Flujo por mes y el filtro Período), en ARS o USD según selector.</v>
       </c>
     </row>
     <row r="4">
@@ -6982,7 +7084,7 @@
         <v>Comisiones/Ventas %</v>
       </c>
       <c r="B6" t="str">
-        <v>Columna: egresos con ef_subitem «Comisiones por Ventas» ÷ ingresos con ef_subitem «Cobranzas por Ventas (Efectivo neto ingresado)» del mes (subítems canónicos EF; alias cortos se normalizan). Sin ef_subitem la fila no entra al ratio. Ayuda al clic en icono de columna e informe PDF (template-flujo-informe-pdf).</v>
+        <v>Fila de ratios: egresos con ef_subitem «Comisiones por Ventas» ÷ ingresos con ef_subitem «Cobranzas por Ventas (Efectivo neto ingresado)» del mes (subítems canónicos EF; alias cortos se normalizan). Sin ef_subitem no entra al ratio. Flecha vs mes anterior. Ayuda e informe PDF (template-flujo-informe-pdf).</v>
       </c>
     </row>
     <row r="7">
@@ -6990,7 +7092,7 @@
         <v>Egresos / Ingresos</v>
       </c>
       <c r="B7" t="str">
-        <v>Ratios del Flujo por mes con denominador siempre = columna Ingresos: Costo dir. / Ingresos (§2), Costo ind. / Ingresos (§3) y Costo total / Ingreso total (Egresos ÷ Ingresos). Total, proyección y Excel con la misma fórmula.</v>
+        <v>Filas de ratios del Flujo (denominador siempre = Ingresos): Costo dir. / Ingresos (§2), Costo ind. / Ingresos (§3) y Costo total / Ingreso total (Egresos ÷ Ingresos). La columna Total de ratios usa solo meses reales (sin proyectados). PDF y Excel con la misma fórmula sobre reales.</v>
       </c>
     </row>
     <row r="8">
@@ -7014,7 +7116,7 @@
         <v>Detalle por mes</v>
       </c>
       <c r="B10" t="str">
-        <v>Clic en una fila de mes abre modal con dos solapas: por categoría (matriz) y por cuenta (matriz).</v>
+        <v>Clic en el encabezado o un importe del mes abre modal con dos solapas: por categoría (matriz) y por cuenta (matriz).</v>
       </c>
     </row>
     <row r="11">
@@ -7601,7 +7703,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C105"/>
+  <dimension ref="A1:C106"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8763,9 +8865,20 @@
         <v>Despliegue v2.61: A eliminar solo Status Pendiente (caja abierta, tesorería o histórico); Confirmado nunca. Flujo de caja: Costo dir./Ingresos, Costo ind./Ingresos y Costo total/Ingreso total con denominador Ingresos. Producción Vercel.</v>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>2.62</v>
+      </c>
+      <c r="B106" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Despliegue v2.62: Flujo de caja tipo Dashboard — filtro Período (último año / año / todo), gráfico G/P Mensual, tabla con meses en columnas e Ingresos/Egresos/G/P + ratios; Total de ratios sin proyectados; PDF A4 apaisado de una página con gráfico de margen a margen y filtros activos remarcados. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C106"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8813,7 +8926,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (Flujo por mes, Resumen, alertas, modal By Categoría / By Cuenta, gráficos de serie mensual). Incluye formatos de moneda y visualizaciones.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, alertas, modal By Categoría / By Cuenta). Incluye PDF de una página con filtros activos y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>
@@ -9074,7 +9187,7 @@
         <v>Frontend</v>
       </c>
       <c r="B2" t="str">
-        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas), Saldos extractos, Impuestos y Matriz EF en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.*, fornitalia-saldos-extractos.*, fornitalia-impuestos.* y fornitalia-matriz-ef.*). Ayuda de menús en scripts/lib/fornitalia-help.js. Novedades de cada versión: scripts/lib/fornitalia-release-blurb.js → fornitalia-release.json. Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia ARS/USD con pdf.js en el navegador.</v>
+        <v>Página dashboard-flujo-caja.html (HTML/CSS/JS). Flujo tipo Dashboard en scripts/lib/fornitalia-flujo-dashboard-ux.js. Gestión de Proyectos, Conciliación Bancaria, Cajas (físicas), Saldos extractos, Impuestos y Matriz EF en componentes aparte (scripts/lib/fornitalia-gestion-proyectos.*, fornitalia-conciliacion-bancaria.*, fornitalia-cajas-fisicas.*, fornitalia-saldos-extractos.*, fornitalia-impuestos.* y fornitalia-matriz-ef.*). Ayuda de menús en scripts/lib/fornitalia-help.js. Novedades de cada versión: scripts/lib/fornitalia-release-blurb.js → fornitalia-release.json. Sin framework; llamadas a Supabase desde el cliente. PDFs Galicia ARS/USD con pdf.js en el navegador.</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
v2.63: alta de perfiles en Seguridad para asignar permisos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E389"/>
+  <dimension ref="A1:E391"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7024,9 +7024,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="390">
+      <c r="A390" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B390" t="str">
+        <v>13:20</v>
+      </c>
+      <c r="C390" t="str">
+        <v>Seguridad: alta de perfiles</v>
+      </c>
+      <c r="D390" t="str">
+        <v>En Seguridad, botón Nuevo perfil para crear roles además de Admin/Encargado/Visor. El perfil nace sin permisos; después se asignan en la grilla y a los usuarios. Se puede eliminar un perfil custom si nadie lo usa. sql/supabase_app_role_gestion_assign_roles.sql.</v>
+      </c>
+      <c r="E390" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B391" t="str">
+        <v>13:25</v>
+      </c>
+      <c r="C391" t="str">
+        <v>Despliegue v2.63 producción</v>
+      </c>
+      <c r="D391" t="str">
+        <v>Push a main y Vercel --prod: Seguridad con alta de perfiles a medida y asignación de permisos. APP_VERSION 2.63.</v>
+      </c>
+      <c r="E391" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E389"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E391"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7052,7 +7086,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total de ratios no incluye proyectados. Proyección como columnas extra si el período incluye el mes en curso. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico a tamaño usable y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total de ratios no incluye proyectados. Proyección como columnas extra si el período incluye el mes en curso. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -7236,7 +7270,7 @@
         <v>Seguridad y roles</v>
       </c>
       <c r="B25" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos granulares desde Supabase: ver_solapa_* (cada solapa del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo por mes + exportar/reportes; un admin puede activar solapas y menús sueltos en Seguridad. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos granulares desde Supabase: ver_solapa_* (cada solapa del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo por mes + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
       </c>
     </row>
     <row r="26">
@@ -7703,7 +7737,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C107"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8876,9 +8910,20 @@
         <v>Despliegue v2.62: Flujo de caja tipo Dashboard — filtro Período (último año / año / todo), gráfico G/P Mensual, tabla con meses en columnas e Ingresos/Egresos/G/P + ratios; Total de ratios sin proyectados; PDF A4 apaisado de una página con gráfico de margen a margen y filtros activos remarcados. Producción Vercel.</v>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>2.63</v>
+      </c>
+      <c r="B107" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Despliegue v2.63: Seguridad — Nuevo perfil para crear roles además de Admin/Encargado/Visor; permisos por grilla; se puede borrar un perfil a medida si nadie lo usa. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C106"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C107"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9038,7 +9083,7 @@
         <v>Seguridad y roles (dashboard)</v>
       </c>
       <c r="B11" t="str">
-        <v>Autenticación email/anónimo, roles Admin/Encargado/Visor, permisos granulares por solapa/menú/acción en Supabase (RPC y RLS), pantalla Seguridad para asignar roles y toggles por ítem (incluido Visor).</v>
+        <v>Autenticación email/anónimo, roles Admin/Encargado/Visor y perfiles a medida, permisos granulares por solapa/menú/acción en Supabase (RPC y RLS), pantalla Seguridad para crear perfiles, asignar roles y toggles por ítem (incluido Visor).</v>
       </c>
       <c r="C11">
         <v>18</v>

</xml_diff>

<commit_message>
v2.64: Flujo de caja como inicio según permiso, y recuperar contraseña.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E391"/>
+  <dimension ref="A1:E394"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7058,9 +7058,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="392">
+      <c r="A392" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B392" t="str">
+        <v>13:35</v>
+      </c>
+      <c r="C392" t="str">
+        <v>Login: recuperar contraseña</v>
+      </c>
+      <c r="D392" t="str">
+        <v>En el login, «¿Olvidaste tu contraseña?» envía un enlace por email. Al abrir el mail se elige una clave nueva y se entra. Site URL / Redirect URLs en docs/SUPABASE_REQUISITOS.md.</v>
+      </c>
+      <c r="E392" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B393" t="str">
+        <v>13:40</v>
+      </c>
+      <c r="C393" t="str">
+        <v>Home es Flujo de caja con permiso</v>
+      </c>
+      <c r="D393" t="str">
+        <v>El ítem Home del menú pasa a Flujo de caja (icono de $). Solo se ve con ver_solapa_flujo. Al entrar, si tiene ese permiso abre Flujo; si no, el primer menú lateral al que tenga acceso. sql/supabase_permiso_flujo_caja_menu.sql.</v>
+      </c>
+      <c r="E393" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B394" t="str">
+        <v>08:09</v>
+      </c>
+      <c r="C394" t="str">
+        <v>Despliegue v2.64 producción</v>
+      </c>
+      <c r="D394" t="str">
+        <v>Push a main y Vercel --prod: Flujo de caja como primer menú (con permiso); si no lo tiene, entra al primer menú habilitado; recuperar contraseña en el login. APP_VERSION 2.64.</v>
+      </c>
+      <c r="E394" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E391"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E394"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7262,7 +7313,7 @@
         <v>Menú lateral</v>
       </c>
       <c r="B24" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Home, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage. Home es el Flujo de caja: cada vez que se vuelve ahí se recargan tesorería, cajas y tipos de cambio.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Flujo de caja (permiso ver_solapa_flujo; icono $), Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage. Al iniciar sesión se abre Flujo de caja si el usuario lo tiene; si no, el primer menú lateral permitido. Cada vez que se vuelve a Flujo se recargan tesorería, cajas y tipos de cambio.</v>
       </c>
     </row>
     <row r="25">
@@ -7270,7 +7321,7 @@
         <v>Seguridad y roles</v>
       </c>
       <c r="B25" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Permisos granulares desde Supabase: ver_solapa_* (cada solapa del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo por mes + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Recuperar contraseña desde el login (enlace por email). Permisos granulares desde Supabase: ver_solapa_flujo (menú y solapa Flujo de caja), ver_solapa_* (resto de solapas del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo de caja + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
       </c>
     </row>
     <row r="26">
@@ -7278,7 +7329,7 @@
         <v>Registro y contraseña</v>
       </c>
       <c r="B26" t="str">
-        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español en pantalla; ayuda bajo el campo y mínimo 8 caracteres en el formulario.</v>
+        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español. Ayuda bajo el campo y mínimo 8 caracteres. En el login, «¿Olvidaste tu contraseña?» envía un enlace por email para elegir una clave nueva (revisar spam, sobre todo Hotmail).</v>
       </c>
     </row>
     <row r="27">
@@ -7486,7 +7537,7 @@
         <v>Botones e iconos unificados</v>
       </c>
       <c r="B52" t="str">
-        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, home, engranaje, usuario), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG. Cada vista de menú muestra en la cabecera el mismo icono que el ítem del sidebar (Home, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad, Mi perfil).</v>
+        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, Flujo de caja / $, engranaje, usuario), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG. Cada vista de menú muestra en la cabecera el mismo icono que el ítem del sidebar (Flujo de caja, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad, Mi perfil).</v>
       </c>
     </row>
     <row r="53">
@@ -7737,7 +7788,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C107"/>
+  <dimension ref="A1:C108"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8921,9 +8972,20 @@
         <v>Despliegue v2.63: Seguridad — Nuevo perfil para crear roles además de Admin/Encargado/Visor; permisos por grilla; se puede borrar un perfil a medida si nadie lo usa. Producción Vercel.</v>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>2.64</v>
+      </c>
+      <c r="B108" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Despliegue v2.64: Home pasa a Flujo de caja (icono $; permiso ver_solapa_flujo); al entrar se abre Flujo si lo tiene y si no el primer menú lateral habilitado; recuperar contraseña desde el login. sql/supabase_permiso_flujo_caja_menu.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C107"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C108"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9083,7 +9145,7 @@
         <v>Seguridad y roles (dashboard)</v>
       </c>
       <c r="B11" t="str">
-        <v>Autenticación email/anónimo, roles Admin/Encargado/Visor y perfiles a medida, permisos granulares por solapa/menú/acción en Supabase (RPC y RLS), pantalla Seguridad para crear perfiles, asignar roles y toggles por ítem (incluido Visor).</v>
+        <v>Autenticación email/anónimo, recuperar contraseña por email, roles Admin/Encargado/Visor y perfiles a medida, permisos granulares por solapa/menú/acción (Flujo de caja como primer menú si hay permiso), pantalla Seguridad para crear perfiles, asignar roles y toggles por ítem (incluido Visor).</v>
       </c>
       <c r="C11">
         <v>18</v>

</xml_diff>

<commit_message>
v2.65: Galicia no retira Imputado al recargar el extracto.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E394"/>
+  <dimension ref="A1:E396"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7109,9 +7109,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="395">
+      <c r="A395" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B395" t="str">
+        <v>09:54</v>
+      </c>
+      <c r="C395" t="str">
+        <v>Galicia: no retirar Imputado</v>
+      </c>
+      <c r="D395" t="str">
+        <v>Al cargar Extracto_CC/CCE ya no se borran movimientos Imputados aunque el Excel de la ventana no los traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso) y ahora no viene; si después llega Imputado, se confirma. sql/supabase_cb_retirar_solo_no_imputado.sql.</v>
+      </c>
+      <c r="E395" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B396" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C396" t="str">
+        <v>Despliegue v2.65 producción</v>
+      </c>
+      <c r="D396" t="str">
+        <v>Push a main y Vercel --prod: Galicia no retira Imputado al recargar el extracto; solo En proceso (u otro no imputado) ausente en este Excel. APP_VERSION 2.65.</v>
+      </c>
+      <c r="E396" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E394"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E396"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7601,7 +7635,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), si un movimiento banco temporal ya no viene en el archivo (cheque en proceso, PDF viejo) se retira; tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -7788,7 +7822,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C108"/>
+  <dimension ref="A1:C109"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -8983,9 +9017,20 @@
         <v>Despliegue v2.64: Home pasa a Flujo de caja (icono $; permiso ver_solapa_flujo); al entrar se abre Flujo si lo tiene y si no el primer menú lateral habilitado; recuperar contraseña desde el login. sql/supabase_permiso_flujo_caja_menu.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>2.65</v>
+      </c>
+      <c r="B109" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Despliegue v2.65: Conciliación Galicia — un movimiento Imputado no se borra al recargar el extracto; solo se retira si al registrarse no era Imputado (p. ej. En proceso) y este Excel ya no lo trae. sql/supabase_cb_retirar_solo_no_imputado.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C108"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C109"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9187,7 +9232,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.66: buscar de conciliación con coma decimal e importe exacto.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E396"/>
+  <dimension ref="A1:E398"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7143,9 +7143,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="397">
+      <c r="A397" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B397" t="str">
+        <v>10:36</v>
+      </c>
+      <c r="C397" t="str">
+        <v>Buscar importe con coma decimal</v>
+      </c>
+      <c r="D397" t="str">
+        <v>En Conciliación Bancaria, el buscar trata la coma como decimal (15,71 o 1.234,56) y filtra el monto exacto (también crédito/débito y el signo). El buscar de conciliación manual usa la misma regla.</v>
+      </c>
+      <c r="E397" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B398" t="str">
+        <v>10:42</v>
+      </c>
+      <c r="C398" t="str">
+        <v>Despliegue v2.66 producción</v>
+      </c>
+      <c r="D398" t="str">
+        <v>Push a main y Vercel --prod: buscar de Conciliación Bancaria con coma decimal e importe exacto. APP_VERSION 2.66.</v>
+      </c>
+      <c r="E398" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E396"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E398"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7635,7 +7669,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar y reconoce coma decimal (15,71) para el importe exacto. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="61">
@@ -7822,7 +7856,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9028,9 +9062,20 @@
         <v>Despliegue v2.65: Conciliación Galicia — un movimiento Imputado no se borra al recargar el extracto; solo se retira si al registrarse no era Imputado (p. ej. En proceso) y este Excel ya no lo trae. sql/supabase_cb_retirar_solo_no_imputado.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>2.66</v>
+      </c>
+      <c r="B110" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Despliegue v2.66: Conciliación Bancaria — el buscar reconoce coma decimal (15,71 / 1.234,56) y filtra el importe exacto; igual en conciliación manual. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C109"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C110"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.67: ratios Sueldos y Costo Financiero MP; PDF Flujo en una página.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E398"/>
+  <dimension ref="A1:E401"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7177,16 +7177,67 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="399">
+      <c r="A399" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B399" t="str">
+        <v>13:22</v>
+      </c>
+      <c r="C399" t="str">
+        <v>Ratios Sueldos y Costo Financiero MP</v>
+      </c>
+      <c r="D399" t="str">
+        <v>Ratios del Negocio en Flujo de caja: Sueldos / Ingresos (egresos categoría Sueldos, sin comisiones de venta) y Costo Financiero MP / Ventas MP (ef_subitem Costo Financiero Mercado Pago ÷ cobranzas por ventas de la caja Mercado Pago). PDF y Excel.</v>
+      </c>
+      <c r="E399" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B400" t="str">
+        <v>14:27</v>
+      </c>
+      <c r="C400" t="str">
+        <v>PDF Flujo: no repetir fila en página 2</v>
+      </c>
+      <c r="D400" t="str">
+        <v>Con los dos ratios nuevos el PDF se iba a una segunda hoja: Chrome reimprimía el encabezado (y el Total G/P, igual a la fila G/P). Queda una sola A4 apaisada: se saca esa fila duplicada, el encabezado no se repite y el recorte usa zoom para que no quede resto.</v>
+      </c>
+      <c r="E400" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B401" t="str">
+        <v>14:32</v>
+      </c>
+      <c r="C401" t="str">
+        <v>Despliegue v2.67 producción</v>
+      </c>
+      <c r="D401" t="str">
+        <v>Push a main y Vercel --prod: Ratios Sueldos / Ingresos y Costo Financiero MP / Ventas MP; PDF de Flujo en una sola hoja sin fila repetida. APP_VERSION 2.67.</v>
+      </c>
+      <c r="E401" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E398"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E401"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B71"/>
+  <dimension ref="A1:B72"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -7205,7 +7256,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total de ratios no incluye proyectados. Proyección como columnas extra si el período incluye el mes en curso. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total de ratios no incluye proyectados. Proyección como columnas extra si el período incluye el mes en curso. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -7242,527 +7293,535 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Egresos / Ingresos</v>
+        <v>Sueldos / Ingresos y Costo Fin. MP</v>
       </c>
       <c r="B7" t="str">
-        <v>Filas de ratios del Flujo (denominador siempre = Ingresos): Costo dir. / Ingresos (§2), Costo ind. / Ingresos (§3) y Costo total / Ingreso total (Egresos ÷ Ingresos). La columna Total de ratios usa solo meses reales (sin proyectados). PDF y Excel con la misma fórmula sobre reales.</v>
+        <v>Ratios del Negocio: Sueldos / Ingresos (egresos de categoría Sueldos, sin comisiones de venta) y Costo Financiero MP / Ventas MP (ef_subitem Costo Financiero Mercado Pago ÷ cobranzas por ventas solo de caja Mercado Pago). PDF y Excel.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Categorías Sueldos y Comisiones</v>
+        <v>Egresos / Ingresos</v>
       </c>
       <c r="B8" t="str">
-        <v>Categoría Sueldos partida en dos: Sueldos (solo sueldos) y Comisiones (según descripción/cat_desc). Sin doble imputación.</v>
+        <v>Filas de ratios del Flujo: Sueldos / Ingresos y Costo dir. / Ingresos (§2), Costo ind. / Ingresos (§3) y Costo total / Ingreso total (Egresos ÷ Ingresos) usan Ingresos como denominador. Costo Financiero MP / Ventas MP usa cobranzas de la caja Mercado Pago. La columna Total de ratios usa solo meses reales (sin proyectados). PDF y Excel con la misma fórmula sobre reales.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Detección comisiones</v>
+        <v>Categorías Sueldos y Comisiones</v>
       </c>
       <c r="B9" t="str">
-        <v>Incluye variante "Comisones" en descripción para clasificar como Comisiones.</v>
+        <v>Categoría Sueldos partida en dos: Sueldos (solo sueldos) y Comisiones (según descripción/cat_desc). Sin doble imputación.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Detalle por mes</v>
+        <v>Detección comisiones</v>
       </c>
       <c r="B10" t="str">
-        <v>Clic en el encabezado o un importe del mes abre modal con dos solapas: por categoría (matriz) y por cuenta (matriz).</v>
+        <v>Incluye variante "Comisones" en descripción para clasificar como Comisiones.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Por categoría (matriz)</v>
+        <v>Detalle por mes</v>
       </c>
       <c r="B11" t="str">
-        <v>Solapa del modal: detalle agrupado por nueva_categoria con fallback a extracto (categoriaDistribucionFlujo); bloques Ingresos / Costo directo / indirecto / Otros costos; Ver para listado de transacciones.</v>
+        <v>Clic en el encabezado o un importe del mes abre modal con dos solapas: por categoría (matriz) y por cuenta (matriz).</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Por cuenta (matriz)</v>
+        <v>Por categoría (matriz)</v>
       </c>
       <c r="B12" t="str">
-        <v>Solapa del modal: detalle agrupado por nueva_cuenta_contable con fallback (cuentaDistribucionFlujo); misma estructura y botón Gráfico.</v>
+        <v>Solapa del modal: detalle agrupado por nueva_categoria con fallback a extracto (categoriaDistribucionFlujo); bloques Ingresos / Costo directo / indirecto / Otros costos; Ver para listado de transacciones.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Gráfico serie mensual</v>
+        <v>Por cuenta (matriz)</v>
       </c>
       <c r="B13" t="str">
-        <v>Botón "Gráfico" en cada fila de categoría o cuenta de matriz: modal con serie mensual (neto por mes) para esa clave, en la moneda seleccionada.</v>
+        <v>Solapa del modal: detalle agrupado por nueva_cuenta_contable con fallback (cuentaDistribucionFlujo); misma estructura y botón Gráfico.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Detalle transacciones</v>
+        <v>Gráfico serie mensual</v>
       </c>
       <c r="B14" t="str">
-        <v>En cada agrupación, listado con monto, descripción y origen (origen_archivo).</v>
+        <v>Botón "Gráfico" en cada fila de categoría o cuenta de matriz: modal con serie mensual (neto por mes) para esa clave, en la moneda seleccionada.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Detalle transacciones (moneda registración)</v>
+        <v>Detalle transacciones</v>
       </c>
       <c r="B15" t="str">
-        <v>En el modal mensual, cada línea muestra el monto en su moneda de registración (US$ / $). Si la moneda seleccionada difiere, se muestra la conversión a la moneda de vista (→) o indica (sin cot.) si falta tipo de cambio.</v>
+        <v>En cada agrupación, listado con monto, descripción y origen (origen_archivo).</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Detalle transacciones (tabla)</v>
+        <v>Detalle transacciones (moneda registración)</v>
       </c>
       <c r="B16" t="str">
-        <v>En el modal mensual, al expandir una categoría/cuenta se muestra una tabla con títulos y filas de transacciones (Fecha, Tipo, Medio, Moneda, Monto, moneda vista, TC, Cliente, Descripción, Observaciones, Origen). Icono ojo por fila (operadores) abre el modal de edición con el detalle completo del registro. Scroll vertical con encabezados fijos en el detalle expandido.</v>
+        <v>En el modal mensual, cada línea muestra el monto en su moneda de registración (US$ / $). Si la moneda seleccionada difiere, se muestra la conversión a la moneda de vista (→) o indica (sin cot.) si falta tipo de cambio.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Detalle transacciones (tipo de cambio)</v>
+        <v>Detalle transacciones (tabla)</v>
       </c>
       <c r="B17" t="str">
-        <v>En el detalle expandido del modal mensual, se muestra la columna TC (según MEP/CCL/Oficial) cuando hay conversión entre moneda registración y moneda vista; si no aplica muestra — y si falta cotización muestra sin cot.</v>
+        <v>En el modal mensual, al expandir una categoría/cuenta se muestra una tabla con títulos y filas de transacciones (Fecha, Tipo, Medio, Moneda, Monto, moneda vista, TC, Cliente, Descripción, Observaciones, Origen). Icono ojo por fila (operadores) abre el modal de edición con el detalle completo del registro. Scroll vertical con encabezados fijos en el detalle expandido.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Alertas por mes</v>
+        <v>Detalle transacciones (tipo de cambio)</v>
       </c>
       <c r="B18" t="str">
-        <v>Avisos: mes sin egresos; sin registros de Sueldos, Comisiones, Alquileres o Impuestos; desvío % de categoría (matriz) vs mes anterior.</v>
+        <v>En el detalle expandido del modal mensual, se muestra la columna TC (según MEP/CCL/Oficial) cuando hay conversión entre moneda registración y moneda vista; si no aplica muestra — y si falta cotización muestra sin cot.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Inclusión por mes (Configuración)</v>
+        <v>Alertas por mes</v>
       </c>
       <c r="B19" t="str">
-        <v>Interruptores por cada mes con movimientos: incluir o excluir del flujo por mes, tarjetas de resumen, Evolución y agregados que usan excluirFilaFlujoOperativo. Persistencia localStorage y columna meses_excluidos en config_dashboard. Sin afectar export de base histórica.</v>
+        <v>Avisos: mes sin egresos; sin registros de Sueldos, Comisiones, Alquileres o Impuestos; desvío % de categoría (matriz) vs mes anterior.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Sin cotización</v>
+        <v>Inclusión por mes (Configuración)</v>
       </c>
       <c r="B20" t="str">
-        <v>Pestaña con transacciones que no tienen tipo de cambio (excluidas del resumen).</v>
+        <v>Interruptores por cada mes con movimientos: incluir o excluir del flujo por mes, tarjetas de resumen, Evolución y agregados que usan excluirFilaFlujoOperativo. Persistencia localStorage y columna meses_excluidos en config_dashboard. Sin afectar export de base histórica.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Exclusiones (flujo operativo)</v>
+        <v>Sin cotización</v>
       </c>
       <c r="B21" t="str">
-        <v>No se incluyen en G/P operativo ni Evolución: apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito; meses desmarcados en Configuración → Inclusión por mes (meses_excluidos en Supabase/localStorage). Status Pendiente sí entra al Flujo. Base histórica y Todas las transacciones siguen completas.</v>
+        <v>Pestaña con transacciones que no tienen tipo de cambio (excluidas del resumen).</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Datos</v>
+        <v>Exclusiones (flujo operativo)</v>
       </c>
       <c r="B22" t="str">
-        <v>Tesorería (Conciliación Bancaria + Cajas físicas) y tipo de cambio desde Supabase (carga paginada). La relación categoría/cuenta/tipo → EF vive en matriz_cat_cuenta_ef. Cotización faltante: se usa la fecha anterior disponible.</v>
+        <v>No se incluyen en G/P operativo ni Evolución: apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito; meses desmarcados en Configuración → Inclusión por mes (meses_excluidos en Supabase/localStorage). Status Pendiente sí entra al Flujo. Base histórica y Todas las transacciones siguen completas.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Tablas y scroll</v>
+        <v>Datos</v>
       </c>
       <c r="B23" t="str">
-        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal. Flujo por mes y Todas las transacciones: clic en el encabezado ordena la columna. Columna Usuario (nombre para mostrar; tooltip con email) en Conciliación, Cajas, Saldos por canal, Impuestos, Matriz EF y Todas las transacciones.</v>
+        <v>Tesorería (Conciliación Bancaria + Cajas físicas) y tipo de cambio desde Supabase (carga paginada). La relación categoría/cuenta/tipo → EF vive en matriz_cat_cuenta_ef. Cotización faltante: se usa la fecha anterior disponible.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Menú lateral</v>
+        <v>Tablas y scroll</v>
       </c>
       <c r="B24" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Flujo de caja (permiso ver_solapa_flujo; icono $), Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage. Al iniciar sesión se abre Flujo de caja si el usuario lo tiene; si no, el primer menú lateral permitido. Cada vez que se vuelve a Flujo se recargan tesorería, cajas y tipos de cambio.</v>
+        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal. Flujo por mes y Todas las transacciones: clic en el encabezado ordena la columna. Columna Usuario (nombre para mostrar; tooltip con email) en Conciliación, Cajas, Saldos por canal, Impuestos, Matriz EF y Todas las transacciones.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Seguridad y roles</v>
+        <v>Menú lateral</v>
       </c>
       <c r="B25" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Recuperar contraseña desde el login (enlace por email). Permisos granulares desde Supabase: ver_solapa_flujo (menú y solapa Flujo de caja), ver_solapa_* (resto de solapas del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo de caja + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Flujo de caja (permiso ver_solapa_flujo; icono $), Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage. Al iniciar sesión se abre Flujo de caja si el usuario lo tiene; si no, el primer menú lateral permitido. Cada vez que se vuelve a Flujo se recargan tesorería, cajas y tipos de cambio.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Registro y contraseña</v>
+        <v>Seguridad y roles</v>
       </c>
       <c r="B26" t="str">
-        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español. Ayuda bajo el campo y mínimo 8 caracteres. En el login, «¿Olvidaste tu contraseña?» envía un enlace por email para elegir una clave nueva (revisar spam, sobre todo Hotmail).</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Recuperar contraseña desde el login (enlace por email). Permisos granulares desde Supabase: ver_solapa_flujo (menú y solapa Flujo de caja), ver_solapa_* (resto de solapas del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo de caja + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Repositorio Git (GitHub)</v>
+        <v>Registro y contraseña</v>
       </c>
       <c r="B27" t="str">
-        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
+        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español. Ayuda bajo el campo y mínimo 8 caracteres. En el login, «¿Olvidaste tu contraseña?» envía un enlace por email para elegir una clave nueva (revisar spam, sobre todo Hotmail).</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>App en producción (Vercel)</v>
+        <v>Repositorio Git (GitHub)</v>
       </c>
       <c r="B28" t="str">
-        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
+        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Exportar a Excel</v>
+        <v>App en producción (Vercel)</v>
       </c>
       <c r="B29" t="str">
-        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, observaciones, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle.</v>
+        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Flujo de despliegue</v>
+        <v>Exportar a Excel</v>
       </c>
       <c r="B30" t="str">
-        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación. En cada despliegue el agente redacta el modal «Nueva versión» (scripts/lib/fornitalia-release-blurb.js → fornitalia-release.json).</v>
+        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, observaciones, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Versiones en bitácora</v>
+        <v>Flujo de despliegue</v>
       </c>
       <c r="B31" t="str">
-        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
+        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación. En cada despliegue el agente redacta el modal «Nueva versión» (scripts/lib/fornitalia-release-blurb.js → fornitalia-release.json).</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Campo moneda (BD)</v>
+        <v>Versiones en bitácora</v>
       </c>
       <c r="B32" t="str">
-        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
+        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Edición desde modal Errores</v>
+        <v>Campo moneda (BD)</v>
       </c>
       <c r="B33" t="str">
-        <v>Retirado: la solapa Errores y su modal de detalle ya no están en el Flujo. La edición de registros sigue en Todas las transacciones.</v>
+        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Campos editado y editado_detalle</v>
+        <v>Edición desde modal Errores</v>
       </c>
       <c r="B34" t="str">
-        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
+        <v>Retirado: la solapa Errores y su modal de detalle ya no están en el Flujo. La edición de registros sigue en Todas las transacciones.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Tipo de error en Errores</v>
+        <v>Campos editado y editado_detalle</v>
       </c>
       <c r="B35" t="str">
-        <v>Retirado: la clasificación de inconsistencia y el tipo de error ya no se calculan ni se listan en el Flujo.</v>
+        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Detección de potencial duplicado</v>
+        <v>Tipo de error en Errores</v>
       </c>
       <c r="B36" t="str">
-        <v>Retirado del Flujo: el modal de comparación Este registro / Posible duplicado ya no existe. Los duplicados de tesorería se gestionan en Conciliación Bancaria → Potenciales duplicados.</v>
+        <v>Retirado: la clasificación de inconsistencia y el tipo de error ya no se calculan ni se listan en el Flujo.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Filtro por tipo de error</v>
+        <v>Detección de potencial duplicado</v>
       </c>
       <c r="B37" t="str">
-        <v>Retirado: el selector Tipo de error de la solapa Errores ya no está en la app.</v>
+        <v>Retirado del Flujo: el modal de comparación Este registro / Posible duplicado ya no existe. Los duplicados de tesorería se gestionan en Conciliación Bancaria → Potenciales duplicados.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Duplicados: condición cliente</v>
+        <v>Filtro por tipo de error</v>
       </c>
       <c r="B38" t="str">
-        <v>Retirado: esa regla de duplicados del Flujo ya no se aplica. Conciliación Bancaria usa su propio criterio (mismo importe, hasta 40 días).</v>
+        <v>Retirado: el selector Tipo de error de la solapa Errores ya no está en la app.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Regla bitácora</v>
+        <v>Duplicados: condición cliente</v>
       </c>
       <c r="B39" t="str">
-        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
+        <v>Retirado: esa regla de duplicados del Flujo ya no se aplica. Conciliación Bancaria usa su propio criterio (mismo importe, hasta 40 días).</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Evolución (tabla dinámica)</v>
+        <v>Regla bitácora</v>
       </c>
       <c r="B40" t="str">
-        <v>Solapa Evolución: Agrupar por = Nueva categoría (matriz) o Nueva cuenta contable (matriz) —prioriza nueva_categoria / nueva_cuenta_contable en BD y si faltan usa extracto—; Período = Diario o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
+        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Estado Financiero (tabla dinámica)</v>
+        <v>Evolución (tabla dinámica)</v>
       </c>
       <c r="B41" t="str">
-        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). AJUSTE DE SALDOS (CAJA) va debajo de FLUJO OPERATIVO GENERADO y entra en (=) FLUJO DE CAJA NETO DEL PERÍODO (D), no en A–C. En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Gráficos y export Excel. Conciliación §7 oculta.</v>
+        <v>Solapa Evolución: Agrupar por = Nueva categoría (matriz) o Nueva cuenta contable (matriz) —prioriza nueva_categoria / nueva_cuenta_contable en BD y si faltan usa extracto—; Período = Diario o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Reportes (menú lateral)</v>
+        <v>Estado Financiero (tabla dinámica)</v>
       </c>
       <c r="B42" t="str">
-        <v>Vista Reportes: exportar Matriz de relaciones desde Supabase. Matriz_Cat_Cuenta_Costo sin exclusiones (suma # Registros = transacciones en sesión); filas verde claro si cat/cuenta vieja tiene relación única a nueva. Cat×cuenta solo Confirmado; proveedores con exclusiones de categoría. Resumen antes de exportar.</v>
+        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). AJUSTE DE SALDOS (CAJA) va debajo de FLUJO OPERATIVO GENERADO y entra en (=) FLUJO DE CAJA NETO DEL PERÍODO (D), no en A–C. En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Gráficos y export Excel. Conciliación §7 oculta.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Evolución: detalle al clic y exportar</v>
+        <v>Reportes (menú lateral)</v>
       </c>
       <c r="B43" t="str">
-        <v>Clic en un valor abre modal con detalle: Fecha, Categoría (matriz), Cuenta (matriz), Descripción, Observaciones, Monto. Exportar Evolución a Excel: primera columna con el mismo criterio de agrupación.</v>
+        <v>Vista Reportes: exportar Matriz de relaciones desde Supabase. Matriz_Cat_Cuenta_Costo sin exclusiones (suma # Registros = transacciones en sesión); filas verde claro si cat/cuenta vieja tiene relación única a nueva. Cat×cuenta solo Confirmado; proveedores con exclusiones de categoría. Resumen antes de exportar.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Exportaciones Excel</v>
+        <v>Evolución: detalle al clic y exportar</v>
       </c>
       <c r="B44" t="str">
-        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Flujo a Excel, Exportar Evolución a Excel y Exportar EF a Excel con el mismo icono y método (SheetJS/xlsx-js-style). Importes como número; % del Flujo y EF como fracción.</v>
+        <v>Clic en un valor abre modal con detalle: Fecha, Categoría (matriz), Cuenta (matriz), Descripción, Observaciones, Monto. Exportar Evolución a Excel: primera columna con el mismo criterio de agrupación.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Evolución: orden ingreso/egreso</v>
+        <v>Exportaciones Excel</v>
       </c>
       <c r="B45" t="str">
-        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica al agrupar por categoría o cuenta de matriz.</v>
+        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Flujo a Excel, Exportar Evolución a Excel y Exportar EF a Excel con el mismo icono y método (SheetJS/xlsx-js-style). Importes como número; % del Flujo y EF como fracción.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Int. por caución</v>
+        <v>Evolución: orden ingreso/egreso</v>
       </c>
       <c r="B46" t="str">
-        <v>Retirado de la app: la columna Caución, el % G/P, el modal de marcha y la carga de Serie_Cauciones ya no están en el Flujo. La fila comercial se conserva por el trabajo histórico.</v>
+        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica al agrupar por categoría o cuenta de matriz.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Todas las transacciones</v>
+        <v>Int. por caución</v>
       </c>
       <c r="B47" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas (incluida Observaciones, después de Descripción). Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) y buscador por id operación, descripción u observaciones. Clic en un encabezado ordena asc/desc. Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa.</v>
+        <v>Retirado de la app: la columna Caución, el % G/P, el modal de marcha y la carga de Serie_Cauciones ya no están en el Flujo. La fila comercial se conserva por el trabajo histórico.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Edición completa de registros</v>
+        <v>Todas las transacciones</v>
       </c>
       <c r="B48" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), ef_item y ef_subitem (estado de flujo), origen archivo, descripción, observaciones, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). En tesorería (cb/cf) observaciones se guarda en raw.observaciones. editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas (incluida Observaciones, después de Descripción). Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) y buscador por id operación, descripción u observaciones. Clic en un encabezado ordena asc/desc. Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Proyección próximos 3 meses</v>
+        <v>Edición completa de registros</v>
       </c>
       <c r="B49" t="str">
-        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), ef_item y ef_subitem (estado de flujo), origen archivo, descripción, observaciones, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). En tesorería (cb/cf) observaciones se guarda en raw.observaciones. editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Int. por caución proyectado</v>
+        <v>Proyección próximos 3 meses</v>
       </c>
       <c r="B50" t="str">
-        <v>Retirado de la app junto con la columna Caución del Flujo.</v>
+        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Disclaimer proyección</v>
+        <v>Int. por caución proyectado</v>
       </c>
       <c r="B51" t="str">
-        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses y ventana rodante.</v>
+        <v>Retirado de la app junto con la columna Caución del Flujo.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Botones e iconos unificados</v>
+        <v>Disclaimer proyección</v>
       </c>
       <c r="B52" t="str">
-        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, Flujo de caja / $, engranaje, usuario), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG. Cada vista de menú muestra en la cabecera el mismo icono que el ítem del sidebar (Flujo de caja, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad, Mi perfil).</v>
+        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses y ventana rodante.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Configuración % G/P en caución</v>
+        <v>Botones e iconos unificados</v>
       </c>
       <c r="B53" t="str">
-        <v>Retirado de Configuración: el combo % G/P acum. en caución ya no se muestra. La columna pct_caucion en config_dashboard queda sin uso.</v>
+        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, Flujo de caja / $, engranaje, usuario), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG. Cada vista de menú muestra en la cabecera el mismo icono que el ítem del sidebar (Flujo de caja, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad, Mi perfil).</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Etiqueta Caución (x% cash)</v>
+        <v>Configuración % G/P en caución</v>
       </c>
       <c r="B54" t="str">
-        <v>Retirado: la columna Caución ya no forma parte del Flujo por mes.</v>
+        <v>Retirado de Configuración: el combo % G/P acum. en caución ya no se muestra. La columna pct_caucion en config_dashboard queda sin uso.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Meses a proyectar</v>
+        <v>Etiqueta Caución (x% cash)</v>
       </c>
       <c r="B55" t="str">
-        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
+        <v>Retirado: la columna Caución ya no forma parte del Flujo por mes.</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Config por usuario en Supabase</v>
+        <v>Meses a proyectar</v>
       </c>
       <c r="B56" t="str">
-        <v>Tabla config_dashboard (user_id, proyección, alertas y meses_excluidos JSON). Se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql; meses excluidos: supabase_config_dashboard_meses_excluidos.sql.</v>
+        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Recorte % (cada lado)</v>
+        <v>Config por usuario en Supabase</v>
       </c>
       <c r="B57" t="str">
-        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
+        <v>Tabla config_dashboard (user_id, proyección, alertas y meses_excluidos JSON). Se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql; meses excluidos: supabase_config_dashboard_meses_excluidos.sql.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Novedades del Negocio</v>
+        <v>Recorte % (cada lado)</v>
       </c>
       <c r="B58" t="str">
-        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
+        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Gestión de Proyectos</v>
+        <v>Novedades del Negocio</v>
       </c>
       <c r="B59" t="str">
-        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Archivos adjuntos por fecha (descripción + archivo en Storage gp-archivos) en proyecto, entregable y tarea; solapa Archivos y hoja Excel. Solapa Horas cons.: conciliación diaria. La solapa activa (To-Do, Gantt, Horas, Archivos) se marca con etiqueta Activo y un contorno más visible. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
+        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Conciliación Bancaria</v>
+        <v>Gestión de Proyectos</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar y reconoce coma decimal (15,71) para el importe exacto. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Archivos adjuntos por fecha (descripción + archivo en Storage gp-archivos) en proyecto, entregable y tarea; solapa Archivos y hoja Excel. Solapa Horas cons.: conciliación diaria. La solapa activa (To-Do, Gantt, Horas, Archivos) se marca con etiqueta Activo y un contorno más visible. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Cajas (físicas)</v>
+        <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Solo Status Pendiente (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar y reconoce coma decimal (15,71) para el importe exacto. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Saldos extractos</v>
+        <v>Cajas (físicas)</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP y Credicoop, mes en curso = último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Solo Status Pendiente (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Impuestos</v>
+        <v>Saldos extractos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca), marcada Activo como el resto de pantallas: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (listado con Observaciones; justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql, sql/supabase_cb_match_impuestos.sql y sql/supabase_imp_tesoreria_observaciones.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP y Credicoop, mes en curso = último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Impuestos</v>
       </c>
       <c r="B64" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca), marcada Activo como el resto de pantallas: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (listado con Observaciones; justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql, sql/supabase_cb_match_impuestos.sql y sql/supabase_imp_tesoreria_observaciones.sql.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B65" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B66" t="str">
-        <v>Retirado: el Flujo ya no reemplaza la tabla transacciones desde un Excel Normalizado. El botón, el modal y el permiso carga_normalizada salieron de la app. Queda el script npm run normalizar-extracto para generar el archivo.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B67" t="str">
-        <v>Retirado: la solapa Excluidos upload y su permiso ya no están en el dashboard. La tabla de auditoría en Supabase se conserva.</v>
+        <v>Retirado: el Flujo ya no reemplaza la tabla transacciones desde un Excel Normalizado. El botón, el modal y el permiso carga_normalizada salieron de la app. Queda el script npm run normalizar-extracto para generar el archivo.</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Matriz EF</v>
+        <v>Log de excluidos en upload</v>
       </c>
       <c r="B68" t="str">
-        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6 ni 1.2 (ajuste de saldos), A–D, 6.1–6.3 ni subítems con relaciones/ratios; códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql, sql/supabase_ef_estructura_abm.sql y sql/supabase_ef_ajuste_saldos_caja.sql.</v>
+        <v>Retirado: la solapa Excluidos upload y su permiso ya no están en el dashboard. La tabla de auditoría en Supabase se conserva.</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Análisis financiero extracto (PDF)</v>
+        <v>Matriz EF</v>
       </c>
       <c r="B69" t="str">
-        <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
+        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6 ni 1.2 (ajuste de saldos), A–D, 6.1–6.3 ni subítems con relaciones/ratios; códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql, sql/supabase_ef_estructura_abm.sql y sql/supabase_ef_ajuste_saldos_caja.sql.</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Usuario en tablas</v>
+        <v>Análisis financiero extracto (PDF)</v>
       </c>
       <c r="B70" t="str">
-        <v>Quién cargó, confirmó, descartó o eliminó: se ve el nombre para mostrar (ej. LB) y al pasar el mouse el email. Lo histórico de tesorería, saldos, impuestos y matriz queda a nombre de LB (lucas.bustos.martin@gmail.com). El consolidado de Saldos extractos no tiene actor por fila. rpc get_usuarios_mostrar. sql/supabase_usuarios_mostrar.sql.</v>
+        <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
+        <v>Usuario en tablas</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Quién cargó, confirmó, descartó o eliminó: se ve el nombre para mostrar (ej. LB) y al pasar el mouse el email. Lo histórico de tesorería, saldos, impuestos y matriz queda a nombre de LB (lucas.bustos.martin@gmail.com). El consolidado de Saldos extractos no tiene actor por fila. rpc get_usuarios_mostrar. sql/supabase_usuarios_mostrar.sql.</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
         <v>Novedades al iniciar sesión</v>
       </c>
-      <c r="B71" t="str">
+      <c r="B72" t="str">
         <v>Tras cada despliegue, al entrar a la app se muestra el modal «Nueva versión» con 2–4 frases de lo que se nota al recargar (logo, badge de versión, lista). Una vez Entendido, no vuelve a aparecer hasta la siguiente versión. El texto lo actualiza el agente en scripts/lib/fornitalia-release-blurb.js; fornitalia-release.json se sirve por red.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B71"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B72"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7856,7 +7915,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:C111"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9073,9 +9132,20 @@
         <v>Despliegue v2.66: Conciliación Bancaria — el buscar reconoce coma decimal (15,71 / 1.234,56) y filtra el importe exacto; igual en conciliación manual. Producción Vercel.</v>
       </c>
     </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>2.67</v>
+      </c>
+      <c r="B111" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Despliegue v2.67: Flujo — Ratios Sueldos / Ingresos y Costo Financiero MP / Ventas MP (solo caja Mercado Pago); PDF A4 apaisado de una página, sin repetir encabezado ni Total G/P. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C110"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C111"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9123,7 +9193,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, alertas, modal By Categoría / By Cuenta). Incluye PDF de una página con filtros activos y formatos de moneda.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). Incluye PDF de una página con filtros activos y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>
@@ -9277,7 +9347,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. El buscar admite coma decimal (15,71) para el importe exacto. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.68: Total de Flujo solo meses reales, antes de las proyecciones.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E401"/>
+  <dimension ref="A1:E403"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7228,9 +7228,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="402">
+      <c r="A402" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B402" t="str">
+        <v>14:48</v>
+      </c>
+      <c r="C402" t="str">
+        <v>Flujo: Total sin proyecciones, luego Proy.</v>
+      </c>
+      <c r="D402" t="str">
+        <v>La columna Total de Flujo (Ingresos, Egresos, G/P y ratios) suma solo meses reales. En pantalla queda después de esos meses y las columnas Proy. a la derecha, para que no parezca que el total las incluye.</v>
+      </c>
+      <c r="E402" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B403" t="str">
+        <v>15:08</v>
+      </c>
+      <c r="C403" t="str">
+        <v>Despliegue v2.68 producción</v>
+      </c>
+      <c r="D403" t="str">
+        <v>Push a main y Vercel --prod: Total de Flujo solo meses reales, a la izquierda de las columnas Proy. APP_VERSION 2.68.</v>
+      </c>
+      <c r="E403" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E401"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E403"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7256,7 +7290,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total de ratios no incluye proyectados. Proyección como columnas extra si el período incluye el mes en curso. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total (Ingresos, Egresos, G/P y ratios) suma solo meses reales y va después de esos meses; las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -7304,7 +7338,7 @@
         <v>Egresos / Ingresos</v>
       </c>
       <c r="B8" t="str">
-        <v>Filas de ratios del Flujo: Sueldos / Ingresos y Costo dir. / Ingresos (§2), Costo ind. / Ingresos (§3) y Costo total / Ingreso total (Egresos ÷ Ingresos) usan Ingresos como denominador. Costo Financiero MP / Ventas MP usa cobranzas de la caja Mercado Pago. La columna Total de ratios usa solo meses reales (sin proyectados). PDF y Excel con la misma fórmula sobre reales.</v>
+        <v>Filas de ratios del Flujo: Sueldos / Ingresos y Costo dir. / Ingresos (§2), Costo ind. / Ingresos (§3) y Costo total / Ingreso total (Egresos ÷ Ingresos) usan Ingresos como denominador. Costo Financiero MP / Ventas MP usa cobranzas de la caja Mercado Pago. La columna Total (montos y ratios) usa solo meses reales, se muestra después de esos meses y las proyecciones van a la derecha. PDF y Excel con la misma fórmula sobre reales.</v>
       </c>
     </row>
     <row r="9">
@@ -7915,7 +7949,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C111"/>
+  <dimension ref="A1:C112"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9143,9 +9177,20 @@
         <v>Despliegue v2.67: Flujo — Ratios Sueldos / Ingresos y Costo Financiero MP / Ventas MP (solo caja Mercado Pago); PDF A4 apaisado de una página, sin repetir encabezado ni Total G/P. Producción Vercel.</v>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>2.68</v>
+      </c>
+      <c r="B112" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Despliegue v2.68: Flujo — columna Total (Ingresos, Egresos, G/P y ratios) suma solo meses reales y se muestra después de esos meses; las columnas Proy. quedan a la derecha. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C111"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C112"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.69: buscar 1000, solapa Todos y carga Galicia más rápida.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E403"/>
+  <dimension ref="A1:E406"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7262,9 +7262,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="B404" t="str">
+        <v>10:25</v>
+      </c>
+      <c r="C404" t="str">
+        <v>Galicia: débito 1000 SIRCREB sí entra</v>
+      </c>
+      <c r="D404" t="str">
+        <v>El registro naranja del Extracto_CC (28/09/2026, Ing. Brutos S/ Cred, débito 1000, REG.RECAU.SIRCREB) ya estaba en Galicia: no lo omite el parser. Queda en Confirmados (conciliación manual). El buscar 1000 no lo mostraba (el entero no se trataba como importe y 1.000,00 no contiene “1000”). Otros IIBB/SIRCREB del mismo Excel también están; el mismo hueco de búsqueda aplica a enteros tipo 2000/3000/4000/6000.</v>
+      </c>
+      <c r="E404" t="str">
+        <v>Diagnostico</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="B405" t="str">
+        <v>10:32</v>
+      </c>
+      <c r="C405" t="str">
+        <v>Conciliación: buscar 1000, Todos y carga Galicia</v>
+      </c>
+      <c r="D405" t="str">
+        <v>El buscar de Conciliación Bancaria trata 1000 y 1.000 como importe exacto (sigue valiendo coma decimal y el texto/ID). Solapa Todos: extracto + tesorería con columna Dónde (clic para ir a esa lista). La carga de Galicia pide los datos en paralelo y evita recargas de más al recalcular sugeridos.</v>
+      </c>
+      <c r="E405" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="B406" t="str">
+        <v>10:36</v>
+      </c>
+      <c r="C406" t="str">
+        <v>Despliegue v2.69 producción</v>
+      </c>
+      <c r="D406" t="str">
+        <v>Push a main y Vercel --prod: Conciliación Bancaria — buscar enteros como 1000; solapa Todos con columna Dónde; carga de Galicia más rápida. APP_VERSION 2.69.</v>
+      </c>
+      <c r="E406" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E403"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E406"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7762,7 +7813,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar y reconoce coma decimal (15,71) para el importe exacto. Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar: un entero (1000) o coma decimal (15,71) encuentran el importe exacto, y también el texto o el ID. Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -7949,7 +8000,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C113"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9188,9 +9239,20 @@
         <v>Despliegue v2.68: Flujo — columna Total (Ingresos, Egresos, G/P y ratios) suma solo meses reales y se muestra después de esos meses; las columnas Proy. quedan a la derecha. Producción Vercel.</v>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>2.69</v>
+      </c>
+      <c r="B113" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="C113" t="str">
+        <v>Despliegue v2.69: Conciliación Bancaria — el buscar trata 1000 / 1.000 como importe; solapa Todos (extracto + tesorería) con columna Dónde; carga de extracto Galicia más rápida. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C112"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C113"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9392,7 +9454,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. El buscar admite coma decimal (15,71) para el importe exacto. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. El buscar admite entero (1000), 1.000 o coma decimal (15,71) para el importe exacto, y también texto/ID. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.70: filtros de importe e ID exactos en conciliación.
El buscar queda texto libre; importe e ID van en el modal de filtros.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E406"/>
+  <dimension ref="A1:E409"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7313,9 +7313,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="B407" t="str">
+        <v>10:48</v>
+      </c>
+      <c r="C407" t="str">
+        <v>Buscar 1000 solo importe exacto</v>
+      </c>
+      <c r="D407" t="str">
+        <v>En Conciliación Bancaria, un número (1000, 1.000 o 15,71) filtra solo movimientos con ese importe (también débito/crédito y el signo). Ya no trae IDs tipo 10000608 ni descripciones que contienen 1000. El texto sin número sigue buscando cliente, concepto e ID.</v>
+      </c>
+      <c r="E407" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="B408" t="str">
+        <v>11:03</v>
+      </c>
+      <c r="C408" t="str">
+        <v>Filtros importe e ID exactos</v>
+      </c>
+      <c r="D408" t="str">
+        <v>En Conciliación Bancaria, el modal Filtros suma Importe exacto e ID exacto. El buscar de la pantalla queda libre para concepto, cliente y observaciones (un 1000 ya no se trata como importe ni como ID).</v>
+      </c>
+      <c r="E408" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="B409" t="str">
+        <v>11:22</v>
+      </c>
+      <c r="C409" t="str">
+        <v>Despliegue v2.70 producción</v>
+      </c>
+      <c r="D409" t="str">
+        <v>Push a main y Vercel --prod: Conciliación Bancaria — Filtros con importe exacto e ID exacto; el buscar queda texto libre. APP_VERSION 2.70.</v>
+      </c>
+      <c r="E409" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E406"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E409"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7813,7 +7864,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar: un entero (1000) o coma decimal (15,71) encuentran el importe exacto, y también el texto o el ID. Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros mes extracto/sistema + categoría + cuenta y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -8000,7 +8051,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C114"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9250,9 +9301,20 @@
         <v>Despliegue v2.69: Conciliación Bancaria — el buscar trata 1000 / 1.000 como importe; solapa Todos (extracto + tesorería) con columna Dónde; carga de extracto Galicia más rápida. Producción Vercel.</v>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>2.70</v>
+      </c>
+      <c r="B114" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Despliegue v2.70: Conciliación Bancaria — Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C113"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C114"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9454,7 +9516,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. El buscar admite entero (1000), 1.000 o coma decimal (15,71) para el importe exacto, y también texto/ID. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.71: sugeridos al abrir conciliación y mensajes de la app.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E409"/>
+  <dimension ref="A1:E413"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7364,16 +7364,84 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="410">
+      <c r="A410" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B410" t="str">
+        <v>12:50</v>
+      </c>
+      <c r="C410" t="str">
+        <v>Sugeridos se recalculan aunque la lista esté vacía</v>
+      </c>
+      <c r="D410" t="str">
+        <v>Al abrir Conciliación Bancaria (o cambiar de caja) se vuelven a armar los sugeridos aunque no haya ninguno. El mismo día también acepta la tolerancia de importe (centavos, $1, $10 o $100), no solo el centavo exacto.</v>
+      </c>
+      <c r="E410" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B411" t="str">
+        <v>13:02</v>
+      </c>
+      <c r="C411" t="str">
+        <v>Confirmación duplicada Galicia 972,40</v>
+      </c>
+      <c r="D411" t="str">
+        <v>La pareja manual extracto 18/09 −972,40 SIRCREB y tesorería 30/09 −972,40 (Lucas Martin Campos) estaba confirmada dos veces, a 3 ms de diferencia, y el recálculo de sugeridos se cancelaba. Se dejó una sola confirmación.</v>
+      </c>
+      <c r="E411" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B412" t="str">
+        <v>13:12</v>
+      </c>
+      <c r="C412" t="str">
+        <v>Mensajes de la app, sin cuadro del navegador</v>
+      </c>
+      <c r="D412" t="str">
+        <v>Confirmaciones y avisos (Confirmar sugerencias, eliminar, errores, exportar vacío, etc.) dejan de usar el cartel del navegador. Pasan a un cuadro de la app, con título, texto y botones con icono. scripts/lib/fornitalia-mensajes.js.</v>
+      </c>
+      <c r="E412" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B413" t="str">
+        <v>14:22</v>
+      </c>
+      <c r="C413" t="str">
+        <v>Despliegue v2.71 producción</v>
+      </c>
+      <c r="D413" t="str">
+        <v>Push a main y Vercel --prod: al abrir Conciliación se rearman los sugeridos aunque la lista esté vacía (también el mismo día con tolerancia de importe); confirmaciones y avisos en un cuadro de la app. APP_VERSION 2.71.</v>
+      </c>
+      <c r="E413" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E409"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E413"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B72"/>
+  <dimension ref="A1:B73"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -7864,7 +7932,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), solo si las fechas no difieren en más de 4 días. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -7955,9 +8023,17 @@
         <v>Tras cada despliegue, al entrar a la app se muestra el modal «Nueva versión» con 2–4 frases de lo que se nota al recargar (logo, badge de versión, lista). Una vez Entendido, no vuelve a aparecer hasta la siguiente versión. El texto lo actualiza el agente en scripts/lib/fornitalia-release-blurb.js; fornitalia-release.json se sirve por red.</v>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Mensajes de confirmación y aviso</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Las preguntas sí/no y los avisos de error o validación se muestran en un cuadro de la app (título, texto y botones con icono), no en el cartel del navegador. Confirmar usa Aceptar y Cancelar; un aviso usa Entendido. Eliminar marca el botón en rojo. Componente: scripts/lib/fornitalia-mensajes.js.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B72"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B73"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8051,7 +8127,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C114"/>
+  <dimension ref="A1:C115"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9312,9 +9388,20 @@
         <v>Despliegue v2.70: Conciliación Bancaria — Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Producción Vercel.</v>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>2.71</v>
+      </c>
+      <c r="B115" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Despliegue v2.71: Conciliación — al abrir la caja se rearman los sugeridos aunque la lista esté vacía, también el mismo día si el importe entra en la tolerancia. Confirmaciones y avisos de toda la app en un cuadro propio (Aceptar / Cancelar), sin el cartel del navegador. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C114"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C115"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.72: A eliminar solo si la fecha del Pendiente entra en el archivo.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E413"/>
+  <dimension ref="A1:E415"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7432,9 +7432,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="414">
+      <c r="A414" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B414" t="str">
+        <v>15:20</v>
+      </c>
+      <c r="C414" t="str">
+        <v>A eliminar solo si la fecha entra en el archivo</v>
+      </c>
+      <c r="D414" t="str">
+        <v>Un Pendiente pasa a A eliminar solo si su fecha cae entre la primera y la última del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Confirmado nunca. sql/supabase_cb_baja_pendiente_rango_fecha.sql.</v>
+      </c>
+      <c r="E414" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B415" t="str">
+        <v>18:32</v>
+      </c>
+      <c r="C415" t="str">
+        <v>Despliegue v2.72 producción</v>
+      </c>
+      <c r="D415" t="str">
+        <v>Push a main y Vercel --prod: A eliminar solo marca un Pendiente cuya fecha cae dentro del Excel cargado (histórico o tesorería, Conciliación y Cajas) y cuyo Id no viene. APP_VERSION 2.72.</v>
+      </c>
+      <c r="E415" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E413"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E415"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7932,7 +7966,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente (caja abierta, entre por tesorería o por el histórico) puede ir a A eliminar: se puede anular en el sistema y desaparecer. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -7940,7 +7974,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Solo Status Pendiente (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Solo Status Pendiente (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -8127,7 +8161,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C115"/>
+  <dimension ref="A1:C116"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9399,9 +9433,20 @@
         <v>Despliegue v2.71: Conciliación — al abrir la caja se rearman los sugeridos aunque la lista esté vacía, también el mismo día si el importe entra en la tolerancia. Confirmaciones y avisos de toda la app en un cuadro propio (Aceptar / Cancelar), sin el cartel del navegador. Producción Vercel.</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>2.72</v>
+      </c>
+      <c r="B116" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Despliegue v2.72: A eliminar solo marca un Pendiente si su fecha está entre la primera y la última del Excel cargado (histórico o tesorería, en Conciliación y en Cajas) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Confirmado nunca. sql/supabase_cb_baja_pendiente_rango_fecha.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C115"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C116"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9603,7 +9648,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, solo los Ids con Status Pendiente (caja abierta) que ya no vienen van a A eliminar; un Confirmado nunca se marca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>
@@ -9631,7 +9676,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B16" t="str">
-        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura), en cualquier tesorería, cierre o histórico) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Tras cada carga se abre el popup de resultado (nuevos, actualizados, sin cambios, omitidos). Apertura de Caja no entra al corte. El histórico no pisa el saldo de tesorería o cierre. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
+        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura), en cualquier tesorería, cierre o histórico) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Tras cada carga se abre el popup de resultado (nuevos, actualizados, sin cambios, omitidos). Un Pendiente pasa a A eliminar solo si su fecha está en el Excel y el Id no viene. Apertura de Caja no entra al corte. El histórico no pisa el saldo de tesorería o cierre. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
       </c>
       <c r="C16">
         <v>8</v>

</xml_diff>

<commit_message>
v2.73: contador en solapas, cartel de carga y A eliminar sin Status.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E415"/>
+  <dimension ref="A1:E418"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7466,9 +7466,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="416">
+      <c r="A416" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B416" t="str">
+        <v>19:00</v>
+      </c>
+      <c r="C416" t="str">
+        <v>A eliminar también con Status vacío</v>
+      </c>
+      <c r="D416" t="str">
+        <v>Además de Pendiente, un movimiento sin Status (como el Id 10003520, ajuste de Galicia ARS) puede ir a A eliminar si su fecha cae en el Excel y el Id no viene. Confirmado nunca. sql/supabase_cb_tesoreria_abierta_pendiente_historico.sql.</v>
+      </c>
+      <c r="E416" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B417" t="str">
+        <v>19:19</v>
+      </c>
+      <c r="C417" t="str">
+        <v>Contador en solapas y cartel de carga</v>
+      </c>
+      <c r="D417" t="str">
+        <v>En Conciliación y Cajas, cada solapa muestra el número de registros (también 0). Mientras corre una carga, un recálculo, una confirmación, una baja o el Excel, queda un cartel hasta que el proceso termina.</v>
+      </c>
+      <c r="E417" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B418" t="str">
+        <v>08:23</v>
+      </c>
+      <c r="C418" t="str">
+        <v>Despliegue v2.73 producción</v>
+      </c>
+      <c r="D418" t="str">
+        <v>Push a main y Vercel --prod: solapas con contador de registros (también 0); cartel de carga hasta que termina el proceso; A eliminar también con Status vacío. APP_VERSION 2.73.</v>
+      </c>
+      <c r="E418" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E415"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E418"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7966,7 +8017,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Solo Status Pendiente puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="62">
@@ -7974,7 +8025,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Solo Status Pendiente (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
       </c>
     </row>
     <row r="63">
@@ -8161,7 +8212,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C117"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9444,9 +9495,20 @@
         <v>Despliegue v2.72: A eliminar solo marca un Pendiente si su fecha está entre la primera y la última del Excel cargado (histórico o tesorería, en Conciliación y en Cajas) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Confirmado nunca. sql/supabase_cb_baja_pendiente_rango_fecha.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>2.73</v>
+      </c>
+      <c r="B117" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Despliegue v2.73: Conciliación y Cajas — cada solapa muestra el contador de registros (también 0). Cartel de carga hasta que termina cargar, recalcular, confirmar, eliminar o el Excel. A eliminar también con Status vacío, si la fecha cae en el archivo y el Id no viene. Confirmado nunca. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C116"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C117"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9648,7 +9710,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
       </c>
       <c r="C14">
         <v>24</v>
@@ -9676,7 +9738,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B16" t="str">
-        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura), en cualquier tesorería, cierre o histórico) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Tras cada carga se abre el popup de resultado (nuevos, actualizados, sin cambios, omitidos). Un Pendiente pasa a A eliminar solo si su fecha está en el Excel y el Id no viene. Apertura de Caja no entra al corte. El histórico no pisa el saldo de tesorería o cierre. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
+        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura), en cualquier tesorería, cierre o histórico) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Tras cada carga se abre el popup de resultado (nuevos, actualizados, sin cambios, omitidos). Un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha está en el Excel y el Id no viene. Apertura de Caja no entra al corte. El histórico no pisa el saldo de tesorería o cierre. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
       </c>
       <c r="C16">
         <v>8</v>

</xml_diff>

<commit_message>
v2.74: Mercado Pago controla el mes con el resumen de cuenta.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E418"/>
+  <dimension ref="A1:E421"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7517,9 +7517,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="419">
+      <c r="A419" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B419" t="str">
+        <v>09:13</v>
+      </c>
+      <c r="C419" t="str">
+        <v>Mercado Pago: resumen de fin de mes</v>
+      </c>
+      <c r="D419" t="str">
+        <v>Se eliminó la última carta de saldo (balance_letter del 30/09/2026, $ 68.955.143,71). En Saldos extractos, Mercado Pago deja de cargar cartas y lee el resumen de cuenta mensual: no da de alta movimientos. Verifica que cada ID de operación esté en el extracto ya cargado y que el saldo final cierre con el saldo inicial más esos movimientos. Después se borró toda la serie de cartas para recargarla con el resumen.</v>
+      </c>
+      <c r="E419" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B420" t="str">
+        <v>09:33</v>
+      </c>
+      <c r="C420" t="str">
+        <v>Mercado Pago: se borran las cartas</v>
+      </c>
+      <c r="D420" t="str">
+        <v>Se eliminaron las 16 cartas de saldo de Mercado Pago (MP_Saldos_ de junio 2025 a septiembre 2026). La serie queda vacía para cargarla de nuevo con el resumen de cuenta, mes por mes. Los movimientos del extracto Excel no se tocaron.</v>
+      </c>
+      <c r="E420" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B421" t="str">
+        <v>09:47</v>
+      </c>
+      <c r="C421" t="str">
+        <v>Despliegue v2.74 producción</v>
+      </c>
+      <c r="D421" t="str">
+        <v>Push a main y Vercel --prod: Saldos extractos de Mercado Pago lee el resumen de cuenta de fin de mes. No da de alta movimientos; verifica que cada operación esté cargada y que el saldo cierre. APP_VERSION 2.74.</v>
+      </c>
+      <c r="E421" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E418"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E421"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8033,7 +8084,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: PDF Carta de saldo (MP_Saldos_YYYYMMDD) con saldo total, disponible y a liberar; variación vs la carta anterior. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP y Credicoop, mes en curso = último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el día a día entra por el Excel del extracto. El PDF resumen de cuenta (fin de mes) no da de alta movimientos: verifica que cada ID de operación esté en la app y que el saldo final cierre con el saldo inicial más esos movimientos. La serie de cartas se vació para volver a cargarla con ese resumen, mes por mes. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP y Credicoop, mes en curso = último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="64">
@@ -8212,7 +8263,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C117"/>
+  <dimension ref="A1:C118"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9506,9 +9557,20 @@
         <v>Despliegue v2.73: Conciliación y Cajas — cada solapa muestra el contador de registros (también 0). Cartel de carga hasta que termina cargar, recalcular, confirmar, eliminar o el Excel. A eliminar también con Status vacío, si la fecha cae en el archivo y el Id no viene. Confirmado nunca. Producción Vercel.</v>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>2.74</v>
+      </c>
+      <c r="B118" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Despliegue v2.74: Saldos extractos Mercado Pago — el PDF de fin de mes es el resumen de cuenta. No da de alta movimientos: verifica que cada operación esté en la app y que el saldo final cierre. Se vació la serie de cartas (junio 2025 a septiembre 2026) para recargarla mes a mes. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C117"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C118"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9724,7 +9786,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En Galicia, mes en curso = saldo corrido del extracto (saldo real del banco). En MP y Credicoop, último corte + créditos − débitos. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (resumen de cuenta de fin de mes: verifica movimientos y saldo; la serie de cartas se vació para recargarla mes a mes), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En Galicia, mes en curso = saldo corrido del extracto (saldo real del banco). En MP y Credicoop, último corte + créditos − débitos. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>

</xml_diff>

<commit_message>
v2.75: ratio Sueldos + Cargas Sociales sobre cobranzas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E421"/>
+  <dimension ref="A1:E423"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7568,9 +7568,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="422">
+      <c r="A422" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B422" t="str">
+        <v>12:28</v>
+      </c>
+      <c r="C422" t="str">
+        <v>Ratio Sueldos + Cargas Sociales / Cobranzas</v>
+      </c>
+      <c r="D422" t="str">
+        <v>En Flujo de caja, Ratios del Negocio suma Sueldos (Neto / Bolsillo) + Cargas Sociales y lo divide por Cobranzas por Ventas (efectivo neto ingresado). Misma fila en el PDF y en el Excel. La columna Total usa solo meses reales.</v>
+      </c>
+      <c r="E422" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B423" t="str">
+        <v>14:50</v>
+      </c>
+      <c r="C423" t="str">
+        <v>Despliegue v2.75 producción</v>
+      </c>
+      <c r="D423" t="str">
+        <v>Push a main y Vercel --prod: Flujo de caja con el ratio Sueldos + Cargas Sociales / Cobranzas. PDF y Excel. APP_VERSION 2.75.</v>
+      </c>
+      <c r="E423" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E421"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E423"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7596,7 +7630,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total (Ingresos, Egresos, G/P y ratios) suma solo meses reales y va después de esos meses; las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas); Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total (Ingresos, Egresos, G/P y ratios) suma solo meses reales y va después de esos meses; las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -7636,7 +7670,7 @@
         <v>Sueldos / Ingresos y Costo Fin. MP</v>
       </c>
       <c r="B7" t="str">
-        <v>Ratios del Negocio: Sueldos / Ingresos (egresos de categoría Sueldos, sin comisiones de venta) y Costo Financiero MP / Ventas MP (ef_subitem Costo Financiero Mercado Pago ÷ cobranzas por ventas solo de caja Mercado Pago). PDF y Excel.</v>
+        <v>Ratios del Negocio: Sueldos / Ingresos (egresos de categoría Sueldos, sin comisiones de venta), Sueldos + Cargas Sociales / Cobranzas (ef_subitem Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas, efectivo neto ingresado) y Costo Financiero MP / Ventas MP (ef_subitem Costo Financiero Mercado Pago ÷ cobranzas por ventas solo de caja Mercado Pago). PDF y Excel.</v>
       </c>
     </row>
     <row r="8">
@@ -8263,7 +8297,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C118"/>
+  <dimension ref="A1:C119"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9568,9 +9602,20 @@
         <v>Despliegue v2.74: Saldos extractos Mercado Pago — el PDF de fin de mes es el resumen de cuenta. No da de alta movimientos: verifica que cada operación esté en la app y que el saldo final cierre. Se vació la serie de cartas (junio 2025 a septiembre 2026) para recargarla mes a mes. Producción Vercel.</v>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>2.75</v>
+      </c>
+      <c r="B119" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Despliegue v2.75: Flujo de caja — ratio Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas, efectivo neto ingresado). Total solo meses reales. PDF y Excel. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C118"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C119"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9618,7 +9663,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). Incluye PDF de una página con filtros activos y formatos de moneda.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). Incluye PDF de una página con filtros activos y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>

</xml_diff>

<commit_message>
v2.76: el mes en curso no distorsiona el Total ni la tendencia.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E423"/>
+  <dimension ref="A1:E426"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7602,9 +7602,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="424">
+      <c r="A424" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B424" t="str">
+        <v>16:22</v>
+      </c>
+      <c r="C424" t="str">
+        <v>Mes en curso fuera del Total y del gráfico</v>
+      </c>
+      <c r="D424" t="str">
+        <v>En Flujo de caja el mes en curso queda en celeste en la tabla y en la barra del gráfico G/P. No entra en las tarjetas, en la columna Total, en los ratios, en el PDF ni en el Excel, ni en las variaciones y la tendencia. La proyección también toma solo meses cerrados.</v>
+      </c>
+      <c r="E424" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B425" t="str">
+        <v>16:34</v>
+      </c>
+      <c r="C425" t="str">
+        <v>G/P del mes en curso en el gráfico</v>
+      </c>
+      <c r="D425" t="str">
+        <v>Sobre la barra celeste del mes en curso, el gráfico G/P Mensual muestra el resultado en millones, con signo si es ganancia o pérdida, igual que el resto de la serie. Sigue fuera de la variación y de la tendencia.</v>
+      </c>
+      <c r="E425" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B426" t="str">
+        <v>16:40</v>
+      </c>
+      <c r="C426" t="str">
+        <v>Despliegue v2.76 producción</v>
+      </c>
+      <c r="D426" t="str">
+        <v>Push a main y Vercel --prod: en Flujo de caja el mes en curso queda en celeste, fuera del Total, de los ratios, de la variación y de la tendencia. La barra muestra el G/P en millones. APP_VERSION 2.76.</v>
+      </c>
+      <c r="E426" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E423"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E426"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7630,7 +7681,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas); Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total (Ingresos, Egresos, G/P y ratios) suma solo meses reales y va después de esos meses; las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas); Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total (Ingresos, Egresos, G/P y ratios) suma meses cerrados y va después de esos meses: el mes en curso se marca en celeste y no entra al Total, ni a las variaciones y la tendencia del gráfico, ni a la base de la proyección. Sobre esa barra se ve el G/P del mes en millones. Las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -7638,7 +7689,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Tres tarjetas: Ingresos totales, Egresos totales y G/P operativo (misma base operativa que la tabla Flujo por mes y el filtro Período), en ARS o USD según selector.</v>
+        <v>Tres tarjetas: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector.</v>
       </c>
     </row>
     <row r="4">
@@ -8297,7 +8348,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9613,9 +9664,20 @@
         <v>Despliegue v2.75: Flujo de caja — ratio Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas, efectivo neto ingresado). Total solo meses reales. PDF y Excel. Producción Vercel.</v>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>2.76</v>
+      </c>
+      <c r="B120" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Despliegue v2.76: Flujo de caja — el mes en curso se marca en celeste y no entra en las tarjetas, el Total, los ratios, el PDF ni el Excel. En el gráfico esa barra muestra el G/P en millones y no participa de la variación ni de la tendencia. La proyección usa solo meses cerrados. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C119"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C120"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.77: Mercado Pago vuelve a la carta de saldo.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E426"/>
+  <dimension ref="A1:E429"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7653,9 +7653,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="427">
+      <c r="A427" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B427" t="str">
+        <v>18:39</v>
+      </c>
+      <c r="C427" t="str">
+        <v>Mercado Pago vuelve a la carta de saldo</v>
+      </c>
+      <c r="D427" t="str">
+        <v>Saldos extractos de Mercado Pago deja el resumen de cuenta (solo traía el disponible) y vuelve a la carta de saldo. El corte es el saldo total, con el dinero a liberar. Al 30/09/2026 el cierre es $ 68.955.143,71. Se restauró la serie de cartas (junio 2025 a septiembre 2026) y se agregó la carta al 30/09. El mes en curso parte de ese saldo total y suma los movimientos del extracto desde el día siguiente. Se borraron los 16 resúmenes de cuenta.</v>
+      </c>
+      <c r="E427" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B428" t="str">
+        <v>18:46</v>
+      </c>
+      <c r="C428" t="str">
+        <v>Carta de Mercado Pago al 01/10</v>
+      </c>
+      <c r="D428" t="str">
+        <v>La carta al 30/09/2026 ($ 68.955.143,71 de saldo total) queda como período 01/10/2026, igual que el resto de la serie (día 1). El mes en curso sigue partiendo de ese saldo y suma los movimientos del extracto desde el 01/10.</v>
+      </c>
+      <c r="E428" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B429" t="str">
+        <v>18:51</v>
+      </c>
+      <c r="C429" t="str">
+        <v>Despliegue v2.77 producción</v>
+      </c>
+      <c r="D429" t="str">
+        <v>Push a main y Vercel --prod: Saldos extractos de Mercado Pago vuelve a la carta de saldo (saldo total, con el dinero a liberar). La última carta queda al 01/10/2026. El mes en curso parte de ese saldo y suma los movimientos del extracto. APP_VERSION 2.77.</v>
+      </c>
+      <c r="E429" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E426"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E429"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8169,7 +8220,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el día a día entra por el Excel del extracto. El PDF resumen de cuenta (fin de mes) no da de alta movimientos: verifica que cada ID de operación esté en la app y que el saldo final cierre con el saldo inicial más esos movimientos. La serie de cartas se vació para volver a cargarla con ese resumen, mes por mes. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP y Credicoop, mes en curso = último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
       </c>
     </row>
     <row r="64">
@@ -8348,7 +8399,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C121"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9675,9 +9726,20 @@
         <v>Despliegue v2.76: Flujo de caja — el mes en curso se marca en celeste y no entra en las tarjetas, el Total, los ratios, el PDF ni el Excel. En el gráfico esa barra muestra el G/P en millones y no participa de la variación ni de la tendencia. La proyección usa solo meses cerrados. Producción Vercel.</v>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>2.77</v>
+      </c>
+      <c r="B121" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Despliegue v2.77: Saldos extractos Mercado Pago — vuelve la carta de saldo. El corte es el saldo total (incluye el dinero a liberar). La última carta queda al 01/10/2026, como el resto de la serie. El mes en curso parte de ese saldo y suma los movimientos del extracto. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C120"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C121"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9893,7 +9955,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (resumen de cuenta de fin de mes: verifica movimientos y saldo; la serie de cartas se vació para recargarla mes a mes), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En Galicia, mes en curso = saldo corrido del extracto (saldo real del banco). En MP y Credicoop, último corte + créditos − débitos. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo: saldo total, con el dinero a liberar; el resumen de cuenta no se usa), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En Galicia, mes en curso = saldo corrido del extracto (saldo real del banco). En MP, mes en curso = saldo total de la última carta + movimientos del extracto. En Credicoop, último corte + créditos − débitos. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>

</xml_diff>

<commit_message>
v2.78: ID Venta e ID Compra en cajas y en Todas las transacciones.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E429"/>
+  <dimension ref="A1:E431"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7704,9 +7704,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="430">
+      <c r="A430" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B430" t="str">
+        <v>14:45</v>
+      </c>
+      <c r="C430" t="str">
+        <v>ID Venta e ID Compra en movimientos</v>
+      </c>
+      <c r="D430" t="str">
+        <v>El histórico movimientos-historico guarda ID Venta e ID Compra en las cajas de banco y en las cajas físicas. Se ven en las tablas y se filtran en Filtros, y también en Flujo de caja → Todas las transacciones. El Excel de esos listados los incluye. sql/supabase_movimientos_id_venta_id_compra.sql.</v>
+      </c>
+      <c r="E430" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B431" t="str">
+        <v>15:16</v>
+      </c>
+      <c r="C431" t="str">
+        <v>Despliegue v2.78 producción</v>
+      </c>
+      <c r="D431" t="str">
+        <v>Push a main y Vercel --prod: ID Venta e ID Compra del histórico se ven y se filtran en las cajas de banco, en las cajas físicas y en Flujo de caja → Todas las transacciones. El Excel de esos listados los incluye. APP_VERSION 2.78.</v>
+      </c>
+      <c r="E431" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E429"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E431"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8100,7 +8134,7 @@
         <v>Todas las transacciones</v>
       </c>
       <c r="B48" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas (incluida Observaciones, después de Descripción). Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) y buscador por id operación, descripción u observaciones. Clic en un encabezado ordena asc/desc. Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas (incluida Observaciones, después de Descripción). Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) y buscador por id operación, descripción u observaciones. Clic en un encabezado ordena asc/desc. Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa. Columnas ID Venta e ID Compra (histórico), con filtro exacto.</v>
       </c>
     </row>
     <row r="49">
@@ -8204,7 +8238,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
     </row>
     <row r="62">
@@ -8212,7 +8246,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
     </row>
     <row r="63">
@@ -8399,7 +8433,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C121"/>
+  <dimension ref="A1:C122"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9737,9 +9771,20 @@
         <v>Despliegue v2.77: Saldos extractos Mercado Pago — vuelve la carta de saldo. El corte es el saldo total (incluye el dinero a liberar). La última carta queda al 01/10/2026, como el resto de la serie. El mes en curso parte de ese saldo y suma los movimientos del extracto. Producción Vercel.</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>2.78</v>
+      </c>
+      <c r="B122" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Despliegue v2.78: ID Venta e ID Compra del histórico se ven en las tablas de las cajas de banco, de las cajas físicas y de Flujo de caja → Todas las transacciones. Se filtran en Filtros y salen en el Excel de esos listados. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C121"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C122"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9941,7 +9986,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
       <c r="C14">
         <v>24</v>
@@ -9969,7 +10014,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B16" t="str">
-        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura), en cualquier tesorería, cierre o histórico) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Tras cada carga se abre el popup de resultado (nuevos, actualizados, sin cambios, omitidos). Un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha está en el Excel y el Id no viene. Apertura de Caja no entra al corte. El histórico no pisa el saldo de tesorería o cierre. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad.</v>
+        <v>Menú de cajas no conciliables. Efectivo-f (ARS) (efectivo pesos), Morba-s/f (ARS) (Transferencia Morba), Efectivo-f (USD) (efectivo dólar pesificado al MEP) y Efectivo-s/f ARS/USD (Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura), en cualquier tesorería, cierre o histórico) con tesorería abierta, cierre de caja e histórico por Id, sin extracto ni match. Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Tras cada carga se abre el popup de resultado (nuevos, actualizados, sin cambios, omitidos). Un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha está en el Excel y el Id no viene. Apertura de Caja no entra al corte. El histórico no pisa el saldo de tesorería o cierre. El saldo de corte alimenta Saldos extractos. Excel y permisos en Seguridad. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
       <c r="C16">
         <v>8</v>

</xml_diff>

<commit_message>
v2.79: el saldo de Efectivo y Morba no cuenta movimientos eliminados.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E431"/>
+  <dimension ref="A1:E433"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7738,9 +7738,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="432">
+      <c r="A432" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B432" t="str">
+        <v>15:47</v>
+      </c>
+      <c r="C432" t="str">
+        <v>Saldos sin movimientos eliminados</v>
+      </c>
+      <c r="D432" t="str">
+        <v>En Efectivo (ARS y USD) y Morba, el saldo de Saldos extractos y la comparación de Tesorería saldos se rearman si un corte no cierra con los movimientos que siguen en la caja. Lo eliminado o marcado A eliminar no entra. Morba deja el corte del 01/10 y vuelve al cierre que sí encadena ($ 3.075.920,42).</v>
+      </c>
+      <c r="E432" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B433" t="str">
+        <v>15:50</v>
+      </c>
+      <c r="C433" t="str">
+        <v>Despliegue v2.79 producción</v>
+      </c>
+      <c r="D433" t="str">
+        <v>Push a main y Vercel --prod: en Efectivo y Morba el saldo se rearma con los movimientos que siguen en la caja. Lo eliminado no entra en Saldos extractos ni en Tesorería saldos. APP_VERSION 2.79.</v>
+      </c>
+      <c r="E433" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E431"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E433"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8254,7 +8288,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
       </c>
     </row>
     <row r="64">
@@ -8433,7 +8467,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C122"/>
+  <dimension ref="A1:C123"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9782,9 +9816,20 @@
         <v>Despliegue v2.78: ID Venta e ID Compra del histórico se ven en las tablas de las cajas de banco, de las cajas físicas y de Flujo de caja → Todas las transacciones. Se filtran en Filtros y salen en el Excel de esos listados. Producción Vercel.</v>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>2.79</v>
+      </c>
+      <c r="B123" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Despliegue v2.79: Efectivo y Morba — el saldo se rearma con los movimientos que siguen en la caja. Lo eliminado no entra en Saldos extractos ni en la comparación de Tesorería saldos. Morba vuelve al cierre que cierra con esos movimientos. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C122"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C123"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.80: Galicia toma el cierre del último extracto y la columna pasa a Saldo Tesorería Fornitalia.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E433"/>
+  <dimension ref="A1:E436"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7772,9 +7772,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="434">
+      <c r="A434" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B434" t="str">
+        <v>15:57</v>
+      </c>
+      <c r="C434" t="str">
+        <v>Columna Saldo Tesorería Fornitalia</v>
+      </c>
+      <c r="D434" t="str">
+        <v>En Saldos extractos, el cuadro Tesorería vs mes en curso cambia el encabezado Saldo Excel por Saldo Tesorería Fornitalia. Queda para el próximo despliegue.</v>
+      </c>
+      <c r="E434" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="str">
+        <v>04/10/2026</v>
+      </c>
+      <c r="B435" t="str">
+        <v>10:10</v>
+      </c>
+      <c r="C435" t="str">
+        <v>Galicia: mes en curso solo del último extracto</v>
+      </c>
+      <c r="D435" t="str">
+        <v>En la comparación de Tesorería saldos, Galicia ARS/USD toma el saldo de cierre del último extracto cargado ese día. No compara el número de fila entre archivos distintos (el extracto (4) en la fila 332 pisaba al (5), que cierra en $ 202.872.555,08). La tesorería no entra en esa columna.</v>
+      </c>
+      <c r="E435" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="str">
+        <v>04/10/2026</v>
+      </c>
+      <c r="B436" t="str">
+        <v>10:34</v>
+      </c>
+      <c r="C436" t="str">
+        <v>Despliegue v2.80 producción</v>
+      </c>
+      <c r="D436" t="str">
+        <v>Push a main y Vercel --prod: la comparación muestra Saldo Tesorería Fornitalia, y el mes en curso de Galicia toma el cierre del último extracto, sin mezclar la tesorería. APP_VERSION 2.80.</v>
+      </c>
+      <c r="E436" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E433"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E436"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8288,7 +8339,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido de la última fila del extracto (el saldo real del banco) más lo posterior a esa fecha; no se re-suman todos los movimientos (así no se infla por re-subidas o cheques en proceso). En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo de cierre del último extracto cargado ese día más lo posterior a esa fecha; no se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
       </c>
     </row>
     <row r="64">
@@ -8467,7 +8518,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C123"/>
+  <dimension ref="A1:C124"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9827,9 +9878,20 @@
         <v>Despliegue v2.79: Efectivo y Morba — el saldo se rearma con los movimientos que siguen en la caja. Lo eliminado no entra en Saldos extractos ni en la comparación de Tesorería saldos. Morba vuelve al cierre que cierra con esos movimientos. Producción Vercel.</v>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>2.80</v>
+      </c>
+      <c r="B124" t="str">
+        <v>04/10/2026</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Despliegue v2.80: Tesorería vs mes en curso — la columna se llama Saldo Tesorería Fornitalia. En Galicia, el mes en curso es el saldo de cierre del último extracto cargado; la tesorería no se mezcla. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C123"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C124"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10045,7 +10107,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo: saldo total, con el dinero a liberar; el resumen de cuenta no se usa), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En Galicia, mes en curso = saldo corrido del extracto (saldo real del banco). En MP, mes en curso = saldo total de la última carta + movimientos del extracto. En Credicoop, último corte + créditos − débitos. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo: saldo total, con el dinero a liberar; el resumen de cuenta no se usa), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En Galicia, mes en curso = saldo de cierre del último extracto cargado (el del banco); la tesorería no se suma. En MP, mes en curso = saldo total de la última carta + movimientos del extracto. En Credicoop, último corte + créditos − débitos. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>

</xml_diff>

<commit_message>
v2.81: descartar un potencial duplicado no lo pasa a Confirmados.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E436"/>
+  <dimension ref="A1:E438"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7823,9 +7823,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="437">
+      <c r="A437" t="str">
+        <v>05/10/2026</v>
+      </c>
+      <c r="B437" t="str">
+        <v>14:40</v>
+      </c>
+      <c r="C437" t="str">
+        <v>Descartar duplicado no confirma</v>
+      </c>
+      <c r="D437" t="str">
+        <v>Al leer el extracto de Galicia, un potencial duplicado de tesorería (mismo importe, hasta 40 días) no se propone como conciliación. Descartarlo no lo pasa a Confirmados: si había una pareja automática, vuelve a Sugeridos. Una conciliación manual no se toca.</v>
+      </c>
+      <c r="E437" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="str">
+        <v>05/10/2026</v>
+      </c>
+      <c r="B438" t="str">
+        <v>14:53</v>
+      </c>
+      <c r="C438" t="str">
+        <v>Despliegue v2.81 producción</v>
+      </c>
+      <c r="D438" t="str">
+        <v>Push a main y Vercel --prod: descartar un potencial duplicado no lo pasa a Confirmados; si había pareja automática vuelve a Sugeridos. Mientras está en Potenciales duplicados no se propone. APP_VERSION 2.81.</v>
+      </c>
+      <c r="E438" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E436"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E438"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8323,7 +8357,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. Descartarlo no lo pasa a Confirmados: si había una pareja automática, vuelve a Sugeridos. Una conciliación manual no se toca. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
     </row>
     <row r="62">
@@ -8518,7 +8552,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C124"/>
+  <dimension ref="A1:C125"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9889,9 +9923,20 @@
         <v>Despliegue v2.80: Tesorería vs mes en curso — la columna se llama Saldo Tesorería Fornitalia. En Galicia, el mes en curso es el saldo de cierre del último extracto cargado; la tesorería no se mezcla. Producción Vercel.</v>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>2.81</v>
+      </c>
+      <c r="B125" t="str">
+        <v>05/10/2026</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Despliegue v2.81: Conciliación — un potencial duplicado de tesorería no se propone al leer el extracto. Descartarlo no lo pasa a Confirmados: la pareja automática vuelve a Sugeridos. Una conciliación manual no se toca. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C124"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C125"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10093,7 +10138,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados; descartar no los pasa a Confirmados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.82: descartar un potencial duplicado no toca conciliaciones ya hechas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E438"/>
+  <dimension ref="A1:E440"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7857,9 +7857,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="439">
+      <c r="A439" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="B439" t="str">
+        <v>13:14</v>
+      </c>
+      <c r="C439" t="str">
+        <v>Duplicados no tocan lo conciliado</v>
+      </c>
+      <c r="D439" t="str">
+        <v>Potenciales duplicados solo mira tesorería que todavía no está conciliada. Un movimiento ya confirmado no entra en el grupo. Descartar solo lo saca de la lista: no modifica ninguna conciliación ya hecha, ni automática ni manual.</v>
+      </c>
+      <c r="E439" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="B440" t="str">
+        <v>13:20</v>
+      </c>
+      <c r="C440" t="str">
+        <v>Despliegue v2.82 producción</v>
+      </c>
+      <c r="D440" t="str">
+        <v>Push a main y Vercel --prod: Potenciales duplicados solo lista tesorería sin conciliar. Descartar no modifica ninguna conciliación ya hecha. APP_VERSION 2.82.</v>
+      </c>
+      <c r="E440" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E438"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E440"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8357,7 +8391,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. Descartarlo no lo pasa a Confirmados: si había una pareja automática, vuelve a Sugeridos. Una conciliación manual no se toca. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
     </row>
     <row r="62">
@@ -8552,7 +8586,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C125"/>
+  <dimension ref="A1:C126"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9934,9 +9968,20 @@
         <v>Despliegue v2.81: Conciliación — un potencial duplicado de tesorería no se propone al leer el extracto. Descartarlo no lo pasa a Confirmados: la pareja automática vuelve a Sugeridos. Una conciliación manual no se toca. Producción Vercel.</v>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>2.82</v>
+      </c>
+      <c r="B126" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Despliegue v2.82: Conciliación — Potenciales duplicados solo muestra tesorería que todavía no está conciliada. Un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C125"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C126"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10138,7 +10183,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados; descartar no los pasa a Confirmados). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados; el listado solo mira tesorería sin conciliar y descartar no toca las conciliaciones ya hechas). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.83: cada perfil elige qué secciones ve en Flujo de caja.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E440"/>
+  <dimension ref="A1:E442"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7891,9 +7891,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="441">
+      <c r="A441" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="B441" t="str">
+        <v>13:52</v>
+      </c>
+      <c r="C441" t="str">
+        <v>Secciones de Flujo de caja por perfil</v>
+      </c>
+      <c r="D441" t="str">
+        <v>En Seguridad → Flujo de caja se elige qué ve cada perfil: Cards, Flujo por mes, Todas las transacciones, Evolución y Estado financiero. Cargar tesorería histórica es un permiso aparte y el botón queda arriba, junto a Exportar Base Histórica, aunque esa solapa esté oculta. sql/supabase_flujo_secciones_por_perfil.sql.</v>
+      </c>
+      <c r="E441" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="B442" t="str">
+        <v>13:57</v>
+      </c>
+      <c r="C442" t="str">
+        <v>Despliegue v2.83 producción</v>
+      </c>
+      <c r="D442" t="str">
+        <v>Push a main y Vercel --prod: en Flujo de caja cada perfil elige Cards, Flujo por mes, Todas las transacciones, Evolución y Estado financiero. Cargar tesorería histórica queda arriba, junto a Exportar Base Histórica. APP_VERSION 2.83.</v>
+      </c>
+      <c r="E442" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E440"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E442"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8111,7 +8145,7 @@
         <v>Seguridad y roles</v>
       </c>
       <c r="B26" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Recuperar contraseña desde el login (enlace por email). Permisos granulares desde Supabase: ver_solapa_flujo (menú y solapa Flujo de caja), ver_solapa_* (resto de solapas del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo de caja + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Recuperar contraseña desde el login (enlace por email). Permisos granulares desde Supabase: ver_solapa_flujo (menú y solapa Flujo de caja), ver_solapa_* (resto de solapas del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo de caja + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. En Flujo de caja el perfil define Cards, Flujo por mes, Todas las transacciones, Evolución, Estado financiero y el botón Cargar tesorería histórica (arriba, junto a Exportar Base Histórica). Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
       </c>
     </row>
     <row r="27">
@@ -8586,7 +8620,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C127"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9979,9 +10013,20 @@
         <v>Despliegue v2.82: Conciliación — Potenciales duplicados solo muestra tesorería que todavía no está conciliada. Un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Producción Vercel.</v>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>2.83</v>
+      </c>
+      <c r="B127" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Despliegue v2.83: Flujo de caja — cada perfil elige si ve Cards, Flujo por mes, Todas las transacciones, Evolución y Estado financiero. Cargar tesorería histórica queda arriba, junto a Exportar Base Histórica, aunque Flujo por mes esté oculto. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C126"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C127"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10141,7 +10186,7 @@
         <v>Seguridad y roles (dashboard)</v>
       </c>
       <c r="B11" t="str">
-        <v>Autenticación email/anónimo, recuperar contraseña por email, roles Admin/Encargado/Visor y perfiles a medida, permisos granulares por solapa/menú/acción (Flujo de caja como primer menú si hay permiso), pantalla Seguridad para crear perfiles, asignar roles y toggles por ítem (incluido Visor).</v>
+        <v>Autenticación email/anónimo, recuperar contraseña por email, roles Admin/Encargado/Visor y perfiles a medida, permisos granulares por solapa/menú/acción (Flujo de caja como primer menú si hay permiso; dentro, Cards, Flujo por mes, Todas las transacciones, Evolución, Estado financiero y Cargar tesorería histórica se prenden por perfil), pantalla Seguridad para crear perfiles, asignar roles y toggles por ítem (incluido Visor).</v>
       </c>
       <c r="C11">
         <v>18</v>

</xml_diff>

<commit_message>
v2.84: torta de la posición de caja en Flujo, con el total en millones y en el PDF.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E442"/>
+  <dimension ref="A1:E445"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7925,9 +7925,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="443">
+      <c r="A443" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B443" t="str">
+        <v>09:30</v>
+      </c>
+      <c r="C443" t="str">
+        <v>Torta de posición de caja</v>
+      </c>
+      <c r="D443" t="str">
+        <v>En Flujo de caja, a la derecha de las tres tarjetas, un gráfico de torta con la posición de hoy: Galicia, Mercado Pago, Credicoop, Efectivo (Efectivo-f ARS + USD) y Resto (Efectivo sin factura ARS y USD + Morba). Monto en millones y porcentaje, en dos columnas alineadas. Las tarjetas no se estiran.</v>
+      </c>
+      <c r="E443" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B444" t="str">
+        <v>09:45</v>
+      </c>
+      <c r="C444" t="str">
+        <v>Solapas y total en la torta</v>
+      </c>
+      <c r="D444" t="str">
+        <v>Las solapas de Flujo de caja quedan alineadas al borde inferior de la torta, para dejar más alto el gráfico de G/P. El subtítulo muestra el total de la posición en millones (Hoy · mes · XX M pesos). Esa torta también entra en el reporte PDF.</v>
+      </c>
+      <c r="E444" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B445" t="str">
+        <v>10:54</v>
+      </c>
+      <c r="C445" t="str">
+        <v>Despliegue v2.84 producción</v>
+      </c>
+      <c r="D445" t="str">
+        <v>Push a main y Vercel --prod: en Flujo de caja, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Las solapas quedan al borde de la torta y el PDF la incluye. APP_VERSION 2.84.</v>
+      </c>
+      <c r="E445" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E442"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E445"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7961,7 +8012,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Tres tarjetas: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector.</v>
+        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total en millones. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
       </c>
     </row>
     <row r="4">
@@ -8620,7 +8671,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C127"/>
+  <dimension ref="A1:C128"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10024,9 +10075,20 @@
         <v>Despliegue v2.83: Flujo de caja — cada perfil elige si ve Cards, Flujo por mes, Todas las transacciones, Evolución y Estado financiero. Cargar tesorería histórica queda arriba, junto a Exportar Base Histórica, aunque Flujo por mes esté oculto. Producción Vercel.</v>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>2.84</v>
+      </c>
+      <c r="B128" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="C128" t="str">
+        <v>Despliegue v2.84: Flujo de caja — torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Las solapas quedan al borde inferior de la torta y el gráfico de G/P tiene más lugar. El PDF de Flujo incluye esa torta. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C127"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C128"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10074,7 +10136,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). Incluye PDF de una página con filtros activos y formatos de moneda.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>

</xml_diff>

<commit_message>
v2.85: con USD, la torta, el gráfico de G/P y la tabla usan el dólar seleccionado.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E445"/>
+  <dimension ref="A1:E447"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -7976,9 +7976,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="446">
+      <c r="A446" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B446" t="str">
+        <v>11:03</v>
+      </c>
+      <c r="C446" t="str">
+        <v>Dólar en torta, gráfico y tabla</v>
+      </c>
+      <c r="D446" t="str">
+        <v>Al pasar el selector a USD, la torta de posición, el gráfico G/P y la tabla de Flujo por mes quedan en el dólar elegido (MEP, CCL u oficial). La torta divide la posición en pesos por la cotización de hoy. El gráfico y la tabla usan esa misma cotización en cada movimiento.</v>
+      </c>
+      <c r="E446" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B447" t="str">
+        <v>11:07</v>
+      </c>
+      <c r="C447" t="str">
+        <v>Despliegue v2.85 producción</v>
+      </c>
+      <c r="D447" t="str">
+        <v>Push a main y Vercel --prod: con USD, la torta de posición, el gráfico G/P y la tabla de Flujo quedan en el dólar elegido (MEP, CCL u oficial). APP_VERSION 2.85.</v>
+      </c>
+      <c r="E447" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E445"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E447"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8012,7 +8046,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total en millones. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
+        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total en millones. Con USD, la torta, el gráfico G/P y la tabla usan el dólar elegido (MEP, CCL u oficial). Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
       </c>
     </row>
     <row r="4">
@@ -8671,7 +8705,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C128"/>
+  <dimension ref="A1:C129"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10086,9 +10120,20 @@
         <v>Despliegue v2.84: Flujo de caja — torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Las solapas quedan al borde inferior de la torta y el gráfico de G/P tiene más lugar. El PDF de Flujo incluye esa torta. Producción Vercel.</v>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>2.85</v>
+      </c>
+      <c r="B129" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="C129" t="str">
+        <v>Despliegue v2.85: Flujo de caja — al elegir USD, la torta de posición, el gráfico G/P y la tabla usan el dólar seleccionado (MEP, CCL u oficial). En pesos no cambia. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C128"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C129"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10136,7 +10181,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Con USD, la torta, el gráfico G/P y la tabla usan el dólar elegido (MEP, CCL u oficial). Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>

</xml_diff>

<commit_message>
v2.86: con USD, la torta de posición muestra miles de dólares.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E447"/>
+  <dimension ref="A1:E449"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8010,9 +8010,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="448">
+      <c r="A448" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B448" t="str">
+        <v>11:11</v>
+      </c>
+      <c r="C448" t="str">
+        <v>Torta en dólares en miles</v>
+      </c>
+      <c r="D448" t="str">
+        <v>Con USD, la torta de posición muestra los montos en miles (por ejemplo 135 mil dólares MEP), no en millones. En pesos sigue en millones.</v>
+      </c>
+      <c r="E448" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B449" t="str">
+        <v>11:16</v>
+      </c>
+      <c r="C449" t="str">
+        <v>Despliegue v2.86 producción</v>
+      </c>
+      <c r="D449" t="str">
+        <v>Push a main y Vercel --prod: con USD, la torta de posición muestra miles de dólares (MEP, CCL u oficial). En pesos sigue en millones. APP_VERSION 2.86.</v>
+      </c>
+      <c r="E449" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E447"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E449"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8046,7 +8080,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total en millones. Con USD, la torta, el gráfico G/P y la tabla usan el dólar elegido (MEP, CCL u oficial). Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
+        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total. Con USD, la torta muestra miles de dólares (MEP, CCL u oficial); el gráfico G/P y la tabla usan ese mismo dólar. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
       </c>
     </row>
     <row r="4">
@@ -8705,7 +8739,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C129"/>
+  <dimension ref="A1:C130"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10131,9 +10165,20 @@
         <v>Despliegue v2.85: Flujo de caja — al elegir USD, la torta de posición, el gráfico G/P y la tabla usan el dólar seleccionado (MEP, CCL u oficial). En pesos no cambia. Producción Vercel.</v>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>2.86</v>
+      </c>
+      <c r="B130" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="C130" t="str">
+        <v>Despliegue v2.86: Flujo de caja — con USD, la torta de posición muestra los montos en miles de dólares (MEP, CCL u oficial). En pesos sigue en millones. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C129"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C130"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10181,7 +10226,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Con USD, la torta, el gráfico G/P y la tabla usan el dólar elegido (MEP, CCL u oficial). Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Con USD, la torta muestra miles de dólares (MEP, CCL u oficial); el gráfico G/P y la tabla usan ese mismo dólar. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>

</xml_diff>

<commit_message>
v2.87: el mes en curso de Galicia no suma un cheque todavía no imputado.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E449"/>
+  <dimension ref="A1:E451"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8044,9 +8044,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="450">
+      <c r="A450" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B450" t="str">
+        <v>11:28</v>
+      </c>
+      <c r="C450" t="str">
+        <v>Saldo extracto sin no imputados</v>
+      </c>
+      <c r="D450" t="str">
+        <v>En Saldos extractos, el mes en curso de Galicia no suma un movimiento que el banco todavía no imputó. El 09/10 hay un cheque Acred. Cheque 48hs En Proceso de $ 2.266.220 (estado Pendiente): el saldo pasa de $ 216.277.938,07 a $ 214.011.718,07. Mercado Pago y Credicoop no cambian.</v>
+      </c>
+      <c r="E450" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B451" t="str">
+        <v>11:41</v>
+      </c>
+      <c r="C451" t="str">
+        <v>Despliegue v2.87 producción</v>
+      </c>
+      <c r="D451" t="str">
+        <v>Push a main y Vercel --prod: el mes en curso de Galicia no suma un cheque o movimiento que el banco todavía no imputó. El cheque del 09/10 ($ 2.266.220) queda afuera y el saldo pasa a $ 214.011.718,07. APP_VERSION 2.87.</v>
+      </c>
+      <c r="E451" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E449"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E451"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8560,7 +8594,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo de cierre del último extracto cargado ese día más lo posterior a esa fecha; no se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
       </c>
     </row>
     <row r="64">
@@ -8739,7 +8773,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C130"/>
+  <dimension ref="A1:C131"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10176,9 +10210,20 @@
         <v>Despliegue v2.86: Flujo de caja — con USD, la torta de posición muestra los montos en miles de dólares (MEP, CCL u oficial). En pesos sigue en millones. Producción Vercel.</v>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>2.87</v>
+      </c>
+      <c r="B131" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="C131" t="str">
+        <v>Despliegue v2.87: Saldos extractos — el mes en curso de Galicia no suma un cheque o movimiento que el banco todavía no imputó. El cheque del 09/10 ($ 2.266.220, En proceso) queda afuera y el saldo pasa a $ 214.011.718,07. Ese saldo también entra en la torta de posición. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C130"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C131"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10394,7 +10439,7 @@
         <v>Saldos extractos bancarios</v>
       </c>
       <c r="B15" t="str">
-        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo: saldo total, con el dinero a liberar; el resumen de cuenta no se usa), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En Galicia, mes en curso = saldo de cierre del último extracto cargado (el del banco); la tesorería no se suma. En MP, mes en curso = saldo total de la última carta + movimientos del extracto. En Credicoop, último corte + créditos − débitos. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
+        <v>Menú de saldos de cierre: Mercado Pago (carta de saldo: saldo total, con el dinero a liberar; el resumen de cuenta no se usa), Galicia (ARS, resumen PDF), Galicia (USD, PDF Extracto_Cuentas_Galicia_… o Extracto_CCE pesificado al MEP), Credicoop (corte desde tesorería, sin extractos históricos), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD) (cajas físicas desde Cajas) y posición consolidada mensual. En Galicia, mes en curso = saldo corrido del último movimiento Imputado (un cheque Pendiente o En proceso no entra); la tesorería no se suma. En MP, mes en curso = saldo total de la última carta + movimientos del extracto. En Credicoop, último corte + créditos − débitos. En cajas USD, debajo del saldo en pesos se ve el monto en dólares. Reporte PDF de la vista activa (cards, gráfico y tabla). Promedios de saldo y variación, Excel y permisos en Seguridad.</v>
       </c>
       <c r="C15">
         <v>12</v>

</xml_diff>

<commit_message>
v2.88: con USD, torta, gráfico y tabla usan la cotización de hoy.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E451"/>
+  <dimension ref="A1:E456"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8078,9 +8078,94 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="452">
+      <c r="A452" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B452" t="str">
+        <v>12:05</v>
+      </c>
+      <c r="C452" t="str">
+        <v>Dólar a una sola cotización</v>
+      </c>
+      <c r="D452" t="str">
+        <v>Con USD, la posición de caja, el gráfico G/P y la tabla de Flujo usan una sola cotización: la de hoy del dólar elegido (MEP, CCL u oficial), o la inmediata anterior. Los pesos se dividen por esa cotización; lo que ya está en dólares no se vuelve a convertir. La cotización se ve debajo del selector y en la torta.</v>
+      </c>
+      <c r="E452" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B453" t="str">
+        <v>12:37</v>
+      </c>
+      <c r="C453" t="str">
+        <v>Cotización desde la tabla global</v>
+      </c>
+      <c r="D453" t="str">
+        <v>El dólar del Flujo, de Saldos extractos y de Cajas se lee de tipos_cambio_global de Sistema Contable (al día). La copia local de Fornitalia quedaba en el 27/02/2026. Si esa tabla no responde, se usa la copia local.</v>
+      </c>
+      <c r="E453" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B454" t="str">
+        <v>12:43</v>
+      </c>
+      <c r="C454" t="str">
+        <v>Cotización fuera de la fila de filtros</v>
+      </c>
+      <c r="D454" t="str">
+        <v>En dólares, la cotización ya no va debajo del selector: esa fila queda en una sola línea, alineada como en pesos. El valor sigue en la torta y en el texto del gráfico.</v>
+      </c>
+      <c r="E454" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B455" t="str">
+        <v>12:47</v>
+      </c>
+      <c r="C455" t="str">
+        <v>Selector de dólar en una línea</v>
+      </c>
+      <c r="D455" t="str">
+        <v>La leyenda del selector pasa de Conversión a dólar a Dólar, para que moneda, dólar, período y botones entren en una sola fila.</v>
+      </c>
+      <c r="E455" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B456" t="str">
+        <v>12:49</v>
+      </c>
+      <c r="C456" t="str">
+        <v>Despliegue v2.88 producción</v>
+      </c>
+      <c r="D456" t="str">
+        <v>Push a main y Vercel --prod: con USD, la torta, el gráfico y la tabla usan la cotización de hoy del dólar elegido (hoy MEP 1.541,03). El selector dice Dólar y la fila queda en una sola línea. APP_VERSION 2.88.</v>
+      </c>
+      <c r="E456" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E451"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E456"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8114,7 +8199,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total. Con USD, la torta muestra miles de dólares (MEP, CCL u oficial); el gráfico G/P y la tabla usan ese mismo dólar. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
+        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total. Con USD, la torta, el gráfico G/P y la tabla usan una sola cotización del dólar elegido (la de hoy, o la inmediata anterior): los pesos se dividen por esa cotización y lo que ya está en dólares no se vuelve a convertir. La cotización se ve debajo del selector y se lee de la tabla global de Sistema Contable. La torta, en dólares, muestra miles. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
       </c>
     </row>
     <row r="4">
@@ -8773,7 +8858,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C131"/>
+  <dimension ref="A1:C132"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10221,9 +10306,20 @@
         <v>Despliegue v2.87: Saldos extractos — el mes en curso de Galicia no suma un cheque o movimiento que el banco todavía no imputó. El cheque del 09/10 ($ 2.266.220, En proceso) queda afuera y el saldo pasa a $ 214.011.718,07. Ese saldo también entra en la torta de posición. Producción Vercel.</v>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>2.88</v>
+      </c>
+      <c r="B132" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="C132" t="str">
+        <v>Despliegue v2.88: con USD, la torta, el gráfico G/P y la tabla usan una sola cotización, la de hoy del dólar elegido (hoy MEP 1.541,03). El selector dice Dólar y la fila de filtros queda en una sola línea. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C131"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C132"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10271,7 +10367,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Con USD, la torta muestra miles de dólares (MEP, CCL u oficial); el gráfico G/P y la tabla usan ese mismo dólar. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Con USD, la torta, el gráfico G/P y la tabla usan una sola cotización del dólar elegido (la de hoy, o la inmediata anterior): los pesos se dividen por esa cotización y lo que ya está en dólares no se vuelve a convertir. La cotización se ve debajo del selector y se lee de la tabla global de Sistema Contable. La torta, en dólares, muestra miles. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>

</xml_diff>

<commit_message>
v2.89: en pesos, la torta pesifica los dólares con la cotización de hoy.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E456"/>
+  <dimension ref="A1:E458"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8163,9 +8163,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="457">
+      <c r="A457" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B457" t="str">
+        <v>13:23</v>
+      </c>
+      <c r="C457" t="str">
+        <v>Torta en pesos con la cotización de hoy</v>
+      </c>
+      <c r="D457" t="str">
+        <v>En ARS, la torta de posición pesifica los dólares con la misma cotización de hoy del dólar elegido (o la inmediata anterior) que al ver en dólares. El subtítulo queda Hoy · mes · total · MEP 1.541,22.</v>
+      </c>
+      <c r="E457" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B458" t="str">
+        <v>13:37</v>
+      </c>
+      <c r="C458" t="str">
+        <v>Despliegue v2.89 producción</v>
+      </c>
+      <c r="D458" t="str">
+        <v>Push a main y Vercel --prod: en pesos, la torta pesifica los dólares con la cotización de hoy del dólar elegido (hoy MEP 1.541,22) y la muestra en el subtítulo. Es la misma que al ver en dólares. APP_VERSION 2.89.</v>
+      </c>
+      <c r="E458" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E456"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E458"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8199,7 +8233,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total. Con USD, la torta, el gráfico G/P y la tabla usan una sola cotización del dólar elegido (la de hoy, o la inmediata anterior): los pesos se dividen por esa cotización y lo que ya está en dólares no se vuelve a convertir. La cotización se ve debajo del selector y se lee de la tabla global de Sistema Contable. La torta, en dólares, muestra miles. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
+        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total y la cotización. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable y se ve en el subtítulo de la torta. La torta, en dólares, muestra miles. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
       </c>
     </row>
     <row r="4">
@@ -8858,7 +8892,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C132"/>
+  <dimension ref="A1:C133"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10317,9 +10351,20 @@
         <v>Despliegue v2.88: con USD, la torta, el gráfico G/P y la tabla usan una sola cotización, la de hoy del dólar elegido (hoy MEP 1.541,03). El selector dice Dólar y la fila de filtros queda en una sola línea. Producción Vercel.</v>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>2.89</v>
+      </c>
+      <c r="B133" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="C133" t="str">
+        <v>Despliegue v2.89: en pesos, la torta de posición pesifica los dólares con la cotización de hoy del dólar elegido (hoy MEP 1.541,22), o la del día anterior, y la muestra en el subtítulo. Es la misma cotización que al ver en dólares. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C132"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C133"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10367,7 +10412,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total en el subtítulo. Con USD, la torta, el gráfico G/P y la tabla usan una sola cotización del dólar elegido (la de hoy, o la inmediata anterior): los pesos se dividen por esa cotización y lo que ya está en dólares no se vuelve a convertir. La cotización se ve debajo del selector y se lee de la tabla global de Sistema Contable. La torta, en dólares, muestra miles. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total y la cotización en el subtítulo. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable. La torta, en dólares, muestra miles. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>

</xml_diff>

<commit_message>
v2.90: cajas FCI Galicia en conciliación, saldos y torta.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E458"/>
+  <dimension ref="A1:E460"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8197,9 +8197,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="459">
+      <c r="A459" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="B459" t="str">
+        <v>12:53</v>
+      </c>
+      <c r="C459" t="str">
+        <v>Cajas FCI Galicia (ARS) y (USD)</v>
+      </c>
+      <c r="D459" t="str">
+        <v>Dos cajas nuevas en Conciliación Bancaria: FCI Galicia (ARS) y FCI Galicia (USD). La tesorería se carga igual que el resto (histórico con Caja FCI Galicia (ARS) o (USD)). No hay extracto propio: las sugerencias usan el extracto de Galicia de la misma moneda. En Saldos extractos entran como solapas y columnas del consolidado (el USD se pesifica al MEP). En la torta de Flujo de caja, FCI suma pesos y dólares con la misma cotización de hoy. sql/supabase_cb_fci_galicia.sql.</v>
+      </c>
+      <c r="E459" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="B460" t="str">
+        <v>13:17</v>
+      </c>
+      <c r="C460" t="str">
+        <v>Despliegue v2.90 producción</v>
+      </c>
+      <c r="D460" t="str">
+        <v>Push a main y Vercel --prod: cajas FCI Galicia (ARS) y FCI Galicia (USD) en Conciliación (sugerencias contra el extracto de Galicia), en Saldos extractos y en la torta de posición. APP_VERSION 2.90.</v>
+      </c>
+      <c r="E460" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E458"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E460"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8233,7 +8267,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total y la cotización. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable y se ve en el subtítulo de la torta. La torta, en dólares, muestra miles. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
+        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, FCI, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total y la cotización. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable y se ve en el subtítulo de la torta. La torta, en dólares, muestra miles. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
       </c>
     </row>
     <row r="4">
@@ -8697,7 +8731,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja) y Credicoop (botón negro). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja), Credicoop (botón negro) y FCI Galicia (ARS)/(USD) (verde). FCI carga solo tesorería (histórico con Caja FCI Galicia (ARS) o (USD)); las sugerencias salen del extracto de Galicia de la misma moneda, sin extracto propio. La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
     </row>
     <row r="62">
@@ -8713,7 +8747,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
       </c>
     </row>
     <row r="64">
@@ -8892,7 +8926,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C134"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10362,9 +10396,20 @@
         <v>Despliegue v2.89: en pesos, la torta de posición pesifica los dólares con la cotización de hoy del dólar elegido (hoy MEP 1.541,22), o la del día anterior, y la muestra en el subtítulo. Es la misma cotización que al ver en dólares. Producción Vercel.</v>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>2.90</v>
+      </c>
+      <c r="B134" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="C134" t="str">
+        <v>Despliegue v2.90: cajas FCI Galicia (ARS) y FCI Galicia (USD). En Conciliación se carga la tesorería y las sugerencias salen del extracto de Galicia de la misma moneda. Entran en Saldos extractos (solapas y consolidado) y en la torta de posición, pesificadas o dolarizadas con la cotización de hoy. sql/supabase_cb_fci_galicia.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C133"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C134"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10412,7 +10457,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, Efectivo y Resto) en millones y porcentaje, con el total y la cotización en el subtítulo. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable. La torta, en dólares, muestra miles. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, FCI, Efectivo y Resto) en millones y porcentaje, con el total y la cotización en el subtítulo. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable. La torta, en dólares, muestra miles. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>
@@ -10566,7 +10611,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro). En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados; el listado solo mira tesorería sin conciliar y descartar no toca las conciliaciones ya hechas). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro, FCI Galicia ARS y USD en verde). FCI no tiene extracto propio: la tesorería se concilia contra el extracto de Galicia de la misma moneda. En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados; el listado solo mira tesorería sin conciliar y descartar no toca las conciliaciones ya hechas). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
       <c r="C14">
         <v>24</v>

</xml_diff>

<commit_message>
v2.91: el mes en curso pesifica los dólares al MEP de hoy, igual que la torta.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E460"/>
+  <dimension ref="A1:E463"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8231,9 +8231,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="461">
+      <c r="A461" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="B461" t="str">
+        <v>13:29</v>
+      </c>
+      <c r="C461" t="str">
+        <v>FCI sin movimientos no es saldo 0</v>
+      </c>
+      <c r="D461" t="str">
+        <v>En Tesorería vs mes en curso, FCI Galicia (ARS) y (USD) se leían como la cuenta Galicia y el mes en curso tomaba ese saldo (diferencia de $ 215.847.791,48). Sin suscripciones ni rescates el mes en curso queda vacío. Si el archivo trae 0, coincide.</v>
+      </c>
+      <c r="E461" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="B462" t="str">
+        <v>13:39</v>
+      </c>
+      <c r="C462" t="str">
+        <v>Mes en curso al MEP de hoy</v>
+      </c>
+      <c r="D462" t="str">
+        <v>En Saldos extractos, el mes en curso pesifica los dólares (Galicia USD, FCI USD y efectivo en dólares) al MEP de hoy, o al inmediato anterior. Es la misma cotización de la torta de Flujo de caja, así el total consolidado y la torta coinciden. Los meses cerrados quedan al MEP de cada fecha.</v>
+      </c>
+      <c r="E462" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="B463" t="str">
+        <v>13:42</v>
+      </c>
+      <c r="C463" t="str">
+        <v>Despliegue v2.91 producción</v>
+      </c>
+      <c r="D463" t="str">
+        <v>Push a main y Vercel --prod: FCI sin movimientos no se compara con Galicia; el mes en curso de Saldos extractos pesifica los dólares al MEP de hoy, igual que la torta. APP_VERSION 2.91.</v>
+      </c>
+      <c r="E463" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E460"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E463"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8747,7 +8798,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. El mes en curso del consolidado pesifica todos los dólares al MEP de hoy (o el inmediato anterior), la misma cotización de la torta; los meses cerrados no se recalculan. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
       </c>
     </row>
     <row r="64">
@@ -8926,7 +8977,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10407,9 +10458,20 @@
         <v>Despliegue v2.90: cajas FCI Galicia (ARS) y FCI Galicia (USD). En Conciliación se carga la tesorería y las sugerencias salen del extracto de Galicia de la misma moneda. Entran en Saldos extractos (solapas y consolidado) y en la torta de posición, pesificadas o dolarizadas con la cotización de hoy. sql/supabase_cb_fci_galicia.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>2.91</v>
+      </c>
+      <c r="B135" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="C135" t="str">
+        <v>Despliegue v2.91: FCI sin suscripciones no marca diferencia en Tesorería vs mes en curso (ya no se lee como la cuenta Galicia). El mes en curso de Saldos extractos pesifica los dólares al MEP de hoy, o al inmediato anterior, la misma cotización de la torta. Los meses cerrados no se recalculan. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C134"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C135"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.92: la cotización y los Excel usan el día de hoy en Argentina.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E463"/>
+  <dimension ref="A1:E465"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8282,9 +8282,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="464">
+      <c r="A464" t="str">
+        <v>11/10/2026</v>
+      </c>
+      <c r="B464" t="str">
+        <v>15:00</v>
+      </c>
+      <c r="C464" t="str">
+        <v>Fechas siempre en horario argentino</v>
+      </c>
+      <c r="D464" t="str">
+        <v>El día de negocio (hoy, mes en curso, cotización, cortes y nombres de Excel) sale del calendario de Argentina. Una fecha sin hora no se corre al día anterior. La cotización de hoy se lee primero: el 11/10/2026 el MEP global es 1.539,28; si la torta decía “del 10/10” era porque no había entrado la fila de hoy.</v>
+      </c>
+      <c r="E464" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="str">
+        <v>11/10/2026</v>
+      </c>
+      <c r="B465" t="str">
+        <v>15:06</v>
+      </c>
+      <c r="C465" t="str">
+        <v>Despliegue v2.92 producción</v>
+      </c>
+      <c r="D465" t="str">
+        <v>Push a main y Vercel --prod: el día de hoy, la cotización y los Excel usan el calendario de Argentina. La torta toma el MEP de hoy (11/10, 1.539,28) o el inmediato anterior, con esa fecha a la vista. APP_VERSION 2.92.</v>
+      </c>
+      <c r="E465" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E463"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E465"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8977,7 +9011,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C135"/>
+  <dimension ref="A1:C136"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10469,9 +10503,20 @@
         <v>Despliegue v2.91: FCI sin suscripciones no marca diferencia en Tesorería vs mes en curso (ya no se lee como la cuenta Galicia). El mes en curso de Saldos extractos pesifica los dólares al MEP de hoy, o al inmediato anterior, la misma cotización de la torta. Los meses cerrados no se recalculan. Producción Vercel.</v>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>2.92</v>
+      </c>
+      <c r="B136" t="str">
+        <v>11/10/2026</v>
+      </c>
+      <c r="C136" t="str">
+        <v>Despliegue v2.92: el día de hoy, el mes en curso y los Excel usan el calendario de Argentina. La cotización del Flujo es la de hoy (MEP 1.539,28 del 11/10) o la inmediata anterior, con la fecha a la vista. Una fecha sin hora no se corre al día anterior. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C135"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C136"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.93: el histórico marca en A eliminar lo que ya no viene en las cajas físicas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E465"/>
+  <dimension ref="A1:E467"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8316,9 +8316,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="466">
+      <c r="A466" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B466" t="str">
+        <v>08:59</v>
+      </c>
+      <c r="C466" t="str">
+        <v>Histórico: A eliminar también en cajas físicas</v>
+      </c>
+      <c r="D466" t="str">
+        <v>El Excel movimientos-historico trae columna Monto y en Efectivo, Morba y el resto de cajas físicas se leía como un cierre: no buscaba Ids que ya no vienen. El Id 10003755 (Morba, 08/10/2026, Pendiente, −33,77) quedó afuera de A eliminar por eso. Ahora el histórico marca Pendiente o Status vacío ausente en todas las cajas, de banco y físicas. Confirmado y un archivo de cierre no se marcan. sql/supabase_cf_historico_no_es_cierre.sql. Hay que volver a cargar el mismo histórico para que aparezcan.</v>
+      </c>
+      <c r="E466" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B467" t="str">
+        <v>09:02</v>
+      </c>
+      <c r="C467" t="str">
+        <v>Despliegue v2.93 producción</v>
+      </c>
+      <c r="D467" t="str">
+        <v>Push a main y Vercel --prod: al cargar el histórico, Efectivo, Morba y el resto de cajas físicas marcan en A eliminar el Pendiente que ya no viene, igual que las cajas de banco. Confirmado no se elimina. APP_VERSION 2.93.</v>
+      </c>
+      <c r="E467" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E465"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E467"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9011,7 +9045,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C136"/>
+  <dimension ref="A1:C137"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10514,9 +10548,20 @@
         <v>Despliegue v2.92: el día de hoy, el mes en curso y los Excel usan el calendario de Argentina. La cotización del Flujo es la de hoy (MEP 1.539,28 del 11/10) o la inmediata anterior, con la fecha a la vista. Una fecha sin hora no se corre al día anterior. Producción Vercel.</v>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>2.93</v>
+      </c>
+      <c r="B137" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="C137" t="str">
+        <v>Despliegue v2.93: al cargar el histórico, Efectivo, Morba y el resto de cajas físicas marcan en A eliminar el Pendiente cuyo Id ya no viene, igual que las cajas de banco. El 10003755 (Morba, 08/10) entra al volver a cargar ese archivo. Confirmado y un cierre no se marcan. sql/supabase_cf_historico_no_es_cierre.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C136"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C137"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.94: el histórico de cajas físicas vuelve a conservar el monto.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E467"/>
+  <dimension ref="A1:E469"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8350,9 +8350,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="468">
+      <c r="A468" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B468" t="str">
+        <v>09:22</v>
+      </c>
+      <c r="C468" t="str">
+        <v>Importes de cajas físicas vueltos a cargar</v>
+      </c>
+      <c r="D468" t="str">
+        <v>La carga del histórico de las 09:05 dejó en 0 el importe de Efectivo-f, Efectivo s/f y Morba (el archivo trae Monto y, al dejar de leerse como cierre, no se tomaba esa columna). Se repusieron 766 movimientos desde movimientos-historico_2026-10-12.xlsx. En dólares se pesificó con el MEP que ya tenía cada fila (el egreso de 4.000 USD del 11/10 queda en −6.157.120). Las cajas de banco no se tocaron. El parser vuelve a leer Monto en el histórico. No volver a cargar ese archivo en el sitio publicado hasta el próximo despliegue: la versión en línea todavía lo pone en 0.</v>
+      </c>
+      <c r="E468" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B469" t="str">
+        <v>09:25</v>
+      </c>
+      <c r="C469" t="str">
+        <v>Despliegue v2.94 producción</v>
+      </c>
+      <c r="D469" t="str">
+        <v>Push a main y Vercel --prod: el histórico de cajas físicas vuelve a tomar la columna Monto (en dólares se pesifica al MEP de la fecha). Los importes que quedaron en 0 a las 09:05 ya están repuestos. Se puede volver a cargar el mismo archivo. APP_VERSION 2.94.</v>
+      </c>
+      <c r="E469" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E467"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E469"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8858,7 +8892,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. El histórico conserva la columna Monto (en dólares se pesifica al MEP de la fecha).</v>
       </c>
     </row>
     <row r="63">
@@ -9045,7 +9079,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C137"/>
+  <dimension ref="A1:C138"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10559,9 +10593,20 @@
         <v>Despliegue v2.93: al cargar el histórico, Efectivo, Morba y el resto de cajas físicas marcan en A eliminar el Pendiente cuyo Id ya no viene, igual que las cajas de banco. El 10003755 (Morba, 08/10) entra al volver a cargar ese archivo. Confirmado y un cierre no se marcan. sql/supabase_cf_historico_no_es_cierre.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>2.94</v>
+      </c>
+      <c r="B138" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="C138" t="str">
+        <v>Despliegue v2.94: el histórico de Efectivo y Morba vuelve a leer la columna Monto. La carga de las 09:05 había dejado esos importes en 0; se repusieron 766 movimientos (el egreso de 4.000 USD del 11/10 queda en −6.157.120). Se puede volver a cargar el mismo archivo. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C137"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C138"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.94: el saldo de las cajas físicas sale de crédito y débito.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E469"/>
+  <dimension ref="A1:E470"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8375,18 +8375,35 @@
         <v>09:25</v>
       </c>
       <c r="C469" t="str">
+        <v>Saldo de cajas físicas desde crédito y débito</v>
+      </c>
+      <c r="D469" t="str">
+        <v>La carga del histórico de las 09:05 dejó en 0 el corte de Efectivo sin factura (ARS y USD). Tesorería vs mes en curso mostraba $ 0 contra $ 1.386.000. Ese saldo, igual que Efectivo-f y Morba, se rearma con los créditos y débitos de la caja si el corte no cierra. Efectivo sin factura queda en $ 1.386.000 y 1.600 USD. El consolidado de las demás cajas no cambia.</v>
+      </c>
+      <c r="E469" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B470" t="str">
+        <v>09:32</v>
+      </c>
+      <c r="C470" t="str">
         <v>Despliegue v2.94 producción</v>
       </c>
-      <c r="D469" t="str">
-        <v>Push a main y Vercel --prod: el histórico de cajas físicas vuelve a tomar la columna Monto (en dólares se pesifica al MEP de la fecha). Los importes que quedaron en 0 a las 09:05 ya están repuestos. Se puede volver a cargar el mismo archivo. APP_VERSION 2.94.</v>
-      </c>
-      <c r="E469" t="str">
+      <c r="D470" t="str">
+        <v>Push a main y Vercel --prod: el histórico de cajas físicas vuelve a tomar la columna Monto. El saldo de cada caja física, también Efectivo sin factura, se rearma con créditos y débitos si el corte no cierra. APP_VERSION 2.94.</v>
+      </c>
+      <c r="E470" t="str">
         <v>Despliegue</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E469"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E470"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -10601,7 +10618,7 @@
         <v>12/10/2026</v>
       </c>
       <c r="C138" t="str">
-        <v>Despliegue v2.94: el histórico de Efectivo y Morba vuelve a leer la columna Monto. La carga de las 09:05 había dejado esos importes en 0; se repusieron 766 movimientos (el egreso de 4.000 USD del 11/10 queda en −6.157.120). Se puede volver a cargar el mismo archivo. Producción Vercel.</v>
+        <v>Despliegue v2.94: el histórico de Efectivo y Morba vuelve a leer la columna Monto. La carga de las 09:05 había dejado esos importes en 0; se repusieron 766 movimientos (el egreso de 4.000 USD del 11/10 queda en −6.157.120). El saldo de cada caja física, también Efectivo sin factura, se rearma con créditos y débitos si el corte no cierra ($ 1.386.000 y 1.600 USD). Se puede volver a cargar el mismo archivo. Producción Vercel.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2.95: el saldo de las cajas en dólares queda en dólares.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E470"/>
+  <dimension ref="A1:E473"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8401,9 +8401,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="471">
+      <c r="A471" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B471" t="str">
+        <v>09:46</v>
+      </c>
+      <c r="C471" t="str">
+        <v>Columna Saldo en cada caja física</v>
+      </c>
+      <c r="D471" t="str">
+        <v>En Cajas (físicas) la columna Saldo acumula crédito y débito en orden de fecha. Queda alineada al corte que cierra con esos movimientos, así la última fila coincide con el saldo de la caja (Efectivo sin factura $ 1.386.000). El Excel de la caja usa ese mismo número.</v>
+      </c>
+      <c r="E471" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B472" t="str">
+        <v>10:29</v>
+      </c>
+      <c r="C472" t="str">
+        <v>Cajas en dólares sin convertir por el MEP</v>
+      </c>
+      <c r="D472" t="str">
+        <v>El saldo de Efectivo-f (USD) y Efectivo sin factura (USD) se calcula y se muestra en dólares: la suma de cada movimiento en USD. Tesorería vs mes en curso ya no compara 1.613,68 contra 1.600 (eso era los pesos guardados divididos por el MEP de hoy). En Saldos extractos esas dos cajas muestran el saldo en dólares; debajo queda el importe en pesos ya registrado. El consolidado no vuelve a pesificar ese efectivo.</v>
+      </c>
+      <c r="E472" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B473" t="str">
+        <v>10:30</v>
+      </c>
+      <c r="C473" t="str">
+        <v>Despliegue v2.95 producción</v>
+      </c>
+      <c r="D473" t="str">
+        <v>Push a main y Vercel --prod: la columna Saldo de cada caja física suma los movimientos. En dólares ese saldo, Saldos extractos y la comparación con tesorería quedan en dólares (1.600, no 1.613,68). APP_VERSION 2.95.</v>
+      </c>
+      <c r="E473" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E470"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E473"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8909,7 +8960,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. El histórico conserva la columna Monto (en dólares se pesifica al MEP de la fecha).</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. El histórico conserva la columna Monto (en dólares se pesifica al MEP de la fecha). La columna Saldo de cada caja acumula crédito y débito en orden de fecha, alineada al corte que cierra con esos movimientos. En las cajas en dólares esa columna y la tarjeta de saldo son la suma en USD, sin dividir los pesos por el tipo de cambio.</v>
       </c>
     </row>
     <row r="63">
@@ -8917,7 +8968,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. El mes en curso del consolidado pesifica todos los dólares al MEP de hoy (o el inmediato anterior), la misma cotización de la torta; los meses cerrados no se recalculan. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD), Efectivo-f (USD) y Efectivo-s/f (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. El mes en curso del consolidado pesifica Galicia USD y FCI USD al MEP de hoy (o el inmediato anterior), la misma cotización de la torta. El efectivo en dólares no se vuelve a pasar por el tipo de cambio: el saldo es la suma en USD. Los meses cerrados no se recalculan. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). En Efectivo-f (USD) y Efectivo-s/f (USD) el saldo, el gráfico, el Excel y la comparación con tesorería están en dólares (suma de los movimientos), con el importe en pesos ya guardado debajo. Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
       </c>
     </row>
     <row r="64">
@@ -9096,7 +9147,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C138"/>
+  <dimension ref="A1:C139"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10621,9 +10672,20 @@
         <v>Despliegue v2.94: el histórico de Efectivo y Morba vuelve a leer la columna Monto. La carga de las 09:05 había dejado esos importes en 0; se repusieron 766 movimientos (el egreso de 4.000 USD del 11/10 queda en −6.157.120). El saldo de cada caja física, también Efectivo sin factura, se rearma con créditos y débitos si el corte no cierra ($ 1.386.000 y 1.600 USD). Se puede volver a cargar el mismo archivo. Producción Vercel.</v>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>2.95</v>
+      </c>
+      <c r="B139" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="C139" t="str">
+        <v>Despliegue v2.95: en cada caja física la columna Saldo suma crédito y débito en orden de fecha. En Efectivo-f (USD) y Efectivo sin factura (USD) ese saldo, Saldos extractos y Tesorería vs mes en curso quedan en dólares (1.600, no 1.613,68 por dividir los pesos por el MEP de hoy). El consolidado no vuelve a pesificar ese efectivo. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C138"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C139"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.96: el histórico muestra el Id que falta y se puede deshacer una anulación de Mercado Pago.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E473"/>
+  <dimension ref="A1:E476"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8452,9 +8452,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="474">
+      <c r="A474" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B474" t="str">
+        <v>17:45</v>
+      </c>
+      <c r="C474" t="str">
+        <v>Deshacer anulación de Mercado Pago</v>
+      </c>
+      <c r="D474" t="str">
+        <v>En Conciliación, solapa Mercado Pago Anulados, se puede deshacer un par (cobro y devolución, o impuesto y anulación). Los dos movimientos vuelven al extracto y se pueden conciliar. Abajo quedan las anulaciones deshechas para volver a marcarlas. sql/supabase_cb_mp_anulacion_deshecha.sql.</v>
+      </c>
+      <c r="E474" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="str">
+        <v>13/10/2026</v>
+      </c>
+      <c r="B475" t="str">
+        <v>17:55</v>
+      </c>
+      <c r="C475" t="str">
+        <v>Histórico: huecos de Id por caja</v>
+      </c>
+      <c r="D475" t="str">
+        <v>Al cargar movimientos-historico, un Pendiente (o sin estado) cuyo Id corta la secuencia del archivo se detecta: si los Id van del 1 al 10 y falta el 8, aparece el 8. En el resultado, las cajas físicas se listan por caja con Eliminar para confirmar. Mercado Pago, Galicia, Credicoop y FCI siguen yendo a A eliminar de cada caja. sql/supabase_historico_huecos_secuencia.sql.</v>
+      </c>
+      <c r="E475" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="str">
+        <v>13/10/2026</v>
+      </c>
+      <c r="B476" t="str">
+        <v>18:27</v>
+      </c>
+      <c r="C476" t="str">
+        <v>Despliegue v2.96 producción</v>
+      </c>
+      <c r="D476" t="str">
+        <v>Push a main y Vercel --prod: el histórico muestra el Id pendiente que corta la secuencia, las cajas físicas se confirman con Eliminar y el resto queda en A eliminar. En Mercado Pago se puede deshacer una anulación. APP_VERSION 2.96.</v>
+      </c>
+      <c r="E476" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E473"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E476"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8952,7 +9003,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja), Credicoop (botón negro) y FCI Galicia (ARS)/(USD) (verde). FCI carga solo tesorería (histórico con Caja FCI Galicia (ARS) o (USD)); las sugerencias salen del extracto de Galicia de la misma moneda, sin extracto propio. La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja), Credicoop (botón negro) y FCI Galicia (ARS)/(USD) (verde). FCI carga solo tesorería (histórico con Caja FCI Galicia (ARS) o (USD)); las sugerencias salen del extracto de Galicia de la misma moneda, sin extracto propio. La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. En el histórico, además, un Id que corta la secuencia del archivo (del menor al mayor) también va a A eliminar de esa caja (Mercado Pago, Galicia, Credicoop y FCI). Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. Se puede deshacer esa anulación: los dos movimientos vuelven al extracto y se pueden conciliar; abajo quedan para volver a anularlos (sql/supabase_cb_mp_anulacion_deshecha.sql). En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
     </row>
     <row r="62">
@@ -8960,7 +9011,7 @@
         <v>Cajas (físicas)</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. El histórico conserva la columna Monto (en dólares se pesifica al MEP de la fecha). La columna Saldo de cada caja acumula crédito y débito en orden de fecha, alineada al corte que cierra con esos movimientos. En las cajas en dólares esa columna y la tarjeta de saldo son la suma en USD, sin dividir los pesos por el tipo de cambio.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. En el histórico, un Pendiente cuyo Id corta la secuencia del archivo (del menor al mayor: si falta el 8 entre 1 y 10, se muestra el 8) aparece en el resultado agrupado por caja física, con Eliminar para confirmar. Mercado Pago, Galicia, Credicoop y FCI siguen yendo a A eliminar de cada caja. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. El histórico conserva la columna Monto (en dólares se pesifica al MEP de la fecha). La columna Saldo de cada caja acumula crédito y débito en orden de fecha, alineada al corte que cierra con esos movimientos. En las cajas en dólares esa columna y la tarjeta de saldo son la suma en USD, sin dividir los pesos por el tipo de cambio.</v>
       </c>
     </row>
     <row r="63">
@@ -9147,7 +9198,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10683,9 +10734,20 @@
         <v>Despliegue v2.95: en cada caja física la columna Saldo suma crédito y débito en orden de fecha. En Efectivo-f (USD) y Efectivo sin factura (USD) ese saldo, Saldos extractos y Tesorería vs mes en curso quedan en dólares (1.600, no 1.613,68 por dividir los pesos por el MEP de hoy). El consolidado no vuelve a pesificar ese efectivo. Producción Vercel.</v>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>2.96</v>
+      </c>
+      <c r="B140" t="str">
+        <v>13/10/2026</v>
+      </c>
+      <c r="C140" t="str">
+        <v>Despliegue v2.96: al cargar el histórico, un Pendiente cuyo Id corta la secuencia (si van del 1 al 10 y falta el 8, se muestra el 8) aparece por caja física con Eliminar para confirmar. Mercado Pago, Galicia, Credicoop y FCI quedan en A eliminar de cada caja. En Mercado Pago se puede deshacer una anulación y los dos movimientos vuelven al extracto. sql/supabase_historico_huecos_secuencia.sql y sql/supabase_cb_mp_anulacion_deshecha.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C139"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C140"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.97: el Estado Financiero muestra el promedio de los últimos 12 meses cerrados.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E476"/>
+  <dimension ref="A1:E478"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8503,9 +8503,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="477">
+      <c r="A477" t="str">
+        <v>14/10/2026</v>
+      </c>
+      <c r="B477" t="str">
+        <v>12:20</v>
+      </c>
+      <c r="C477" t="str">
+        <v>Estado Financiero: promedio mensual</v>
+      </c>
+      <c r="D477" t="str">
+        <v>En Estado Financiero, antes de Total, la columna Avg Mensual muestra el promedio de los últimos 12 meses cerrados móviles (el mes en curso no entra; un mes sin movimientos cuenta como cero). El signo de ayuda del encabezado lo aclara. El Excel de EF incluye la misma columna, con el importe numérico.</v>
+      </c>
+      <c r="E477" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="str">
+        <v>14/10/2026</v>
+      </c>
+      <c r="B478" t="str">
+        <v>12:20</v>
+      </c>
+      <c r="C478" t="str">
+        <v>Despliegue v2.97 producción</v>
+      </c>
+      <c r="D478" t="str">
+        <v>Push a main y Vercel --prod: Estado Financiero muestra Avg Mensual antes de Total, promedio de los últimos 12 meses cerrados. APP_VERSION 2.97.</v>
+      </c>
+      <c r="E478" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E476"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E478"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8851,7 +8885,7 @@
         <v>Estado Financiero (tabla dinámica)</v>
       </c>
       <c r="B42" t="str">
-        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). AJUSTE DE SALDOS (CAJA) va debajo de FLUJO OPERATIVO GENERADO y entra en (=) FLUJO DE CAJA NETO DEL PERÍODO (D), no en A–C. En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Gráficos y export Excel. Conciliación §7 oculta.</v>
+        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). AJUSTE DE SALDOS (CAJA) va debajo de FLUJO OPERATIVO GENERADO y entra en (=) FLUJO DE CAJA NETO DEL PERÍODO (D), no en A–C. En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Antes de Total, Avg Mensual es el promedio de los últimos 12 meses cerrados móviles (el mes en curso no entra; un mes sin movimientos cuenta como cero). Gráficos y export Excel. Conciliación §7 oculta.</v>
       </c>
     </row>
     <row r="43">
@@ -9198,7 +9232,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C141"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10745,9 +10779,20 @@
         <v>Despliegue v2.96: al cargar el histórico, un Pendiente cuyo Id corta la secuencia (si van del 1 al 10 y falta el 8, se muestra el 8) aparece por caja física con Eliminar para confirmar. Mercado Pago, Galicia, Credicoop y FCI quedan en A eliminar de cada caja. En Mercado Pago se puede deshacer una anulación y los dos movimientos vuelven al extracto. sql/supabase_historico_huecos_secuencia.sql y sql/supabase_cb_mp_anulacion_deshecha.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>2.97</v>
+      </c>
+      <c r="B141" t="str">
+        <v>14/10/2026</v>
+      </c>
+      <c r="C141" t="str">
+        <v>Despliegue v2.97: en Estado Financiero, antes de Total, la columna Avg Mensual es el promedio de los últimos 12 meses cerrados móviles. El mes en curso no entra y un mes sin movimientos cuenta como cero. El Excel del Estado Financiero incluye esa columna. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C140"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C141"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.98: en Matriz EF se pueden borrar las relaciones sin movimientos.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E478"/>
+  <dimension ref="A1:E482"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8537,9 +8537,77 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="479">
+      <c r="A479" t="str">
+        <v>15/10/2026</v>
+      </c>
+      <c r="B479" t="str">
+        <v>18:12</v>
+      </c>
+      <c r="C479" t="str">
+        <v>Caja efectivo dólar: factura sí o no</v>
+      </c>
+      <c r="D479" t="str">
+        <v>Sobre Caja_Efectivo_Dolar_Con_Factura.xlsx se cruzó Movimientos con Factura por el mismo ID Venta. Tiene factura: Y si Tipo de cambio × Monto coincide con el total de la factura (igual o a menos del 1% / $100), N si ese ID no está en Factura, NI si el ID está pero el importe no coincide. docs/Caja_Efectivo_Dolar_Con_Factura_resultado.xlsx.</v>
+      </c>
+      <c r="E479" t="str">
+        <v>Analisis</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="B480" t="str">
+        <v>08:14</v>
+      </c>
+      <c r="C480" t="str">
+        <v>Días de cobro por monto de venta</v>
+      </c>
+      <c r="D480" t="str">
+        <v>Con movimientos-historico_2026-10-17, solo ingresos de Ventas con ID Venta ya confirmados: días del primer al último cobro y porcentaje del importe que entra cada 30 días, por rango de monto. docs/Analisis_Cobro_Ventas_por_Monto_2026-10-17.docx.</v>
+      </c>
+      <c r="E480" t="str">
+        <v>Analisis</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="B481" t="str">
+        <v>10:15</v>
+      </c>
+      <c r="C481" t="str">
+        <v>Matriz EF: borrar relaciones sin movimientos</v>
+      </c>
+      <c r="D481" t="str">
+        <v>En Relaciones, el tacho borra una relación solo si no tiene movimientos de tesorería; si tiene, queda el candado. En Estructura EF, un subítem que no es fórmula se puede borrar aunque tenga relaciones, si ninguna tiene movimientos: esas relaciones se van con el renglón.</v>
+      </c>
+      <c r="E481" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="B482" t="str">
+        <v>10:55</v>
+      </c>
+      <c r="C482" t="str">
+        <v>Despliegue v2.98 producción</v>
+      </c>
+      <c r="D482" t="str">
+        <v>Push a main y Vercel --prod: en Matriz EF se borra una relación sin movimientos y, en Estructura EF, el renglón se va junto con esas relaciones. APP_VERSION 2.98.</v>
+      </c>
+      <c r="E482" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E478"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E482"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9101,7 +9169,7 @@
         <v>Matriz EF</v>
       </c>
       <c r="B69" t="str">
-        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6 ni 1.2 (ajuste de saldos), A–D, 6.1–6.3 ni subítems con relaciones/ratios; códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql, sql/supabase_ef_estructura_abm.sql y sql/supabase_ef_ajuste_saldos_caja.sql.</v>
+        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6 ni 1.2 (ajuste de saldos), A–D, 6.1–6.3 ni ratios. Una relación sin movimientos se borra desde Relaciones; un subítem se borra junto con sus relaciones si ninguna tiene movimientos. Códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql, sql/supabase_ef_estructura_abm.sql y sql/supabase_ef_ajuste_saldos_caja.sql.</v>
       </c>
     </row>
     <row r="70">
@@ -9232,7 +9300,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C142"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10790,9 +10858,20 @@
         <v>Despliegue v2.97: en Estado Financiero, antes de Total, la columna Avg Mensual es el promedio de los últimos 12 meses cerrados móviles. El mes en curso no entra y un mes sin movimientos cuenta como cero. El Excel del Estado Financiero incluye esa columna. Producción Vercel.</v>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>2.98</v>
+      </c>
+      <c r="B142" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="C142" t="str">
+        <v>Despliegue v2.98: en Matriz EF, Relaciones, el tacho borra una relación solo si no tiene movimientos; si tiene, queda el candado con la cantidad. En Estructura EF un subítem que no es fórmula se borra junto con esas relaciones vacías. Las secciones, totales y fórmulas siguen protegidos. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C141"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C142"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.99: en Flujo por mes se ve qué parte de los ingresos entra con factura y qué parte sin factura.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E482"/>
+  <dimension ref="A1:E485"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8605,9 +8605,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="483">
+      <c r="A483" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="B483" t="str">
+        <v>11:56</v>
+      </c>
+      <c r="C483" t="str">
+        <v>Precio de venta para ganancia neta 20% y 25%</v>
+      </c>
+      <c r="D483" t="str">
+        <v>Sobre el Estado Financiero al 17/10/2026, meses cerrados julio 2025 a septiembre 2026: la ganancia neta es 18,0% de lo cobrado. Para el 20% hay que subir el precio 2,9% y para el 25%, 10,9%, vendiendo la misma cantidad. docs/Analisis_Aumento_Precio_Venta_EF_2026-10-17.docx.</v>
+      </c>
+      <c r="E483" t="str">
+        <v>Analisis</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="B484" t="str">
+        <v>12:40</v>
+      </c>
+      <c r="C484" t="str">
+        <v>Flujo: ingresos con factura y sin factura</v>
+      </c>
+      <c r="D484" t="str">
+        <v>En Ratios del Negocio, Ingresos c/f / Ingresos (Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop) e Ingresos s/f / Ingresos (el resto). Los dos suman 100%. También en el Excel y el PDF.</v>
+      </c>
+      <c r="E484" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="B485" t="str">
+        <v>20:10</v>
+      </c>
+      <c r="C485" t="str">
+        <v>Despliegue v2.99 producción</v>
+      </c>
+      <c r="D485" t="str">
+        <v>Push a main y Vercel --prod: en Flujo por mes, Ingresos c/f / Ingresos e Ingresos s/f / Ingresos. Los dos suman 100%. APP_VERSION 2.99.</v>
+      </c>
+      <c r="E485" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E482"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E485"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8633,7 +8684,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas); Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. La columna Total (Ingresos, Egresos, G/P y ratios) suma meses cerrados y va después de esos meses: el mes en curso se marca en celeste y no entra al Total, ni a las variaciones y la tendencia del gráfico, ni a la base de la proyección. Sobre esa barra se ve el G/P del mes en millones. Las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas); Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. Ingresos c/f / Ingresos e Ingresos s/f / Ingresos parten el mes: c/f es Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop; s/f es el resto. Los dos suman 100%. Ingresos c/f / Ingresos e Ingresos s/f / Ingresos parten el mes: c/f es Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop; s/f es el resto. Los dos suman 100%. La columna Total (Ingresos, Egresos, G/P y ratios) suma meses cerrados y va después de esos meses: el mes en curso se marca en celeste y no entra al Total, ni a las variaciones y la tendencia del gráfico, ni a la base de la proyección. Sobre esa barra se ve el G/P del mes en millones. Las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -9300,7 +9351,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C142"/>
+  <dimension ref="A1:C143"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10869,9 +10920,20 @@
         <v>Despliegue v2.98: en Matriz EF, Relaciones, el tacho borra una relación solo si no tiene movimientos; si tiene, queda el candado con la cantidad. En Estructura EF un subítem que no es fórmula se borra junto con esas relaciones vacías. Las secciones, totales y fórmulas siguen protegidos. Producción Vercel.</v>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>2.99</v>
+      </c>
+      <c r="B143" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="C143" t="str">
+        <v>Despliegue v2.99: en Flujo por mes, dos ratios nuevos. Ingresos c/f / Ingresos (Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop) e Ingresos s/f / Ingresos (el resto de las cajas). Entre los dos suman 100%. También en el Excel y el PDF. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C142"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C143"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.100: hay un menú To-Do y en Seguridad se elige quién lo ve y quién crea tareas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E485"/>
+  <dimension ref="A1:E493"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8656,16 +8656,152 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="486">
+      <c r="A486" t="str">
+        <v>19/10/2026</v>
+      </c>
+      <c r="B486" t="str">
+        <v>10:03</v>
+      </c>
+      <c r="C486" t="str">
+        <v>Balance certificado vs Estado Financiero</v>
+      </c>
+      <c r="D486" t="str">
+        <v>Cruce del balance al 31/01/2026 (en blanco, moneda homogénea) con la caja de julio 2025 a enero 2026. Margen, sueldos y publicidad correlacionan; la caja de siete meses ya empata el año facturado. docs/Analisis_Balance_vs_Estado_Financiero_2026-10-19.docx.</v>
+      </c>
+      <c r="E486" t="str">
+        <v>Analisis</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="str">
+        <v>20/10/2026</v>
+      </c>
+      <c r="B487" t="str">
+        <v>09:19</v>
+      </c>
+      <c r="C487" t="str">
+        <v>Consumo de ingresos y caja quieta</v>
+      </c>
+      <c r="D487" t="str">
+        <v>Resumen de julio 2025 a septiembre 2026: 54% costos directos, 25% estructura, 2% impuestos, queda 18%. El excedente de Galicia pesos, arriba de un piso de $25 millones, puesto en un FCI de rescate rinde cerca de $425.000 por mes a la tasa de octubre 2026. docs/Resumen_Consumo_Ingresos_y_Caja_2026-10-20.docx.</v>
+      </c>
+      <c r="E487" t="str">
+        <v>Analisis</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="str">
+        <v>20/10/2026</v>
+      </c>
+      <c r="B488" t="str">
+        <v>09:39</v>
+      </c>
+      <c r="C488" t="str">
+        <v>FCI: Galicia más Mercado Pago</v>
+      </c>
+      <c r="D488" t="str">
+        <v>El interés del fondo suma las dos cuentas, porque Mercado Pago se pasa a Galicia para invertirlo. Promedio conjunto $121 millones; dejando $25 millones, sobran $96 millones y rinden unos $1,5 millones por mes al 19,1%. Misma nota, corregida.</v>
+      </c>
+      <c r="E488" t="str">
+        <v>Analisis</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="str">
+        <v>21/10/2026</v>
+      </c>
+      <c r="B489" t="str">
+        <v>12:21</v>
+      </c>
+      <c r="C489" t="str">
+        <v>Bono adicional dentro de costos indirectos</v>
+      </c>
+      <c r="D489" t="str">
+        <v>En la estructura del Estado Financiero, Bono adicional no remunerativo pasó del orden 14 (código 2.7, entre los directos) al orden 22 (código 3.5), entre Repuestos y Gastos bancarios. El ítem ya decía indirecto; el Estado Financiero lo ubica por el orden.</v>
+      </c>
+      <c r="E489" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="str">
+        <v>22/10/2026</v>
+      </c>
+      <c r="B490" t="str">
+        <v>08:57</v>
+      </c>
+      <c r="C490" t="str">
+        <v>Menú To-Do</v>
+      </c>
+      <c r="D490" t="str">
+        <v>Nueva opción To-Do, igual que Everfit: bandeja, recurrencia, responsable usuario o perfil, matriz por responsable y reasignar. En Seguridad, ver y completar quedan en todos los perfiles; crear, editar y eliminar en Admin y Encargado. sql/supabase_todo.sql.</v>
+      </c>
+      <c r="E490" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="str">
+        <v>22/10/2026</v>
+      </c>
+      <c r="B491" t="str">
+        <v>09:32</v>
+      </c>
+      <c r="C491" t="str">
+        <v>To-Do: columna Tarea y ayuda</v>
+      </c>
+      <c r="D491" t="str">
+        <v>La columna Tarea ocupa el ancho libre de la pantalla. La descripción deja de verse debajo del título y se abre con el ícono de ayuda, igual que el resto de la app.</v>
+      </c>
+      <c r="E491" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="str">
+        <v>22/10/2026</v>
+      </c>
+      <c r="B492" t="str">
+        <v>09:56</v>
+      </c>
+      <c r="C492" t="str">
+        <v>To-Do en Seguridad</v>
+      </c>
+      <c r="D492" t="str">
+        <v>En Permisos por rol, Menús laterales incluye Ver To-Do. El bloque To-Do tiene crear, editar, eliminar y completar, con el mismo interruptor que el resto de la app.</v>
+      </c>
+      <c r="E492" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="str">
+        <v>22/10/2026</v>
+      </c>
+      <c r="B493" t="str">
+        <v>10:06</v>
+      </c>
+      <c r="C493" t="str">
+        <v>Despliegue v2.100 producción</v>
+      </c>
+      <c r="D493" t="str">
+        <v>Push a main y Vercel --prod: menú To-Do y permisos en Seguridad (ver, crear, editar, eliminar, completar). APP_VERSION 2.100.</v>
+      </c>
+      <c r="E493" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E485"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E493"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B73"/>
+  <dimension ref="A1:B74"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -8868,7 +9004,7 @@
         <v>Menú lateral</v>
       </c>
       <c r="B25" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Flujo de caja (permiso ver_solapa_flujo; icono $), Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage. Al iniciar sesión se abre Flujo de caja si el usuario lo tiene; si no, el primer menú lateral permitido. Cada vez que se vuelve a Flujo se recargan tesorería, cajas y tipos de cambio.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Flujo de caja (permiso ver_solapa_flujo; icono $), To-Do (ver_todo), Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage. Al iniciar sesión se abre Flujo de caja si el usuario lo tiene; si no, el primer menú lateral permitido. Cada vez que se vuelve a Flujo se recargan tesorería, cajas y tipos de cambio.</v>
       </c>
     </row>
     <row r="26">
@@ -8876,7 +9012,7 @@
         <v>Seguridad y roles</v>
       </c>
       <c r="B26" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Recuperar contraseña desde el login (enlace por email). Permisos granulares desde Supabase: ver_solapa_flujo (menú y solapa Flujo de caja), ver_solapa_* (resto de solapas del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo de caja + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. En Flujo de caja el perfil define Cards, Flujo por mes, Todas las transacciones, Evolución, Estado financiero y el botón Cargar tesorería histórica (arriba, junto a Exportar Base Histórica). Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Recuperar contraseña desde el login (enlace por email). Permisos granulares desde Supabase: ver_solapa_flujo (menú y solapa Flujo de caja), ver_solapa_* (resto de solapas del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos/todo, crear/editar/eliminar/completar_todo, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo de caja + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. En Flujo de caja el perfil define Cards, Flujo por mes, Todas las transacciones, Evolución, Estado financiero y el botón Cargar tesorería histórica (arriba, junto a Exportar Base Histórica). Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
       </c>
     </row>
     <row r="27">
@@ -9145,119 +9281,127 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Gestión de Proyectos</v>
+        <v>To-Do</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Archivos adjuntos por fecha (descripción + archivo en Storage gp-archivos) en proyecto, entregable y tarea; solapa Archivos y hoja Excel. Solapa Horas cons.: conciliación diaria. La solapa activa (To-Do, Gantt, Horas, Archivos) se marca con etiqueta Activo y un contorno más visible. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
+        <v>Menú To-Do, mismo criterio que Everfit. Bandeja con filtros (abiertas, hoy), tarjetas Pendientes / En curso / Vencidas / Hechas hoy, recurrencia (única, diaria, semanal, mensual, bimestral, trimestral, anual; sin domingos; la diaria se marca hecha desde el día de vencimiento), responsable usuario o perfil. Quien no crea solo ve las suyas o las de su perfil. Admin y Encargado ven la matriz Por responsable. Abajo, si tiene Configuración, reasigna abiertas de un usuario o perfil a otro. Excel con fechas y prioridad numéricas. En Seguridad: ver_todo y completar_todo en todos los perfiles; crear_todo, editar_todo y eliminar_todo en Admin y Encargado (se puede cambiar el toggle). La columna Tarea usa el ancho libre de la pantalla. La descripción se abre con el ícono de ayuda al lado del título.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Conciliación Bancaria</v>
+        <v>Gestión de Proyectos</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja), Credicoop (botón negro) y FCI Galicia (ARS)/(USD) (verde). FCI carga solo tesorería (histórico con Caja FCI Galicia (ARS) o (USD)); las sugerencias salen del extracto de Galicia de la misma moneda, sin extracto propio. La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. En el histórico, además, un Id que corta la secuencia del archivo (del menor al mayor) también va a A eliminar de esa caja (Mercado Pago, Galicia, Credicoop y FCI). Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. Se puede deshacer esa anulación: los dos movimientos vuelven al extracto y se pueden conciliar; abajo quedan para volver a anularlos (sql/supabase_cb_mp_anulacion_deshecha.sql). En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Archivos adjuntos por fecha (descripción + archivo en Storage gp-archivos) en proyecto, entregable y tarea; solapa Archivos y hoja Excel. Solapa Horas cons.: conciliación diaria. La solapa activa (To-Do, Gantt, Horas, Archivos) se marca con etiqueta Activo y un contorno más visible. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Cajas (físicas)</v>
+        <v>Conciliación Bancaria</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. En el histórico, un Pendiente cuyo Id corta la secuencia del archivo (del menor al mayor: si falta el 8 entre 1 y 10, se muestra el 8) aparece en el resultado agrupado por caja física, con Eliminar para confirmar. Mercado Pago, Galicia, Credicoop y FCI siguen yendo a A eliminar de cada caja. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. El histórico conserva la columna Monto (en dólares se pesifica al MEP de la fecha). La columna Saldo de cada caja acumula crédito y débito en orden de fecha, alineada al corte que cierra con esos movimientos. En las cajas en dólares esa columna y la tarjeta de saldo son la suma en USD, sin dividir los pesos por el tipo de cambio.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja), Credicoop (botón negro) y FCI Galicia (ARS)/(USD) (verde). FCI carga solo tesorería (histórico con Caja FCI Galicia (ARS) o (USD)); las sugerencias salen del extracto de Galicia de la misma moneda, sin extracto propio. La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. En el histórico, además, un Id que corta la secuencia del archivo (del menor al mayor) también va a A eliminar de esa caja (Mercado Pago, Galicia, Credicoop y FCI). Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. Se puede deshacer esa anulación: los dos movimientos vuelven al extracto y se pueden conciliar; abajo quedan para volver a anularlos (sql/supabase_cb_mp_anulacion_deshecha.sql). En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Saldos extractos</v>
+        <v>Cajas (físicas)</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. El mes en curso del consolidado pesifica Galicia USD y FCI USD al MEP de hoy (o el inmediato anterior), la misma cotización de la torta. El efectivo en dólares no se vuelve a pasar por el tipo de cambio: el saldo es la suma en USD. Los meses cerrados no se recalculan. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). En Efectivo-f (USD) y Efectivo-s/f (USD) el saldo, el gráfico, el Excel y la comparación con tesorería están en dólares (suma de los movimientos), con el importe en pesos ya guardado debajo. Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. En el histórico, un Pendiente cuyo Id corta la secuencia del archivo (del menor al mayor: si falta el 8 entre 1 y 10, se muestra el 8) aparece en el resultado agrupado por caja física, con Eliminar para confirmar. Mercado Pago, Galicia, Credicoop y FCI siguen yendo a A eliminar de cada caja. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. El histórico conserva la columna Monto (en dólares se pesifica al MEP de la fecha). La columna Saldo de cada caja acumula crédito y débito en orden de fecha, alineada al corte que cierra con esos movimientos. En las cajas en dólares esa columna y la tarjeta de saldo son la suma en USD, sin dividir los pesos por el tipo de cambio.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Impuestos</v>
+        <v>Saldos extractos</v>
       </c>
       <c r="B64" t="str">
-        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca), marcada Activo como el resto de pantallas: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (listado con Observaciones; justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql, sql/supabase_cb_match_impuestos.sql y sql/supabase_imp_tesoreria_observaciones.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. El mes en curso del consolidado pesifica Galicia USD y FCI USD al MEP de hoy (o el inmediato anterior), la misma cotización de la torta. El efectivo en dólares no se vuelve a pasar por el tipo de cambio: el saldo es la suma en USD. Los meses cerrados no se recalculan. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). En Efectivo-f (USD) y Efectivo-s/f (USD) el saldo, el gráfico, el Excel y la comparación con tesorería están en dólares (suma de los movimientos), con el importe en pesos ya guardado debajo. Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Impuestos</v>
       </c>
       <c r="B65" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca), marcada Activo como el resto de pantallas: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (listado con Observaciones; justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql, sql/supabase_cb_match_impuestos.sql y sql/supabase_imp_tesoreria_observaciones.sql.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B66" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B67" t="str">
-        <v>Retirado: el Flujo ya no reemplaza la tabla transacciones desde un Excel Normalizado. El botón, el modal y el permiso carga_normalizada salieron de la app. Queda el script npm run normalizar-extracto para generar el archivo.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B68" t="str">
-        <v>Retirado: la solapa Excluidos upload y su permiso ya no están en el dashboard. La tabla de auditoría en Supabase se conserva.</v>
+        <v>Retirado: el Flujo ya no reemplaza la tabla transacciones desde un Excel Normalizado. El botón, el modal y el permiso carga_normalizada salieron de la app. Queda el script npm run normalizar-extracto para generar el archivo.</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Matriz EF</v>
+        <v>Log de excluidos en upload</v>
       </c>
       <c r="B69" t="str">
-        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6 ni 1.2 (ajuste de saldos), A–D, 6.1–6.3 ni ratios. Una relación sin movimientos se borra desde Relaciones; un subítem se borra junto con sus relaciones si ninguna tiene movimientos. Códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql, sql/supabase_ef_estructura_abm.sql y sql/supabase_ef_ajuste_saldos_caja.sql.</v>
+        <v>Retirado: la solapa Excluidos upload y su permiso ya no están en el dashboard. La tabla de auditoría en Supabase se conserva.</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Análisis financiero extracto (PDF)</v>
+        <v>Matriz EF</v>
       </c>
       <c r="B70" t="str">
-        <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
+        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6 ni 1.2 (ajuste de saldos), A–D, 6.1–6.3 ni ratios. Una relación sin movimientos se borra desde Relaciones; un subítem se borra junto con sus relaciones si ninguna tiene movimientos. Códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql, sql/supabase_ef_estructura_abm.sql y sql/supabase_ef_ajuste_saldos_caja.sql.</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Usuario en tablas</v>
+        <v>Análisis financiero extracto (PDF)</v>
       </c>
       <c r="B71" t="str">
-        <v>Quién cargó, confirmó, descartó o eliminó: se ve el nombre para mostrar (ej. LB) y al pasar el mouse el email. Lo histórico de tesorería, saldos, impuestos y matriz queda a nombre de LB (lucas.bustos.martin@gmail.com). El consolidado de Saldos extractos no tiene actor por fila. rpc get_usuarios_mostrar. sql/supabase_usuarios_mostrar.sql.</v>
+        <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Novedades al iniciar sesión</v>
+        <v>Usuario en tablas</v>
       </c>
       <c r="B72" t="str">
-        <v>Tras cada despliegue, al entrar a la app se muestra el modal «Nueva versión» con 2–4 frases de lo que se nota al recargar (logo, badge de versión, lista). Una vez Entendido, no vuelve a aparecer hasta la siguiente versión. El texto lo actualiza el agente en scripts/lib/fornitalia-release-blurb.js; fornitalia-release.json se sirve por red.</v>
+        <v>Quién cargó, confirmó, descartó o eliminó: se ve el nombre para mostrar (ej. LB) y al pasar el mouse el email. Lo histórico de tesorería, saldos, impuestos y matriz queda a nombre de LB (lucas.bustos.martin@gmail.com). El consolidado de Saldos extractos no tiene actor por fila. rpc get_usuarios_mostrar. sql/supabase_usuarios_mostrar.sql.</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
+        <v>Novedades al iniciar sesión</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Tras cada despliegue, al entrar a la app se muestra el modal «Nueva versión» con 2–4 frases de lo que se nota al recargar (logo, badge de versión, lista). Una vez Entendido, no vuelve a aparecer hasta la siguiente versión. El texto lo actualiza el agente en scripts/lib/fornitalia-release-blurb.js; fornitalia-release.json se sirve por red.</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
         <v>Mensajes de confirmación y aviso</v>
       </c>
-      <c r="B73" t="str">
+      <c r="B74" t="str">
         <v>Las preguntas sí/no y los avisos de error o validación se muestran en un cuadro de la app (título, texto y botones con icono), no en el cartel del navegador. Confirmar usa Aceptar y Cancelar; un aviso usa Entendido. Eliminar marca el botón en rojo. Componente: scripts/lib/fornitalia-mensajes.js.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B74"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9351,7 +9495,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C143"/>
+  <dimension ref="A1:C144"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -10931,16 +11075,27 @@
         <v>Despliegue v2.99: en Flujo por mes, dos ratios nuevos. Ingresos c/f / Ingresos (Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop) e Ingresos s/f / Ingresos (el resto de las cajas). Entre los dos suman 100%. También en el Excel y el PDF. Producción Vercel.</v>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>2.100</v>
+      </c>
+      <c r="B144" t="str">
+        <v>22/10/2026</v>
+      </c>
+      <c r="C144" t="str">
+        <v>Despliegue v2.100: menú To-Do, con bandeja, recurrencia, responsable por usuario o perfil, matriz por responsable y reasignar. En Seguridad se elige quién ve el menú y quién puede crear, editar, eliminar o completar. La descripción se abre con el ícono de ayuda y la columna Tarea usa el ancho libre. sql/supabase_todo.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C143"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C144"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -11214,9 +11369,23 @@
         <v/>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>To-Do</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Bandeja de tareas como Everfit: recurrencia, responsable usuario o perfil, matriz por responsable, reasignación y permisos ver/crear/editar/eliminar/completar en Seguridad.</v>
+      </c>
+      <c r="C20">
+        <v>16</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.101: en To-Do se puede filtrar por recurrencia.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E493"/>
+  <dimension ref="A1:E495"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8792,9 +8792,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="494">
+      <c r="A494" t="str">
+        <v>23/10/2026</v>
+      </c>
+      <c r="B494" t="str">
+        <v>10:14</v>
+      </c>
+      <c r="C494" t="str">
+        <v>To-Do: filtro Recurrencia</v>
+      </c>
+      <c r="D494" t="str">
+        <v>En los filtros de la bandeja se puede elegir Única, Diaria, Semanal, Mensual, Bimestral, Trimestral o Anual. Recorta la tabla, las tarjetas, la matriz y el Excel. Todas deja el listado como estaba.</v>
+      </c>
+      <c r="E494" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="str">
+        <v>23/10/2026</v>
+      </c>
+      <c r="B495" t="str">
+        <v>10:43</v>
+      </c>
+      <c r="C495" t="str">
+        <v>Despliegue v2.101 producción</v>
+      </c>
+      <c r="D495" t="str">
+        <v>Push a main y Vercel --prod: filtro Recurrencia en To-Do. APP_VERSION 2.101.</v>
+      </c>
+      <c r="E495" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E493"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E495"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9284,7 +9318,7 @@
         <v>To-Do</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú To-Do, mismo criterio que Everfit. Bandeja con filtros (abiertas, hoy), tarjetas Pendientes / En curso / Vencidas / Hechas hoy, recurrencia (única, diaria, semanal, mensual, bimestral, trimestral, anual; sin domingos; la diaria se marca hecha desde el día de vencimiento), responsable usuario o perfil. Quien no crea solo ve las suyas o las de su perfil. Admin y Encargado ven la matriz Por responsable. Abajo, si tiene Configuración, reasigna abiertas de un usuario o perfil a otro. Excel con fechas y prioridad numéricas. En Seguridad: ver_todo y completar_todo en todos los perfiles; crear_todo, editar_todo y eliminar_todo en Admin y Encargado (se puede cambiar el toggle). La columna Tarea usa el ancho libre de la pantalla. La descripción se abre con el ícono de ayuda al lado del título.</v>
+        <v>Menú To-Do, mismo criterio que Everfit. Bandeja con filtros (abiertas, hoy, recurrencia), tarjetas Pendientes / En curso / Vencidas / Hechas hoy, recurrencia (única, diaria, semanal, mensual, bimestral, trimestral, anual; sin domingos; la diaria se marca hecha desde el día de vencimiento), responsable usuario o perfil. Quien no crea solo ve las suyas o las de su perfil. Admin y Encargado ven la matriz Por responsable. Abajo, si tiene Configuración, reasigna abiertas de un usuario o perfil a otro. Excel con fechas y prioridad numéricas. En Seguridad: ver_todo y completar_todo en todos los perfiles; crear_todo, editar_todo y eliminar_todo en Admin y Encargado (se puede cambiar el toggle). La columna Tarea usa el ancho libre de la pantalla. La descripción se abre con el ícono de ayuda al lado del título.</v>
       </c>
     </row>
     <row r="61">
@@ -9495,7 +9529,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C145"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11086,9 +11120,20 @@
         <v>Despliegue v2.100: menú To-Do, con bandeja, recurrencia, responsable por usuario o perfil, matriz por responsable y reasignar. En Seguridad se elige quién ve el menú y quién puede crear, editar, eliminar o completar. La descripción se abre con el ícono de ayuda y la columna Tarea usa el ancho libre. sql/supabase_todo.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>2.101</v>
+      </c>
+      <c r="B145" t="str">
+        <v>23/10/2026</v>
+      </c>
+      <c r="C145" t="str">
+        <v>Despliegue v2.101: en To-Do, filtro de Recurrencia (Única, Diaria, Semanal, Mensual, Bimestral, Trimestral o Anual). Recorta la bandeja, las tarjetas, la matriz por responsable y el Excel. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C144"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C145"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.102: hay una agenda de pagos en Flujo de caja.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E495"/>
+  <dimension ref="A1:E502"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8826,16 +8826,135 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="496">
+      <c r="A496" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B496" t="str">
+        <v>09:00</v>
+      </c>
+      <c r="C496" t="str">
+        <v>Agenda de pagos</v>
+      </c>
+      <c r="D496" t="str">
+        <v>Solapa Agenda de pagos en Flujo de caja. Con los egresos de los últimos 3 meses estima las próximas 4 semanas: primero las series con ID compra (categoría y proveedor) y también las frecuentes sin ID compra. Cada barra es el total de la semana; el clic muestra el detalle. Ya pagado no mira el importe: en esa semana ya hay un egreso con ID compra al mismo proveedor. Las series sin ID compra no se marcan. En Seguridad, el perfil que ve Flujo por mes también ve esta solapa.</v>
+      </c>
+      <c r="E496" t="str">
+        <v>Implementacion</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B497" t="str">
+        <v>09:15</v>
+      </c>
+      <c r="C497" t="str">
+        <v>Agenda de pagos: estimado, impuestos y solapa inicial</v>
+      </c>
+      <c r="D497" t="str">
+        <v>El importe usa los últimos 3 pagos y el más reciente pesa más. Impuestos de hasta $ 500.000 no entran. Al abrir Flujo de caja, Agenda de pagos es la primera solapa y la vista inicial; si el perfil no la tiene, se abre la primera solapa que sí puede ver.</v>
+      </c>
+      <c r="E497" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B498" t="str">
+        <v>09:18</v>
+      </c>
+      <c r="C498" t="str">
+        <v>Agenda de pagos: sin gastos bancarios</v>
+      </c>
+      <c r="D498" t="str">
+        <v>Gastos bancarios no entra en la agenda. Es movimiento habitual del negocio, no un pago a agendar.</v>
+      </c>
+      <c r="E498" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B499" t="str">
+        <v>09:30</v>
+      </c>
+      <c r="C499" t="str">
+        <v>Agenda de pagos: cuenta contable y sueldos</v>
+      </c>
+      <c r="D499" t="str">
+        <v>Cada serie se abre también por cuenta contable. Sueldos y Jornales se proyecta el día 1, cada 30 días, solo con la carga oportuna desde septiembre (el 1/10/2026 deja el próximo el 1/11). La registración anterior no mueve la fecha ni el importe.</v>
+      </c>
+      <c r="E499" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B500" t="str">
+        <v>09:40</v>
+      </c>
+      <c r="C500" t="str">
+        <v>Agenda de pagos: Sueldos y Jornales a pagar</v>
+      </c>
+      <c r="D500" t="str">
+        <v>La cuenta es Sueldos y Jornales a pagar. El estimado usa la primera semana del último mes (1 al 6/10/2026, unos $ 14,8 millones) y el próximo pago queda el 1/11.</v>
+      </c>
+      <c r="E500" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B501" t="str">
+        <v>09:48</v>
+      </c>
+      <c r="C501" t="str">
+        <v>Agenda de pagos: semanas de lunes a viernes</v>
+      </c>
+      <c r="D501" t="str">
+        <v>Las 4 semanas se muestran de lunes a viernes. Si el estimado cae sábado o domingo, el pago pasa al lunes siguiente. El 1/11/2026 es domingo, así que Sueldos y Jornales queda el 2/11.</v>
+      </c>
+      <c r="E501" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B502" t="str">
+        <v>10:00</v>
+      </c>
+      <c r="C502" t="str">
+        <v>Despliegue v2.102 producción</v>
+      </c>
+      <c r="D502" t="str">
+        <v>Push a main y Vercel --prod: solapa Agenda de pagos, primera en Flujo de caja. Estimado de 4 semanas de lunes a viernes, por categoría, cuenta contable y proveedor. Sueldos y Jornales a pagar el primer día hábil. APP_VERSION 2.102.</v>
+      </c>
+      <c r="E502" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E495"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E502"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B74"/>
+  <dimension ref="A1:B75"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="85.83203125" customWidth="1"/>
@@ -8995,447 +9114,455 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Inclusión por mes (Configuración)</v>
+        <v>Agenda de pagos</v>
       </c>
       <c r="B20" t="str">
-        <v>Interruptores por cada mes con movimientos: incluir o excluir del flujo por mes, tarjetas de resumen, Evolución y agregados que usan excluirFilaFlujoOperativo. Persistencia localStorage y columna meses_excluidos en config_dashboard. Sin afectar export de base histórica.</v>
+        <v>Primera solapa de Flujo de caja y vista al entrar, si el perfil la tiene. Estima egresos de las próximas 4 semanas con los últimos 3 meses. El importe sale de los últimos 3 pagos de ese proveedor y categoría, con más peso en el más reciente. Prioriza series con ID compra. También entran pagos frecuentes sin ID compra. Impuestos de hasta $ 500.000 y Gastos bancarios no entran. Cada serie se abre por categoría y cuenta contable. Sueldos y Jornales se estima el día 1, cada 30 días, con los pagos cargados desde septiembre de 2026. Barras por semana (ámbar por pagar, verde ya pagado) y total al pie de cada semana. Ya pagado: en esa semana ya hubo un egreso con ID compra al mismo proveedor, sin comparar el monto. No aplica a series sin ID compra. Permiso ver_solapa_agenda_pagos en Seguridad.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Sin cotización</v>
+        <v>Inclusión por mes (Configuración)</v>
       </c>
       <c r="B21" t="str">
-        <v>Pestaña con transacciones que no tienen tipo de cambio (excluidas del resumen).</v>
+        <v>Interruptores por cada mes con movimientos: incluir o excluir del flujo por mes, tarjetas de resumen, Evolución y agregados que usan excluirFilaFlujoOperativo. Persistencia localStorage y columna meses_excluidos en config_dashboard. Sin afectar export de base histórica.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Exclusiones (flujo operativo)</v>
+        <v>Sin cotización</v>
       </c>
       <c r="B22" t="str">
-        <v>No se incluyen en G/P operativo ni Evolución: apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito; meses desmarcados en Configuración → Inclusión por mes (meses_excluidos en Supabase/localStorage). Status Pendiente sí entra al Flujo. Base histórica y Todas las transacciones siguen completas.</v>
+        <v>Pestaña con transacciones que no tienen tipo de cambio (excluidas del resumen).</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Datos</v>
+        <v>Exclusiones (flujo operativo)</v>
       </c>
       <c r="B23" t="str">
-        <v>Tesorería (Conciliación Bancaria + Cajas físicas) y tipo de cambio desde Supabase (carga paginada). La relación categoría/cuenta/tipo → EF vive en matriz_cat_cuenta_ef. Cotización faltante: se usa la fecha anterior disponible.</v>
+        <v>No se incluyen en G/P operativo ni Evolución: apertura/cierre (categoría o heurística en fila); Transferencia ni Deposito/Depósito; meses desmarcados en Configuración → Inclusión por mes (meses_excluidos en Supabase/localStorage). Status Pendiente sí entra al Flujo. Base histórica y Todas las transacciones siguen completas.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Tablas y scroll</v>
+        <v>Datos</v>
       </c>
       <c r="B24" t="str">
-        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal. Flujo por mes y Todas las transacciones: clic en el encabezado ordena la columna. Columna Usuario (nombre para mostrar; tooltip con email) en Conciliación, Cajas, Saldos por canal, Impuestos, Matriz EF y Todas las transacciones.</v>
+        <v>Tesorería (Conciliación Bancaria + Cajas físicas) y tipo de cambio desde Supabase (carga paginada). La relación categoría/cuenta/tipo → EF vive en matriz_cat_cuenta_ef. Cotización faltante: se usa la fecha anterior disponible.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Menú lateral</v>
+        <v>Tablas y scroll</v>
       </c>
       <c r="B25" t="str">
-        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Flujo de caja (permiso ver_solapa_flujo; icono $), To-Do (ver_todo), Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage. Al iniciar sesión se abre Flujo de caja si el usuario lo tiene; si no, el primer menú lateral permitido. Cada vez que se vuelve a Flujo se recargan tesorería, cajas y tipos de cambio.</v>
+        <v>Encabezados de columna anclados (sticky) al desplazarse. Flujo por mes: scroll vertical de la página (sin caja con max-height) para llegar bien al pie de la tabla; scroll horizontal en el wrap si hace falta. Otras solapas listas anchas con scroll horizontal. Flujo por mes y Todas las transacciones: clic en el encabezado ordena la columna. Columna Usuario (nombre para mostrar; tooltip con email) en Conciliación, Cajas, Saldos por canal, Impuestos, Matriz EF y Todas las transacciones.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Seguridad y roles</v>
+        <v>Menú lateral</v>
       </c>
       <c r="B26" t="str">
-        <v>Login con email/contraseña, registro o invitado anónimo (visor). Recuperar contraseña desde el login (enlace por email). Permisos granulares desde Supabase: ver_solapa_flujo (menú y solapa Flujo de caja), ver_solapa_* (resto de solapas del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos/todo, crear/editar/eliminar/completar_todo, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo de caja + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. En Flujo de caja el perfil define Cards, Flujo por mes, Todas las transacciones, Evolución, Estado financiero y el botón Cargar tesorería histórica (arriba, junto a Exportar Base Histórica). Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
+        <v>Sidebar izquierdo colapsable/expandible; botón toggle (▶/◀); Flujo de caja (permiso ver_solapa_flujo; icono $), To-Do (ver_todo), Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad (solo admin con permiso), Mi perfil, Cerrar sesión; estado expandido en localStorage. Al iniciar sesión se abre Flujo de caja si el usuario lo tiene; si no, el primer menú lateral permitido. Cada vez que se vuelve a Flujo se recargan tesorería, cajas y tipos de cambio.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Registro y contraseña</v>
+        <v>Seguridad y roles</v>
       </c>
       <c r="B27" t="str">
-        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español. Ayuda bajo el campo y mínimo 8 caracteres. En el login, «¿Olvidaste tu contraseña?» envía un enlace por email para elegir una clave nueva (revisar spam, sobre todo Hotmail).</v>
+        <v>Login con email/contraseña, registro o invitado anónimo (visor). Recuperar contraseña desde el login (enlace por email). Permisos granulares desde Supabase: ver_solapa_flujo (menú y solapa Flujo de caja), ver_solapa_* (resto de solapas del dashboard), ver_novedades/configuracion/reportes/gestion_proyectos/todo, crear/editar/eliminar/completar_todo, crear/editar/eliminar_proyecto, exportar_base_historica, editar_registros, assign_roles. Visor por defecto: Flujo de caja + exportar/reportes. Un admin puede crear perfiles nuevos (Nuevo perfil), activar solapas y menús por perfil, y asignarlos a usuarios. En Flujo de caja el perfil define Cards, Flujo por mes, Todas las transacciones, Evolución, Estado financiero, Agenda de pagos y el botón Cargar tesorería histórica (arriba, junto a Exportar Base Histórica). Admin, Encargado y Visor no se eliminan. Encargado/Admin: pack operador + Gestión de Proyectos. dashboard_operador se conserva como compatibilidad legacy. Sin SQL de seguridad, modo acceso completo. Tabla Usuarios: email, nombre para mostrar (iniciales) y rol; Mi perfil para el propio usuario.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Repositorio Git (GitHub)</v>
+        <v>Registro y contraseña</v>
       </c>
       <c r="B28" t="str">
-        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
+        <v>Si Supabase rechaza la contraseña (débil o en listas de filtrados), el mensaje se muestra en español. Ayuda bajo el campo y mínimo 8 caracteres. En el login, «¿Olvidaste tu contraseña?» envía un enlace por email para elegir una clave nueva (revisar spam, sobre todo Hotmail).</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>App en producción (Vercel)</v>
+        <v>Repositorio Git (GitHub)</v>
       </c>
       <c r="B29" t="str">
-        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
+        <v>Repo: https://github.com/lucasbustosmartin-coder/fornitalia. Rama main. .gitignore excluye node_modules, .venv, .env. Para actualizar: git add . ; git commit -m "mensaje" ; git push origin main.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Exportar a Excel</v>
+        <v>App en producción (Vercel)</v>
       </c>
       <c r="B30" t="str">
-        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, observaciones, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle.</v>
+        <v>URL pública: https://fornitalia.vercel.app/ (vercel.json reescribe / al dashboard). Cada push a main en GitHub dispara redeploy automático en Vercel. Proyecto: fornitalia, equipo Lucas Bustos, plan Hobby.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Flujo de despliegue</v>
+        <v>Exportar a Excel</v>
       </c>
       <c r="B31" t="str">
-        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación. En cada despliegue el agente redacta el modal «Nueva versión» (scripts/lib/fornitalia-release-blurb.js → fornitalia-release.json).</v>
+        <v>Botón en la barra de la tabla (solo icono). Exporta la tabla de transacciones tal como está en Supabase: una hoja "Transacciones" con columnas fecha, mes, anio, tipo_movimiento, monto (valor numérico para fórmulas), status, medio_pago, moneda, descripcion, observaciones, cliente, categoria, cat_desc, origen_archivo, cuenta_contable, editado, editado_detalle.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Versiones en bitácora</v>
+        <v>Flujo de despliegue</v>
       </c>
       <c r="B32" t="str">
-        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
+        <v>Al terminar cada tarea: el usuario prueba en local y confirma; recién entonces el asistente hace git add, commit y push (Vercel redepliega automático). No se despliega hasta confirmación. En cada despliegue el agente redacta el modal «Nueva versión» (scripts/lib/fornitalia-release-blurb.js → fornitalia-release.json).</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Campo moneda (BD)</v>
+        <v>Versiones en bitácora</v>
       </c>
       <c r="B33" t="str">
-        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
+        <v>Hoja "Versiones" en Bitacora_tareas.xlsx: registro incremental (1.0, 1.1, …) con fecha y descripción de cada despliegue a Git/Vercel.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Edición desde modal Errores</v>
+        <v>Campo moneda (BD)</v>
       </c>
       <c r="B34" t="str">
-        <v>Retirado: la solapa Errores y su modal de detalle ya no están en el Flujo. La edición de registros sigue en Todas las transacciones.</v>
+        <v>Columna moneda en tabla transacciones (ARS/USD). Si está informada, el dashboard la usa salvo reglas de negocio: Mercado Pago y Transferencia Morba siempre ARS para conversión (también morva por typo). Si moneda vacía, infiere desde textos/medio (dólar → USD). Export a Excel incluye moneda.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Campos editado y editado_detalle</v>
+        <v>Edición desde modal Errores</v>
       </c>
       <c r="B35" t="str">
-        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
+        <v>Retirado: la solapa Errores y su modal de detalle ya no están en el Flujo. La edición de registros sigue en Todas las transacciones.</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Tipo de error en Errores</v>
+        <v>Campos editado y editado_detalle</v>
       </c>
       <c r="B36" t="str">
-        <v>Retirado: la clasificación de inconsistencia y el tipo de error ya no se calculan ni se listan en el Flujo.</v>
+        <v>En transacciones: editado (boolean) y editado_detalle (texto, ej. "Categoria, Descripcion, Cuenta Contable"). Migración supabase_transacciones_editado.sql. Export Excel los incluye.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Detección de potencial duplicado</v>
+        <v>Tipo de error en Errores</v>
       </c>
       <c r="B37" t="str">
-        <v>Retirado del Flujo: el modal de comparación Este registro / Posible duplicado ya no existe. Los duplicados de tesorería se gestionan en Conciliación Bancaria → Potenciales duplicados.</v>
+        <v>Retirado: la clasificación de inconsistencia y el tipo de error ya no se calculan ni se listan en el Flujo.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Filtro por tipo de error</v>
+        <v>Detección de potencial duplicado</v>
       </c>
       <c r="B38" t="str">
-        <v>Retirado: el selector Tipo de error de la solapa Errores ya no está en la app.</v>
+        <v>Retirado del Flujo: el modal de comparación Este registro / Posible duplicado ya no existe. Los duplicados de tesorería se gestionan en Conciliación Bancaria → Potenciales duplicados.</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Duplicados: condición cliente</v>
+        <v>Filtro por tipo de error</v>
       </c>
       <c r="B39" t="str">
-        <v>Retirado: esa regla de duplicados del Flujo ya no se aplica. Conciliación Bancaria usa su propio criterio (mismo importe, hasta 40 días).</v>
+        <v>Retirado: el selector Tipo de error de la solapa Errores ya no está en la app.</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Regla bitácora</v>
+        <v>Duplicados: condición cliente</v>
       </c>
       <c r="B40" t="str">
-        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
+        <v>Retirado: esa regla de duplicados del Flujo ya no se aplica. Conciliación Bancaria usa su propio criterio (mismo importe, hasta 40 días).</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Evolución (tabla dinámica)</v>
+        <v>Regla bitácora</v>
       </c>
       <c r="B41" t="str">
-        <v>Solapa Evolución: Agrupar por = Nueva categoría (matriz) o Nueva cuenta contable (matriz) —prioriza nueva_categoria / nueva_cuenta_contable en BD y si faltan usa extracto—; Período = Diario o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
+        <v>Actualizar todas las solapas necesarias: Log (siempre que haya tarea), Resumen (si cambia funcionalidad), Presupuesto (si agrega o cambia entregable comercial), Versiones (en despliegue). Regenerar Excel tras editar crear-bitacora-excel.js.</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Estado Financiero (tabla dinámica)</v>
+        <v>Evolución (tabla dinámica)</v>
       </c>
       <c r="B42" t="str">
-        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). AJUSTE DE SALDOS (CAJA) va debajo de FLUJO OPERATIVO GENERADO y entra en (=) FLUJO DE CAJA NETO DEL PERÍODO (D), no en A–C. En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Antes de Total, Avg Mensual es el promedio de los últimos 12 meses cerrados móviles (el mes en curso no entra; un mes sin movimientos cuenta como cero). Gráficos y export Excel. Conciliación §7 oculta.</v>
+        <v>Solapa Evolución: Agrupar por = Nueva categoría (matriz) o Nueva cuenta contable (matriz) —prioriza nueva_categoria / nueva_cuenta_contable en BD y si faltan usa extracto—; Período = Diario o Mensual (MM-YYYY). Columnas = períodos, celdas = neto en moneda seleccionada, columna Total.</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Reportes (menú lateral)</v>
+        <v>Estado Financiero (tabla dinámica)</v>
       </c>
       <c r="B43" t="str">
-        <v>Vista Reportes: exportar Matriz de relaciones desde Supabase. Matriz_Cat_Cuenta_Costo sin exclusiones (suma # Registros = transacciones en sesión); filas verde claro si cat/cuenta vieja tiene relación única a nueva. Cat×cuenta solo Confirmado; proveedores con exclusiones de categoría. Resumen antes de exportar.</v>
+        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). AJUSTE DE SALDOS (CAJA) va debajo de FLUJO OPERATIVO GENERADO y entra en (=) FLUJO DE CAJA NETO DEL PERÍODO (D), no en A–C. En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Antes de Total, Avg Mensual es el promedio de los últimos 12 meses cerrados móviles (el mes en curso no entra; un mes sin movimientos cuenta como cero). Gráficos y export Excel. Conciliación §7 oculta.</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Evolución: detalle al clic y exportar</v>
+        <v>Reportes (menú lateral)</v>
       </c>
       <c r="B44" t="str">
-        <v>Clic en un valor abre modal con detalle: Fecha, Categoría (matriz), Cuenta (matriz), Descripción, Observaciones, Monto. Exportar Evolución a Excel: primera columna con el mismo criterio de agrupación.</v>
+        <v>Vista Reportes: exportar Matriz de relaciones desde Supabase. Matriz_Cat_Cuenta_Costo sin exclusiones (suma # Registros = transacciones en sesión); filas verde claro si cat/cuenta vieja tiene relación única a nueva. Cat×cuenta solo Confirmado; proveedores con exclusiones de categoría. Resumen antes de exportar.</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Exportaciones Excel</v>
+        <v>Evolución: detalle al clic y exportar</v>
       </c>
       <c r="B45" t="str">
-        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Flujo a Excel, Exportar Evolución a Excel y Exportar EF a Excel con el mismo icono y método (SheetJS/xlsx-js-style). Importes como número; % del Flujo y EF como fracción.</v>
+        <v>Clic en un valor abre modal con detalle: Fecha, Categoría (matriz), Cuenta (matriz), Descripción, Observaciones, Monto. Exportar Evolución a Excel: primera columna con el mismo criterio de agrupación.</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Evolución: orden ingreso/egreso</v>
+        <v>Exportaciones Excel</v>
       </c>
       <c r="B46" t="str">
-        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica al agrupar por categoría o cuenta de matriz.</v>
+        <v>Todas las exportaciones incluyen una fila título con la moneda. Exportar Base Histórica (icono Excel) en la línea del selector de moneda; Exportar Flujo a Excel, Exportar Evolución a Excel y Exportar EF a Excel con el mismo icono y método (SheetJS/xlsx-js-style). Importes como número; % del Flujo y EF como fracción.</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Int. por caución</v>
+        <v>Evolución: orden ingreso/egreso</v>
       </c>
       <c r="B47" t="str">
-        <v>Retirado de la app: la columna Caución, el % G/P, el modal de marcha y la carga de Serie_Cauciones ya no están en el Flujo. La fila comercial se conserva por el trabajo histórico.</v>
+        <v>En la tabla Evolución las filas se muestran primero las de ingreso (total &gt;= 0) y luego las de egreso (total &lt; 0); dentro de cada grupo orden alfabético. Aplica al agrupar por categoría o cuenta de matriz.</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Todas las transacciones</v>
+        <v>Int. por caución</v>
       </c>
       <c r="B48" t="str">
-        <v>Solapa que lista todas las transacciones con todas las columnas (incluida Observaciones, después de Descripción). Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) y buscador por id operación, descripción u observaciones. Clic en un encabezado ordena asc/desc. Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa. Columnas ID Venta e ID Compra (histórico), con filtro exacto.</v>
+        <v>Retirado de la app: la columna Caución, el % G/P, el modal de marcha y la carga de Serie_Cauciones ya no están en el Flujo. La fila comercial se conserva por el trabajo histórico.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Edición completa de registros</v>
+        <v>Todas las transacciones</v>
       </c>
       <c r="B49" t="str">
-        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), ef_item y ef_subitem (estado de flujo), origen archivo, descripción, observaciones, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). En tesorería (cb/cf) observaciones se guarda en raw.observaciones. editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
+        <v>Solapa que lista todas las transacciones con todas las columnas (incluida Observaciones, después de Descripción). Filtros por mes, categoría nueva (BD), cuenta nueva (BD), cliente, tipo (Ingreso/Egreso) y buscador por id operación, descripción u observaciones. Clic en un encabezado ordena asc/desc. Tabla: categoría/cuenta del extracto (vieja) y nueva en BD en columnas separadas. Botón Editar por registro abre modal de edición completa. Columnas ID Venta e ID Compra (histórico), con filtro exacto.</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Proyección próximos 3 meses</v>
+        <v>Edición completa de registros</v>
       </c>
       <c r="B50" t="str">
-        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
+        <v>Modal de edición con todos los campos: fecha, mes, año, tipo movimiento, monto, moneda, status, medio pago, categoría, nueva categoría (matriz), cuenta contable, nueva cuenta contable (matriz), costo_directo y costo_indirecto (Y/N o vacío), ef_item y ef_subitem (estado de flujo), origen archivo, descripción, observaciones, cliente (combo con valores existentes en BD), cat_desc, id_origen, id_operación. Combos para campos normalizados (valores existentes en BD). En tesorería (cb/cf) observaciones se guarda en raw.observaciones. editado y editado_detalle al guardar. Tras guardar OK: recarga datos, recalcula flujo, y si el modal de detalle del mes sigue abierto se vuelve a armar ese modal para no mostrar HTML viejo.</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Int. por caución proyectado</v>
+        <v>Proyección próximos 3 meses</v>
       </c>
       <c r="B51" t="str">
-        <v>Retirado de la app junto con la columna Caución del Flujo.</v>
+        <v>Debajo del total real en Flujo por mes: "Próximos 3 meses proyectados" con ventana rodante. Configuración (sidebar): método (Mediana/Promedio) y meses de historia (3, 6, 12, 24). Ingresos, egresos, G/P y ratios proyectados por mes.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Disclaimer proyección</v>
+        <v>Int. por caución proyectado</v>
       </c>
       <c r="B52" t="str">
-        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses y ventana rodante.</v>
+        <v>Retirado de la app junto con la columna Caución del Flujo.</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Botones e iconos unificados</v>
+        <v>Disclaimer proyección</v>
       </c>
       <c r="B53" t="str">
-        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, Flujo de caja / $, engranaje, usuario), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG. Cada vista de menú muestra en la cabecera el mismo icono que el ítem del sidebar (Flujo de caja, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad, Mi perfil).</v>
+        <v>Debajo de las filas proyectadas, texto en letra chica y gris oscuro que explica la metodología: Mediana/Promedio de N meses y ventana rodante.</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Configuración % G/P en caución</v>
+        <v>Botones e iconos unificados</v>
       </c>
       <c r="B54" t="str">
-        <v>Retirado de Configuración: el combo % G/P acum. en caución ya no se muestra. La columna pct_caucion en config_dashboard queda sin uso.</v>
+        <v>Todos los botones con mismo estilo: icono SVG + texto. Sidebar (chevron, Flujo de caja / $, engranaje, usuario), tabs con iconos, exportar con icono descarga, modales con iconos (Guardar, Cerrar, Excluir, Eliminar). Iconos solos (cerrar, editar, alerta) en SVG. Cada vista de menú muestra en la cabecera el mismo icono que el ítem del sidebar (Flujo de caja, Gestión de Proyectos, Reportes, Novedades, Configuración, Seguridad, Mi perfil).</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Etiqueta Caución (x% cash)</v>
+        <v>Configuración % G/P en caución</v>
       </c>
       <c r="B55" t="str">
-        <v>Retirado: la columna Caución ya no forma parte del Flujo por mes.</v>
+        <v>Retirado de Configuración: el combo % G/P acum. en caución ya no se muestra. La columna pct_caucion en config_dashboard queda sin uso.</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Meses a proyectar</v>
+        <v>Etiqueta Caución (x% cash)</v>
       </c>
       <c r="B56" t="str">
-        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
+        <v>Retirado: la columna Caución ya no forma parte del Flujo por mes.</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Config por usuario en Supabase</v>
+        <v>Meses a proyectar</v>
       </c>
       <c r="B57" t="str">
-        <v>Tabla config_dashboard (user_id, proyección, alertas y meses_excluidos JSON). Se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql; meses excluidos: supabase_config_dashboard_meses_excluidos.sql.</v>
+        <v>En Configuración: combo Meses a proyectar (1, 2, 3, 4, 5, 6, 12). Flujo por mes y Evolución muestran esa cantidad de columnas/filas proyectadas.</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Recorte % (cada lado)</v>
+        <v>Config por usuario en Supabase</v>
       </c>
       <c r="B58" t="str">
-        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
+        <v>Tabla config_dashboard (user_id, proyección, alertas y meses_excluidos JSON). Se sincroniza al cargar y al guardar; la config persiste por usuario en la base. Migración: supabase_config_dashboard.sql; meses excluidos: supabase_config_dashboard_meses_excluidos.sql.</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Novedades del Negocio</v>
+        <v>Recorte % (cada lado)</v>
       </c>
       <c r="B59" t="str">
-        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
+        <v>En Configuración, combo Recorte % (cada lado) (0, 5, 10, 15, 20, 25) visible solo cuando el método es Promedio recortado. Más % = más suavizado. Persistido en config_dashboard (proyeccion_recorte).</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>To-Do</v>
+        <v>Novedades del Negocio</v>
       </c>
       <c r="B60" t="str">
-        <v>Menú To-Do, mismo criterio que Everfit. Bandeja con filtros (abiertas, hoy, recurrencia), tarjetas Pendientes / En curso / Vencidas / Hechas hoy, recurrencia (única, diaria, semanal, mensual, bimestral, trimestral, anual; sin domingos; la diaria se marca hecha desde el día de vencimiento), responsable usuario o perfil. Quien no crea solo ve las suyas o las de su perfil. Admin y Encargado ven la matriz Por responsable. Abajo, si tiene Configuración, reasigna abiertas de un usuario o perfil a otro. Excel con fechas y prioridad numéricas. En Seguridad: ver_todo y completar_todo en todos los perfiles; crear_todo, editar_todo y eliminar_todo en Admin y Encargado (se puede cambiar el toggle). La columna Tarea usa el ancho libre de la pantalla. La descripción se abre con el ícono de ayuda al lado del título.</v>
+        <v>Ítem en sidebar que abre una vista con importadores de hornos y comercios de venta de hornos en Argentina (Buenos Aires). Datos recuperados por IA (Edge Function con Gemini + google_search). Nombre, dirección, teléfono y web por contacto.</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Gestión de Proyectos</v>
+        <v>To-Do</v>
       </c>
       <c r="B61" t="str">
-        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Archivos adjuntos por fecha (descripción + archivo en Storage gp-archivos) en proyecto, entregable y tarea; solapa Archivos y hoja Excel. Solapa Horas cons.: conciliación diaria. La solapa activa (To-Do, Gantt, Horas, Archivos) se marca con etiqueta Activo y un contorno más visible. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
+        <v>Menú To-Do, mismo criterio que Everfit. Bandeja con filtros (abiertas, hoy, recurrencia), tarjetas Pendientes / En curso / Vencidas / Hechas hoy, recurrencia (única, diaria, semanal, mensual, bimestral, trimestral, anual; sin domingos; la diaria se marca hecha desde el día de vencimiento), responsable usuario o perfil. Quien no crea solo ve las suyas o las de su perfil. Admin y Encargado ven la matriz Por responsable. Abajo, si tiene Configuración, reasigna abiertas de un usuario o perfil a otro. Excel con fechas y prioridad numéricas. En Seguridad: ver_todo y completar_todo en todos los perfiles; crear_todo, editar_todo y eliminar_todo en Admin y Encargado (se puede cambiar el toggle). La columna Tarea usa el ancho libre de la pantalla. La descripción se abre con el ícono de ayuda al lado del título.</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Conciliación Bancaria</v>
+        <v>Gestión de Proyectos</v>
       </c>
       <c r="B62" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja), Credicoop (botón negro) y FCI Galicia (ARS)/(USD) (verde). FCI carga solo tesorería (histórico con Caja FCI Galicia (ARS) o (USD)); las sugerencias salen del extracto de Galicia de la misma moneda, sin extracto propio. La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. En el histórico, además, un Id que corta la secuencia del archivo (del menor al mayor) también va a A eliminar de esa caja (Mercado Pago, Galicia, Credicoop y FCI). Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. Se puede deshacer esa anulación: los dos movimientos vuelven al extracto y se pueden conciliar; abajo quedan para volver a anularlos (sql/supabase_cb_mp_anulacion_deshecha.sql). En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Menú lateral (permiso ver_gestion_proyectos). ABM de planes: Proyecto → Entregables (nombre, alcance, fechas, responsable usuario o perfil) → Tareas (misma metadata) y Dependencias (viñeta + responsable). Las horas son las realmente consumidas por fecha en el proyecto (gp_proyecto_hora), el entregable (gp_entregable_hora) y/o las tareas (gp_tarea_hora), cada fila con observaciones; el total del proyecto es propias + entregables + tareas (RPC gp_guardar_horas_*). Archivos adjuntos por fecha (descripción + archivo en Storage gp-archivos) en proyecto, entregable y tarea; solapa Archivos y hoja Excel. Solapa Horas cons.: conciliación diaria. La solapa activa (To-Do, Gantt, Horas, Archivos) se marca con etiqueta Activo y un contorno más visible. Alerta si una tarea o las horas superan el deadline del entregable o del proyecto. El responsable de usuario se muestra como nombre corto / iniciales (no el email; el correo va en el tooltip). Solapa To-Do: tabla jerárquica expandable o solo entregables (entregable en negrita, tareas y dependencias en peso normal), cards de pendientes/en curso/vencidas, cambio de estado. Ordenar entregables por fecha, nombre, estado o manual (flechas ↑↓ persistidas). Solapa Gantt one-page: anillo de avance, SPI ponderado por horas consumidas (propias del proyecto + entregables/tareas; sin horas no diluye) vs calendario, barras con % y horas consumidas (reales, no planificadas); export Excel (Plan/Resumen/Horas cons./Gantt gráfico con barras de color como el PDF, sin unos, importes, % y horas numéricos) y PDF (impresión en la misma pestaña, sin pop-up). Permisos crear_proyecto / editar_proyecto / eliminar_proyecto en Seguridad. Componente: scripts/lib/fornitalia-gestion-proyectos.js + .css. SQL: sql/supabase_gestion_proyectos.sql, sql/supabase_user_profiles_nombre_usuario.sql, sql/supabase_gp_tarea_horas_alocadas.sql, sql/supabase_gp_tarea_hora.sql, sql/supabase_gp_entregable_hora.sql, sql/supabase_gp_proyecto_hora.sql, sql/supabase_gp_observaciones_y_horas_rls.sql y sql/supabase_gp_hora_observaciones.sql.</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Cajas (físicas)</v>
+        <v>Conciliación Bancaria</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. En el histórico, un Pendiente cuyo Id corta la secuencia del archivo (del menor al mayor: si falta el 8 entre 1 y 10, se muestra el 8) aparece en el resultado agrupado por caja física, con Eliminar para confirmar. Mercado Pago, Galicia, Credicoop y FCI siguen yendo a A eliminar de cada caja. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. El histórico conserva la columna Monto (en dólares se pesifica al MEP de la fecha). La columna Saldo de cada caja acumula crédito y débito en orden de fecha, alineada al corte que cierra con esos movimientos. En las cajas en dólares esa columna y la tarjeta de saldo son la suma en USD, sin dividir los pesos por el tipo de cambio.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja), Credicoop (botón negro) y FCI Galicia (ARS)/(USD) (verde). FCI carga solo tesorería (histórico con Caja FCI Galicia (ARS) o (USD)); las sugerencias salen del extracto de Galicia de la misma moneda, sin extracto propio. La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. En el histórico, además, un Id que corta la secuencia del archivo (del menor al mayor) también va a A eliminar de esa caja (Mercado Pago, Galicia, Credicoop y FCI). Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. Se puede deshacer esa anulación: los dos movimientos vuelven al extracto y se pueden conciliar; abajo quedan para volver a anularlos (sql/supabase_cb_mp_anulacion_deshecha.sql). En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Saldos extractos</v>
+        <v>Cajas (físicas)</v>
       </c>
       <c r="B64" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. El mes en curso del consolidado pesifica Galicia USD y FCI USD al MEP de hoy (o el inmediato anterior), la misma cotización de la torta. El efectivo en dólares no se vuelve a pasar por el tipo de cambio: el saldo es la suma en USD. Los meses cerrados no se recalculan. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). En Efectivo-f (USD) y Efectivo-s/f (USD) el saldo, el gráfico, el Excel y la comparación con tesorería están en dólares (suma de los movimientos), con el importe en pesos ya guardado debajo. Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
+        <v>Menú lateral (permiso ver_cajas_fisicas). Cajas que no se concilian con extracto bancario. Solapas Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS) y Efectivo-s/f (USD). La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico se puede cargar de a una caja acá o, para todas juntas, desde Flujo de caja. El histórico Caja Efectivo … sin factura entra a s/f (USD si Moneda es USD o Caja = Efectivo Dolar (sin factura)). Caja = Efectivo Pesos (sin factura) / Efectivo Dolar (sin factura) se reconoce en cualquier tesorería, cierre o histórico (también si se sube desde Conciliación Bancaria) y el saldo va a Saldos extractos. En USD los importes se pesifican al MEP de tipo_de_cambio (fecha del movimiento o última cotización anterior); la grilla muestra ARS, USD original y TC. Upload con columna Id (alta o actualización, sin duplicar); si el archivo no es de la solapa activa, pide cambiar de solapa. El histórico movimientos-historico_… también se puede cargar: solo entran las filas de esa caja física. Apertura de Caja no se carga ni entra al corte de Saldos extractos. El histórico carga movimientos y no pisa el saldo de tesorería o cierre. Status Anulado no se carga (si el Id ya existía, se elimina). Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente; Status Pendiente sí se da de alta. Status Pendiente o sin Status (caja abierta) que ya no viene va a A eliminar; un Confirmado nunca. Tras cada carga se abre el mismo popup que en Conciliación Bancaria (nuevos, actualizados, sin cambios, a eliminar y omitidos). Encabezados de tabla ordenan asc/desc. Columna Observaciones (después de Descripción; viene del Excel / raw). Filtros en modal: mes, tipo, categoría y cuenta contable (opciones dinámicas; badge con cantidad activa); el buscar amplio sigue en la toolbar. El saldo de corte alimenta Saldos extractos. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene. En el histórico, un Pendiente cuyo Id corta la secuencia del archivo (del menor al mayor: si falta el 8 entre 1 y 10, se muestra el 8) aparece en el resultado agrupado por caja física, con Eliminar para confirmar. Mercado Pago, Galicia, Credicoop y FCI siguen yendo a A eliminar de cada caja. Excel del listado visible con los filtros (importes numéricos, fechas serial Argentina). Permisos cargar_cajas_fisicas y exportar_cajas_fisicas. Componente: scripts/lib/fornitalia-cajas-fisicas.js + .css. SQL: sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cf_borrar_apertura_caja.sql, sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_borrar_saldos_historico_apertura.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. El histórico conserva la columna Monto (en dólares se pesifica al MEP de la fecha). La columna Saldo de cada caja acumula crédito y débito en orden de fecha, alineada al corte que cierra con esos movimientos. En las cajas en dólares esa columna y la tarjeta de saldo son la suma en USD, sin dividir los pesos por el tipo de cambio.</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Impuestos</v>
+        <v>Saldos extractos</v>
       </c>
       <c r="B65" t="str">
-        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca), marcada Activo como el resto de pantallas: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (listado con Observaciones; justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql, sql/supabase_cb_match_impuestos.sql y sql/supabase_imp_tesoreria_observaciones.sql.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. El mes en curso del consolidado pesifica Galicia USD y FCI USD al MEP de hoy (o el inmediato anterior), la misma cotización de la torta. El efectivo en dólares no se vuelve a pasar por el tipo de cambio: el saldo es la suma en USD. Los meses cerrados no se recalculan. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). En Efectivo-f (USD) y Efectivo-s/f (USD) el saldo, el gráfico, el Excel y la comparación con tesorería están en dólares (suma de los movimientos), con el importe en pesos ya guardado debajo. Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Normalización de extracto bancario</v>
+        <v>Impuestos</v>
       </c>
       <c r="B66" t="str">
-        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
+        <v>Menú lateral (permiso ver_impuestos). Primera solapa Mercado Pago (azul de marca), marcada Activo como el resto de pantallas: combo de régimen (CIBBPP = IIBB Reg. General Buenos Aires; CIBCPP = IIBB Rég. General CABA; CIVAPP = Percepción IVA) para cargar el Excel de percepción. Se guarda por Número de movimiento (sin duplicar) y se cruza con el extracto MP de Conciliación Bancaria: columnas En extracto y Conciliado (confirmado, No requiere o conciliación manual con tesorería). Conciliación manual: no conciliadas por tipo de archivo, seleccionar todas y cruzarlas con un único movimiento de tesorería Mercado Pago (listado con Observaciones; justificación); el tesorería queda en Confirmados de Conciliación Bancaria con badge Conciliación manual de impuestos (sin match del cargo del extracto). La card Percibido muestra debajo el monto no conciliado. Modal Filtros (como Cajas) con Mes, En extracto MP y Conciliado; el buscar queda en la toolbar. Tabla, KPIs y Excel respetan esos filtros. Encabezados ordenables. Permisos cargar_impuestos y exportar_impuestos. Componente: scripts/lib/fornitalia-impuestos.js + .css. SQL: sql/supabase_impuestos.sql, sql/supabase_impuestos_conciliacion_manual.sql, sql/supabase_cb_match_impuestos.sql y sql/supabase_imp_tesoreria_observaciones.sql.</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Informe inconsistencias datos legacy (cliente)</v>
+        <v>Normalización de extracto bancario</v>
       </c>
       <c r="B67" t="str">
-        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
+        <v>npm run normalizar-extracto: lee Fornitalia_Movimientos.xlsx (o Extracto legado), hoja Normalizado con fecha_iso, tipo, medio, categoría, cuenta, moneda inferida, monto_original, tipo_cambio, monto_ars, id_cierre_caja, id_comprobante_pago, id_impuesto, cat_desc cuando vienen del export.</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Upload de extracto normalizado</v>
+        <v>Informe inconsistencias datos legacy (cliente)</v>
       </c>
       <c r="B68" t="str">
-        <v>Retirado: el Flujo ya no reemplaza la tabla transacciones desde un Excel Normalizado. El botón, el modal y el permiso carga_normalizada salieron de la app. Queda el script npm run normalizar-extracto para generar el archivo.</v>
+        <v>docs/ANALISIS_NORMALIZACION_DATOS_LEGACY_FORNITALIA.md alineado a Fornitalia_Movimientos.xlsx, §0 validaciones IDs/CatDesc, pipeline normalizar-extracto. Regenerar HTML+PDF: npm run informe-normalizacion (informe-normalizacion-solo-html solo si hace falta iterar sin Playwright).</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Log de excluidos en upload</v>
+        <v>Upload de extracto normalizado</v>
       </c>
       <c r="B69" t="str">
-        <v>Retirado: la solapa Excluidos upload y su permiso ya no están en el dashboard. La tabla de auditoría en Supabase se conserva.</v>
+        <v>Retirado: el Flujo ya no reemplaza la tabla transacciones desde un Excel Normalizado. El botón, el modal y el permiso carga_normalizada salieron de la app. Queda el script npm run normalizar-extracto para generar el archivo.</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Matriz EF</v>
+        <v>Log de excluidos en upload</v>
       </c>
       <c r="B70" t="str">
-        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6 ni 1.2 (ajuste de saldos), A–D, 6.1–6.3 ni ratios. Una relación sin movimientos se borra desde Relaciones; un subítem se borra junto con sus relaciones si ninguna tiene movimientos. Códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql, sql/supabase_ef_estructura_abm.sql y sql/supabase_ef_ajuste_saldos_caja.sql.</v>
+        <v>Retirado: la solapa Excluidos upload y su permiso ya no están en el dashboard. La tabla de auditoría en Supabase se conserva.</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Análisis financiero extracto (PDF)</v>
+        <v>Matriz EF</v>
       </c>
       <c r="B71" t="str">
-        <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
+        <v>Menú lateral (permiso ver_matriz_ef). ABM de relaciones categoría + cuenta contable + tipo Ingreso/Egreso → ítem y subítem del Estado Financiero, y ABM del árbol ef_estructura (solapa Estructura EF: secciones, subítems y totales). La solapa activa (Relaciones, Sin relación, Estructura EF) se marca con etiqueta Activo. Validaciones: no borrar 1–6 ni 1.2 (ajuste de saldos), A–D, 6.1–6.3 ni ratios. Una relación sin movimientos se borra desde Relaciones; un subítem se borra junto con sus relaciones si ninguna tiene movimientos. Códigos únicos; rename en cascada a matriz. Nombres = tesorería. Encabezados ordenan la grilla. Sin relación lista pares del Flujo sin fila. Permiso editar_matriz_ef. Componente: scripts/lib/fornitalia-matriz-ef.js + .css. SQL: sql/supabase_cb_credicoop_cajas_sf_matriz_ef.sql, sql/supabase_ef_estructura_abm.sql y sql/supabase_ef_ajuste_saldos_caja.sql.</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Usuario en tablas</v>
+        <v>Análisis financiero extracto (PDF)</v>
       </c>
       <c r="B72" t="str">
-        <v>Quién cargó, confirmó, descartó o eliminó: se ve el nombre para mostrar (ej. LB) y al pasar el mouse el email. Lo histórico de tesorería, saldos, impuestos y matriz queda a nombre de LB (lucas.bustos.martin@gmail.com). El consolidado de Saldos extractos no tiene actor por fila. rpc get_usuarios_mostrar. sql/supabase_usuarios_mostrar.sql.</v>
+        <v>npm run analisis-financiero-pdf: métricas desde Fornitalia_Movimientos.xlsx (fallback Extracto legado); ARS vía MontoCambio/Monto en $, TC por fila o MEP; exclusiones y USD sin conversión. Sección ventas: ranking por vendedor desde Resumen_Operaciones (Tabla, Vendedor_RO) por N° operación; ranking proxy por producto (detalle hasta mes cierre feb 2026). Ver docs/ANALISIS_FINANCIERO_EXTRACTO_README.md.</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Novedades al iniciar sesión</v>
+        <v>Usuario en tablas</v>
       </c>
       <c r="B73" t="str">
-        <v>Tras cada despliegue, al entrar a la app se muestra el modal «Nueva versión» con 2–4 frases de lo que se nota al recargar (logo, badge de versión, lista). Una vez Entendido, no vuelve a aparecer hasta la siguiente versión. El texto lo actualiza el agente en scripts/lib/fornitalia-release-blurb.js; fornitalia-release.json se sirve por red.</v>
+        <v>Quién cargó, confirmó, descartó o eliminó: se ve el nombre para mostrar (ej. LB) y al pasar el mouse el email. Lo histórico de tesorería, saldos, impuestos y matriz queda a nombre de LB (lucas.bustos.martin@gmail.com). El consolidado de Saldos extractos no tiene actor por fila. rpc get_usuarios_mostrar. sql/supabase_usuarios_mostrar.sql.</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
+        <v>Novedades al iniciar sesión</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Tras cada despliegue, al entrar a la app se muestra el modal «Nueva versión» con 2–4 frases de lo que se nota al recargar (logo, badge de versión, lista). Una vez Entendido, no vuelve a aparecer hasta la siguiente versión. El texto lo actualiza el agente en scripts/lib/fornitalia-release-blurb.js; fornitalia-release.json se sirve por red.</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
         <v>Mensajes de confirmación y aviso</v>
       </c>
-      <c r="B74" t="str">
+      <c r="B75" t="str">
         <v>Las preguntas sí/no y los avisos de error o validación se muestran en un cuadro de la app (título, texto y botones con icono), no en el cartel del navegador. Confirmar usa Aceptar y Cancelar; un aviso usa Entendido. Eliminar marca el botón en rojo. Componente: scripts/lib/fornitalia-mensajes.js.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B75"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9529,7 +9656,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C145"/>
+  <dimension ref="A1:C146"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11131,16 +11258,27 @@
         <v>Despliegue v2.101: en To-Do, filtro de Recurrencia (Única, Diaria, Semanal, Mensual, Bimestral, Trimestral o Anual). Recorta la bandeja, las tarjetas, la matriz por responsable y el Excel. Producción Vercel.</v>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>2.102</v>
+      </c>
+      <c r="B146" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="C146" t="str">
+        <v>Despliegue v2.102: Agenda de pagos, primera solapa de Flujo de caja. Estima las próximas 4 semanas de lunes a viernes, por categoría, cuenta contable y proveedor. Sueldos y Jornales a pagar usa la primera semana del último mes y cae el primer día hábil (el 1/11/2026 pasa al 2/11). Impuestos de hasta $ 500.000 y gastos bancarios no entran. Si el cálculo cae sábado o domingo, el pago pasa al lunes. En Seguridad se puede ocultar la solapa. sql/supabase_agenda_pagos_permiso.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C145"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C146"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="90.83203125" customWidth="1"/>
@@ -11428,9 +11566,23 @@
         <v/>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Agenda de pagos</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Solapa inicial de Flujo de caja: estimado de las próximas 4 semanas según los últimos 3 pagos del proveedor (el más reciente pesa más), por categoría y cuenta contable, sin impuestos de hasta $ 500.000 ni gastos bancarios. Sueldos y Jornales el día 1, cada 30 días, desde septiembre. Con lo ya pagado al mismo proveedor.</v>
+      </c>
+      <c r="C21">
+        <v>8</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.103: en Agenda de pagos cada semana suma un colchón de entre 5% y 30% del estimado.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E502"/>
+  <dimension ref="A1:E506"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -8945,9 +8945,77 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="503">
+      <c r="A503" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B503" t="str">
+        <v>10:08</v>
+      </c>
+      <c r="C503" t="str">
+        <v>Agenda de pagos: colchón por dispersión</v>
+      </c>
+      <c r="D503" t="str">
+        <v>Cada semana suma un colchón de liquidez igual al desvío de los egresos de esa misma semana del mes en los últimos 6 meses. El cálculo sale de la historia y cambia con los datos. Se ve en la barra y en el total de la semana, aparte del estimado.</v>
+      </c>
+      <c r="E503" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B504" t="str">
+        <v>10:18</v>
+      </c>
+      <c r="C504" t="str">
+        <v>Agenda de pagos: colchón sin Mercaderías</v>
+      </c>
+      <c r="D504" t="str">
+        <v>La cuenta Mercaderías sale del desvío del colchón. Son compras grandes, en promedio cada unos 3 meses, y no son el pago habitual. El colchón queda sobre el resto de los egresos de esa semana del mes. Si esa compra cae en las 4 semanas, sigue en el estimado.</v>
+      </c>
+      <c r="E504" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B505" t="str">
+        <v>10:25</v>
+      </c>
+      <c r="C505" t="str">
+        <v>Agenda de pagos: colchón como porcentaje</v>
+      </c>
+      <c r="D505" t="str">
+        <v>El colchón dejó de ser el desvío en pesos de toda la semana, que daba decenas de millones. Ahora es un adicional del estimado de esa semana, entre 5% y 30%. La semana del mes más pareja queda en 5% y la más variable en 30%. Mercaderías sigue fuera de la dispersión.</v>
+      </c>
+      <c r="E505" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="B506" t="str">
+        <v>10:35</v>
+      </c>
+      <c r="C506" t="str">
+        <v>Despliegue v2.103 producción</v>
+      </c>
+      <c r="D506" t="str">
+        <v>Push a main y Vercel --prod: en Agenda de pagos cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes. Mercaderías no entra. APP_VERSION 2.103.</v>
+      </c>
+      <c r="E506" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E502"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E506"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9117,7 +9185,7 @@
         <v>Agenda de pagos</v>
       </c>
       <c r="B20" t="str">
-        <v>Primera solapa de Flujo de caja y vista al entrar, si el perfil la tiene. Estima egresos de las próximas 4 semanas con los últimos 3 meses. El importe sale de los últimos 3 pagos de ese proveedor y categoría, con más peso en el más reciente. Prioriza series con ID compra. También entran pagos frecuentes sin ID compra. Impuestos de hasta $ 500.000 y Gastos bancarios no entran. Cada serie se abre por categoría y cuenta contable. Sueldos y Jornales se estima el día 1, cada 30 días, con los pagos cargados desde septiembre de 2026. Barras por semana (ámbar por pagar, verde ya pagado) y total al pie de cada semana. Ya pagado: en esa semana ya hubo un egreso con ID compra al mismo proveedor, sin comparar el monto. No aplica a series sin ID compra. Permiso ver_solapa_agenda_pagos en Seguridad.</v>
+        <v>Primera solapa de Flujo de caja y vista al entrar, si el perfil la tiene. Estima egresos de las próximas 4 semanas con los últimos 3 meses. El importe sale de los últimos 3 pagos de ese proveedor y categoría, con más peso en el más reciente. Prioriza series con ID compra. También entran pagos frecuentes sin ID compra. Impuestos de hasta $ 500.000 y Gastos bancarios no entran. Cada serie se abre por categoría y cuenta contable. Sueldos y Jornales se estima el día 1, cada 30 días, con los pagos cargados desde septiembre de 2026. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses. La más pareja queda en 5% y la más variable en 30%. La cuenta Mercaderías no entra en esa dispersión. Barras por semana (ámbar por pagar, azul colchón, verde ya pagado) y total al pie de cada semana. Ya pagado: en esa semana ya hubo un egreso con ID compra al mismo proveedor, sin comparar el monto. No aplica a series sin ID compra. Permiso ver_solapa_agenda_pagos en Seguridad.</v>
       </c>
     </row>
     <row r="21">
@@ -9656,7 +9724,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C146"/>
+  <dimension ref="A1:C147"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11269,9 +11337,20 @@
         <v>Despliegue v2.102: Agenda de pagos, primera solapa de Flujo de caja. Estima las próximas 4 semanas de lunes a viernes, por categoría, cuenta contable y proveedor. Sueldos y Jornales a pagar usa la primera semana del último mes y cae el primer día hábil (el 1/11/2026 pasa al 2/11). Impuestos de hasta $ 500.000 y gastos bancarios no entran. Si el cálculo cae sábado o domingo, el pago pasa al lunes. En Seguridad se puede ocultar la solapa. sql/supabase_agenda_pagos_permiso.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>2.103</v>
+      </c>
+      <c r="B147" t="str">
+        <v>24/10/2026</v>
+      </c>
+      <c r="C147" t="str">
+        <v>Despliegue v2.103: en Agenda de pagos cada semana suma un colchón de liquidez. Es un adicional del estimado de esa semana, entre 5% y 30%, según la dispersión de esa semana del mes en los últimos 6 meses. La más pareja queda en 5% y la más variable en 30%. La cuenta Mercaderías no entra en el colchón. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C146"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C147"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11571,7 +11650,7 @@
         <v>Agenda de pagos</v>
       </c>
       <c r="B21" t="str">
-        <v>Solapa inicial de Flujo de caja: estimado de las próximas 4 semanas según los últimos 3 pagos del proveedor (el más reciente pesa más), por categoría y cuenta contable, sin impuestos de hasta $ 500.000 ni gastos bancarios. Sueldos y Jornales el día 1, cada 30 días, desde septiembre. Con lo ya pagado al mismo proveedor.</v>
+        <v>Solapa inicial de Flujo de caja: estimado de las próximas 4 semanas según los últimos 3 pagos del proveedor (el más reciente pesa más), por categoría y cuenta contable, sin impuestos de hasta $ 500.000 ni gastos bancarios. Sueldos y Jornales el día 1, cada 30 días, desde septiembre. Con lo ya pagado al mismo proveedor. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses, sin la cuenta Mercaderías.</v>
       </c>
       <c r="C21">
         <v>8</v>

</xml_diff>

<commit_message>
v2.104: el efectivo en dólares del mes en curso se pesifica al MEP de hoy.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E506"/>
+  <dimension ref="A1:E508"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -9013,9 +9013,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="507">
+      <c r="A507" t="str">
+        <v>25/10/2026</v>
+      </c>
+      <c r="B507" t="str">
+        <v>09:11</v>
+      </c>
+      <c r="C507" t="str">
+        <v>Saldos extractos: efectivo dólar del mes en curso al MEP de hoy</v>
+      </c>
+      <c r="D507" t="str">
+        <v>Efectivo-f (USD) mostraba pesos negativos (unos −2,8 millones) con US$ 1.200 porque el consolidado sumaba cada movimiento al MEP del día, no los 1.200 dólares de hoy. En el mes en curso, Efectivo-f (USD) y Efectivo sin factura (USD) se pesifican al MEP de hoy, igual que la posición de caja de Flujo de caja. Los meses cerrados no se recalculan.</v>
+      </c>
+      <c r="E507" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="str">
+        <v>25/10/2026</v>
+      </c>
+      <c r="B508" t="str">
+        <v>09:14</v>
+      </c>
+      <c r="C508" t="str">
+        <v>Despliegue v2.104 producción</v>
+      </c>
+      <c r="D508" t="str">
+        <v>Push a main y Vercel --prod: en el mes en curso, Efectivo-f (USD) y Efectivo sin factura (USD) se pesifican al MEP de hoy. El saldo actual del consolidado coincide con la posición de caja. APP_VERSION 2.104.</v>
+      </c>
+      <c r="E508" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E506"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E508"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9545,7 +9579,7 @@
         <v>Saldos extractos</v>
       </c>
       <c r="B65" t="str">
-        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. El mes en curso del consolidado pesifica Galicia USD y FCI USD al MEP de hoy (o el inmediato anterior), la misma cotización de la torta. El efectivo en dólares no se vuelve a pasar por el tipo de cambio: el saldo es la suma en USD. Los meses cerrados no se recalculan. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). En Efectivo-f (USD) y Efectivo-s/f (USD) el saldo, el gráfico, el Excel y la comparación con tesorería están en dólares (suma de los movimientos), con el importe en pesos ya guardado debajo. Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
+        <v>Menú lateral (permiso ver_saldos_extractos). Solapas Mercado Pago (azul de marca), Galicia (ARS) y Galicia (USD) (naranja), FCI Galicia (ARS) y FCI Galicia (USD), Efectivo-f (ARS), Morba-s/f (ARS), Efectivo-f (USD), Efectivo-s/f (ARS), Efectivo-s/f (USD) y Consolidado. FCI es la suma corrida de la tesorería de suscripción y rescate (sin extracto propio); el USD se pesifica al MEP y el consolidado y la torta de Flujo lo incluyen. El mes en curso del consolidado pesifica Galicia USD, FCI USD, Efectivo-f (USD) y Efectivo sin factura (USD) al MEP de hoy (o el inmediato anterior), la misma cotización de la torta de Flujo de caja, para que el saldo actual coincida con la posición de caja. Los meses cerrados no se recalculan. MP: el corte es la carta de saldo (saldo total, incluye el saldo a liberar). El resumen de cuenta no se usa porque solo trae el disponible. El día a día entra por el Excel del extracto. El mes en curso parte del saldo total de la última carta y suma los movimientos banco desde el día siguiente. Galicia (ARS): el día a día entra por el Excel Extracto_CC. El PDF solo verifica movimientos del período que el banco no metió en el resumen. Un corte nuevo = último corte + movimientos Excel. Los extractos ya cargados no se recalculan. Galicia (USD): PDF Extracto_Cuentas_Galicia_… (Cuenta Corriente Especial en dólares) o Excel Extracto_CCE…; el saldo en USD se pesifica al MEP de tipo_de_cambio (fecha de cierre o última cotización anterior) y entra en ARS al consolidado. En Galicia (ARS/USD), el mes en curso (celeste) es el saldo corrido del último movimiento Imputado del extracto, más lo posterior a esa fecha que también esté Imputado; un cheque Pendiente o En proceso no entra. No se compara la fila entre archivos distintos ni se suma la tesorería. En MP, mes en curso = saldo total de la última carta + movimientos del extracto posteriores. En Credicoop, último corte + crédito − débito. Botón Tesorería saldos: sube tesoreria_saldos_YYYY-MM-DD.xlsx y compara el saldo de cada caja con el mes en curso (tilde verde si coincide; cruz roja con la diferencia si no; en cajas dólar se compara US$). En Galicia (USD) el saldo en pesos lleva debajo el monto en dólares (US$, letra chica). En Efectivo-f (USD) y Efectivo-s/f (USD) el saldo, el gráfico, el Excel y la comparación con tesorería están en dólares (suma de los movimientos), con el importe en pesos ya guardado debajo. Botón PDF: reporte gráfico de la vista activa (cards, gráfico y tabla) indicando la solapa Activo. Las cajas físicas se actualizan desde el menú Cajas (físicas) con tesorería o cierre (Apertura de Caja no entra; el histórico no pisa el corte); Efectivo-f (USD) entra en ARS (MEP). Credicoop (caja banco, botón negro) no tiene extractos históricos: el corte se arma con tesorería de Conciliación Bancaria (sin Apertura) y entra al consolidado. Carga de varios archivos, se reconocen de a uno y se guardan juntos sin duplicar ni borrar previos (clave canal+cuenta+fecha). Consolidado: posición mensual Galicia (ARS) + Galicia (USD) + MP + Efectivo-f (ARS) + Morba-s/f (ARS) + Efectivo-f (USD) (si un canal no tiene corte ese mes, se arrastra el saldo anterior). KPIs: cantidad, último saldo, variación del período (con el filtro Desde/Hasta debajo), promedio de saldo (cuánto queda en las cuentas) y promedio de variación; cada card tiene icono de ayuda. Gráfico de línea y Excel (importes numéricos, fechas serial Argentina). Permisos cargar_saldos_extractos y exportar_saldos_extractos. Componente: scripts/lib/fornitalia-saldos-extractos.js + .css. SQL: sql/supabase_saldos_extractos.sql, sql/supabase_saldos_extractos_mercadopago.sql, sql/supabase_cajas_fisicas.sql, sql/supabase_cajas_fisicas_morba.sql, sql/supabase_cajas_fisicas_dolar.sql, sql/supabase_cb_galicia_usd.sql, sql/supabase_eb_saldo_credicoop.sql, sql/supabase_eb_saldo_mes_en_curso.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. Un corte de Efectivo o Morba que no cierra con los movimientos que siguen en la caja se rearma: lo eliminado no entra al saldo.</v>
       </c>
     </row>
     <row r="66">
@@ -9724,7 +9758,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C147"/>
+  <dimension ref="A1:C148"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11348,9 +11382,20 @@
         <v>Despliegue v2.103: en Agenda de pagos cada semana suma un colchón de liquidez. Es un adicional del estimado de esa semana, entre 5% y 30%, según la dispersión de esa semana del mes en los últimos 6 meses. La más pareja queda en 5% y la más variable en 30%. La cuenta Mercaderías no entra en el colchón. Producción Vercel.</v>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>2.104</v>
+      </c>
+      <c r="B148" t="str">
+        <v>25/10/2026</v>
+      </c>
+      <c r="C148" t="str">
+        <v>Despliegue v2.104: en Saldos extractos, el mes en curso pesifica Efectivo-f (USD) y Efectivo sin factura (USD) al MEP de hoy. Efectivo-f (USD) deja de mostrar pesos negativos cuando todavía hay dólares en caja. El saldo actual del consolidado coincide con la posición de caja de Flujo de caja. Los meses cerrados no se recalculan. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C147"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C148"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.105: en Flujo por mes los ratios c/f y s/f usan solo cobranzas por ventas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E508"/>
+  <dimension ref="A1:E510"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -9047,9 +9047,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="509">
+      <c r="A509" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="B509" t="str">
+        <v>09:02</v>
+      </c>
+      <c r="C509" t="str">
+        <v>Ratios c/f y s/f solo con cobranzas por ventas</v>
+      </c>
+      <c r="D509" t="str">
+        <v>Ingresos c/f / Ingresos e Ingresos s/f / Ingresos dejan afuera el resto de los ingresos. Entran los movimientos con subítem Cobranzas por Ventas, o con categoría Ventas. c/f y s/f siguen partiendo esas cobranzas y suman 100%.</v>
+      </c>
+      <c r="E509" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="B510" t="str">
+        <v>09:04</v>
+      </c>
+      <c r="C510" t="str">
+        <v>Despliegue v2.105 producción</v>
+      </c>
+      <c r="D510" t="str">
+        <v>Push a main y Vercel --prod: en Flujo por mes, Ingresos c/f / Ingresos e Ingresos s/f / Ingresos usan solo cobranzas por ventas (subítem Cobranzas por Ventas o categoría Ventas). Los dos suman 100% de esas cobranzas. APP_VERSION 2.105.</v>
+      </c>
+      <c r="E510" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E508"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E510"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9075,7 +9109,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas); Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. Ingresos c/f / Ingresos e Ingresos s/f / Ingresos parten el mes: c/f es Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop; s/f es el resto. Los dos suman 100%. Ingresos c/f / Ingresos e Ingresos s/f / Ingresos parten el mes: c/f es Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop; s/f es el resto. Los dos suman 100%. La columna Total (Ingresos, Egresos, G/P y ratios) suma meses cerrados y va después de esos meses: el mes en curso se marca en celeste y no entra al Total, ni a las variaciones y la tendencia del gráfico, ni a la base de la proyección. Sobre esa barra se ve el G/P del mes en millones. Las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas); Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. Ingresos c/f / Ingresos e Ingresos s/f / Ingresos parten solo las cobranzas por ventas (subítem Cobranzas por Ventas, o categoría Ventas): c/f es Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop; s/f es el resto de esas cobranzas. Los dos suman 100% de esas cobranzas. La columna Total (Ingresos, Egresos, G/P y ratios) suma meses cerrados y va después de esos meses: el mes en curso se marca en celeste y no entra al Total, ni a las variaciones y la tendencia del gráfico, ni a la base de la proyección. Sobre esa barra se ve el G/P del mes en millones. Las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -9758,7 +9792,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C148"/>
+  <dimension ref="A1:C149"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11393,9 +11427,20 @@
         <v>Despliegue v2.104: en Saldos extractos, el mes en curso pesifica Efectivo-f (USD) y Efectivo sin factura (USD) al MEP de hoy. Efectivo-f (USD) deja de mostrar pesos negativos cuando todavía hay dólares en caja. El saldo actual del consolidado coincide con la posición de caja de Flujo de caja. Los meses cerrados no se recalculan. Producción Vercel.</v>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>2.105</v>
+      </c>
+      <c r="B149" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="C149" t="str">
+        <v>Despliegue v2.105: en Flujo por mes, Ingresos c/f / Ingresos e Ingresos s/f / Ingresos usan solo cobranzas por ventas (subítem Cobranzas por Ventas o categoría Ventas). Entre los dos suman 100% de esas cobranzas. También en el Excel y el PDF. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C148"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C149"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.106: la agenda conserva el día ya pasado y Conciliación no pisa a quien ya está conciliando.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E510"/>
+  <dimension ref="A1:E514"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -9081,9 +9081,77 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="511">
+      <c r="A511" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="B511" t="str">
+        <v>11:50</v>
+      </c>
+      <c r="C511" t="str">
+        <v>Agenda de pagos: no borrar el día que ya pasó</v>
+      </c>
+      <c r="D511" t="str">
+        <v>En la semana en curso, un estimado de ayer sigue en la agenda. El pago no cae justo en esa fecha, así que la fila no se saca porque el día ya pasó. Si en la semana hubo un pago al proveedor, el estado pasa a Ya pagado y la fila sigue en la tabla.</v>
+      </c>
+      <c r="E511" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="B512" t="str">
+        <v>11:58</v>
+      </c>
+      <c r="C512" t="str">
+        <v>Agenda de pagos: pagado por categoría y cuenta</v>
+      </c>
+      <c r="D512" t="str">
+        <v>Una fila sin proveedor, como Compras Mercado Pago / Libre y Publicidad y Propaganda, pasa a Ya pagado si en esa semana entró un egreso de esa categoría y esa cuenta. Se toma una sola fila y el importe queda el del pago, no el estimado.</v>
+      </c>
+      <c r="E512" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="B513" t="str">
+        <v>12:46</v>
+      </c>
+      <c r="C513" t="str">
+        <v>Conciliación: entrar no pisa a quien ya está conciliando</v>
+      </c>
+      <c r="D513" t="str">
+        <v>Abrir Conciliación o cambiar de solapa solo lee las sugerencias. Ya no las borra y las vuelve a armar. Se rearman al cargar un archivo o con Recalcular. Esa escritura espera si otra persona está confirmando el mismo canal, y no saca la fila que esa persona ya tiene tomada. sql/supabase_cb_sugerencias_concurrentes.sql.</v>
+      </c>
+      <c r="E513" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="B514" t="str">
+        <v>12:51</v>
+      </c>
+      <c r="C514" t="str">
+        <v>Despliegue v2.106 producción</v>
+      </c>
+      <c r="D514" t="str">
+        <v>Push a main y Vercel --prod: en Agenda de pagos un día de la semana en curso sigue aunque ya haya pasado, y un pago de la misma categoría y cuenta deja una fila en Ya pagado con el importe real. En Conciliación, entrar no rearma las sugerencias de quien ya está conciliando. APP_VERSION 2.106.</v>
+      </c>
+      <c r="E514" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E510"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E514"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9253,7 +9321,7 @@
         <v>Agenda de pagos</v>
       </c>
       <c r="B20" t="str">
-        <v>Primera solapa de Flujo de caja y vista al entrar, si el perfil la tiene. Estima egresos de las próximas 4 semanas con los últimos 3 meses. El importe sale de los últimos 3 pagos de ese proveedor y categoría, con más peso en el más reciente. Prioriza series con ID compra. También entran pagos frecuentes sin ID compra. Impuestos de hasta $ 500.000 y Gastos bancarios no entran. Cada serie se abre por categoría y cuenta contable. Sueldos y Jornales se estima el día 1, cada 30 días, con los pagos cargados desde septiembre de 2026. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses. La más pareja queda en 5% y la más variable en 30%. La cuenta Mercaderías no entra en esa dispersión. Barras por semana (ámbar por pagar, azul colchón, verde ya pagado) y total al pie de cada semana. Ya pagado: en esa semana ya hubo un egreso con ID compra al mismo proveedor, sin comparar el monto. No aplica a series sin ID compra. Permiso ver_solapa_agenda_pagos en Seguridad.</v>
+        <v>Primera solapa de Flujo de caja y vista al entrar, si el perfil la tiene. Estima egresos de las próximas 4 semanas con los últimos 3 meses. El importe sale de los últimos 3 pagos de ese proveedor y categoría, con más peso en el más reciente. Prioriza series con ID compra. También entran pagos frecuentes sin ID compra. Impuestos de hasta $ 500.000 y Gastos bancarios no entran. Cada serie se abre por categoría y cuenta contable. Sueldos y Jornales se estima el día 1, cada 30 días, con los pagos cargados desde septiembre de 2026. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses. La más pareja queda en 5% y la más variable en 30%. La cuenta Mercaderías no entra en esa dispersión. Barras por semana (ámbar por pagar, azul colchón, verde ya pagado) y total al pie de cada semana. Ya pagado: en esa semana ya hubo un egreso con ID compra al mismo proveedor, sin comparar el monto, y la fila sigue en la tabla. Sin ID compra, un pago de la misma categoría y cuenta contable toma una fila de esa semana, le pone el importe real y la deja en Ya pagado. Un día de la semana en curso no se saca porque ya pasó. No aplica a series sin ID compra. Permiso ver_solapa_agenda_pagos en Seguridad.</v>
       </c>
     </row>
     <row r="21">
@@ -9597,7 +9665,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B63" t="str">
-        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja), Credicoop (botón negro) y FCI Galicia (ARS)/(USD) (verde). FCI carga solo tesorería (histórico con Caja FCI Galicia (ARS) o (USD)); las sugerencias salen del extracto de Galicia de la misma moneda, sin extracto propio. La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. En el histórico, además, un Id que corta la secuencia del archivo (del menor al mayor) también va a A eliminar de esa caja (Mercado Pago, Galicia, Credicoop y FCI). Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. Se puede deshacer esa anulación: los dos movimientos vuelven al extracto y se pueden conciliar; abajo quedan para volver a anularlos (sql/supabase_cb_mp_anulacion_deshecha.sql). En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Menú lateral (permiso ver_conciliacion_bancaria). El banco (Galicia / Mercado Pago) es la fuente de verdad: lo que no está ahí no está. Tesorería son los movimientos administrativos de la app; Sugeridos / Solo banco / Solo sistema muestran las diferencias. Solapas Mercado Pago (azul de marca #009EE3), Galicia (ARS), Galicia (USD) (naranja), Credicoop (botón negro) y FCI Galicia (ARS)/(USD) (verde). FCI carga solo tesorería (histórico con Caja FCI Galicia (ARS) o (USD)); las sugerencias salen del extracto de Galicia de la misma moneda, sin extracto propio. La solapa y el listado en uso se marcan con etiqueta Activo y un contorno más visible. El histórico movimientos-historico_… también se puede cargar una sola vez desde Flujo de caja (reparte bancos y cajas físicas) y recálcula sugeridos en cada canal, igual que si se cargara tesorería en cada solapa. En cada canal: dos uploads (extracto banco y tesorería sistema). La carga es incremental para tesorería y para MP. En Galicia (Excel CC/CCE), un movimiento Imputado no se borra aunque el archivo de la ventana no lo traiga. Solo se retira si al entrar no estaba Imputado (p. ej. En proceso / cheque en proceso) y este Excel ya no lo trae; si después viene Imputado, se confirma. Tesorería no se toca. Si el ID ya existe no se inserta de nuevo (MP: Número de Movimiento; Galicia: fecha + débito/crédito + descripción, sin saldo — el banco cambia el saldo entre exportaciones). Apertura de Caja no se sube (tesorería). También se reconoce el Excel de cierre de caja: Fecha/Tipo/Monto e Id único (p. ej. cierre_CIERRE-…); Ingreso→crédito, Egreso→débito; historial de caja ya cerrada. El histórico movimientos-historico_… (Id, Fecha, Tipo, Caja, Monto) entra como tesorería: la columna Caja reparte Mercado Pago, Galicia ARS, Galicia USD y Credicoop; Efectivo con factura y Morba no se cargan acá (van a Cajas físicas). Caja Efectivo Pesos (sin factura) y Efectivo Dolar (sin factura) sí se desvían a Cajas físicas Efectivo-s/f (ARS/USD) y actualizan Saldos extractos. Tras cada carga se abre un popup con cuántos registros son nuevos (y sus Ids), cuántos cambiaron, cuántos ya estaban, Sugeridos por caja aunque sea 0 (para ver que el recálculo corrió) y qué se omitió. Si el Id ya existe, categoría y cuenta se actualizan aunque el Excel traiga Status Pendiente (Status Pendiente sí se da de alta). Status Anulado no se carga: se omite y, si ese Id ya estaba, se elimina (también la conciliación asociada). El Id hace alta o actualización (origen_id id|{Id}) sin duplicar ni dejar datos viejos; si ya existía tesorería sin Id, se adopta ese registro y se actualizan categoría y cuenta. La columna Caja (Transferencia Galicia / Transferencia Galicia Dolar / Mercado Pago) elige el canal; si el archivo no trae Id, sigue valiendo el prefijo MP_… / Galicia_… . Totales del pie no se cargan. Tesorería tesoreria_*.xlsx (Mercado Pago, Galicia ARS y Galicia Dolar) con columna Id hace alta o actualización por origen_id id|{Id} (si cambió categoría, cuenta u otro dato, se actualiza el mismo movimiento; filas sin Id no se cargan). Si el archivo no trae columna Id, no duplica por fecha, monto, descripción, categoría, cuenta y cliente. Al subir un cierre o tesorería con Id, se adoptan o retiran tesorerías viejas del mismo movimiento. Si un Id de tesorería abierta (tesoreria_*.xlsx) no viene en el nuevo archivo, el movimiento pasa a la solapa A eliminar (Id, fecha, importe, categoría, cuenta contable, descripción) para confirmar la baja definitiva (también borra la conciliación asociada); el movimiento queda en Tesorería eliminada. El cierre de caja no entra. Status Pendiente o sin Status puede ir a A eliminar, y solo si su fecha cae dentro del rango del Excel cargado (histórico o tesorería) y el Id no viene. En el histórico, además, un Id que corta la secuencia del archivo (del menor al mayor) también va a A eliminar de esa caja (Mercado Pago, Galicia, Credicoop y FCI). Si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. La lectura desde Supabase pagina de a 1000 filas para no truncar el listado. MP: Número de Movimiento + tesorería hoja MercadoPago. Galicia (ARS): extracto Excel CC o PDF Extracto_Cuentas_Galicia_… (fecha+débito/crédito+concepto; no duplica vs lo ya cargado si solo cambió el saldo) + tesorería tesoreria_transferencia_galicia (Tipo/Fecha/Crédito/Débito e Id; no se confunde con el extracto). Galicia (USD): extracto Excel Extracto_CCE… o el mismo PDF Extracto_Cuentas_Galicia_… de Cuenta Corriente Especial en dólares (se detecta por el título; no se mezcla con ARS) y tesorería tesoreria_transferencia_galicia_dolar_… o cierre_CIERRE-… / cierre_DOL-… con Caja = Transferencia Galicia Dolar y Moneda USD; los importes se concilian en USD y el saldo de corte se pesifica al MEP en Saldos extractos. En un PDF Galicia nuevo el corte = último corte + movimientos del Excel; el PDF no da de alta movimientos (solo verifica). Los cortes ya cargados no se recalculan. Filtros en modal: mes de extracto, mes de sistema, categoría, cuenta contable, importe exacto e ID exacto (opciones dinámicas; badge con cantidad activa); el buscar de la toolbar es texto libre (concepto, cliente, observaciones). Solapa Todos: extracto y tesorería juntos, con columna Dónde (Sugeridos, Confirmados, Solo banco, etc.; clic para ir). Las cards muestran cantidad y, debajo, la suma algebraica de importes del listado filtrado. Solapa Potenciales duplicados: tesorería con el mismo importe y hasta 40 días de diferencia (2 o más registros; el ojito muestra todos los datos de cada uno). Se puede descartar un grupo para que no vuelva a entrar (mismo conjunto de IDs; un movimiento nuevo sí lo muestra); Duplicados descartados permite deshacer. Mientras el grupo sigue en Potenciales duplicados, el extracto no lo propone. El listado solo incluye tesorería sin conciliar: un movimiento ya confirmado no entra. Descartar no modifica ninguna conciliación ya hecha. Encabezados de tabla ordenan asc/desc. La app sugiere matches por mismo importe con tolerancia según el tamaño (centavos si el monto es chico; $1 / $10 / $100 si es más grande), el mismo día o hasta 4 días de diferencia. Al abrir la caja o cambiar de solapa se vuelven a armar esas parejas aunque Sugeridos esté vacía. Si coinciden monto y fecha exactos, el criterio se muestra en verde. y, si el monto se repite, por coincidencia de concepto en la descripción (IVA/IIBB/SIRTAC-SIRCREB, Ganancias, Ley 25.413, para no cruzar impuestos). SIRTAC/SIRCREB se trata como IIBB. Si el importe deja un solo candidato, igual se sugiere aunque el concepto impositivo no coincida. El usuario confirma o descarta. En Sugeridos, un check Confirmar todos los listados confirma las visibles (con filtros) de una vez. En Mercado Pago, los pares del extracto con la misma operación relacionada e importes opuestos (cobro/devolución, impuesto/anulación) van a la solapa Mercado Pago Anulados y no entran a la conciliación ni al match manual, porque no existen en tesorería. Se puede deshacer esa anulación: los dos movimientos vuelven al extracto y se pueden conciliar; abajo quedan para volver a anularlos (sql/supabase_cb_mp_anulacion_deshecha.sql). En Confirmados, botón de acción para deshacer (vuelve a Sugeridos). Conciliación manual: se eligen uno o más movimientos de extracto y uno o más de tesorería (clic para sumar o quitar; mismo modal de filtros (mes extracto/sistema, categoría, cuenta, importe exacto e ID exacto) y buscar por lado; si ya estaban activos en la vista, el modal los hereda; encabezados ordenan asc/desc; extracto muestra Contraparte y tesorería Descripción), o dos o más del mismo extracto sin tesorería (crédito y débito que se compensan, p. ej. transferencia por error y devolución). La diferencia es suma extracto − suma tesorería (aunque sea mayor a $1; si no hay tesorería, es la suma neta del extracto) y queda un solo confirmado (justificación, diferencia, usuario y fecha). En Sugeridos, Confirmados, Solo sistema y Conciliación manual (tesorería) hay columnas Observaciones, Categoría y Cuenta contable de tesorería; el extracto del modal muestra Contraparte y tesorería Descripción. En Confirmados se muestran el crédito y el débito (no la suma neta en cero). La conciliación manual de Impuestos deja el tesorería MP en Confirmados con criterio Conciliación manual de impuestos (sin líneas de extracto de retención). Ojito para ver el detalle de todos los movimientos del grupo. En Solo sistema, icono de papelera (permiso cargar_conciliacion_bancaria) para eliminar un movimiento de tesorería que no esté conciliado. En Solo banco (Galicia), la misma papelera elimina un movimiento del extracto que no esté conciliado. En Mercado Pago, Galicia (ARS) y Galicia (USD), Solo banco y Solo sistema permiten marcar No requiere conciliación de a uno, varios o todos los listados (una justificación para el lote; no se borra; solapa No requiere con origen Extracto o Tesorería; se puede deshacer). Botón Excel (verde) exporta el listado visible con los filtros activos (importes numéricos, fechas serial Argentina). El recálculo de sugerencias al cargar no corta por timeout: el solapamiento se chequea una vez por statement (un movimiento no puede estar en dos conciliaciones activas) y el recálculo omite pares ya confirmados, duplicados y con más de 4 días (sql/supabase_cb_reemplazar_sugerencias_filtra_confirmados.sql). Permisos cargar_conciliacion_bancaria y confirmar_conciliacion_bancaria. Componente: scripts/lib/fornitalia-conciliacion-bancaria.js + .css. SQL: sql/supabase_conciliacion_bancaria.sql, sql/supabase_conciliacion_bancaria_manual.sql, sql/supabase_conciliacion_bancaria_manual_grupo.sql, sql/supabase_cb_retirar_tesoreria_duplicada_por_cierre.sql, sql/supabase_cb_borrar_tesoreria_abierta_sin_id.sql, sql/supabase_cb_tesoreria_abierta_pendiente_baja.sql, sql/supabase_cb_upload_sin_timeout.sql, sql/supabase_cb_borrar_movimiento_banco_galicia.sql, sql/supabase_cb_retirar_extracto_banco_ausente.sql, sql/supabase_cb_retirar_solo_no_imputado.sql, sql/supabase_cb_confirmar_manual_solo_extracto.sql y sql/supabase_cb_mp_no_requiere_conciliacion.sql y sql/supabase_cb_mp_no_requiere_conciliacion_lote.sql y sql/supabase_cb_no_requiere_conciliacion_galicia.sql y sql/supabase_cb_no_requiere_conciliacion_sistema.sql y sql/supabase_cb_confirmar_sugeridos.sql y sql/supabase_cb_galicia_usd.sql y sql/supabase_cb_dup_tesoreria_descartar.sql y sql/supabase_cb_dup_tesoreria_descartar_lote.sql y sql/supabase_cb_tesoreria_eliminada.sql y sql/supabase_tesoreria_omitir_anulado.sql y sql/supabase_eb_guardar_saldos_regla_movimientos.sql. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros. Entrar o cambiar de solapa solo lee las sugerencias ya guardadas y no las vuelve a armar. Se rearman al cargar un archivo o con Recalcular, y esa escritura espera si otra persona está confirmando ese canal.</v>
       </c>
     </row>
     <row r="64">
@@ -9792,7 +9860,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C149"/>
+  <dimension ref="A1:C150"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11438,9 +11506,20 @@
         <v>Despliegue v2.105: en Flujo por mes, Ingresos c/f / Ingresos e Ingresos s/f / Ingresos usan solo cobranzas por ventas (subítem Cobranzas por Ventas o categoría Ventas). Entre los dos suman 100% de esas cobranzas. También en el Excel y el PDF. Producción Vercel.</v>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>2.106</v>
+      </c>
+      <c r="B150" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="C150" t="str">
+        <v>Despliegue v2.106: en Agenda de pagos un día de la semana en curso sigue aunque ya haya pasado. Si entró un pago de la misma categoría y cuenta, una fila queda Ya pagado con el importe real. En Conciliación, entrar o cambiar de solapa no rearma las sugerencias de quien ya está conciliando. sql/supabase_cb_sugerencias_concurrentes.sql. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C149"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C150"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11642,7 +11721,7 @@
         <v>Conciliación Bancaria</v>
       </c>
       <c r="B14" t="str">
-        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro, FCI Galicia ARS y USD en verde). FCI no tiene extracto propio: la tesorería se concilia contra el extracto de Galicia de la misma moneda. En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados; el listado solo mira tesorería sin conciliar y descartar no toca las conciliaciones ya hechas). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
+        <v>Módulo de conciliación extracto vs tesorería (Mercado Pago en azul de marca, Galicia ARS y USD en naranja, Credicoop en negro, FCI Galicia ARS y USD en verde). FCI no tiene extracto propio: la tesorería se concilia contra el extracto de Galicia de la misma moneda. En Galicia, un Imputado no se borra al recargar el extracto; solo se retira si al entrar no era Imputado. Filtros con importe exacto e ID exacto; el buscar queda libre para concepto, cliente y observaciones. Solapa Todos con columna Dónde. Uploads por ID sin duplicar (Galicia ARS: Excel CC o PDF Extracto_Cuentas_Galicia_… en pesos; Galicia USD: Excel Extracto_CCE… o el mismo PDF de Cuenta Corriente Especial en dólares, y tesorería tesoreria_transferencia_galicia_dolar / cierre_CIERRE o cierre_DOL con Caja Transferencia Galicia Dolar, importes en USD; Credicoop: tesorería tesoreria_transferencia_credicoop o histórico Caja Transferencia Credicoop). Cards con cantidad y suma algebraica del listado filtrado. Solapa Potenciales duplicados (mismo importe de tesorería y hasta 40 días; se descartan de a uno, varios o todos los listados para que no vuelvan a entrar, con deshacer en Duplicados descartados; el listado solo mira tesorería sin conciliar y descartar no toca las conciliaciones ya hechas). Sugerencias de match, conciliación manual N:M (varios extractos con una o más tesorerías, o dos o más movimientos del mismo extracto sin tesorería; en el modal el extracto muestra Contraparte y tesorería Descripción; en Confirmados se ven crédito y débito, no la suma neta) con justificación de diferencia, deshacer confirmados (vuelve a Sugeridos), orden de columnas, detalle con ojito, confirmación y export Excel del listado filtrado. Incluye el Excel de cierre de caja (cierre_CIERRE) y el histórico movimientos-historico_… como tesorería (Caja reparte canales; popup de resumen de carga). Si el Id ya existe se actualizan categoría y cuenta aunque el Excel traiga Pendiente. Al cargar tesorería o histórico, un Pendiente o un movimiento sin Status pasa a A eliminar solo si su fecha cae dentro del Excel y el Id no viene; si el archivo no cubre esa fecha, no se marca. Un Confirmado nunca. En Solo banco (Galicia) se puede eliminar un movimiento del extracto no conciliado. En Mercado Pago, Solo banco puede marcar No requiere conciliación (justificación; no se borra; solapa propia) y los pares autoanulados del extracto (misma operación relacionada e importes opuestos) se listan aparte y no se concilian. Permisos en Seguridad. Entrar a la pantalla no rearma las sugerencias de quien ya está conciliando. ID Venta e ID Compra del histórico se ven en la tabla y se filtran en Filtros.</v>
       </c>
       <c r="C14">
         <v>24</v>
@@ -11740,7 +11819,7 @@
         <v>Agenda de pagos</v>
       </c>
       <c r="B21" t="str">
-        <v>Solapa inicial de Flujo de caja: estimado de las próximas 4 semanas según los últimos 3 pagos del proveedor (el más reciente pesa más), por categoría y cuenta contable, sin impuestos de hasta $ 500.000 ni gastos bancarios. Sueldos y Jornales el día 1, cada 30 días, desde septiembre. Con lo ya pagado al mismo proveedor. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses, sin la cuenta Mercaderías.</v>
+        <v>Solapa inicial de Flujo de caja: estimado de 4 semanas desde el lunes en curso (un día de esta semana sigue aunque ya haya pasado; si hubo un pago de la misma categoría y cuenta, una fila pasa a Ya pagado con el importe real), según los últimos 3 pagos del proveedor (el más reciente pesa más), por categoría y cuenta contable, sin impuestos de hasta $ 500.000 ni gastos bancarios. Sueldos y Jornales el día 1, cada 30 días, desde septiembre. Con lo ya pagado al mismo proveedor. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses, sin la cuenta Mercaderías.</v>
       </c>
       <c r="C21">
         <v>8</v>

</xml_diff>

<commit_message>
v2.107: Flujo de caja ya no se corta cuando hay más pagos que filas.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E514"/>
+  <dimension ref="A1:E516"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -9149,9 +9149,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="515">
+      <c r="A515" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="B515" t="str">
+        <v>17:18</v>
+      </c>
+      <c r="C515" t="str">
+        <v>Flujo de caja: el error de fecha al marcar pagado</v>
+      </c>
+      <c r="D515" t="str">
+        <v>Si en la semana había más pagos que filas de la misma categoría y cuenta, Flujo de caja cortaba con «Cannot read properties of undefined (reading fecha)». Ahora se marcan las filas que hay, con el importe real, y los pagos de más no cortan el tablero.</v>
+      </c>
+      <c r="E515" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="B516" t="str">
+        <v>17:35</v>
+      </c>
+      <c r="C516" t="str">
+        <v>Despliegue v2.107 producción</v>
+      </c>
+      <c r="D516" t="str">
+        <v>Push a main y Vercel --prod: Flujo de caja deja de cortarse cuando en la semana hay más pagos que filas de la misma categoría y cuenta. Se marcan las filas que hay, con el importe real. APP_VERSION 2.107.</v>
+      </c>
+      <c r="E516" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E514"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E516"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9321,7 +9355,7 @@
         <v>Agenda de pagos</v>
       </c>
       <c r="B20" t="str">
-        <v>Primera solapa de Flujo de caja y vista al entrar, si el perfil la tiene. Estima egresos de las próximas 4 semanas con los últimos 3 meses. El importe sale de los últimos 3 pagos de ese proveedor y categoría, con más peso en el más reciente. Prioriza series con ID compra. También entran pagos frecuentes sin ID compra. Impuestos de hasta $ 500.000 y Gastos bancarios no entran. Cada serie se abre por categoría y cuenta contable. Sueldos y Jornales se estima el día 1, cada 30 días, con los pagos cargados desde septiembre de 2026. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses. La más pareja queda en 5% y la más variable en 30%. La cuenta Mercaderías no entra en esa dispersión. Barras por semana (ámbar por pagar, azul colchón, verde ya pagado) y total al pie de cada semana. Ya pagado: en esa semana ya hubo un egreso con ID compra al mismo proveedor, sin comparar el monto, y la fila sigue en la tabla. Sin ID compra, un pago de la misma categoría y cuenta contable toma una fila de esa semana, le pone el importe real y la deja en Ya pagado. Un día de la semana en curso no se saca porque ya pasó. No aplica a series sin ID compra. Permiso ver_solapa_agenda_pagos en Seguridad.</v>
+        <v>Primera solapa de Flujo de caja y vista al entrar, si el perfil la tiene. Estima egresos de las próximas 4 semanas con los últimos 3 meses. El importe sale de los últimos 3 pagos de ese proveedor y categoría, con más peso en el más reciente. Prioriza series con ID compra. También entran pagos frecuentes sin ID compra. Impuestos de hasta $ 500.000 y Gastos bancarios no entran. Cada serie se abre por categoría y cuenta contable. Sueldos y Jornales se estima el día 1, cada 30 días, con los pagos cargados desde septiembre de 2026. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses. La más pareja queda en 5% y la más variable en 30%. La cuenta Mercaderías no entra en esa dispersión. Barras por semana (ámbar por pagar, azul colchón, verde ya pagado) y total al pie de cada semana. Ya pagado: en esa semana ya hubo un egreso con ID compra al mismo proveedor, sin comparar el monto, y la fila sigue en la tabla. Sin ID compra, un pago de la misma categoría y cuenta contable toma una fila de esa semana, le pone el importe real y la deja en Ya pagado. Si hay más pagos que filas, se marcan las que hay y el tablero sigue. Un día de la semana en curso no se saca porque ya pasó. Permiso ver_solapa_agenda_pagos en Seguridad.</v>
       </c>
     </row>
     <row r="21">
@@ -9860,7 +9894,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C150"/>
+  <dimension ref="A1:C151"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11517,9 +11551,20 @@
         <v>Despliegue v2.106: en Agenda de pagos un día de la semana en curso sigue aunque ya haya pasado. Si entró un pago de la misma categoría y cuenta, una fila queda Ya pagado con el importe real. En Conciliación, entrar o cambiar de solapa no rearma las sugerencias de quien ya está conciliando. sql/supabase_cb_sugerencias_concurrentes.sql. Producción Vercel.</v>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>2.107</v>
+      </c>
+      <c r="B151" t="str">
+        <v>27/10/2026</v>
+      </c>
+      <c r="C151" t="str">
+        <v>Despliegue v2.107: Flujo de caja deja de mostrar el error al abrir cuando en la semana hay más pagos que filas de la misma categoría y cuenta. Se marcan las filas que hay, con el importe real, y el tablero sigue. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C150"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C151"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
v2.108: los importes en millones muestran un decimal.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E516"/>
+  <dimension ref="A1:E518"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -9183,9 +9183,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="517">
+      <c r="A517" t="str">
+        <v>28/10/2026</v>
+      </c>
+      <c r="B517" t="str">
+        <v>14:34</v>
+      </c>
+      <c r="C517" t="str">
+        <v>Millones con un decimal</v>
+      </c>
+      <c r="D517" t="str">
+        <v>Todo importe en millones muestra un decimal: la torta de posición, su total, el PDF y las etiquetas del gráfico G/P. $ 200.423.092 se ve como 200,4 M, no como 200 M. En dólares la torta sigue en miles.</v>
+      </c>
+      <c r="E517" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="str">
+        <v>28/10/2026</v>
+      </c>
+      <c r="B518" t="str">
+        <v>17:19</v>
+      </c>
+      <c r="C518" t="str">
+        <v>Despliegue v2.108 producción</v>
+      </c>
+      <c r="D518" t="str">
+        <v>Push a main y Vercel --prod: todo importe en millones muestra un decimal. En la posición de caja, $ 200.423.092 se ve como 200,4 M. También el total, el gráfico de G/P y el PDF. APP_VERSION 2.108.</v>
+      </c>
+      <c r="E518" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E516"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E518"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9211,7 +9245,7 @@
         <v>Flujo de caja por mes</v>
       </c>
       <c r="B2" t="str">
-        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas); Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. Ingresos c/f / Ingresos e Ingresos s/f / Ingresos parten solo las cobranzas por ventas (subítem Cobranzas por Ventas, o categoría Ventas): c/f es Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop; s/f es el resto de esas cobranzas. Los dos suman 100% de esas cobranzas. La columna Total (Ingresos, Egresos, G/P y ratios) suma meses cerrados y va después de esos meses: el mes en curso se marca en celeste y no entra al Total, ni a las variaciones y la tendencia del gráfico, ni a la base de la proyección. Sobre esa barra se ve el G/P del mes en millones. Las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
+        <v>Vista tipo Dashboard: filtro Período (último año por defecto, un año o todo el histórico), gráfico G/P Mensual (barras + tendencia vs mes anterior) y tabla con meses en columnas, filas Ingresos / Egresos / G/P y debajo Ratios del Negocio. Alimentada por tesorería (cb_movimiento origen=sistema + cf_movimiento) unida a la Matriz EF. Incluye Status Pendiente. Botón Cargar tesorería histórica: el Excel movimientos-historico_… se reparte a todas las cajas. Ratios: Comisiones/Ventas % por subítems EF; Sueldos / Ingresos; Sueldos + Cargas Sociales / Cobranzas (Sueldos Neto/Bolsillo + Cargas Sociales ÷ Cobranzas por Ventas); Costo Financiero MP / Ventas MP (solo caja Mercado Pago); Costo dir./Ingresos = §2 ÷ Ingresos; Costo ind./Ingresos = §3 ÷ Ingresos; Costo total/Ingreso total = Egresos ÷ Ingresos. Ingresos c/f / Ingresos e Ingresos s/f / Ingresos parten solo las cobranzas por ventas (subítem Cobranzas por Ventas, o categoría Ventas): c/f es Efectivo Pesos, Efectivo Dólar, Mercado Pago, Transferencia Galicia, Transferencia Galicia Dólar y Transferencia Credicoop; s/f es el resto de esas cobranzas. Los dos suman 100% de esas cobranzas. La columna Total (Ingresos, Egresos, G/P y ratios) suma meses cerrados y va después de esos meses: el mes en curso se marca en celeste y no entra al Total, ni a las variaciones y la tendencia del gráfico, ni a la base de la proyección. Sobre esa barra se ve el G/P del mes en millones, con un decimal. Las columnas Proy. quedan a la derecha y no entran al Total. Meses excluidos por Configuración no aparecen. Clic en un mes (encabezado o importe) abre el detalle. PDF de una sola página (A4 apaisado) con filtros activos remarcados; gráfico de margen a margen (sangría chica) y columnas de la tabla ajustadas al contenido. Exportar Flujo a Excel (importes numéricos, % como fracción).</v>
       </c>
     </row>
     <row r="3">
@@ -9219,7 +9253,7 @@
         <v>Resumen global</v>
       </c>
       <c r="B3" t="str">
-        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, FCI, Efectivo y Resto) en millones y porcentaje; el subtítulo incluye el total y la cotización. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable y se ve en el subtítulo de la torta. La torta, en dólares, muestra miles. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
+        <v>Tres tarjetas al ancho del número: Ingresos totales, Egresos totales y G/P operativo (misma base que la columna Total del Flujo: meses cerrados del período, sin el mes en curso), en ARS o USD según selector. A la derecha, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, FCI, Efectivo y Resto) en millones con un decimal (200,4 M) y porcentaje; el subtítulo incluye el total y la cotización. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable y se ve en el subtítulo de la torta. La torta, en dólares, muestra miles. Las solapas quedan al borde inferior de la torta. El PDF de Flujo incluye esa torta.</v>
       </c>
     </row>
     <row r="4">
@@ -9894,7 +9928,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C151"/>
+  <dimension ref="A1:C152"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11562,9 +11596,20 @@
         <v>Despliegue v2.107: Flujo de caja deja de mostrar el error al abrir cuando en la semana hay más pagos que filas de la misma categoría y cuenta. Se marcan las filas que hay, con el importe real, y el tablero sigue. Producción Vercel.</v>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>2.108</v>
+      </c>
+      <c r="B152" t="str">
+        <v>28/10/2026</v>
+      </c>
+      <c r="C152" t="str">
+        <v>Despliegue v2.108: todo importe en millones muestra un decimal. En la posición de caja, $ 200.423.092 se ve como 200,4 M. Lo mismo en el total, en el gráfico de G/P y en el PDF. En dólares la torta sigue en miles. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C151"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C152"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11612,7 +11657,7 @@
         <v>Dashboard flujo de caja</v>
       </c>
       <c r="B3" t="str">
-        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, FCI, Efectivo y Resto) en millones y porcentaje, con el total y la cotización en el subtítulo. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable. La torta, en dólares, muestra miles. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
+        <v>Diseño y desarrollo del dashboard mensual (filtro Período, gráfico G/P Mensual, tabla con meses en columnas, Resumen, Ratios del Negocio incluyendo Sueldos/Ingresos, Sueldos + Cargas Sociales/Cobranzas y Costo Financiero MP/Ventas MP, alertas, modal By Categoría / By Cuenta). A la derecha de las tarjetas, torta de la posición de caja de hoy (Galicia, Mercado Pago, Credicoop, FCI, Efectivo y Resto) en millones con un decimal (200,4 M) y porcentaje, con el total y la cotización en el subtítulo. En pesos, los dólares de la torta se pesifican con la cotización de hoy del dólar elegido (o la inmediata anterior). Con USD, la torta, el gráfico G/P y la tabla usan esa misma cotización: los pesos se dividen por ella y lo que ya está en dólares no se vuelve a convertir. La cotización se lee de la tabla global de Sistema Contable. La torta, en dólares, muestra miles. Incluye PDF de una página con filtros activos, esa torta y formatos de moneda.</v>
       </c>
       <c r="C3">
         <v>25</v>

</xml_diff>

<commit_message>
v2.109: la agenda incluye comisiones de fin de mes y descuenta el pago adelantado.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E518"/>
+  <dimension ref="A1:E521"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -9217,9 +9217,60 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="519">
+      <c r="A519" t="str">
+        <v>29/10/2026</v>
+      </c>
+      <c r="B519" t="str">
+        <v>09:33</v>
+      </c>
+      <c r="C519" t="str">
+        <v>Costeo hornos de banda ARG</v>
+      </c>
+      <c r="D519" t="str">
+        <v>docs/Costeo_Hornos_de_Banda_ARG_2026.xlsx. Solo la solapa ARG del costeo original, con controles para tipo de cambio, múltiplo, costo de importación, comisión, impuesto a las ganancias y gastos indirectos. La flecha mueve la variable y, si se escribe un valor exacto, ese número manda. Precio, comisión, impuesto y utilidad se recalculan en los seis modelos. Con los valores de origen los importes coinciden con el archivo original.</v>
+      </c>
+      <c r="E519" t="str">
+        <v>Entregable</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="str">
+        <v>29/10/2026</v>
+      </c>
+      <c r="B520" t="str">
+        <v>19:03</v>
+      </c>
+      <c r="C520" t="str">
+        <v>Agenda de pagos: comisiones y pago adelantado</v>
+      </c>
+      <c r="D520" t="str">
+        <v>Comisiones de venta se proyectan en la última semana del mes. Si esa semana ya se pagaron, la fila queda Ya pagado con la suma real. Si un gasto entra antes de la semana prevista, se agrega Ya pagado esa semana con el importe real y se descuenta de la proyección siguiente. Vale para sueldos y para el resto de los gastos.</v>
+      </c>
+      <c r="E520" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="str">
+        <v>30/10/2026</v>
+      </c>
+      <c r="B521" t="str">
+        <v>07:27</v>
+      </c>
+      <c r="C521" t="str">
+        <v>Despliegue v2.109 producción</v>
+      </c>
+      <c r="D521" t="str">
+        <v>Push a main y Vercel --prod: en Agenda de pagos las comisiones de venta caen en la última semana del mes. Si ya se pagaron, la fila queda Ya pagado con el importe real. Un gasto que entra antes de lo previsto se ve pagado esa semana y se descuenta de la proyección siguiente. APP_VERSION 2.109.</v>
+      </c>
+      <c r="E521" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E518"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E521"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9389,7 +9440,7 @@
         <v>Agenda de pagos</v>
       </c>
       <c r="B20" t="str">
-        <v>Primera solapa de Flujo de caja y vista al entrar, si el perfil la tiene. Estima egresos de las próximas 4 semanas con los últimos 3 meses. El importe sale de los últimos 3 pagos de ese proveedor y categoría, con más peso en el más reciente. Prioriza series con ID compra. También entran pagos frecuentes sin ID compra. Impuestos de hasta $ 500.000 y Gastos bancarios no entran. Cada serie se abre por categoría y cuenta contable. Sueldos y Jornales se estima el día 1, cada 30 días, con los pagos cargados desde septiembre de 2026. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses. La más pareja queda en 5% y la más variable en 30%. La cuenta Mercaderías no entra en esa dispersión. Barras por semana (ámbar por pagar, azul colchón, verde ya pagado) y total al pie de cada semana. Ya pagado: en esa semana ya hubo un egreso con ID compra al mismo proveedor, sin comparar el monto, y la fila sigue en la tabla. Sin ID compra, un pago de la misma categoría y cuenta contable toma una fila de esa semana, le pone el importe real y la deja en Ya pagado. Si hay más pagos que filas, se marcan las que hay y el tablero sigue. Un día de la semana en curso no se saca porque ya pasó. Permiso ver_solapa_agenda_pagos en Seguridad.</v>
+        <v>Primera solapa de Flujo de caja y vista al entrar, si el perfil la tiene. Estima egresos de las próximas 4 semanas con los últimos 3 meses. El importe sale de los últimos 3 pagos de ese proveedor y categoría, con más peso en el más reciente. Prioriza series con ID compra. También entran pagos frecuentes sin ID compra. Impuestos de hasta $ 500.000 y Gastos bancarios no entran. Cada serie se abre por categoría y cuenta contable. Sueldos y Jornales se estima el día 1, cada 30 días, con los pagos cargados desde septiembre de 2026. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses. La más pareja queda en 5% y la más variable en 30%. La cuenta Mercaderías no entra en esa dispersión. Barras por semana (ámbar por pagar, azul colchón, verde ya pagado) y total al pie de cada semana. Ya pagado: en esa semana ya hubo un egreso con ID compra al mismo proveedor, sin comparar el monto, y la fila sigue en la tabla. Sin ID compra, un pago de la misma categoría y cuenta contable toma una fila de esa semana, le pone el importe real y la deja en Ya pagado. Si hay más pagos que filas, se marcan las que hay y el tablero sigue. Un día de la semana en curso no se saca porque ya pasó. Comisiones de venta se proyectan en la última semana del mes; si esa semana ya se pagaron, la fila queda Ya pagado con la suma real. Si un gasto entra antes de la semana prevista, se agrega Ya pagado esa semana con el importe real y se descuenta de la proyección siguiente. Permiso ver_solapa_agenda_pagos en Seguridad.</v>
       </c>
     </row>
     <row r="21">
@@ -9928,7 +9979,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C152"/>
+  <dimension ref="A1:C153"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11607,9 +11658,20 @@
         <v>Despliegue v2.108: todo importe en millones muestra un decimal. En la posición de caja, $ 200.423.092 se ve como 200,4 M. Lo mismo en el total, en el gráfico de G/P y en el PDF. En dólares la torta sigue en miles. Producción Vercel.</v>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>2.109</v>
+      </c>
+      <c r="B153" t="str">
+        <v>30/10/2026</v>
+      </c>
+      <c r="C153" t="str">
+        <v>Despliegue v2.109: en Agenda de pagos las comisiones de venta caen en la última semana del mes. Si ya se pagaron, la fila queda Ya pagado con el importe real. Un gasto que entra antes de lo previsto se ve pagado esa semana y se descuenta de la proyección siguiente. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C152"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C153"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -11909,7 +11971,7 @@
         <v>Agenda de pagos</v>
       </c>
       <c r="B21" t="str">
-        <v>Solapa inicial de Flujo de caja: estimado de 4 semanas desde el lunes en curso (un día de esta semana sigue aunque ya haya pasado; si hubo un pago de la misma categoría y cuenta, una fila pasa a Ya pagado con el importe real), según los últimos 3 pagos del proveedor (el más reciente pesa más), por categoría y cuenta contable, sin impuestos de hasta $ 500.000 ni gastos bancarios. Sueldos y Jornales el día 1, cada 30 días, desde septiembre. Con lo ya pagado al mismo proveedor. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses, sin la cuenta Mercaderías.</v>
+        <v>Solapa inicial de Flujo de caja: estimado de 4 semanas desde el lunes en curso (un día de esta semana sigue aunque ya haya pasado; si hubo un pago de la misma categoría y cuenta, una fila pasa a Ya pagado con el importe real), según los últimos 3 pagos del proveedor (el más reciente pesa más), por categoría y cuenta contable, sin impuestos de hasta $ 500.000 ni gastos bancarios. Sueldos y Jornales el día 1, cada 30 días, desde septiembre. Comisiones de venta en la última semana del mes. Si un gasto entra antes de lo previsto, queda pagado esa semana con el importe real y se descuenta de la proyección siguiente. Con lo ya pagado al mismo proveedor. Cada semana suma un colchón de entre 5% y 30% del estimado, según la dispersión de esa semana del mes en los últimos 6 meses, sin la cuenta Mercaderías.</v>
       </c>
       <c r="C21">
         <v>8</v>

</xml_diff>

<commit_message>
v2.110: el Estado Financiero cierra como el de la empresa.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Bitacora_tareas.xlsx
+++ b/Bitacora_tareas.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E521"/>
+  <dimension ref="A1:E523"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -9268,9 +9268,43 @@
         <v>Despliegue</v>
       </c>
     </row>
+    <row r="522">
+      <c r="A522" t="str">
+        <v>30/10/2026</v>
+      </c>
+      <c r="B522" t="str">
+        <v>10:43</v>
+      </c>
+      <c r="C522" t="str">
+        <v>Estado Financiero alineado al de la empresa</v>
+      </c>
+      <c r="D522" t="str">
+        <v>El margen bruto incluye el ajuste de saldos de caja. El flujo de caja neto del período suma los intereses del FCI, además de la financiación. El detalle de cada total lista las mismas partidas que la fórmula, así la suma cierra con la celda.</v>
+      </c>
+      <c r="E522" t="str">
+        <v>Ajuste</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="str">
+        <v>30/10/2026</v>
+      </c>
+      <c r="B523" t="str">
+        <v>10:48</v>
+      </c>
+      <c r="C523" t="str">
+        <v>Despliegue v2.110 producción</v>
+      </c>
+      <c r="D523" t="str">
+        <v>Push a main y Vercel --prod: en el Estado Financiero el margen bruto incluye el ajuste de caja y el flujo de caja neto del período suma los intereses del FCI. En octubre ese total queda en línea con el resultado de la empresa. El detalle de cada total cierra con la celda. APP_VERSION 2.110.</v>
+      </c>
+      <c r="E523" t="str">
+        <v>Despliegue</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E521"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E523"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9624,7 +9658,7 @@
         <v>Estado Financiero (tabla dinámica)</v>
       </c>
       <c r="B43" t="str">
-        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). AJUSTE DE SALDOS (CAJA) va debajo de FLUJO OPERATIVO GENERADO y entra en (=) FLUJO DE CAJA NETO DEL PERÍODO (D), no en A–C. En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Antes de Total, Avg Mensual es el promedio de los últimos 12 meses cerrados móviles (el mes en curso no entra; un mes sin movimientos cuenta como cero). Gráficos y export Excel. Conciliación §7 oculta.</v>
+        <v>Solapa Estado Financiero: estructura desde Supabase ef_estructura (ABM en Matriz EF → Estructura EF). Montos desde tesorería por ef_subitem (matriz categoría + cuenta; Ingreso y Egreso del mismo par pegan en la misma línea). El margen bruto incluye el ajuste de saldos de caja. El flujo de caja neto del período suma la financiación completa, intereses del FCI incluidos. El detalle de cada total cierra con la celda. En ARS, USD × MEP de la fecha. Clic en importe: detalle con Observaciones e Ids. Antes de Total, Avg Mensual es el promedio de los últimos 12 meses cerrados móviles (el mes en curso no entra; un mes sin movimientos cuenta como cero). Gráficos y export Excel. Conciliación §7 oculta.</v>
       </c>
     </row>
     <row r="44">
@@ -9979,7 +10013,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C153"/>
+  <dimension ref="A1:C154"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -11669,9 +11703,20 @@
         <v>Despliegue v2.109: en Agenda de pagos las comisiones de venta caen en la última semana del mes. Si ya se pagaron, la fila queda Ya pagado con el importe real. Un gasto que entra antes de lo previsto se ve pagado esa semana y se descuenta de la proyección siguiente. Producción Vercel.</v>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>2.110</v>
+      </c>
+      <c r="B154" t="str">
+        <v>30/10/2026</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Despliegue v2.110: en el Estado Financiero el margen bruto incluye el ajuste de caja y el flujo de caja neto del período suma los intereses del FCI. En octubre ese total queda en línea con el resultado de la empresa. El detalle de cada total cierra con la celda. Producción Vercel.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C153"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C154"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>